<commit_message>
Resolve Day 2 pending items
Confirmed with the user:

- 70g chocolate bar was not eaten (had whey with water instead). Row
  removed from meals.csv rather than left pending.
- Pre-workout not taken as of the last check. Stays pending, so it still
  counts toward no total.

Day 2 totals are unchanged, since neither item was ever counted. Added the
dinner headroom read now that the bar is off the table.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1091,39 +1091,39 @@
       </c>
       <c r="B14" s="12" t="inlineStr">
         <is>
-          <t>Snack</t>
+          <t>Supplement</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
         <is>
-          <t>Chocolate bar 70g (2 x 35g king-size)</t>
+          <t>Pre-workout scoop</t>
         </is>
       </c>
       <c r="D14" s="14" t="n">
-        <v>335</v>
+        <v>5</v>
       </c>
       <c r="E14" s="14" t="n">
-        <v>335</v>
+        <v>15</v>
       </c>
       <c r="F14" s="15">
         <f>AVERAGE(D14:E14)</f>
         <v/>
       </c>
       <c r="G14" s="16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H14" s="16" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I14" s="17">
         <f>AVERAGE(G14:H14)</f>
         <v/>
       </c>
       <c r="J14" s="16" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="K14" s="16" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="L14" s="17">
         <f>AVERAGE(J14:K14)</f>
@@ -1136,62 +1136,7 @@
       </c>
       <c r="N14" s="13" t="inlineStr">
         <is>
-          <t>UNCONFIRMED - asked about it then had whey with water instead; ~36 g sugar</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="11" t="n">
-        <v>46270</v>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>Supplement</t>
-        </is>
-      </c>
-      <c r="C15" s="13" t="inlineStr">
-        <is>
-          <t>Pre-workout scoop</t>
-        </is>
-      </c>
-      <c r="D15" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="E15" s="14" t="n">
-        <v>15</v>
-      </c>
-      <c r="F15" s="15">
-        <f>AVERAGE(D15:E15)</f>
-        <v/>
-      </c>
-      <c r="G15" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="17">
-        <f>AVERAGE(G15:H15)</f>
-        <v/>
-      </c>
-      <c r="J15" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" s="17">
-        <f>AVERAGE(J15:K15)</f>
-        <v/>
-      </c>
-      <c r="M15" s="12" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="N15" s="13" t="inlineStr">
-        <is>
-          <t>UNCONFIRMED - planned only; no label seen</t>
+          <t>Planned but not taken as of last check - confirm before logging</t>
         </is>
       </c>
     </row>
@@ -1307,11 +1252,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$15,Meals!$A$5:$A$15,$A5,Meals!$M$5:$M$15,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$14,Meals!$A$5:$A$14,$A5,Meals!$M$5:$M$14,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$15,Meals!$A$5:$A$15,$A5,Meals!$M$5:$M$15,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$14,Meals!$A$5:$A$14,$A5,Meals!$M$5:$M$14,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -1319,11 +1264,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$15,Meals!$A$5:$A$15,$A5,Meals!$M$5:$M$15,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$14,Meals!$A$5:$A$14,$A5,Meals!$M$5:$M$14,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$15,Meals!$A$5:$A$15,$A5,Meals!$M$5:$M$15,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$14,Meals!$A$5:$A$14,$A5,Meals!$M$5:$M$14,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -1331,11 +1276,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$15,Meals!$A$5:$A$15,$A5,Meals!$M$5:$M$15,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$14,Meals!$A$5:$A$14,$A5,Meals!$M$5:$M$14,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$15,Meals!$A$5:$A$15,$A5,Meals!$M$5:$M$15,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$14,Meals!$A$5:$A$14,$A5,Meals!$M$5:$M$14,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -1343,11 +1288,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$15,$A5,Meals!$M$5:$M$15,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$14,$A5,Meals!$M$5:$M$14,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$15,$A5,Meals!$M$5:$M$15,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$14,$A5,Meals!$M$5:$M$14,"pending")</f>
         <v/>
       </c>
     </row>
@@ -1356,11 +1301,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="20">
-        <f>SUMIFS(Meals!$D$5:$D$15,Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$14,Meals!$A$5:$A$14,$A6,Meals!$M$5:$M$14,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="20">
-        <f>SUMIFS(Meals!$E$5:$E$15,Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$14,Meals!$A$5:$A$14,$A6,Meals!$M$5:$M$14,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="20">
@@ -1368,11 +1313,11 @@
         <v/>
       </c>
       <c r="E6" s="21">
-        <f>SUMIFS(Meals!$G$5:$G$15,Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$14,Meals!$A$5:$A$14,$A6,Meals!$M$5:$M$14,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="21">
-        <f>SUMIFS(Meals!$H$5:$H$15,Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$14,Meals!$A$5:$A$14,$A6,Meals!$M$5:$M$14,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="21">
@@ -1380,11 +1325,11 @@
         <v/>
       </c>
       <c r="H6" s="21">
-        <f>SUMIFS(Meals!$J$5:$J$15,Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$14,Meals!$A$5:$A$14,$A6,Meals!$M$5:$M$14,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="21">
-        <f>SUMIFS(Meals!$K$5:$K$15,Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$14,Meals!$A$5:$A$14,$A6,Meals!$M$5:$M$14,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="21">
@@ -1392,11 +1337,11 @@
         <v/>
       </c>
       <c r="K6" s="19">
-        <f>COUNTIFS(Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$14,$A6,Meals!$M$5:$M$14,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="19">
-        <f>COUNTIFS(Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$14,$A6,Meals!$M$5:$M$14,"pending")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Log 3 uzhunnu vada with coconut chutney on Day 2
Adds the meal at 480-650 kcal, 11.5-17 g protein, 29-40 g fat, and a
reference row for uzhunnu vada (130-180 kcal each) so it is costed the
same way next time.

Day 2 now totals 1,680-2,260 kcal (mid 1,970), overtaking Day 1's 1,808
midpoint, with fat at 78 g against Day 1's 67.5 g.

Also stops verify_tracker.py carrying a date past the end of its own Day
section, so tables under a later heading can never be read as that day's
totals.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1086,55 +1086,110 @@
       <c r="N13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="n">
+      <c r="A14" s="4" t="n">
         <v>46270</v>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>3 uzhunnu vada + coconut chutney</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>480</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>650</v>
+      </c>
+      <c r="F14" s="8">
+        <f>AVERAGE(D14:E14)</f>
+        <v/>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H14" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="I14" s="10">
+        <f>AVERAGE(G14:H14)</f>
+        <v/>
+      </c>
+      <c r="J14" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="K14" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="L14" s="10">
+        <f>AVERAGE(J14:K14)</f>
+        <v/>
+      </c>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N14" s="6" t="inlineStr">
+        <is>
+          <t>Coconut chutney included this time (skipped at breakfast both days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>Supplement</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="C15" s="13" t="inlineStr">
         <is>
           <t>Pre-workout scoop</t>
         </is>
       </c>
-      <c r="D14" s="14" t="n">
+      <c r="D15" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="E14" s="14" t="n">
+      <c r="E15" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="F14" s="15">
-        <f>AVERAGE(D14:E14)</f>
-        <v/>
-      </c>
-      <c r="G14" s="16" t="n">
+      <c r="F15" s="15">
+        <f>AVERAGE(D15:E15)</f>
+        <v/>
+      </c>
+      <c r="G15" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="H14" s="16" t="n">
+      <c r="H15" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="I14" s="17">
-        <f>AVERAGE(G14:H14)</f>
-        <v/>
-      </c>
-      <c r="J14" s="16" t="n">
+      <c r="I15" s="17">
+        <f>AVERAGE(G15:H15)</f>
+        <v/>
+      </c>
+      <c r="J15" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="K14" s="16" t="n">
+      <c r="K15" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="L14" s="17">
-        <f>AVERAGE(J14:K14)</f>
-        <v/>
-      </c>
-      <c r="M14" s="12" t="inlineStr">
+      <c r="L15" s="17">
+        <f>AVERAGE(J15:K15)</f>
+        <v/>
+      </c>
+      <c r="M15" s="12" t="inlineStr">
         <is>
           <t>pending</t>
         </is>
       </c>
-      <c r="N14" s="13" t="inlineStr">
+      <c r="N15" s="13" t="inlineStr">
         <is>
           <t>Planned but not taken as of last check - confirm before logging</t>
         </is>
@@ -1252,11 +1307,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$14,Meals!$A$5:$A$14,$A5,Meals!$M$5:$M$14,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$15,Meals!$A$5:$A$15,$A5,Meals!$M$5:$M$15,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$14,Meals!$A$5:$A$14,$A5,Meals!$M$5:$M$14,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$15,Meals!$A$5:$A$15,$A5,Meals!$M$5:$M$15,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -1264,11 +1319,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$14,Meals!$A$5:$A$14,$A5,Meals!$M$5:$M$14,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$15,Meals!$A$5:$A$15,$A5,Meals!$M$5:$M$15,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$14,Meals!$A$5:$A$14,$A5,Meals!$M$5:$M$14,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$15,Meals!$A$5:$A$15,$A5,Meals!$M$5:$M$15,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -1276,11 +1331,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$14,Meals!$A$5:$A$14,$A5,Meals!$M$5:$M$14,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$15,Meals!$A$5:$A$15,$A5,Meals!$M$5:$M$15,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$14,Meals!$A$5:$A$14,$A5,Meals!$M$5:$M$14,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$15,Meals!$A$5:$A$15,$A5,Meals!$M$5:$M$15,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -1288,11 +1343,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$14,$A5,Meals!$M$5:$M$14,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$15,$A5,Meals!$M$5:$M$15,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$14,$A5,Meals!$M$5:$M$14,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$15,$A5,Meals!$M$5:$M$15,"pending")</f>
         <v/>
       </c>
     </row>
@@ -1301,11 +1356,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="20">
-        <f>SUMIFS(Meals!$D$5:$D$14,Meals!$A$5:$A$14,$A6,Meals!$M$5:$M$14,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$15,Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="20">
-        <f>SUMIFS(Meals!$E$5:$E$14,Meals!$A$5:$A$14,$A6,Meals!$M$5:$M$14,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$15,Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="20">
@@ -1313,11 +1368,11 @@
         <v/>
       </c>
       <c r="E6" s="21">
-        <f>SUMIFS(Meals!$G$5:$G$14,Meals!$A$5:$A$14,$A6,Meals!$M$5:$M$14,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$15,Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="21">
-        <f>SUMIFS(Meals!$H$5:$H$14,Meals!$A$5:$A$14,$A6,Meals!$M$5:$M$14,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$15,Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="21">
@@ -1325,11 +1380,11 @@
         <v/>
       </c>
       <c r="H6" s="21">
-        <f>SUMIFS(Meals!$J$5:$J$14,Meals!$A$5:$A$14,$A6,Meals!$M$5:$M$14,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$15,Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="21">
-        <f>SUMIFS(Meals!$K$5:$K$14,Meals!$A$5:$A$14,$A6,Meals!$M$5:$M$14,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$15,Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="21">
@@ -1337,11 +1392,11 @@
         <v/>
       </c>
       <c r="K6" s="19">
-        <f>COUNTIFS(Meals!$A$5:$A$14,$A6,Meals!$M$5:$M$14,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="19">
-        <f>COUNTIFS(Meals!$A$5:$A$14,$A6,Meals!$M$5:$M$14,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"pending")</f>
         <v/>
       </c>
     </row>
@@ -1626,7 +1681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1894,14 +1949,14 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Kadala curry (1 container)</t>
+          <t>Uzhunnu vada / medu vada (1)</t>
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>200</v>
+        <v>130</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>300</v>
+        <v>180</v>
       </c>
       <c r="D13" s="8">
         <f>AVERAGE(B13:C13)</f>
@@ -1909,22 +1964,26 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>~8-10 g</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr"/>
+          <t>~3.5-5 g each</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>Deep-fried urad dal - protein-bearing but fat-dense</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Fish fry (1 piece pan-fried)</t>
+          <t>Kadala curry (1 container)</t>
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>220</v>
+        <v>300</v>
       </c>
       <c r="D14" s="8">
         <f>AVERAGE(B14:C14)</f>
@@ -1932,7 +1991,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>~15-20 g</t>
+          <t>~8-10 g</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr"/>
@@ -1940,14 +1999,14 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Barik/basmati rice (half container cooked)</t>
+          <t>Fish fry (1 piece pan-fried)</t>
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="C15" s="7" t="n">
-        <v>280</v>
+        <v>220</v>
       </c>
       <c r="D15" s="8">
         <f>AVERAGE(B15:C15)</f>
@@ -1955,7 +2014,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>~4-5 g</t>
+          <t>~15-20 g</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr"/>
@@ -1963,14 +2022,14 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in water)</t>
+          <t>Barik/basmati rice (half container cooked)</t>
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>120</v>
+        <v>280</v>
       </c>
       <c r="D16" s="8">
         <f>AVERAGE(B16:C16)</f>
@@ -1978,7 +2037,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
+          <t>~4-5 g</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr"/>
@@ -1986,14 +2045,14 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in black coffee no sugar)</t>
+          <t>Whey scoop (in water)</t>
         </is>
       </c>
       <c r="B17" s="7" t="n">
         <v>100</v>
       </c>
       <c r="C17" s="7" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="D17" s="8">
         <f>AVERAGE(B17:C17)</f>
@@ -2009,14 +2068,14 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Cashew/almond biscuit (1)</t>
+          <t>Whey scoop (in black coffee no sugar)</t>
         </is>
       </c>
       <c r="B18" s="7" t="n">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>38</v>
+        <v>130</v>
       </c>
       <c r="D18" s="8">
         <f>AVERAGE(B18:C18)</f>
@@ -2024,7 +2083,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>~0.5 g</t>
+          <t>~20-25 g</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr"/>
@@ -2032,14 +2091,14 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (~50g standard)</t>
+          <t>Cashew/almond biscuit (1)</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>245</v>
+        <v>38</v>
       </c>
       <c r="C19" s="7" t="n">
-        <v>250</v>
+        <v>38</v>
       </c>
       <c r="D19" s="8">
         <f>AVERAGE(B19:C19)</f>
@@ -2047,7 +2106,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>~4 g</t>
+          <t>~0.5 g</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr"/>
@@ -2055,14 +2114,14 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (70g king-size)</t>
+          <t>Chocolate bar (~50g standard)</t>
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>335</v>
+        <v>245</v>
       </c>
       <c r="C20" s="7" t="n">
-        <v>335</v>
+        <v>250</v>
       </c>
       <c r="D20" s="8">
         <f>AVERAGE(B20:C20)</f>
@@ -2070,7 +2129,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>~6 g</t>
+          <t>~4 g</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr"/>
@@ -2078,14 +2137,14 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Pre-workout scoop</t>
+          <t>Chocolate bar (70g king-size)</t>
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>5</v>
+        <v>335</v>
       </c>
       <c r="C21" s="7" t="n">
-        <v>15</v>
+        <v>335</v>
       </c>
       <c r="D21" s="8">
         <f>AVERAGE(B21:C21)</f>
@@ -2093,10 +2152,33 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
+          <t>~6 g</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Pre-workout scoop</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C22" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D22" s="8">
+        <f>AVERAGE(B22:C22)</f>
+        <v/>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
           <t>0 g</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>Negligible</t>
         </is>

</xml_diff>

<commit_message>
Add Targets sheet deriving calorie and macro targets from body stats
Set from 91.5 kg / 162.5 cm / 33 y / male: BMR 1,771 (Mifflin-St Jeor),
maintenance ~2,567 at a 1.45 activity multiplier, calorie target ~2,020 at
a 550/day deficit for 0.5 kg/week.

The Targets sheet holds weight, height, age, multiplier and deficit as
input cells and derives everything else with formulas, so updating the
weight re-derives maintenance, the target and the carb allowance. The
Daily sheet gains a "vs target" column and Trends gains deficit and
implied-loss rows, all referencing those cells.

Raises the protein band from 90-130 g to 130-145 g (~2.1 g/kg estimated
lean mass), which is what a 6-day split in a deficit needs to hold muscle.
Both logged days fall short of the new floor.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -10,7 +10,8 @@
     <sheet name="Meals" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Daily" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Trends" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Reference" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Targets" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Reference" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,9 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="+#,##0;-#,##0;0"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -117,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -145,13 +147,21 @@
     <xf numFmtId="165" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="1" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1209,7 +1219,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1224,6 +1234,7 @@
     <col width="9" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1301,6 +1312,11 @@
           <t>Pending items</t>
         </is>
       </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>vs target (mid)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="18" t="n">
@@ -1350,59 +1366,67 @@
         <f>COUNTIFS(Meals!$A$5:$A$15,$A5,Meals!$M$5:$M$15,"pending")</f>
         <v/>
       </c>
+      <c r="M5" s="19">
+        <f>D5-Targets!$B$16</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="n">
+      <c r="A6" s="20" t="n">
         <v>46270</v>
       </c>
-      <c r="B6" s="20">
+      <c r="B6" s="21">
         <f>SUMIFS(Meals!$D$5:$D$15,Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
         <v/>
       </c>
-      <c r="C6" s="20">
+      <c r="C6" s="21">
         <f>SUMIFS(Meals!$E$5:$E$15,Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
         <v/>
       </c>
-      <c r="D6" s="20">
+      <c r="D6" s="21">
         <f>AVERAGE(B6:C6)</f>
         <v/>
       </c>
-      <c r="E6" s="21">
+      <c r="E6" s="22">
         <f>SUMIFS(Meals!$G$5:$G$15,Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
         <v/>
       </c>
-      <c r="F6" s="21">
+      <c r="F6" s="22">
         <f>SUMIFS(Meals!$H$5:$H$15,Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
         <v/>
       </c>
-      <c r="G6" s="21">
+      <c r="G6" s="22">
         <f>AVERAGE(E6:F6)</f>
         <v/>
       </c>
-      <c r="H6" s="21">
+      <c r="H6" s="22">
         <f>SUMIFS(Meals!$J$5:$J$15,Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
         <v/>
       </c>
-      <c r="I6" s="21">
+      <c r="I6" s="22">
         <f>SUMIFS(Meals!$K$5:$K$15,Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
         <v/>
       </c>
-      <c r="J6" s="21">
+      <c r="J6" s="22">
         <f>AVERAGE(H6:I6)</f>
         <v/>
       </c>
-      <c r="K6" s="19">
+      <c r="K6" s="20">
         <f>COUNTIFS(Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
         <v/>
       </c>
-      <c r="L6" s="19">
+      <c r="L6" s="20">
         <f>COUNTIFS(Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"pending")</f>
+        <v/>
+      </c>
+      <c r="M6" s="23">
+        <f>D6-Targets!$B$16</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A2:M2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1432,102 +1456,110 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="22" t="inlineStr">
-        <is>
-          <t>Assumptions</t>
+    <row r="2">
+      <c r="A2" s="24" t="inlineStr">
+        <is>
+          <t>Targets come from the Targets sheet - change them there, not here.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="inlineStr">
-        <is>
-          <t>Protein target low (g/day)</t>
-        </is>
-      </c>
-      <c r="B4" s="24" t="n">
-        <v>90</v>
-      </c>
-      <c r="C4" s="25" t="inlineStr">
-        <is>
-          <t>Source: stated by user (adjust to bodyweight). Yellow = edit me.</t>
+      <c r="A4" s="25" t="inlineStr">
+        <is>
+          <t>Overall</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="inlineStr">
-        <is>
-          <t>Protein target high (g/day)</t>
-        </is>
-      </c>
-      <c r="B5" s="24" t="n">
-        <v>130</v>
+      <c r="A5" s="26" t="inlineStr">
+        <is>
+          <t>Days logged</t>
+        </is>
+      </c>
+      <c r="B5" s="18">
+        <f>COUNT(Daily!$A$5:$A$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="26" t="inlineStr">
+        <is>
+          <t>Avg calories/day (mid)</t>
+        </is>
+      </c>
+      <c r="B6" s="8">
+        <f>IFERROR(AVERAGE(Daily!$D$5:$D$6),0)</f>
+        <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="22" t="inlineStr">
-        <is>
-          <t>Overall</t>
-        </is>
+      <c r="A7" s="26" t="inlineStr">
+        <is>
+          <t>Avg protein/day (mid, g)</t>
+        </is>
+      </c>
+      <c r="B7" s="10">
+        <f>IFERROR(AVERAGE(Daily!$G$5:$G$6),0)</f>
+        <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="inlineStr">
-        <is>
-          <t>Days logged</t>
-        </is>
-      </c>
-      <c r="B8" s="18">
-        <f>COUNT(Daily!$A$5:$A$6)</f>
+      <c r="A8" s="26" t="inlineStr">
+        <is>
+          <t>Avg fat/day (mid, g)</t>
+        </is>
+      </c>
+      <c r="B8" s="10">
+        <f>IFERROR(AVERAGE(Daily!$J$5:$J$6),0)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="inlineStr">
-        <is>
-          <t>Avg calories/day (mid)</t>
-        </is>
-      </c>
-      <c r="B9" s="8">
-        <f>IFERROR(AVERAGE(Daily!$D$5:$D$6),0)</f>
+      <c r="A9" s="26" t="inlineStr">
+        <is>
+          <t>Avg vs calorie target</t>
+        </is>
+      </c>
+      <c r="B9" s="19">
+        <f>IFERROR(B6-Targets!$B$16,0)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="inlineStr">
-        <is>
-          <t>Avg protein/day (mid, g)</t>
-        </is>
-      </c>
-      <c r="B10" s="10">
-        <f>IFERROR(AVERAGE(Daily!$G$5:$G$6),0)</f>
+      <c r="A10" s="26" t="inlineStr">
+        <is>
+          <t>Avg deficit vs maintenance</t>
+        </is>
+      </c>
+      <c r="B10" s="19">
+        <f>IFERROR(Targets!$B$15-B6,0)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="inlineStr">
-        <is>
-          <t>Avg fat/day (mid, g)</t>
-        </is>
-      </c>
-      <c r="B11" s="10">
-        <f>IFERROR(AVERAGE(Daily!$J$5:$J$6),0)</f>
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>Implied loss (kg/week)</t>
+        </is>
+      </c>
+      <c r="B11" s="27">
+        <f>IFERROR((Targets!$B$15-B6)*7/Targets!$B$11,0)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="inlineStr">
+      <c r="A12" s="26" t="inlineStr">
         <is>
           <t>Days hitting protein target</t>
         </is>
       </c>
       <c r="B12" s="18">
-        <f>COUNTIFS(Daily!$G$5:$G$6,"&gt;="&amp;$B$4)</f>
+        <f>COUNTIFS(Daily!$G$5:$G$6,"&gt;="&amp;Targets!$B$20)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="inlineStr">
+      <c r="A13" s="26" t="inlineStr">
         <is>
           <t>Total pending (unconfirmed) items</t>
         </is>
@@ -1538,7 +1570,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="22" t="inlineStr">
+      <c r="A15" s="25" t="inlineStr">
         <is>
           <t>Weekly (week starting Monday)</t>
         </is>
@@ -1601,7 +1633,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="22" t="inlineStr">
+      <c r="A19" s="25" t="inlineStr">
         <is>
           <t>Monthly</t>
         </is>
@@ -1664,7 +1696,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="25" t="inlineStr">
+      <c r="A23" s="24" t="inlineStr">
         <is>
           <t>Averages cover only the days present in the log; a part-logged day (today's dinner still to come) drags its average down.</t>
         </is>
@@ -1676,6 +1708,299 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="66" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Targets</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Edit the yellow input cells only. BMR uses Mifflin-St Jeor, the equation recommended for this purpose. Everything below the inputs is a formula, so dropping the weight here re-derives maintenance, the calorie target and the carb allowance automatically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="25" t="inlineStr">
+        <is>
+          <t>Inputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="26" t="inlineStr">
+        <is>
+          <t>Weight (kg)</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="n">
+        <v>91.5</v>
+      </c>
+      <c r="C5" s="28" t="inlineStr">
+        <is>
+          <t>Source: stated by user, 2026-09-05. Update as it changes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="26" t="inlineStr">
+        <is>
+          <t>Height (cm)</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="n">
+        <v>162.5</v>
+      </c>
+      <c r="C6" s="28" t="inlineStr">
+        <is>
+          <t>Source: stated by user.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="26" t="inlineStr">
+        <is>
+          <t>Age (years)</t>
+        </is>
+      </c>
+      <c r="B7" s="29" t="n">
+        <v>33</v>
+      </c>
+      <c r="C7" s="28" t="inlineStr">
+        <is>
+          <t>Source: stated by user (turns 33 on 2026-09-15).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="26" t="inlineStr">
+        <is>
+          <t>Sex constant</t>
+        </is>
+      </c>
+      <c r="B8" s="29" t="n">
+        <v>5</v>
+      </c>
+      <c r="C8" s="28" t="inlineStr">
+        <is>
+          <t>Mifflin-St Jeor term: +5 male, -161 female.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="26" t="inlineStr">
+        <is>
+          <t>Activity multiplier</t>
+        </is>
+      </c>
+      <c r="B9" s="30" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="C9" s="28" t="inlineStr">
+        <is>
+          <t>1.45 = desk job plus 6 lifting sessions/week. Lifting burns less than cardio-based charts assume; raise it only if the scale says so.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="26" t="inlineStr">
+        <is>
+          <t>Daily deficit (kcal)</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="n">
+        <v>550</v>
+      </c>
+      <c r="C10" s="28" t="inlineStr">
+        <is>
+          <t>550/day = 0.5 kg/week. Assumption, not a measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>kcal per kg of body fat</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="n">
+        <v>7700</v>
+      </c>
+      <c r="C11" s="28" t="inlineStr">
+        <is>
+          <t>Standard 7,700 kcal/kg conversion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="25" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>BMR (Mifflin-St Jeor)</t>
+        </is>
+      </c>
+      <c r="B14" s="8">
+        <f>10*B5+6.25*B6-5*B7+B8</f>
+        <v/>
+      </c>
+      <c r="C14" s="28" t="inlineStr">
+        <is>
+          <t>Resting burn: what the body uses doing nothing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>Maintenance (TDEE)</t>
+        </is>
+      </c>
+      <c r="B15" s="8">
+        <f>B14*B9</f>
+        <v/>
+      </c>
+      <c r="C15" s="28" t="inlineStr">
+        <is>
+          <t>Estimate. The scale over 2-3 weeks is the real measurement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="25" t="inlineStr">
+        <is>
+          <t>CALORIE TARGET</t>
+        </is>
+      </c>
+      <c r="B16" s="31">
+        <f>B15-B10</f>
+        <v/>
+      </c>
+      <c r="C16" s="28" t="inlineStr">
+        <is>
+          <t>The number to eat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="26" t="inlineStr">
+        <is>
+          <t>Projected loss (kg/week)</t>
+        </is>
+      </c>
+      <c r="B17" s="27">
+        <f>B10*7/B11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="26" t="inlineStr">
+        <is>
+          <t>BMI</t>
+        </is>
+      </c>
+      <c r="B18" s="10">
+        <f>B5/(B6/100)^2</f>
+        <v/>
+      </c>
+      <c r="C18" s="28" t="inlineStr">
+        <is>
+          <t>Worth a GP or dietitian check alongside this plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="25" t="inlineStr">
+        <is>
+          <t>Macros at the calorie target</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>Protein target low (g)</t>
+        </is>
+      </c>
+      <c r="B21" s="29" t="n">
+        <v>130</v>
+      </c>
+      <c r="C21" s="28" t="inlineStr">
+        <is>
+          <t>~2.1 g/kg of estimated lean mass - the level that protects muscle in a deficit while training 6 days.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="26" t="inlineStr">
+        <is>
+          <t>Protein target high (g)</t>
+        </is>
+      </c>
+      <c r="B22" s="29" t="n">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="26" t="inlineStr">
+        <is>
+          <t>Fat floor (g)</t>
+        </is>
+      </c>
+      <c r="B23" s="29" t="n">
+        <v>55</v>
+      </c>
+      <c r="C23" s="28" t="inlineStr">
+        <is>
+          <t>~0.6 g/kg. A floor for hormone health, not a goal to hit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="26" t="inlineStr">
+        <is>
+          <t>Carb allowance (g)</t>
+        </is>
+      </c>
+      <c r="B24" s="18">
+        <f>(B16-B21*4-B23*9)/4</f>
+        <v/>
+      </c>
+      <c r="C24" s="28" t="inlineStr">
+        <is>
+          <t>Whatever is left once protein and the fat floor are paid for. Fuels the PPL work.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Log pineapple juice as Day 2 dinner and close out the day
Fresh pineapple juice, ~350-450 ml, no added sugar: 175-240 kcal, 1-2 g
protein, negligible fat, ~35-45 g natural sugar. Added a reference row for
it.

Day 2 finishes at 1,855-2,500 kcal (mid 2,177.5), 158 over the ~2,020
target, with protein at 107.25 g against the 130 g floor and fat at
78.25 g against the 55 g floor.

Two-day average is now 1,993 kcal, within 25 kcal of target, implying
~0.52 kg/week. Reframed the trends read around the evening meal slot,
which is what decided both days.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -948,39 +948,39 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Lunch</t>
+          <t>Dinner</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Fish fry + ~half container barik rice + sambar + veg raita + red chutney + veg side</t>
+          <t>Fresh pineapple juice (~350-450 ml takeaway cup) - no added sugar</t>
         </is>
       </c>
       <c r="D11" s="7" t="n">
-        <v>590</v>
+        <v>175</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>840</v>
+        <v>240</v>
       </c>
       <c r="F11" s="8">
         <f>AVERAGE(D11:E11)</f>
         <v/>
       </c>
       <c r="G11" s="9" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="I11" s="10">
         <f>AVERAGE(G11:H11)</f>
         <v/>
       </c>
       <c r="J11" s="9" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>33</v>
+        <v>0.5</v>
       </c>
       <c r="L11" s="10">
         <f>AVERAGE(J11:K11)</f>
@@ -991,7 +991,11 @@
           <t>logged</t>
         </is>
       </c>
-      <c r="N11" s="6" t="inlineStr"/>
+      <c r="N11" s="6" t="inlineStr">
+        <is>
+          <t>Juice only - no solid food at dinner. ~35-45 g natural sugar; no fibre; ~1.5 g protein</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
@@ -999,39 +1003,39 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Snack</t>
+          <t>Lunch</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Black coffee + 1 whey scoop (no sugar)</t>
+          <t>Fish fry + ~half container barik rice + sambar + veg raita + red chutney + veg side</t>
         </is>
       </c>
       <c r="D12" s="7" t="n">
-        <v>100</v>
+        <v>590</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>130</v>
+        <v>840</v>
       </c>
       <c r="F12" s="8">
         <f>AVERAGE(D12:E12)</f>
         <v/>
       </c>
       <c r="G12" s="9" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="H12" s="9" t="n">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="I12" s="10">
         <f>AVERAGE(G12:H12)</f>
         <v/>
       </c>
       <c r="J12" s="9" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="K12" s="9" t="n">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="L12" s="10">
         <f>AVERAGE(J12:K12)</f>
@@ -1055,14 +1059,14 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>1 whey scoop + water</t>
+          <t>Black coffee + 1 whey scoop (no sugar)</t>
         </is>
       </c>
       <c r="D13" s="7" t="n">
         <v>100</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="F13" s="8">
         <f>AVERAGE(D13:E13)</f>
@@ -1082,7 +1086,7 @@
         <v>1</v>
       </c>
       <c r="K13" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L13" s="10">
         <f>AVERAGE(J13:K13)</f>
@@ -1106,34 +1110,34 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>3 uzhunnu vada + coconut chutney</t>
+          <t>1 whey scoop + water</t>
         </is>
       </c>
       <c r="D14" s="7" t="n">
-        <v>480</v>
+        <v>100</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>650</v>
+        <v>120</v>
       </c>
       <c r="F14" s="8">
         <f>AVERAGE(D14:E14)</f>
         <v/>
       </c>
       <c r="G14" s="9" t="n">
-        <v>11.5</v>
+        <v>20</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="I14" s="10">
         <f>AVERAGE(G14:H14)</f>
         <v/>
       </c>
       <c r="J14" s="9" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="K14" s="9" t="n">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="L14" s="10">
         <f>AVERAGE(J14:K14)</f>
@@ -1144,62 +1148,113 @@
           <t>logged</t>
         </is>
       </c>
-      <c r="N14" s="6" t="inlineStr">
+      <c r="N14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>3 uzhunnu vada + coconut chutney</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>480</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>650</v>
+      </c>
+      <c r="F15" s="8">
+        <f>AVERAGE(D15:E15)</f>
+        <v/>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H15" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="I15" s="10">
+        <f>AVERAGE(G15:H15)</f>
+        <v/>
+      </c>
+      <c r="J15" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="K15" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="L15" s="10">
+        <f>AVERAGE(J15:K15)</f>
+        <v/>
+      </c>
+      <c r="M15" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N15" s="6" t="inlineStr">
         <is>
           <t>Coconut chutney included this time (skipped at breakfast both days)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="11" t="n">
+    <row r="16">
+      <c r="A16" s="11" t="n">
         <v>46270</v>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>Supplement</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
+      <c r="C16" s="13" t="inlineStr">
         <is>
           <t>Pre-workout scoop</t>
         </is>
       </c>
-      <c r="D15" s="14" t="n">
+      <c r="D16" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="E15" s="14" t="n">
+      <c r="E16" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="F15" s="15">
-        <f>AVERAGE(D15:E15)</f>
-        <v/>
-      </c>
-      <c r="G15" s="16" t="n">
+      <c r="F16" s="15">
+        <f>AVERAGE(D16:E16)</f>
+        <v/>
+      </c>
+      <c r="G16" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="H15" s="16" t="n">
+      <c r="H16" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="I15" s="17">
-        <f>AVERAGE(G15:H15)</f>
-        <v/>
-      </c>
-      <c r="J15" s="16" t="n">
+      <c r="I16" s="17">
+        <f>AVERAGE(G16:H16)</f>
+        <v/>
+      </c>
+      <c r="J16" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="K15" s="16" t="n">
+      <c r="K16" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="L15" s="17">
-        <f>AVERAGE(J15:K15)</f>
-        <v/>
-      </c>
-      <c r="M15" s="12" t="inlineStr">
+      <c r="L16" s="17">
+        <f>AVERAGE(J16:K16)</f>
+        <v/>
+      </c>
+      <c r="M16" s="12" t="inlineStr">
         <is>
           <t>pending</t>
         </is>
       </c>
-      <c r="N15" s="13" t="inlineStr">
+      <c r="N16" s="13" t="inlineStr">
         <is>
           <t>Planned but not taken as of last check - confirm before logging</t>
         </is>
@@ -1323,11 +1378,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$15,Meals!$A$5:$A$15,$A5,Meals!$M$5:$M$15,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$16,Meals!$A$5:$A$16,$A5,Meals!$M$5:$M$16,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$15,Meals!$A$5:$A$15,$A5,Meals!$M$5:$M$15,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$16,Meals!$A$5:$A$16,$A5,Meals!$M$5:$M$16,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -1335,11 +1390,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$15,Meals!$A$5:$A$15,$A5,Meals!$M$5:$M$15,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$16,Meals!$A$5:$A$16,$A5,Meals!$M$5:$M$16,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$15,Meals!$A$5:$A$15,$A5,Meals!$M$5:$M$15,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$16,Meals!$A$5:$A$16,$A5,Meals!$M$5:$M$16,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -1347,11 +1402,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$15,Meals!$A$5:$A$15,$A5,Meals!$M$5:$M$15,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$16,Meals!$A$5:$A$16,$A5,Meals!$M$5:$M$16,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$15,Meals!$A$5:$A$15,$A5,Meals!$M$5:$M$15,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$16,Meals!$A$5:$A$16,$A5,Meals!$M$5:$M$16,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -1359,11 +1414,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$15,$A5,Meals!$M$5:$M$15,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$16,$A5,Meals!$M$5:$M$16,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$15,$A5,Meals!$M$5:$M$15,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$16,$A5,Meals!$M$5:$M$16,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -1376,11 +1431,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$15,Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$16,Meals!$A$5:$A$16,$A6,Meals!$M$5:$M$16,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$15,Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$16,Meals!$A$5:$A$16,$A6,Meals!$M$5:$M$16,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -1388,11 +1443,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$15,Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$16,Meals!$A$5:$A$16,$A6,Meals!$M$5:$M$16,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$15,Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$16,Meals!$A$5:$A$16,$A6,Meals!$M$5:$M$16,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -1400,11 +1455,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$15,Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$16,Meals!$A$5:$A$16,$A6,Meals!$M$5:$M$16,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$15,Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$16,Meals!$A$5:$A$16,$A6,Meals!$M$5:$M$16,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -1412,11 +1467,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$16,$A6,Meals!$M$5:$M$16,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$15,$A6,Meals!$M$5:$M$15,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$16,$A6,Meals!$M$5:$M$16,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -2006,7 +2061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2370,14 +2425,14 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in water)</t>
+          <t>Fresh pineapple juice (350-450 ml)</t>
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>100</v>
+        <v>175</v>
       </c>
       <c r="C17" s="7" t="n">
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="D17" s="8">
         <f>AVERAGE(B17:C17)</f>
@@ -2385,22 +2440,26 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr"/>
+          <t>~1-2 g</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>No added sugar but ~35-45 g natural sugar; no fibre; almost no protein</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in black coffee no sugar)</t>
+          <t>Whey scoop (in water)</t>
         </is>
       </c>
       <c r="B18" s="7" t="n">
         <v>100</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="D18" s="8">
         <f>AVERAGE(B18:C18)</f>
@@ -2416,14 +2475,14 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Cashew/almond biscuit (1)</t>
+          <t>Whey scoop (in black coffee no sugar)</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C19" s="7" t="n">
-        <v>38</v>
+        <v>130</v>
       </c>
       <c r="D19" s="8">
         <f>AVERAGE(B19:C19)</f>
@@ -2431,7 +2490,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>~0.5 g</t>
+          <t>~20-25 g</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr"/>
@@ -2439,14 +2498,14 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (~50g standard)</t>
+          <t>Cashew/almond biscuit (1)</t>
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>245</v>
+        <v>38</v>
       </c>
       <c r="C20" s="7" t="n">
-        <v>250</v>
+        <v>38</v>
       </c>
       <c r="D20" s="8">
         <f>AVERAGE(B20:C20)</f>
@@ -2454,7 +2513,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>~4 g</t>
+          <t>~0.5 g</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr"/>
@@ -2462,14 +2521,14 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (70g king-size)</t>
+          <t>Chocolate bar (~50g standard)</t>
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>335</v>
+        <v>245</v>
       </c>
       <c r="C21" s="7" t="n">
-        <v>335</v>
+        <v>250</v>
       </c>
       <c r="D21" s="8">
         <f>AVERAGE(B21:C21)</f>
@@ -2477,7 +2536,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>~6 g</t>
+          <t>~4 g</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr"/>
@@ -2485,14 +2544,14 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Pre-workout scoop</t>
+          <t>Chocolate bar (70g king-size)</t>
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>5</v>
+        <v>335</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>15</v>
+        <v>335</v>
       </c>
       <c r="D22" s="8">
         <f>AVERAGE(B22:C22)</f>
@@ -2500,10 +2559,33 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
+          <t>~6 g</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Pre-workout scoop</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C23" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D23" s="8">
+        <f>AVERAGE(B23:C23)</f>
+        <v/>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
           <t>0 g</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="F23" s="6" t="inlineStr">
         <is>
           <t>Negligible</t>
         </is>

</xml_diff>

<commit_message>
Add reference estimates for late-night protein options
Greek yogurt, boiled egg, paneer and cucumber, so a late snack can be
costed consistently when one gets logged.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -2061,7 +2061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2475,14 +2475,14 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in black coffee no sugar)</t>
+          <t>Greek yogurt (200 g plain low-fat)</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="C19" s="7" t="n">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="D19" s="8">
         <f>AVERAGE(B19:C19)</f>
@@ -2490,22 +2490,26 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr"/>
+          <t>~18-20 g</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>Casein - digests slowly; good overnight</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Cashew/almond biscuit (1)</t>
+          <t>Boiled egg (1 large)</t>
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>38</v>
+        <v>70</v>
       </c>
       <c r="C20" s="7" t="n">
-        <v>38</v>
+        <v>78</v>
       </c>
       <c r="D20" s="8">
         <f>AVERAGE(B20:C20)</f>
@@ -2513,22 +2517,26 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>~0.5 g</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr"/>
+          <t>~6-6.5 g</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>~5 g fat each</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (~50g standard)</t>
+          <t>Paneer (50 g full-fat)</t>
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>245</v>
+        <v>130</v>
       </c>
       <c r="C21" s="7" t="n">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="D21" s="8">
         <f>AVERAGE(B21:C21)</f>
@@ -2536,22 +2544,26 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>~4 g</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr"/>
+          <t>~8-9 g</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>Fat-dense for the protein it gives</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (70g king-size)</t>
+          <t>Cucumber (1 medium)</t>
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>335</v>
+        <v>25</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>335</v>
+        <v>30</v>
       </c>
       <c r="D22" s="8">
         <f>AVERAGE(B22:C22)</f>
@@ -2559,22 +2571,26 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>~6 g</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr"/>
+          <t>~1.5 g</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>Volume with almost no calories</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Pre-workout scoop</t>
+          <t>Whey scoop (in black coffee no sugar)</t>
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="C23" s="7" t="n">
-        <v>15</v>
+        <v>130</v>
       </c>
       <c r="D23" s="8">
         <f>AVERAGE(B23:C23)</f>
@@ -2582,10 +2598,102 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
+          <t>~20-25 g</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Cashew/almond biscuit (1)</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="n">
+        <v>38</v>
+      </c>
+      <c r="C24" s="7" t="n">
+        <v>38</v>
+      </c>
+      <c r="D24" s="8">
+        <f>AVERAGE(B24:C24)</f>
+        <v/>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>~0.5 g</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Chocolate bar (~50g standard)</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="n">
+        <v>245</v>
+      </c>
+      <c r="C25" s="7" t="n">
+        <v>250</v>
+      </c>
+      <c r="D25" s="8">
+        <f>AVERAGE(B25:C25)</f>
+        <v/>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>~4 g</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Chocolate bar (70g king-size)</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="n">
+        <v>335</v>
+      </c>
+      <c r="C26" s="7" t="n">
+        <v>335</v>
+      </c>
+      <c r="D26" s="8">
+        <f>AVERAGE(B26:C26)</f>
+        <v/>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>~6 g</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Pre-workout scoop</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C27" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D27" s="8">
+        <f>AVERAGE(B27:C27)</f>
+        <v/>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
           <t>0 g</t>
         </is>
       </c>
-      <c r="F23" s="6" t="inlineStr">
+      <c r="F27" s="6" t="inlineStr">
         <is>
           <t>Negligible</t>
         </is>

</xml_diff>

<commit_message>
Add grilled chicken and grill-side reference estimates
Breast (100 g and 150 g skinless), quarter with skin, toum and khubz, so a
grill order can be costed consistently. Toum and khubz are the items that
quietly double a grilled chicken order.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -2061,7 +2061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2402,14 +2402,14 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Barik/basmati rice (half container cooked)</t>
+          <t>Grilled chicken breast (100 g skinless)</t>
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>200</v>
+        <v>160</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>280</v>
+        <v>180</v>
       </c>
       <c r="D16" s="8">
         <f>AVERAGE(B16:C16)</f>
@@ -2417,22 +2417,26 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>~4-5 g</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr"/>
+          <t>~30-32 g</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Best protein-per-calorie item in this list</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Fresh pineapple juice (350-450 ml)</t>
+          <t>Grilled chicken breast (150 g skinless)</t>
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>175</v>
+        <v>240</v>
       </c>
       <c r="C17" s="7" t="n">
-        <v>240</v>
+        <v>270</v>
       </c>
       <c r="D17" s="8">
         <f>AVERAGE(B17:C17)</f>
@@ -2440,26 +2444,22 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>~1-2 g</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>No added sugar but ~35-45 g natural sugar; no fibre; almost no protein</t>
-        </is>
-      </c>
+          <t>~45-48 g</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in water)</t>
+          <t>Grilled chicken quarter (skin on)</t>
         </is>
       </c>
       <c r="B18" s="7" t="n">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>120</v>
+        <v>320</v>
       </c>
       <c r="D18" s="8">
         <f>AVERAGE(B18:C18)</f>
@@ -2467,22 +2467,26 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr"/>
+          <t>~28-33 g</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Skin adds ~12-15 g fat over breast</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Greek yogurt (200 g plain low-fat)</t>
+          <t>Garlic sauce / toum (1 tbsp)</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
       <c r="C19" s="7" t="n">
-        <v>140</v>
+        <v>110</v>
       </c>
       <c r="D19" s="8">
         <f>AVERAGE(B19:C19)</f>
@@ -2490,26 +2494,26 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>~18-20 g</t>
+          <t>0 g</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>Casein - digests slowly; good overnight</t>
+          <t>Essentially emulsified oil - the hidden cost at a grill</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Boiled egg (1 large)</t>
+          <t>Khubz / pita (1 large)</t>
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>70</v>
+        <v>250</v>
       </c>
       <c r="C20" s="7" t="n">
-        <v>78</v>
+        <v>300</v>
       </c>
       <c r="D20" s="8">
         <f>AVERAGE(B20:C20)</f>
@@ -2517,26 +2521,22 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>~6-6.5 g</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>~5 g fat each</t>
-        </is>
-      </c>
+          <t>~8-9 g</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Paneer (50 g full-fat)</t>
+          <t>Barik/basmati rice (half container cooked)</t>
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>130</v>
+        <v>200</v>
       </c>
       <c r="C21" s="7" t="n">
-        <v>150</v>
+        <v>280</v>
       </c>
       <c r="D21" s="8">
         <f>AVERAGE(B21:C21)</f>
@@ -2544,26 +2544,22 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>~8-9 g</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>Fat-dense for the protein it gives</t>
-        </is>
-      </c>
+          <t>~4-5 g</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Cucumber (1 medium)</t>
+          <t>Fresh pineapple juice (350-450 ml)</t>
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>25</v>
+        <v>175</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>30</v>
+        <v>240</v>
       </c>
       <c r="D22" s="8">
         <f>AVERAGE(B22:C22)</f>
@@ -2571,26 +2567,26 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>~1.5 g</t>
+          <t>~1-2 g</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>Volume with almost no calories</t>
+          <t>No added sugar but ~35-45 g natural sugar; no fibre; almost no protein</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in black coffee no sugar)</t>
+          <t>Whey scoop (in water)</t>
         </is>
       </c>
       <c r="B23" s="7" t="n">
         <v>100</v>
       </c>
       <c r="C23" s="7" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="D23" s="8">
         <f>AVERAGE(B23:C23)</f>
@@ -2606,14 +2602,14 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Cashew/almond biscuit (1)</t>
+          <t>Greek yogurt (200 g plain low-fat)</t>
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>38</v>
+        <v>120</v>
       </c>
       <c r="C24" s="7" t="n">
-        <v>38</v>
+        <v>140</v>
       </c>
       <c r="D24" s="8">
         <f>AVERAGE(B24:C24)</f>
@@ -2621,22 +2617,26 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>~0.5 g</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr"/>
+          <t>~18-20 g</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>Casein - digests slowly; good overnight</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (~50g standard)</t>
+          <t>Boiled egg (1 large)</t>
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>245</v>
+        <v>70</v>
       </c>
       <c r="C25" s="7" t="n">
-        <v>250</v>
+        <v>78</v>
       </c>
       <c r="D25" s="8">
         <f>AVERAGE(B25:C25)</f>
@@ -2644,22 +2644,26 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>~4 g</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr"/>
+          <t>~6-6.5 g</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>~5 g fat each</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (70g king-size)</t>
+          <t>Paneer (50 g full-fat)</t>
         </is>
       </c>
       <c r="B26" s="7" t="n">
-        <v>335</v>
+        <v>130</v>
       </c>
       <c r="C26" s="7" t="n">
-        <v>335</v>
+        <v>150</v>
       </c>
       <c r="D26" s="8">
         <f>AVERAGE(B26:C26)</f>
@@ -2667,22 +2671,26 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>~6 g</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr"/>
+          <t>~8-9 g</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>Fat-dense for the protein it gives</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Pre-workout scoop</t>
+          <t>Cucumber (1 medium)</t>
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="C27" s="7" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="D27" s="8">
         <f>AVERAGE(B27:C27)</f>
@@ -2690,10 +2698,129 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
+          <t>~1.5 g</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>Volume with almost no calories</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Whey scoop (in black coffee no sugar)</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C28" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="D28" s="8">
+        <f>AVERAGE(B28:C28)</f>
+        <v/>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>~20-25 g</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Cashew/almond biscuit (1)</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="n">
+        <v>38</v>
+      </c>
+      <c r="C29" s="7" t="n">
+        <v>38</v>
+      </c>
+      <c r="D29" s="8">
+        <f>AVERAGE(B29:C29)</f>
+        <v/>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>~0.5 g</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Chocolate bar (~50g standard)</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>245</v>
+      </c>
+      <c r="C30" s="7" t="n">
+        <v>250</v>
+      </c>
+      <c r="D30" s="8">
+        <f>AVERAGE(B30:C30)</f>
+        <v/>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>~4 g</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>Chocolate bar (70g king-size)</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="n">
+        <v>335</v>
+      </c>
+      <c r="C31" s="7" t="n">
+        <v>335</v>
+      </c>
+      <c r="D31" s="8">
+        <f>AVERAGE(B31:C31)</f>
+        <v/>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>~6 g</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>Pre-workout scoop</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C32" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D32" s="8">
+        <f>AVERAGE(B32:C32)</f>
+        <v/>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
           <t>0 g</t>
         </is>
       </c>
-      <c r="F27" s="6" t="inlineStr">
+      <c r="F32" s="6" t="inlineStr">
         <is>
           <t>Negligible</t>
         </is>

</xml_diff>

<commit_message>
Log Day 3 breakfast: 3 porotta with kadala curry
680-1,050 kcal (mid 865), 20-28 g protein, 31-52 g fat. Heaviest single
meal in the log: 43% of the day's calorie target and 75% of a day's fat
floor for 24 g of protein.

Adds a budget table for the rest of Day 3 - 1,152 kcal remaining with
106 g of protein still to find.

Trends averages are temporarily depressed by the part-logged day; the
Trends sheet already carries a note about that.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1260,6 +1260,61 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Breakfast</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>3 maida porotta + kadala curry</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>680</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>1050</v>
+      </c>
+      <c r="F17" s="8">
+        <f>AVERAGE(D17:E17)</f>
+        <v/>
+      </c>
+      <c r="G17" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="H17" s="9" t="n">
+        <v>28</v>
+      </c>
+      <c r="I17" s="10">
+        <f>AVERAGE(G17:H17)</f>
+        <v/>
+      </c>
+      <c r="J17" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="K17" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="L17" s="10">
+        <f>AVERAGE(J17:K17)</f>
+        <v/>
+      </c>
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N17" s="6" t="inlineStr">
+        <is>
+          <t>Up from 2 porotta on Day 1; heaviest single meal in the log so far</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:N2"/>
@@ -1274,7 +1329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1378,11 +1433,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$16,Meals!$A$5:$A$16,$A5,Meals!$M$5:$M$16,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$17,Meals!$A$5:$A$17,$A5,Meals!$M$5:$M$17,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$16,Meals!$A$5:$A$16,$A5,Meals!$M$5:$M$16,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$17,Meals!$A$5:$A$17,$A5,Meals!$M$5:$M$17,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -1390,11 +1445,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$16,Meals!$A$5:$A$16,$A5,Meals!$M$5:$M$16,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$17,Meals!$A$5:$A$17,$A5,Meals!$M$5:$M$17,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$16,Meals!$A$5:$A$16,$A5,Meals!$M$5:$M$16,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$17,Meals!$A$5:$A$17,$A5,Meals!$M$5:$M$17,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -1402,11 +1457,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$16,Meals!$A$5:$A$16,$A5,Meals!$M$5:$M$16,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$17,Meals!$A$5:$A$17,$A5,Meals!$M$5:$M$17,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$16,Meals!$A$5:$A$16,$A5,Meals!$M$5:$M$16,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$17,Meals!$A$5:$A$17,$A5,Meals!$M$5:$M$17,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -1414,11 +1469,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$16,$A5,Meals!$M$5:$M$16,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$17,$A5,Meals!$M$5:$M$17,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$16,$A5,Meals!$M$5:$M$16,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$17,$A5,Meals!$M$5:$M$17,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -1431,11 +1486,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$16,Meals!$A$5:$A$16,$A6,Meals!$M$5:$M$16,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$17,Meals!$A$5:$A$17,$A6,Meals!$M$5:$M$17,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$16,Meals!$A$5:$A$16,$A6,Meals!$M$5:$M$16,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$17,Meals!$A$5:$A$17,$A6,Meals!$M$5:$M$17,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -1443,11 +1498,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$16,Meals!$A$5:$A$16,$A6,Meals!$M$5:$M$16,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$17,Meals!$A$5:$A$17,$A6,Meals!$M$5:$M$17,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$16,Meals!$A$5:$A$16,$A6,Meals!$M$5:$M$16,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$17,Meals!$A$5:$A$17,$A6,Meals!$M$5:$M$17,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -1455,11 +1510,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$16,Meals!$A$5:$A$16,$A6,Meals!$M$5:$M$16,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$17,Meals!$A$5:$A$17,$A6,Meals!$M$5:$M$17,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$16,Meals!$A$5:$A$16,$A6,Meals!$M$5:$M$16,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$17,Meals!$A$5:$A$17,$A6,Meals!$M$5:$M$17,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -1467,15 +1522,68 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$16,$A6,Meals!$M$5:$M$16,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$17,$A6,Meals!$M$5:$M$17,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$16,$A6,Meals!$M$5:$M$16,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$17,$A6,Meals!$M$5:$M$17,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
         <f>D6-Targets!$B$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="18" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B7" s="8">
+        <f>SUMIFS(Meals!$D$5:$D$17,Meals!$A$5:$A$17,$A7,Meals!$M$5:$M$17,"logged")</f>
+        <v/>
+      </c>
+      <c r="C7" s="8">
+        <f>SUMIFS(Meals!$E$5:$E$17,Meals!$A$5:$A$17,$A7,Meals!$M$5:$M$17,"logged")</f>
+        <v/>
+      </c>
+      <c r="D7" s="8">
+        <f>AVERAGE(B7:C7)</f>
+        <v/>
+      </c>
+      <c r="E7" s="10">
+        <f>SUMIFS(Meals!$G$5:$G$17,Meals!$A$5:$A$17,$A7,Meals!$M$5:$M$17,"logged")</f>
+        <v/>
+      </c>
+      <c r="F7" s="10">
+        <f>SUMIFS(Meals!$H$5:$H$17,Meals!$A$5:$A$17,$A7,Meals!$M$5:$M$17,"logged")</f>
+        <v/>
+      </c>
+      <c r="G7" s="10">
+        <f>AVERAGE(E7:F7)</f>
+        <v/>
+      </c>
+      <c r="H7" s="10">
+        <f>SUMIFS(Meals!$J$5:$J$17,Meals!$A$5:$A$17,$A7,Meals!$M$5:$M$17,"logged")</f>
+        <v/>
+      </c>
+      <c r="I7" s="10">
+        <f>SUMIFS(Meals!$K$5:$K$17,Meals!$A$5:$A$17,$A7,Meals!$M$5:$M$17,"logged")</f>
+        <v/>
+      </c>
+      <c r="J7" s="10">
+        <f>AVERAGE(H7:I7)</f>
+        <v/>
+      </c>
+      <c r="K7" s="18">
+        <f>COUNTIFS(Meals!$A$5:$A$17,$A7,Meals!$M$5:$M$17,"logged")</f>
+        <v/>
+      </c>
+      <c r="L7" s="18">
+        <f>COUNTIFS(Meals!$A$5:$A$17,$A7,Meals!$M$5:$M$17,"pending")</f>
+        <v/>
+      </c>
+      <c r="M7" s="19">
+        <f>D7-Targets!$B$16</f>
         <v/>
       </c>
     </row>
@@ -1532,7 +1640,7 @@
         </is>
       </c>
       <c r="B5" s="18">
-        <f>COUNT(Daily!$A$5:$A$6)</f>
+        <f>COUNT(Daily!$A$5:$A$7)</f>
         <v/>
       </c>
     </row>
@@ -1543,7 +1651,7 @@
         </is>
       </c>
       <c r="B6" s="8">
-        <f>IFERROR(AVERAGE(Daily!$D$5:$D$6),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$D$5:$D$7),0)</f>
         <v/>
       </c>
     </row>
@@ -1554,7 +1662,7 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>IFERROR(AVERAGE(Daily!$G$5:$G$6),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$G$5:$G$7),0)</f>
         <v/>
       </c>
     </row>
@@ -1565,7 +1673,7 @@
         </is>
       </c>
       <c r="B8" s="10">
-        <f>IFERROR(AVERAGE(Daily!$J$5:$J$6),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$J$5:$J$7),0)</f>
         <v/>
       </c>
     </row>
@@ -1609,7 +1717,7 @@
         </is>
       </c>
       <c r="B12" s="18">
-        <f>COUNTIFS(Daily!$G$5:$G$6,"&gt;="&amp;Targets!$B$20)</f>
+        <f>COUNTIFS(Daily!$G$5:$G$7,"&gt;="&amp;Targets!$B$20)</f>
         <v/>
       </c>
     </row>
@@ -1620,7 +1728,7 @@
         </is>
       </c>
       <c r="B13" s="18">
-        <f>SUM(Daily!$L$5:$L$6)</f>
+        <f>SUM(Daily!$L$5:$L$7)</f>
         <v/>
       </c>
     </row>
@@ -1671,19 +1779,19 @@
         <v>46271</v>
       </c>
       <c r="C17" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$6,"&gt;="&amp;$A17,Daily!$A$5:$A$6,"&lt;="&amp;$B17)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$7,"&gt;="&amp;$A17,Daily!$A$5:$A$7,"&lt;="&amp;$B17)</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$6,Daily!$A$5:$A$6,"&gt;="&amp;$A17,Daily!$A$5:$A$6,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$7,Daily!$A$5:$A$7,"&gt;="&amp;$A17,Daily!$A$5:$A$7,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$6,Daily!$A$5:$A$6,"&gt;="&amp;$A17,Daily!$A$5:$A$6,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$7,Daily!$A$5:$A$7,"&gt;="&amp;$A17,Daily!$A$5:$A$7,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$6,Daily!$A$5:$A$6,"&gt;="&amp;$A17,Daily!$A$5:$A$6,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$7,Daily!$A$5:$A$7,"&gt;="&amp;$A17,Daily!$A$5:$A$7,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
     </row>
@@ -1734,19 +1842,19 @@
         <v>46295</v>
       </c>
       <c r="C21" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$6,"&gt;="&amp;$A21,Daily!$A$5:$A$6,"&lt;="&amp;$B21)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$7,"&gt;="&amp;$A21,Daily!$A$5:$A$7,"&lt;="&amp;$B21)</f>
         <v/>
       </c>
       <c r="D21" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$6,Daily!$A$5:$A$6,"&gt;="&amp;$A21,Daily!$A$5:$A$6,"&lt;="&amp;$B21),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$7,Daily!$A$5:$A$7,"&gt;="&amp;$A21,Daily!$A$5:$A$7,"&lt;="&amp;$B21),0)</f>
         <v/>
       </c>
       <c r="E21" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$6,Daily!$A$5:$A$6,"&gt;="&amp;$A21,Daily!$A$5:$A$6,"&lt;="&amp;$B21),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$7,Daily!$A$5:$A$7,"&gt;="&amp;$A21,Daily!$A$5:$A$7,"&lt;="&amp;$B21),0)</f>
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$6,Daily!$A$5:$A$6,"&gt;="&amp;$A21,Daily!$A$5:$A$6,"&lt;="&amp;$B21),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$7,Daily!$A$5:$A$7,"&gt;="&amp;$A21,Daily!$A$5:$A$7,"&lt;="&amp;$B21),0)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct Day 3 breakfast to 2 porotta
Three were served, two were eaten - the third was left deliberately for
calories. Recalculated to 520-800 kcal (mid 660), 15-21 g protein,
23-38 g fat, matching how Day 1's identical dish was costed.

That is 205 kcal and 11 g of fat less than the served plate, and leaves
1,357 kcal and 112 g of protein for the rest of the day.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -1271,34 +1271,34 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>3 maida porotta + kadala curry</t>
+          <t>2 maida porotta + kadala curry</t>
         </is>
       </c>
       <c r="D17" s="7" t="n">
-        <v>680</v>
+        <v>520</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>1050</v>
+        <v>800</v>
       </c>
       <c r="F17" s="8">
         <f>AVERAGE(D17:E17)</f>
         <v/>
       </c>
       <c r="G17" s="9" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H17" s="9" t="n">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="I17" s="10">
         <f>AVERAGE(G17:H17)</f>
         <v/>
       </c>
       <c r="J17" s="9" t="n">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="K17" s="9" t="n">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="L17" s="10">
         <f>AVERAGE(J17:K17)</f>
@@ -1311,7 +1311,7 @@
       </c>
       <c r="N17" s="6" t="inlineStr">
         <is>
-          <t>Up from 2 porotta on Day 1; heaviest single meal in the log so far</t>
+          <t>Ate 2 of the 3 served - deliberately cut one for calories; costed identically to Day 1 dinner</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add reference estimate for the Honest Bowl chicken and rice bowl
550-710 kcal, 42-48 g protein, 9-18 g fat, with the side sauce costed
separately since it is the variable part. Not logged - the meal is planned,
not eaten.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -2169,7 +2169,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2560,14 +2560,14 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Grilled chicken quarter (skin on)</t>
+          <t>Honest Bowl - Grilled Chicken and Rice Bowl</t>
         </is>
       </c>
       <c r="B18" s="7" t="n">
-        <v>250</v>
+        <v>550</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>320</v>
+        <v>710</v>
       </c>
       <c r="D18" s="8">
         <f>AVERAGE(B18:C18)</f>
@@ -2575,26 +2575,26 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>~28-33 g</t>
+          <t>42-48 g</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>Skin adds ~12-15 g fat over breast</t>
+          <t>Menu states 42 g protein; chicken + jasmine rice + sweet potato. Sauce served separately</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Garlic sauce / toum (1 tbsp)</t>
+          <t>Brown/mushroom sauce (side pot)</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="C19" s="7" t="n">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="D19" s="8">
         <f>AVERAGE(B19:C19)</f>
@@ -2602,26 +2602,26 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>0 g</t>
+          <t>~1-2 g</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>Essentially emulsified oil - the hidden cost at a grill</t>
+          <t>Often cream or butter based - the variable in a bowl like this</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Khubz / pita (1 large)</t>
+          <t>Grilled chicken quarter (skin on)</t>
         </is>
       </c>
       <c r="B20" s="7" t="n">
         <v>250</v>
       </c>
       <c r="C20" s="7" t="n">
-        <v>300</v>
+        <v>320</v>
       </c>
       <c r="D20" s="8">
         <f>AVERAGE(B20:C20)</f>
@@ -2629,22 +2629,26 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>~8-9 g</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr"/>
+          <t>~28-33 g</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Skin adds ~12-15 g fat over breast</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Barik/basmati rice (half container cooked)</t>
+          <t>Garlic sauce / toum (1 tbsp)</t>
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>200</v>
+        <v>90</v>
       </c>
       <c r="C21" s="7" t="n">
-        <v>280</v>
+        <v>110</v>
       </c>
       <c r="D21" s="8">
         <f>AVERAGE(B21:C21)</f>
@@ -2652,22 +2656,26 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>~4-5 g</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr"/>
+          <t>0 g</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>Essentially emulsified oil - the hidden cost at a grill</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Fresh pineapple juice (350-450 ml)</t>
+          <t>Khubz / pita (1 large)</t>
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>175</v>
+        <v>250</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="D22" s="8">
         <f>AVERAGE(B22:C22)</f>
@@ -2675,26 +2683,22 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>~1-2 g</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>No added sugar but ~35-45 g natural sugar; no fibre; almost no protein</t>
-        </is>
-      </c>
+          <t>~8-9 g</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in water)</t>
+          <t>Barik/basmati rice (half container cooked)</t>
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="C23" s="7" t="n">
-        <v>120</v>
+        <v>280</v>
       </c>
       <c r="D23" s="8">
         <f>AVERAGE(B23:C23)</f>
@@ -2702,7 +2706,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
+          <t>~4-5 g</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr"/>
@@ -2710,14 +2714,14 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Greek yogurt (200 g plain low-fat)</t>
+          <t>Fresh pineapple juice (350-450 ml)</t>
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>120</v>
+        <v>175</v>
       </c>
       <c r="C24" s="7" t="n">
-        <v>140</v>
+        <v>240</v>
       </c>
       <c r="D24" s="8">
         <f>AVERAGE(B24:C24)</f>
@@ -2725,26 +2729,26 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>~18-20 g</t>
+          <t>~1-2 g</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>Casein - digests slowly; good overnight</t>
+          <t>No added sugar but ~35-45 g natural sugar; no fibre; almost no protein</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Boiled egg (1 large)</t>
+          <t>Whey scoop (in water)</t>
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="C25" s="7" t="n">
-        <v>78</v>
+        <v>120</v>
       </c>
       <c r="D25" s="8">
         <f>AVERAGE(B25:C25)</f>
@@ -2752,26 +2756,22 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>~6-6.5 g</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>~5 g fat each</t>
-        </is>
-      </c>
+          <t>~20-25 g</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Paneer (50 g full-fat)</t>
+          <t>Greek yogurt (200 g plain low-fat)</t>
         </is>
       </c>
       <c r="B26" s="7" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="C26" s="7" t="n">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="D26" s="8">
         <f>AVERAGE(B26:C26)</f>
@@ -2779,26 +2779,26 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>~8-9 g</t>
+          <t>~18-20 g</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>Fat-dense for the protein it gives</t>
+          <t>Casein - digests slowly; good overnight</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Cucumber (1 medium)</t>
+          <t>Boiled egg (1 large)</t>
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>25</v>
+        <v>70</v>
       </c>
       <c r="C27" s="7" t="n">
-        <v>30</v>
+        <v>78</v>
       </c>
       <c r="D27" s="8">
         <f>AVERAGE(B27:C27)</f>
@@ -2806,26 +2806,26 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>~1.5 g</t>
+          <t>~6-6.5 g</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>Volume with almost no calories</t>
+          <t>~5 g fat each</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in black coffee no sugar)</t>
+          <t>Paneer (50 g full-fat)</t>
         </is>
       </c>
       <c r="B28" s="7" t="n">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="C28" s="7" t="n">
-        <v>130</v>
+        <v>150</v>
       </c>
       <c r="D28" s="8">
         <f>AVERAGE(B28:C28)</f>
@@ -2833,22 +2833,26 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr"/>
+          <t>~8-9 g</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>Fat-dense for the protein it gives</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Cashew/almond biscuit (1)</t>
+          <t>Cucumber (1 medium)</t>
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="C29" s="7" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="D29" s="8">
         <f>AVERAGE(B29:C29)</f>
@@ -2856,22 +2860,26 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>~0.5 g</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="inlineStr"/>
+          <t>~1.5 g</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>Volume with almost no calories</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (~50g standard)</t>
+          <t>Whey scoop (in black coffee no sugar)</t>
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>245</v>
+        <v>100</v>
       </c>
       <c r="C30" s="7" t="n">
-        <v>250</v>
+        <v>130</v>
       </c>
       <c r="D30" s="8">
         <f>AVERAGE(B30:C30)</f>
@@ -2879,7 +2887,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>~4 g</t>
+          <t>~20-25 g</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr"/>
@@ -2887,14 +2895,14 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (70g king-size)</t>
+          <t>Cashew/almond biscuit (1)</t>
         </is>
       </c>
       <c r="B31" s="7" t="n">
-        <v>335</v>
+        <v>38</v>
       </c>
       <c r="C31" s="7" t="n">
-        <v>335</v>
+        <v>38</v>
       </c>
       <c r="D31" s="8">
         <f>AVERAGE(B31:C31)</f>
@@ -2902,7 +2910,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>~6 g</t>
+          <t>~0.5 g</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr"/>
@@ -2910,14 +2918,14 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Pre-workout scoop</t>
+          <t>Chocolate bar (~50g standard)</t>
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>5</v>
+        <v>245</v>
       </c>
       <c r="C32" s="7" t="n">
-        <v>15</v>
+        <v>250</v>
       </c>
       <c r="D32" s="8">
         <f>AVERAGE(B32:C32)</f>
@@ -2925,10 +2933,56 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
+          <t>~4 g</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>Chocolate bar (70g king-size)</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="n">
+        <v>335</v>
+      </c>
+      <c r="C33" s="7" t="n">
+        <v>335</v>
+      </c>
+      <c r="D33" s="8">
+        <f>AVERAGE(B33:C33)</f>
+        <v/>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>~6 g</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>Pre-workout scoop</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C34" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D34" s="8">
+        <f>AVERAGE(B34:C34)</f>
+        <v/>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
           <t>0 g</t>
         </is>
       </c>
-      <c r="F32" s="6" t="inlineStr">
+      <c r="F34" s="6" t="inlineStr">
         <is>
           <t>Negligible</t>
         </is>

</xml_diff>

<commit_message>
Add reference estimates for the tofu bowl and a chicken curry container
Tofu Delight Bowl at 420-560 kcal for the menu-stated 20 g protein, and a
takeaway chicken curry at 280-420 kcal, 20-28 g. Neither is logged - both
are planned, not eaten.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -2169,7 +2169,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2614,14 +2614,14 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Grilled chicken quarter (skin on)</t>
+          <t>Honest Bowl - Tofu Delight Bowl</t>
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>250</v>
+        <v>420</v>
       </c>
       <c r="C20" s="7" t="n">
-        <v>320</v>
+        <v>560</v>
       </c>
       <c r="D20" s="8">
         <f>AVERAGE(B20:C20)</f>
@@ -2629,26 +2629,26 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>~28-33 g</t>
+          <t>~20 g</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>Skin adds ~12-15 g fat over breast</t>
+          <t>Menu states 20 g; jasmine rice + cajun tofu + grilled eggplant. Half the protein of the chicken bowl at the same price</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Garlic sauce / toum (1 tbsp)</t>
+          <t>Chicken curry (1 takeaway container)</t>
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>90</v>
+        <v>280</v>
       </c>
       <c r="C21" s="7" t="n">
-        <v>110</v>
+        <v>420</v>
       </c>
       <c r="D21" s="8">
         <f>AVERAGE(B21:C21)</f>
@@ -2656,26 +2656,26 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>0 g</t>
+          <t>~20-28 g</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>Essentially emulsified oil - the hidden cost at a grill</t>
+          <t>Kerala style; oil and coconut carry most of the calories</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Khubz / pita (1 large)</t>
+          <t>Grilled chicken quarter (skin on)</t>
         </is>
       </c>
       <c r="B22" s="7" t="n">
         <v>250</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>300</v>
+        <v>320</v>
       </c>
       <c r="D22" s="8">
         <f>AVERAGE(B22:C22)</f>
@@ -2683,22 +2683,26 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>~8-9 g</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr"/>
+          <t>~28-33 g</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>Skin adds ~12-15 g fat over breast</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Barik/basmati rice (half container cooked)</t>
+          <t>Garlic sauce / toum (1 tbsp)</t>
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>200</v>
+        <v>90</v>
       </c>
       <c r="C23" s="7" t="n">
-        <v>280</v>
+        <v>110</v>
       </c>
       <c r="D23" s="8">
         <f>AVERAGE(B23:C23)</f>
@@ -2706,22 +2710,26 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>~4-5 g</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="inlineStr"/>
+          <t>0 g</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>Essentially emulsified oil - the hidden cost at a grill</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Fresh pineapple juice (350-450 ml)</t>
+          <t>Khubz / pita (1 large)</t>
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>175</v>
+        <v>250</v>
       </c>
       <c r="C24" s="7" t="n">
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="D24" s="8">
         <f>AVERAGE(B24:C24)</f>
@@ -2729,26 +2737,22 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>~1-2 g</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>No added sugar but ~35-45 g natural sugar; no fibre; almost no protein</t>
-        </is>
-      </c>
+          <t>~8-9 g</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in water)</t>
+          <t>Barik/basmati rice (half container cooked)</t>
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="C25" s="7" t="n">
-        <v>120</v>
+        <v>280</v>
       </c>
       <c r="D25" s="8">
         <f>AVERAGE(B25:C25)</f>
@@ -2756,7 +2760,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
+          <t>~4-5 g</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr"/>
@@ -2764,14 +2768,14 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Greek yogurt (200 g plain low-fat)</t>
+          <t>Fresh pineapple juice (350-450 ml)</t>
         </is>
       </c>
       <c r="B26" s="7" t="n">
-        <v>120</v>
+        <v>175</v>
       </c>
       <c r="C26" s="7" t="n">
-        <v>140</v>
+        <v>240</v>
       </c>
       <c r="D26" s="8">
         <f>AVERAGE(B26:C26)</f>
@@ -2779,26 +2783,26 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>~18-20 g</t>
+          <t>~1-2 g</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>Casein - digests slowly; good overnight</t>
+          <t>No added sugar but ~35-45 g natural sugar; no fibre; almost no protein</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Boiled egg (1 large)</t>
+          <t>Whey scoop (in water)</t>
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="C27" s="7" t="n">
-        <v>78</v>
+        <v>120</v>
       </c>
       <c r="D27" s="8">
         <f>AVERAGE(B27:C27)</f>
@@ -2806,26 +2810,22 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>~6-6.5 g</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>~5 g fat each</t>
-        </is>
-      </c>
+          <t>~20-25 g</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Paneer (50 g full-fat)</t>
+          <t>Greek yogurt (200 g plain low-fat)</t>
         </is>
       </c>
       <c r="B28" s="7" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="C28" s="7" t="n">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="D28" s="8">
         <f>AVERAGE(B28:C28)</f>
@@ -2833,26 +2833,26 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>~8-9 g</t>
+          <t>~18-20 g</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>Fat-dense for the protein it gives</t>
+          <t>Casein - digests slowly; good overnight</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Cucumber (1 medium)</t>
+          <t>Boiled egg (1 large)</t>
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>25</v>
+        <v>70</v>
       </c>
       <c r="C29" s="7" t="n">
-        <v>30</v>
+        <v>78</v>
       </c>
       <c r="D29" s="8">
         <f>AVERAGE(B29:C29)</f>
@@ -2860,26 +2860,26 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>~1.5 g</t>
+          <t>~6-6.5 g</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>Volume with almost no calories</t>
+          <t>~5 g fat each</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in black coffee no sugar)</t>
+          <t>Paneer (50 g full-fat)</t>
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="C30" s="7" t="n">
-        <v>130</v>
+        <v>150</v>
       </c>
       <c r="D30" s="8">
         <f>AVERAGE(B30:C30)</f>
@@ -2887,22 +2887,26 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="inlineStr"/>
+          <t>~8-9 g</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>Fat-dense for the protein it gives</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Cashew/almond biscuit (1)</t>
+          <t>Cucumber (1 medium)</t>
         </is>
       </c>
       <c r="B31" s="7" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="C31" s="7" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="D31" s="8">
         <f>AVERAGE(B31:C31)</f>
@@ -2910,22 +2914,26 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>~0.5 g</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="inlineStr"/>
+          <t>~1.5 g</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>Volume with almost no calories</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (~50g standard)</t>
+          <t>Whey scoop (in black coffee no sugar)</t>
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>245</v>
+        <v>100</v>
       </c>
       <c r="C32" s="7" t="n">
-        <v>250</v>
+        <v>130</v>
       </c>
       <c r="D32" s="8">
         <f>AVERAGE(B32:C32)</f>
@@ -2933,7 +2941,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>~4 g</t>
+          <t>~20-25 g</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr"/>
@@ -2941,14 +2949,14 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (70g king-size)</t>
+          <t>Cashew/almond biscuit (1)</t>
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>335</v>
+        <v>38</v>
       </c>
       <c r="C33" s="7" t="n">
-        <v>335</v>
+        <v>38</v>
       </c>
       <c r="D33" s="8">
         <f>AVERAGE(B33:C33)</f>
@@ -2956,7 +2964,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>~6 g</t>
+          <t>~0.5 g</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr"/>
@@ -2964,14 +2972,14 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Pre-workout scoop</t>
+          <t>Chocolate bar (~50g standard)</t>
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>5</v>
+        <v>245</v>
       </c>
       <c r="C34" s="7" t="n">
-        <v>15</v>
+        <v>250</v>
       </c>
       <c r="D34" s="8">
         <f>AVERAGE(B34:C34)</f>
@@ -2979,10 +2987,56 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
+          <t>~4 g</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>Chocolate bar (70g king-size)</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="n">
+        <v>335</v>
+      </c>
+      <c r="C35" s="7" t="n">
+        <v>335</v>
+      </c>
+      <c r="D35" s="8">
+        <f>AVERAGE(B35:C35)</f>
+        <v/>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>~6 g</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>Pre-workout scoop</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D36" s="8">
+        <f>AVERAGE(B36:C36)</f>
+        <v/>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
           <t>0 g</t>
         </is>
       </c>
-      <c r="F34" s="6" t="inlineStr">
+      <c r="F36" s="6" t="inlineStr">
         <is>
           <t>Negligible</t>
         </is>

</xml_diff>

<commit_message>
Log Day 3 lunch and dinner, close the day, add three-day trend read
Chicken bowl 550-710 kcal / 42-48 g, tofu bowl 420-560 / 18-22 g, chicken
curry 280-420 / 20-28 g. Day 3 finishes at 1,770-2,490 kcal (mid 2,130),
107 g protein, 85 g fat.

Three complete days now average 2,038 kcal (21 above target, a 529/day
deficit implying 0.48 kg/week), 97.6 g protein and 76.9 g fat. Calories are
on target; protein has plateaued at ~107 g and fat has risen every day.
Rewrote the trends section around the swap that resolves both.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1312,6 +1312,171 @@
       <c r="N17" s="6" t="inlineStr">
         <is>
           <t>Ate 2 of the 3 served - deliberately cut one for calories; costed identically to Day 1 dinner</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Dinner</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Honest Bowl - Tofu Delight Bowl</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>420</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>560</v>
+      </c>
+      <c r="F18" s="8">
+        <f>AVERAGE(D18:E18)</f>
+        <v/>
+      </c>
+      <c r="G18" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="H18" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="I18" s="10">
+        <f>AVERAGE(G18:H18)</f>
+        <v/>
+      </c>
+      <c r="J18" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="K18" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="L18" s="10">
+        <f>AVERAGE(J18:K18)</f>
+        <v/>
+      </c>
+      <c r="M18" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N18" s="6" t="inlineStr">
+        <is>
+          <t>Menu states 20 g protein; jasmine rice + cajun tofu + grilled eggplant</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Dinner</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Chicken curry (1 takeaway container)</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>280</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>420</v>
+      </c>
+      <c r="F19" s="8">
+        <f>AVERAGE(D19:E19)</f>
+        <v/>
+      </c>
+      <c r="G19" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="H19" s="9" t="n">
+        <v>28</v>
+      </c>
+      <c r="I19" s="10">
+        <f>AVERAGE(G19:H19)</f>
+        <v/>
+      </c>
+      <c r="J19" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="K19" s="9" t="n">
+        <v>26</v>
+      </c>
+      <c r="L19" s="10">
+        <f>AVERAGE(J19:K19)</f>
+        <v/>
+      </c>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N19" s="6" t="inlineStr">
+        <is>
+          <t>Eaten alongside the tofu bowl</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Honest Bowl - Grilled Chicken and Rice Bowl</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>550</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>710</v>
+      </c>
+      <c r="F20" s="8">
+        <f>AVERAGE(D20:E20)</f>
+        <v/>
+      </c>
+      <c r="G20" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="I20" s="10">
+        <f>AVERAGE(G20:H20)</f>
+        <v/>
+      </c>
+      <c r="J20" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="K20" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="L20" s="10">
+        <f>AVERAGE(J20:K20)</f>
+        <v/>
+      </c>
+      <c r="M20" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N20" s="6" t="inlineStr">
+        <is>
+          <t>Menu states 42 g protein; chicken + jasmine rice + sweet potato</t>
         </is>
       </c>
     </row>
@@ -1433,11 +1598,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$17,Meals!$A$5:$A$17,$A5,Meals!$M$5:$M$17,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$20,Meals!$A$5:$A$20,$A5,Meals!$M$5:$M$20,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$17,Meals!$A$5:$A$17,$A5,Meals!$M$5:$M$17,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$20,Meals!$A$5:$A$20,$A5,Meals!$M$5:$M$20,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -1445,11 +1610,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$17,Meals!$A$5:$A$17,$A5,Meals!$M$5:$M$17,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$20,Meals!$A$5:$A$20,$A5,Meals!$M$5:$M$20,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$17,Meals!$A$5:$A$17,$A5,Meals!$M$5:$M$17,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$20,Meals!$A$5:$A$20,$A5,Meals!$M$5:$M$20,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -1457,11 +1622,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$17,Meals!$A$5:$A$17,$A5,Meals!$M$5:$M$17,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$20,Meals!$A$5:$A$20,$A5,Meals!$M$5:$M$20,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$17,Meals!$A$5:$A$17,$A5,Meals!$M$5:$M$17,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$20,Meals!$A$5:$A$20,$A5,Meals!$M$5:$M$20,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -1469,11 +1634,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$17,$A5,Meals!$M$5:$M$17,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$20,$A5,Meals!$M$5:$M$20,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$17,$A5,Meals!$M$5:$M$17,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$20,$A5,Meals!$M$5:$M$20,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -1486,11 +1651,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$17,Meals!$A$5:$A$17,$A6,Meals!$M$5:$M$17,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$20,Meals!$A$5:$A$20,$A6,Meals!$M$5:$M$20,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$17,Meals!$A$5:$A$17,$A6,Meals!$M$5:$M$17,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$20,Meals!$A$5:$A$20,$A6,Meals!$M$5:$M$20,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -1498,11 +1663,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$17,Meals!$A$5:$A$17,$A6,Meals!$M$5:$M$17,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$20,Meals!$A$5:$A$20,$A6,Meals!$M$5:$M$20,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$17,Meals!$A$5:$A$17,$A6,Meals!$M$5:$M$17,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$20,Meals!$A$5:$A$20,$A6,Meals!$M$5:$M$20,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -1510,11 +1675,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$17,Meals!$A$5:$A$17,$A6,Meals!$M$5:$M$17,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$20,Meals!$A$5:$A$20,$A6,Meals!$M$5:$M$20,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$17,Meals!$A$5:$A$17,$A6,Meals!$M$5:$M$17,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$20,Meals!$A$5:$A$20,$A6,Meals!$M$5:$M$20,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -1522,11 +1687,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$17,$A6,Meals!$M$5:$M$17,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$20,$A6,Meals!$M$5:$M$20,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$17,$A6,Meals!$M$5:$M$17,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$20,$A6,Meals!$M$5:$M$20,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -1539,11 +1704,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$17,Meals!$A$5:$A$17,$A7,Meals!$M$5:$M$17,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$20,Meals!$A$5:$A$20,$A7,Meals!$M$5:$M$20,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$17,Meals!$A$5:$A$17,$A7,Meals!$M$5:$M$17,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$20,Meals!$A$5:$A$20,$A7,Meals!$M$5:$M$20,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -1551,11 +1716,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$17,Meals!$A$5:$A$17,$A7,Meals!$M$5:$M$17,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$20,Meals!$A$5:$A$20,$A7,Meals!$M$5:$M$20,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$17,Meals!$A$5:$A$17,$A7,Meals!$M$5:$M$17,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$20,Meals!$A$5:$A$20,$A7,Meals!$M$5:$M$20,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -1563,11 +1728,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$17,Meals!$A$5:$A$17,$A7,Meals!$M$5:$M$17,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$20,Meals!$A$5:$A$20,$A7,Meals!$M$5:$M$20,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$17,Meals!$A$5:$A$17,$A7,Meals!$M$5:$M$17,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$20,Meals!$A$5:$A$20,$A7,Meals!$M$5:$M$20,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -1575,11 +1740,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$17,$A7,Meals!$M$5:$M$17,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$20,$A7,Meals!$M$5:$M$20,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$17,$A7,Meals!$M$5:$M$17,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$20,$A7,Meals!$M$5:$M$20,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">

</xml_diff>

<commit_message>
Log orange juice on Day 3
155-205 kcal, 2-3 g protein, ~32-40 g natural sugar. Day 3 closes at
1,925-2,695 kcal (mid 2,310), 109.5 g protein, 85.25 g fat.

Three-day average moves to 2,098 kcal (81 above target, 0.43 kg/week) with
protein 98.4 g and fat 77.0 g. Second juice in three days; noted the
combined cost in the Day 3 notes.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1477,6 +1477,61 @@
       <c r="N20" s="6" t="inlineStr">
         <is>
           <t>Menu states 42 g protein; chicken + jasmine rice + sweet potato</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Fresh orange juice (~350-450 ml) - no added sugar</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>155</v>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>205</v>
+      </c>
+      <c r="F21" s="8">
+        <f>AVERAGE(D21:E21)</f>
+        <v/>
+      </c>
+      <c r="G21" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H21" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I21" s="10">
+        <f>AVERAGE(G21:H21)</f>
+        <v/>
+      </c>
+      <c r="J21" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L21" s="10">
+        <f>AVERAGE(J21:K21)</f>
+        <v/>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N21" s="6" t="inlineStr">
+        <is>
+          <t>Second juice in three days; ~32-40 g natural sugar</t>
         </is>
       </c>
     </row>
@@ -1598,11 +1653,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$20,Meals!$A$5:$A$20,$A5,Meals!$M$5:$M$20,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$21,Meals!$A$5:$A$21,$A5,Meals!$M$5:$M$21,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$20,Meals!$A$5:$A$20,$A5,Meals!$M$5:$M$20,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$21,Meals!$A$5:$A$21,$A5,Meals!$M$5:$M$21,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -1610,11 +1665,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$20,Meals!$A$5:$A$20,$A5,Meals!$M$5:$M$20,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$21,Meals!$A$5:$A$21,$A5,Meals!$M$5:$M$21,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$20,Meals!$A$5:$A$20,$A5,Meals!$M$5:$M$20,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$21,Meals!$A$5:$A$21,$A5,Meals!$M$5:$M$21,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -1622,11 +1677,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$20,Meals!$A$5:$A$20,$A5,Meals!$M$5:$M$20,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$21,Meals!$A$5:$A$21,$A5,Meals!$M$5:$M$21,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$20,Meals!$A$5:$A$20,$A5,Meals!$M$5:$M$20,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$21,Meals!$A$5:$A$21,$A5,Meals!$M$5:$M$21,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -1634,11 +1689,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$20,$A5,Meals!$M$5:$M$20,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$21,$A5,Meals!$M$5:$M$21,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$20,$A5,Meals!$M$5:$M$20,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$21,$A5,Meals!$M$5:$M$21,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -1651,11 +1706,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$20,Meals!$A$5:$A$20,$A6,Meals!$M$5:$M$20,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$21,Meals!$A$5:$A$21,$A6,Meals!$M$5:$M$21,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$20,Meals!$A$5:$A$20,$A6,Meals!$M$5:$M$20,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$21,Meals!$A$5:$A$21,$A6,Meals!$M$5:$M$21,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -1663,11 +1718,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$20,Meals!$A$5:$A$20,$A6,Meals!$M$5:$M$20,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$21,Meals!$A$5:$A$21,$A6,Meals!$M$5:$M$21,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$20,Meals!$A$5:$A$20,$A6,Meals!$M$5:$M$20,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$21,Meals!$A$5:$A$21,$A6,Meals!$M$5:$M$21,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -1675,11 +1730,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$20,Meals!$A$5:$A$20,$A6,Meals!$M$5:$M$20,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$21,Meals!$A$5:$A$21,$A6,Meals!$M$5:$M$21,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$20,Meals!$A$5:$A$20,$A6,Meals!$M$5:$M$20,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$21,Meals!$A$5:$A$21,$A6,Meals!$M$5:$M$21,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -1687,11 +1742,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$20,$A6,Meals!$M$5:$M$20,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$21,$A6,Meals!$M$5:$M$21,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$20,$A6,Meals!$M$5:$M$20,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$21,$A6,Meals!$M$5:$M$21,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -1704,11 +1759,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$20,Meals!$A$5:$A$20,$A7,Meals!$M$5:$M$20,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$21,Meals!$A$5:$A$21,$A7,Meals!$M$5:$M$21,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$20,Meals!$A$5:$A$20,$A7,Meals!$M$5:$M$20,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$21,Meals!$A$5:$A$21,$A7,Meals!$M$5:$M$21,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -1716,11 +1771,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$20,Meals!$A$5:$A$20,$A7,Meals!$M$5:$M$20,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$21,Meals!$A$5:$A$21,$A7,Meals!$M$5:$M$21,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$20,Meals!$A$5:$A$20,$A7,Meals!$M$5:$M$20,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$21,Meals!$A$5:$A$21,$A7,Meals!$M$5:$M$21,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -1728,11 +1783,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$20,Meals!$A$5:$A$20,$A7,Meals!$M$5:$M$20,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$21,Meals!$A$5:$A$21,$A7,Meals!$M$5:$M$21,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$20,Meals!$A$5:$A$20,$A7,Meals!$M$5:$M$20,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$21,Meals!$A$5:$A$21,$A7,Meals!$M$5:$M$21,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -1740,11 +1795,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$20,$A7,Meals!$M$5:$M$20,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$21,$A7,Meals!$M$5:$M$21,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$20,$A7,Meals!$M$5:$M$20,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$21,$A7,Meals!$M$5:$M$21,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -2334,7 +2389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2960,14 +3015,14 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in water)</t>
+          <t>Fresh orange juice (350-450 ml)</t>
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>100</v>
+        <v>155</v>
       </c>
       <c r="C27" s="7" t="n">
-        <v>120</v>
+        <v>205</v>
       </c>
       <c r="D27" s="8">
         <f>AVERAGE(B27:C27)</f>
@@ -2975,22 +3030,26 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr"/>
+          <t>~2-3 g</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>No added sugar but ~32-40 g natural sugar; no fibre</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Greek yogurt (200 g plain low-fat)</t>
+          <t>Whey scoop (in water)</t>
         </is>
       </c>
       <c r="B28" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C28" s="7" t="n">
         <v>120</v>
-      </c>
-      <c r="C28" s="7" t="n">
-        <v>140</v>
       </c>
       <c r="D28" s="8">
         <f>AVERAGE(B28:C28)</f>
@@ -2998,26 +3057,22 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>~18-20 g</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>Casein - digests slowly; good overnight</t>
-        </is>
-      </c>
+          <t>~20-25 g</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Boiled egg (1 large)</t>
+          <t>Greek yogurt (200 g plain low-fat)</t>
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>70</v>
+        <v>120</v>
       </c>
       <c r="C29" s="7" t="n">
-        <v>78</v>
+        <v>140</v>
       </c>
       <c r="D29" s="8">
         <f>AVERAGE(B29:C29)</f>
@@ -3025,26 +3080,26 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>~6-6.5 g</t>
+          <t>~18-20 g</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>~5 g fat each</t>
+          <t>Casein - digests slowly; good overnight</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Paneer (50 g full-fat)</t>
+          <t>Boiled egg (1 large)</t>
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>130</v>
+        <v>70</v>
       </c>
       <c r="C30" s="7" t="n">
-        <v>150</v>
+        <v>78</v>
       </c>
       <c r="D30" s="8">
         <f>AVERAGE(B30:C30)</f>
@@ -3052,26 +3107,26 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>~8-9 g</t>
+          <t>~6-6.5 g</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>Fat-dense for the protein it gives</t>
+          <t>~5 g fat each</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Cucumber (1 medium)</t>
+          <t>Paneer (50 g full-fat)</t>
         </is>
       </c>
       <c r="B31" s="7" t="n">
-        <v>25</v>
+        <v>130</v>
       </c>
       <c r="C31" s="7" t="n">
-        <v>30</v>
+        <v>150</v>
       </c>
       <c r="D31" s="8">
         <f>AVERAGE(B31:C31)</f>
@@ -3079,26 +3134,26 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>~1.5 g</t>
+          <t>~8-9 g</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>Volume with almost no calories</t>
+          <t>Fat-dense for the protein it gives</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in black coffee no sugar)</t>
+          <t>Cucumber (1 medium)</t>
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="C32" s="7" t="n">
-        <v>130</v>
+        <v>30</v>
       </c>
       <c r="D32" s="8">
         <f>AVERAGE(B32:C32)</f>
@@ -3106,22 +3161,26 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="inlineStr"/>
+          <t>~1.5 g</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>Volume with almost no calories</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Cashew/almond biscuit (1)</t>
+          <t>Whey scoop (in black coffee no sugar)</t>
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C33" s="7" t="n">
-        <v>38</v>
+        <v>130</v>
       </c>
       <c r="D33" s="8">
         <f>AVERAGE(B33:C33)</f>
@@ -3129,7 +3188,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>~0.5 g</t>
+          <t>~20-25 g</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr"/>
@@ -3137,14 +3196,14 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (~50g standard)</t>
+          <t>Cashew/almond biscuit (1)</t>
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>245</v>
+        <v>38</v>
       </c>
       <c r="C34" s="7" t="n">
-        <v>250</v>
+        <v>38</v>
       </c>
       <c r="D34" s="8">
         <f>AVERAGE(B34:C34)</f>
@@ -3152,7 +3211,7 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>~4 g</t>
+          <t>~0.5 g</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr"/>
@@ -3160,14 +3219,14 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (70g king-size)</t>
+          <t>Chocolate bar (~50g standard)</t>
         </is>
       </c>
       <c r="B35" s="7" t="n">
-        <v>335</v>
+        <v>245</v>
       </c>
       <c r="C35" s="7" t="n">
-        <v>335</v>
+        <v>250</v>
       </c>
       <c r="D35" s="8">
         <f>AVERAGE(B35:C35)</f>
@@ -3175,7 +3234,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>~6 g</t>
+          <t>~4 g</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr"/>
@@ -3183,14 +3242,14 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Pre-workout scoop</t>
+          <t>Chocolate bar (70g king-size)</t>
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>5</v>
+        <v>335</v>
       </c>
       <c r="C36" s="7" t="n">
-        <v>15</v>
+        <v>335</v>
       </c>
       <c r="D36" s="8">
         <f>AVERAGE(B36:C36)</f>
@@ -3198,10 +3257,33 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
+          <t>~6 g</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>Pre-workout scoop</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C37" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D37" s="8">
+        <f>AVERAGE(B37:C37)</f>
+        <v/>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
           <t>0 g</t>
         </is>
       </c>
-      <c r="F36" s="6" t="inlineStr">
+      <c r="F37" s="6" t="inlineStr">
         <is>
           <t>Negligible</t>
         </is>

</xml_diff>

<commit_message>
Add weigh-in tracking and link targets to the latest weight
New weights.csv and a Weights sheet with per-weigh-in change, change since
start and a 7-day trailing average. The Targets sheet's weight cell is now
a formula reading the last entry, so a new weigh-in re-derives BMR,
maintenance, the calorie target and the carb allowance.

First two weigh-ins: 91.5 kg on 09-05, 90.75 kg on 09-07. At 90.75 kg the
target moves from 2,017 to 2,007 kcal.

The 0.75 kg drop is not 0.75 kg of fat - the deficit over the two days the
scale covers accounts for 0.084 kg, so ~89% is water and glycogen. Noted in
the log, and the activity multiplier deliberately left at 1.45.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -9,9 +9,10 @@
   <sheets>
     <sheet name="Meals" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Daily" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Trends" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Targets" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Reference" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Weights" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Trends" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Targets" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Reference" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,12 +21,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="+#,##0;-#,##0;0"/>
+    <numFmt numFmtId="167" formatCode="+0.00;-0.00;0.00"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -67,6 +69,11 @@
     </font>
     <font>
       <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00008000"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -119,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -152,10 +159,13 @@
     <xf numFmtId="3" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1821,6 +1831,131 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Weigh-ins</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Weigh same time, same conditions - first thing, after the toilet, before food or drink. Add a row per weigh-in; the Targets sheet reads the latest entry automatically. Read the trailing average, not the raw number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Weight (kg)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Since start</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Trailing avg (7)</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B5" s="24" t="n">
+        <v>91.5</v>
+      </c>
+      <c r="C5" s="25" t="inlineStr"/>
+      <c r="D5" s="25">
+        <f>B5-$B$5</f>
+        <v/>
+      </c>
+      <c r="E5" s="26">
+        <f>AVERAGE(B5:B5)</f>
+        <v/>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Starting weight - stated by user</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B6" s="24" t="n">
+        <v>90.75</v>
+      </c>
+      <c r="C6" s="25">
+        <f>B6-B5</f>
+        <v/>
+      </c>
+      <c r="D6" s="25">
+        <f>B6-$B$5</f>
+        <v/>
+      </c>
+      <c r="E6" s="26">
+        <f>AVERAGE(B5:B6)</f>
+        <v/>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Morning weigh-in</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="27" t="inlineStr">
+        <is>
+          <t>A drop in the first week is mostly water and glycogen, not fat. Judge the trend over 2-3 weeks, and change the activity multiplier on Targets only then.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1840,21 +1975,21 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="24" t="inlineStr">
+      <c r="A2" s="27" t="inlineStr">
         <is>
           <t>Targets come from the Targets sheet - change them there, not here.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="25" t="inlineStr">
+      <c r="A4" s="28" t="inlineStr">
         <is>
           <t>Overall</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="26" t="inlineStr">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>Days logged</t>
         </is>
@@ -1865,7 +2000,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="26" t="inlineStr">
+      <c r="A6" s="29" t="inlineStr">
         <is>
           <t>Avg calories/day (mid)</t>
         </is>
@@ -1876,7 +2011,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="A7" s="29" t="inlineStr">
         <is>
           <t>Avg protein/day (mid, g)</t>
         </is>
@@ -1887,7 +2022,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="26" t="inlineStr">
+      <c r="A8" s="29" t="inlineStr">
         <is>
           <t>Avg fat/day (mid, g)</t>
         </is>
@@ -1898,7 +2033,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="26" t="inlineStr">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>Avg vs calorie target</t>
         </is>
@@ -1909,7 +2044,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="26" t="inlineStr">
+      <c r="A10" s="29" t="inlineStr">
         <is>
           <t>Avg deficit vs maintenance</t>
         </is>
@@ -1920,18 +2055,18 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="26" t="inlineStr">
+      <c r="A11" s="29" t="inlineStr">
         <is>
           <t>Implied loss (kg/week)</t>
         </is>
       </c>
-      <c r="B11" s="27">
+      <c r="B11" s="26">
         <f>IFERROR((Targets!$B$15-B6)*7/Targets!$B$11,0)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="26" t="inlineStr">
+      <c r="A12" s="29" t="inlineStr">
         <is>
           <t>Days hitting protein target</t>
         </is>
@@ -1942,7 +2077,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="26" t="inlineStr">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>Total pending (unconfirmed) items</t>
         </is>
@@ -1953,7 +2088,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="25" t="inlineStr">
+      <c r="A15" s="28" t="inlineStr">
         <is>
           <t>Weekly (week starting Monday)</t>
         </is>
@@ -2016,7 +2151,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="25" t="inlineStr">
+      <c r="A19" s="28" t="inlineStr">
         <is>
           <t>Monthly</t>
         </is>
@@ -2079,7 +2214,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="24" t="inlineStr">
+      <c r="A23" s="27" t="inlineStr">
         <is>
           <t>Averages cover only the days present in the log; a part-logged day (today's dinner still to come) drags its average down.</t>
         </is>
@@ -2090,7 +2225,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2119,29 +2254,30 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="25" t="inlineStr">
+      <c r="A4" s="28" t="inlineStr">
         <is>
           <t>Inputs</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="26" t="inlineStr">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>Weight (kg)</t>
         </is>
       </c>
-      <c r="B5" s="16" t="n">
-        <v>91.5</v>
-      </c>
-      <c r="C5" s="28" t="inlineStr">
-        <is>
-          <t>Source: stated by user, 2026-09-05. Update as it changes.</t>
+      <c r="B5" s="30">
+        <f>INDEX(Weights!$B$5:$B$500,COUNT(Weights!$B$5:$B$500))</f>
+        <v/>
+      </c>
+      <c r="C5" s="31" t="inlineStr">
+        <is>
+          <t>Latest entry on the Weights sheet - add a weigh-in there and everything below re-derives. Do not type over it.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="26" t="inlineStr">
+      <c r="A6" s="29" t="inlineStr">
         <is>
           <t>Height (cm)</t>
         </is>
@@ -2149,59 +2285,59 @@
       <c r="B6" s="16" t="n">
         <v>162.5</v>
       </c>
-      <c r="C6" s="28" t="inlineStr">
+      <c r="C6" s="31" t="inlineStr">
         <is>
           <t>Source: stated by user.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="A7" s="29" t="inlineStr">
         <is>
           <t>Age (years)</t>
         </is>
       </c>
-      <c r="B7" s="29" t="n">
+      <c r="B7" s="32" t="n">
         <v>33</v>
       </c>
-      <c r="C7" s="28" t="inlineStr">
+      <c r="C7" s="31" t="inlineStr">
         <is>
           <t>Source: stated by user (turns 33 on 2026-09-15).</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="26" t="inlineStr">
+      <c r="A8" s="29" t="inlineStr">
         <is>
           <t>Sex constant</t>
         </is>
       </c>
-      <c r="B8" s="29" t="n">
+      <c r="B8" s="32" t="n">
         <v>5</v>
       </c>
-      <c r="C8" s="28" t="inlineStr">
+      <c r="C8" s="31" t="inlineStr">
         <is>
           <t>Mifflin-St Jeor term: +5 male, -161 female.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="26" t="inlineStr">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>Activity multiplier</t>
         </is>
       </c>
-      <c r="B9" s="30" t="n">
+      <c r="B9" s="33" t="n">
         <v>1.45</v>
       </c>
-      <c r="C9" s="28" t="inlineStr">
+      <c r="C9" s="31" t="inlineStr">
         <is>
           <t>1.45 = desk job plus 6 lifting sessions/week. Lifting burns less than cardio-based charts assume; raise it only if the scale says so.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="26" t="inlineStr">
+      <c r="A10" s="29" t="inlineStr">
         <is>
           <t>Daily deficit (kcal)</t>
         </is>
@@ -2209,14 +2345,14 @@
       <c r="B10" s="14" t="n">
         <v>550</v>
       </c>
-      <c r="C10" s="28" t="inlineStr">
+      <c r="C10" s="31" t="inlineStr">
         <is>
           <t>550/day = 0.5 kg/week. Assumption, not a measurement.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="26" t="inlineStr">
+      <c r="A11" s="29" t="inlineStr">
         <is>
           <t>kcal per kg of body fat</t>
         </is>
@@ -2224,21 +2360,21 @@
       <c r="B11" s="14" t="n">
         <v>7700</v>
       </c>
-      <c r="C11" s="28" t="inlineStr">
+      <c r="C11" s="31" t="inlineStr">
         <is>
           <t>Standard 7,700 kcal/kg conversion.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="25" t="inlineStr">
+      <c r="A13" s="28" t="inlineStr">
         <is>
           <t>Derived</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="26" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>BMR (Mifflin-St Jeor)</t>
         </is>
@@ -2247,14 +2383,14 @@
         <f>10*B5+6.25*B6-5*B7+B8</f>
         <v/>
       </c>
-      <c r="C14" s="28" t="inlineStr">
+      <c r="C14" s="31" t="inlineStr">
         <is>
           <t>Resting burn: what the body uses doing nothing.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="26" t="inlineStr">
+      <c r="A15" s="29" t="inlineStr">
         <is>
           <t>Maintenance (TDEE)</t>
         </is>
@@ -2263,41 +2399,41 @@
         <f>B14*B9</f>
         <v/>
       </c>
-      <c r="C15" s="28" t="inlineStr">
+      <c r="C15" s="31" t="inlineStr">
         <is>
           <t>Estimate. The scale over 2-3 weeks is the real measurement.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="25" t="inlineStr">
+      <c r="A16" s="28" t="inlineStr">
         <is>
           <t>CALORIE TARGET</t>
         </is>
       </c>
-      <c r="B16" s="31">
+      <c r="B16" s="34">
         <f>B15-B10</f>
         <v/>
       </c>
-      <c r="C16" s="28" t="inlineStr">
+      <c r="C16" s="31" t="inlineStr">
         <is>
           <t>The number to eat.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="26" t="inlineStr">
+      <c r="A17" s="29" t="inlineStr">
         <is>
           <t>Projected loss (kg/week)</t>
         </is>
       </c>
-      <c r="B17" s="27">
+      <c r="B17" s="26">
         <f>B10*7/B11</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="26" t="inlineStr">
+      <c r="A18" s="29" t="inlineStr">
         <is>
           <t>BMI</t>
         </is>
@@ -2306,61 +2442,61 @@
         <f>B5/(B6/100)^2</f>
         <v/>
       </c>
-      <c r="C18" s="28" t="inlineStr">
+      <c r="C18" s="31" t="inlineStr">
         <is>
           <t>Worth a GP or dietitian check alongside this plan.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="25" t="inlineStr">
+      <c r="A20" s="28" t="inlineStr">
         <is>
           <t>Macros at the calorie target</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="26" t="inlineStr">
+      <c r="A21" s="29" t="inlineStr">
         <is>
           <t>Protein target low (g)</t>
         </is>
       </c>
-      <c r="B21" s="29" t="n">
+      <c r="B21" s="32" t="n">
         <v>130</v>
       </c>
-      <c r="C21" s="28" t="inlineStr">
+      <c r="C21" s="31" t="inlineStr">
         <is>
           <t>~2.1 g/kg of estimated lean mass - the level that protects muscle in a deficit while training 6 days.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="26" t="inlineStr">
+      <c r="A22" s="29" t="inlineStr">
         <is>
           <t>Protein target high (g)</t>
         </is>
       </c>
-      <c r="B22" s="29" t="n">
+      <c r="B22" s="32" t="n">
         <v>145</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="26" t="inlineStr">
+      <c r="A23" s="29" t="inlineStr">
         <is>
           <t>Fat floor (g)</t>
         </is>
       </c>
-      <c r="B23" s="29" t="n">
+      <c r="B23" s="32" t="n">
         <v>55</v>
       </c>
-      <c r="C23" s="28" t="inlineStr">
+      <c r="C23" s="31" t="inlineStr">
         <is>
           <t>~0.6 g/kg. A floor for hormone health, not a goal to hit.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="26" t="inlineStr">
+      <c r="A24" s="29" t="inlineStr">
         <is>
           <t>Carb allowance (g)</t>
         </is>
@@ -2369,7 +2505,7 @@
         <f>(B16-B21*4-B23*9)/4</f>
         <v/>
       </c>
-      <c r="C24" s="28" t="inlineStr">
+      <c r="C24" s="31" t="inlineStr">
         <is>
           <t>Whatever is left once protein and the fat floor are paid for. Fuels the PPL work.</t>
         </is>
@@ -2383,7 +2519,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Log Day 4 breakfast: 2 appam with potato bhaji
390-520 kcal (mid 455), 8-11 g protein, 10-18 g fat - the lightest
breakfast in the log, 205 kcal and 16 g of fat below yesterday's.

Adds a four-day breakfast comparison: every breakfast so far sits under
3 g of protein per 100 kcal, averaging 12 g, which is the structural
reason no day has reached the 130 g floor.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -537,7 +537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1545,6 +1545,61 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Breakfast</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>2 appam + potato curry (bhaji)</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="n">
+        <v>390</v>
+      </c>
+      <c r="E22" s="7" t="n">
+        <v>520</v>
+      </c>
+      <c r="F22" s="8">
+        <f>AVERAGE(D22:E22)</f>
+        <v/>
+      </c>
+      <c r="G22" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="H22" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="I22" s="10">
+        <f>AVERAGE(G22:H22)</f>
+        <v/>
+      </c>
+      <c r="J22" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="K22" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="L22" s="10">
+        <f>AVERAGE(J22:K22)</f>
+        <v/>
+      </c>
+      <c r="M22" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N22" s="6" t="inlineStr">
+        <is>
+          <t>Lightest breakfast in the log by calories; fourth straight breakfast under 20 g protein</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:N2"/>
@@ -1559,7 +1614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1663,11 +1718,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$21,Meals!$A$5:$A$21,$A5,Meals!$M$5:$M$21,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$22,Meals!$A$5:$A$22,$A5,Meals!$M$5:$M$22,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$21,Meals!$A$5:$A$21,$A5,Meals!$M$5:$M$21,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$22,Meals!$A$5:$A$22,$A5,Meals!$M$5:$M$22,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -1675,11 +1730,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$21,Meals!$A$5:$A$21,$A5,Meals!$M$5:$M$21,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$22,Meals!$A$5:$A$22,$A5,Meals!$M$5:$M$22,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$21,Meals!$A$5:$A$21,$A5,Meals!$M$5:$M$21,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$22,Meals!$A$5:$A$22,$A5,Meals!$M$5:$M$22,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -1687,11 +1742,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$21,Meals!$A$5:$A$21,$A5,Meals!$M$5:$M$21,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$22,Meals!$A$5:$A$22,$A5,Meals!$M$5:$M$22,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$21,Meals!$A$5:$A$21,$A5,Meals!$M$5:$M$21,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$22,Meals!$A$5:$A$22,$A5,Meals!$M$5:$M$22,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -1699,11 +1754,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$21,$A5,Meals!$M$5:$M$21,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$22,$A5,Meals!$M$5:$M$22,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$21,$A5,Meals!$M$5:$M$21,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$22,$A5,Meals!$M$5:$M$22,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -1716,11 +1771,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$21,Meals!$A$5:$A$21,$A6,Meals!$M$5:$M$21,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$22,Meals!$A$5:$A$22,$A6,Meals!$M$5:$M$22,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$21,Meals!$A$5:$A$21,$A6,Meals!$M$5:$M$21,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$22,Meals!$A$5:$A$22,$A6,Meals!$M$5:$M$22,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -1728,11 +1783,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$21,Meals!$A$5:$A$21,$A6,Meals!$M$5:$M$21,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$22,Meals!$A$5:$A$22,$A6,Meals!$M$5:$M$22,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$21,Meals!$A$5:$A$21,$A6,Meals!$M$5:$M$21,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$22,Meals!$A$5:$A$22,$A6,Meals!$M$5:$M$22,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -1740,11 +1795,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$21,Meals!$A$5:$A$21,$A6,Meals!$M$5:$M$21,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$22,Meals!$A$5:$A$22,$A6,Meals!$M$5:$M$22,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$21,Meals!$A$5:$A$21,$A6,Meals!$M$5:$M$21,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$22,Meals!$A$5:$A$22,$A6,Meals!$M$5:$M$22,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -1752,11 +1807,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$21,$A6,Meals!$M$5:$M$21,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$22,$A6,Meals!$M$5:$M$22,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$21,$A6,Meals!$M$5:$M$21,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$22,$A6,Meals!$M$5:$M$22,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -1769,11 +1824,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$21,Meals!$A$5:$A$21,$A7,Meals!$M$5:$M$21,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$22,Meals!$A$5:$A$22,$A7,Meals!$M$5:$M$22,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$21,Meals!$A$5:$A$21,$A7,Meals!$M$5:$M$21,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$22,Meals!$A$5:$A$22,$A7,Meals!$M$5:$M$22,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -1781,11 +1836,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$21,Meals!$A$5:$A$21,$A7,Meals!$M$5:$M$21,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$22,Meals!$A$5:$A$22,$A7,Meals!$M$5:$M$22,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$21,Meals!$A$5:$A$21,$A7,Meals!$M$5:$M$21,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$22,Meals!$A$5:$A$22,$A7,Meals!$M$5:$M$22,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -1793,11 +1848,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$21,Meals!$A$5:$A$21,$A7,Meals!$M$5:$M$21,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$22,Meals!$A$5:$A$22,$A7,Meals!$M$5:$M$22,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$21,Meals!$A$5:$A$21,$A7,Meals!$M$5:$M$21,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$22,Meals!$A$5:$A$22,$A7,Meals!$M$5:$M$22,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -1805,15 +1860,68 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$21,$A7,Meals!$M$5:$M$21,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$22,$A7,Meals!$M$5:$M$22,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$21,$A7,Meals!$M$5:$M$21,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$22,$A7,Meals!$M$5:$M$22,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
         <f>D7-Targets!$B$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="20" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B8" s="21">
+        <f>SUMIFS(Meals!$D$5:$D$22,Meals!$A$5:$A$22,$A8,Meals!$M$5:$M$22,"logged")</f>
+        <v/>
+      </c>
+      <c r="C8" s="21">
+        <f>SUMIFS(Meals!$E$5:$E$22,Meals!$A$5:$A$22,$A8,Meals!$M$5:$M$22,"logged")</f>
+        <v/>
+      </c>
+      <c r="D8" s="21">
+        <f>AVERAGE(B8:C8)</f>
+        <v/>
+      </c>
+      <c r="E8" s="22">
+        <f>SUMIFS(Meals!$G$5:$G$22,Meals!$A$5:$A$22,$A8,Meals!$M$5:$M$22,"logged")</f>
+        <v/>
+      </c>
+      <c r="F8" s="22">
+        <f>SUMIFS(Meals!$H$5:$H$22,Meals!$A$5:$A$22,$A8,Meals!$M$5:$M$22,"logged")</f>
+        <v/>
+      </c>
+      <c r="G8" s="22">
+        <f>AVERAGE(E8:F8)</f>
+        <v/>
+      </c>
+      <c r="H8" s="22">
+        <f>SUMIFS(Meals!$J$5:$J$22,Meals!$A$5:$A$22,$A8,Meals!$M$5:$M$22,"logged")</f>
+        <v/>
+      </c>
+      <c r="I8" s="22">
+        <f>SUMIFS(Meals!$K$5:$K$22,Meals!$A$5:$A$22,$A8,Meals!$M$5:$M$22,"logged")</f>
+        <v/>
+      </c>
+      <c r="J8" s="22">
+        <f>AVERAGE(H8:I8)</f>
+        <v/>
+      </c>
+      <c r="K8" s="20">
+        <f>COUNTIFS(Meals!$A$5:$A$22,$A8,Meals!$M$5:$M$22,"logged")</f>
+        <v/>
+      </c>
+      <c r="L8" s="20">
+        <f>COUNTIFS(Meals!$A$5:$A$22,$A8,Meals!$M$5:$M$22,"pending")</f>
+        <v/>
+      </c>
+      <c r="M8" s="23">
+        <f>D8-Targets!$B$16</f>
         <v/>
       </c>
     </row>
@@ -1956,7 +2064,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1995,7 +2103,7 @@
         </is>
       </c>
       <c r="B5" s="18">
-        <f>COUNT(Daily!$A$5:$A$7)</f>
+        <f>COUNT(Daily!$A$5:$A$8)</f>
         <v/>
       </c>
     </row>
@@ -2006,7 +2114,7 @@
         </is>
       </c>
       <c r="B6" s="8">
-        <f>IFERROR(AVERAGE(Daily!$D$5:$D$7),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$D$5:$D$8),0)</f>
         <v/>
       </c>
     </row>
@@ -2017,7 +2125,7 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>IFERROR(AVERAGE(Daily!$G$5:$G$7),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$G$5:$G$8),0)</f>
         <v/>
       </c>
     </row>
@@ -2028,7 +2136,7 @@
         </is>
       </c>
       <c r="B8" s="10">
-        <f>IFERROR(AVERAGE(Daily!$J$5:$J$7),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$J$5:$J$8),0)</f>
         <v/>
       </c>
     </row>
@@ -2072,7 +2180,7 @@
         </is>
       </c>
       <c r="B12" s="18">
-        <f>COUNTIFS(Daily!$G$5:$G$7,"&gt;="&amp;Targets!$B$20)</f>
+        <f>COUNTIFS(Daily!$G$5:$G$8,"&gt;="&amp;Targets!$B$20)</f>
         <v/>
       </c>
     </row>
@@ -2083,7 +2191,7 @@
         </is>
       </c>
       <c r="B13" s="18">
-        <f>SUM(Daily!$L$5:$L$7)</f>
+        <f>SUM(Daily!$L$5:$L$8)</f>
         <v/>
       </c>
     </row>
@@ -2134,87 +2242,111 @@
         <v>46271</v>
       </c>
       <c r="C17" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$7,"&gt;="&amp;$A17,Daily!$A$5:$A$7,"&lt;="&amp;$B17)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$8,"&gt;="&amp;$A17,Daily!$A$5:$A$8,"&lt;="&amp;$B17)</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$7,Daily!$A$5:$A$7,"&gt;="&amp;$A17,Daily!$A$5:$A$7,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$8,Daily!$A$5:$A$8,"&gt;="&amp;$A17,Daily!$A$5:$A$8,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$7,Daily!$A$5:$A$7,"&gt;="&amp;$A17,Daily!$A$5:$A$7,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$8,Daily!$A$5:$A$8,"&gt;="&amp;$A17,Daily!$A$5:$A$8,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$7,Daily!$A$5:$A$7,"&gt;="&amp;$A17,Daily!$A$5:$A$7,"&lt;="&amp;$B17),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="28" t="inlineStr">
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$8,Daily!$A$5:$A$8,"&gt;="&amp;$A17,Daily!$A$5:$A$8,"&lt;="&amp;$B17),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>46278</v>
+      </c>
+      <c r="C18" s="18">
+        <f>COUNTIFS(Daily!$A$5:$A$8,"&gt;="&amp;$A18,Daily!$A$5:$A$8,"&lt;="&amp;$B18)</f>
+        <v/>
+      </c>
+      <c r="D18" s="8">
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$8,Daily!$A$5:$A$8,"&gt;="&amp;$A18,Daily!$A$5:$A$8,"&lt;="&amp;$B18),0)</f>
+        <v/>
+      </c>
+      <c r="E18" s="10">
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$8,Daily!$A$5:$A$8,"&gt;="&amp;$A18,Daily!$A$5:$A$8,"&lt;="&amp;$B18),0)</f>
+        <v/>
+      </c>
+      <c r="F18" s="10">
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$8,Daily!$A$5:$A$8,"&gt;="&amp;$A18,Daily!$A$5:$A$8,"&lt;="&amp;$B18),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="28" t="inlineStr">
         <is>
           <t>Monthly</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>Month start</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Month end</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>Days logged</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>Avg cal/day (mid)</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>Avg protein/day (mid, g)</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>Avg fat/day (mid, g)</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="4" t="n">
+    <row r="22">
+      <c r="A22" s="4" t="n">
         <v>46266</v>
       </c>
-      <c r="B21" s="4" t="n">
+      <c r="B22" s="4" t="n">
         <v>46295</v>
       </c>
-      <c r="C21" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$7,"&gt;="&amp;$A21,Daily!$A$5:$A$7,"&lt;="&amp;$B21)</f>
-        <v/>
-      </c>
-      <c r="D21" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$7,Daily!$A$5:$A$7,"&gt;="&amp;$A21,Daily!$A$5:$A$7,"&lt;="&amp;$B21),0)</f>
-        <v/>
-      </c>
-      <c r="E21" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$7,Daily!$A$5:$A$7,"&gt;="&amp;$A21,Daily!$A$5:$A$7,"&lt;="&amp;$B21),0)</f>
-        <v/>
-      </c>
-      <c r="F21" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$7,Daily!$A$5:$A$7,"&gt;="&amp;$A21,Daily!$A$5:$A$7,"&lt;="&amp;$B21),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="27" t="inlineStr">
+      <c r="C22" s="18">
+        <f>COUNTIFS(Daily!$A$5:$A$8,"&gt;="&amp;$A22,Daily!$A$5:$A$8,"&lt;="&amp;$B22)</f>
+        <v/>
+      </c>
+      <c r="D22" s="8">
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$8,Daily!$A$5:$A$8,"&gt;="&amp;$A22,Daily!$A$5:$A$8,"&lt;="&amp;$B22),0)</f>
+        <v/>
+      </c>
+      <c r="E22" s="10">
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$8,Daily!$A$5:$A$8,"&gt;="&amp;$A22,Daily!$A$5:$A$8,"&lt;="&amp;$B22),0)</f>
+        <v/>
+      </c>
+      <c r="F22" s="10">
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$8,Daily!$A$5:$A$8,"&gt;="&amp;$A22,Daily!$A$5:$A$8,"&lt;="&amp;$B22),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="27" t="inlineStr">
         <is>
           <t>Averages cover only the days present in the log; a part-logged day (today's dinner still to come) drags its average down.</t>
         </is>
@@ -2525,7 +2657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2639,14 +2771,14 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Sambar (with veg)</t>
+          <t>Appam / palappam (1)</t>
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="D7" s="8">
         <f>AVERAGE(B7:C7)</f>
@@ -2654,26 +2786,26 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>~4-6 g</t>
+          <t>~2.5-3.5 g each</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>Per serving</t>
+          <t>Fermented rice batter with coconut milk</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Coconut chutney (~2 tbsp)</t>
+          <t>Potato bhaji / curry (small bowl)</t>
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>90</v>
+        <v>150</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>110</v>
+        <v>220</v>
       </c>
       <c r="D8" s="8">
         <f>AVERAGE(B8:C8)</f>
@@ -2681,26 +2813,26 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>~1-2 g</t>
+          <t>~3-4 g</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Fat-dense - the usual thing to cut</t>
+          <t>Kerala style; oil and coconut milk carry the calories</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Red/tomato chutney (~2 tbsp)</t>
+          <t>Sambar (with veg)</t>
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>40</v>
+        <v>130</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>70</v>
+        <v>160</v>
       </c>
       <c r="D9" s="8">
         <f>AVERAGE(B9:C9)</f>
@@ -2708,22 +2840,26 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>~1 g</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr"/>
+          <t>~4-6 g</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Per serving</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Chicken biryani (half plate)</t>
+          <t>Coconut chutney (~2 tbsp)</t>
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>450</v>
+        <v>90</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>600</v>
+        <v>110</v>
       </c>
       <c r="D10" s="8">
         <f>AVERAGE(B10:C10)</f>
@@ -2731,26 +2867,26 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>~22-30 g</t>
+          <t>~1-2 g</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>Rice + 2 pieces</t>
+          <t>Fat-dense - the usual thing to cut</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Raita (small)</t>
+          <t>Red/tomato chutney (~2 tbsp)</t>
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C11" s="7" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D11" s="8">
         <f>AVERAGE(B11:C11)</f>
@@ -2758,7 +2894,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>~2-4 g</t>
+          <t>~1 g</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr"/>
@@ -2766,14 +2902,14 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Maida porotta</t>
+          <t>Chicken biryani (half plate)</t>
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>160</v>
+        <v>450</v>
       </c>
       <c r="C12" s="7" t="n">
-        <v>250</v>
+        <v>600</v>
       </c>
       <c r="D12" s="8">
         <f>AVERAGE(B12:C12)</f>
@@ -2781,26 +2917,26 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>~4-6 g each</t>
+          <t>~22-30 g</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>Refined flour + layered oil/ghee</t>
+          <t>Rice + 2 pieces</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Uzhunnu vada / medu vada (1)</t>
+          <t>Raita (small)</t>
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>130</v>
+        <v>50</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>180</v>
+        <v>80</v>
       </c>
       <c r="D13" s="8">
         <f>AVERAGE(B13:C13)</f>
@@ -2808,26 +2944,22 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>~3.5-5 g each</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>Deep-fried urad dal - protein-bearing but fat-dense</t>
-        </is>
-      </c>
+          <t>~2-4 g</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Kadala curry (1 container)</t>
+          <t>Maida porotta</t>
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>200</v>
+        <v>160</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>300</v>
+        <v>250</v>
       </c>
       <c r="D14" s="8">
         <f>AVERAGE(B14:C14)</f>
@@ -2835,22 +2967,26 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>~8-10 g</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr"/>
+          <t>~4-6 g each</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Refined flour + layered oil/ghee</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Fish fry (1 piece pan-fried)</t>
+          <t>Uzhunnu vada / medu vada (1)</t>
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="C15" s="7" t="n">
-        <v>220</v>
+        <v>180</v>
       </c>
       <c r="D15" s="8">
         <f>AVERAGE(B15:C15)</f>
@@ -2858,22 +2994,26 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>~15-20 g</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr"/>
+          <t>~3.5-5 g each</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>Deep-fried urad dal - protein-bearing but fat-dense</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Grilled chicken breast (100 g skinless)</t>
+          <t>Kadala curry (1 container)</t>
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>160</v>
+        <v>200</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>180</v>
+        <v>300</v>
       </c>
       <c r="D16" s="8">
         <f>AVERAGE(B16:C16)</f>
@@ -2881,26 +3021,22 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>~30-32 g</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>Best protein-per-calorie item in this list</t>
-        </is>
-      </c>
+          <t>~8-10 g</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Grilled chicken breast (150 g skinless)</t>
+          <t>Fish fry (1 piece pan-fried)</t>
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>240</v>
+        <v>150</v>
       </c>
       <c r="C17" s="7" t="n">
-        <v>270</v>
+        <v>220</v>
       </c>
       <c r="D17" s="8">
         <f>AVERAGE(B17:C17)</f>
@@ -2908,7 +3044,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>~45-48 g</t>
+          <t>~15-20 g</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr"/>
@@ -2916,14 +3052,14 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Honest Bowl - Grilled Chicken and Rice Bowl</t>
+          <t>Grilled chicken breast (100 g skinless)</t>
         </is>
       </c>
       <c r="B18" s="7" t="n">
-        <v>550</v>
+        <v>160</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>710</v>
+        <v>180</v>
       </c>
       <c r="D18" s="8">
         <f>AVERAGE(B18:C18)</f>
@@ -2931,26 +3067,26 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>42-48 g</t>
+          <t>~30-32 g</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>Menu states 42 g protein; chicken + jasmine rice + sweet potato. Sauce served separately</t>
+          <t>Best protein-per-calorie item in this list</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Brown/mushroom sauce (side pot)</t>
+          <t>Grilled chicken breast (150 g skinless)</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>50</v>
+        <v>240</v>
       </c>
       <c r="C19" s="7" t="n">
-        <v>120</v>
+        <v>270</v>
       </c>
       <c r="D19" s="8">
         <f>AVERAGE(B19:C19)</f>
@@ -2958,26 +3094,22 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>~1-2 g</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>Often cream or butter based - the variable in a bowl like this</t>
-        </is>
-      </c>
+          <t>~45-48 g</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Honest Bowl - Tofu Delight Bowl</t>
+          <t>Honest Bowl - Grilled Chicken and Rice Bowl</t>
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>420</v>
+        <v>550</v>
       </c>
       <c r="C20" s="7" t="n">
-        <v>560</v>
+        <v>710</v>
       </c>
       <c r="D20" s="8">
         <f>AVERAGE(B20:C20)</f>
@@ -2985,26 +3117,26 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>~20 g</t>
+          <t>42-48 g</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>Menu states 20 g; jasmine rice + cajun tofu + grilled eggplant. Half the protein of the chicken bowl at the same price</t>
+          <t>Menu states 42 g protein; chicken + jasmine rice + sweet potato. Sauce served separately</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Chicken curry (1 takeaway container)</t>
+          <t>Brown/mushroom sauce (side pot)</t>
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>280</v>
+        <v>50</v>
       </c>
       <c r="C21" s="7" t="n">
-        <v>420</v>
+        <v>120</v>
       </c>
       <c r="D21" s="8">
         <f>AVERAGE(B21:C21)</f>
@@ -3012,26 +3144,26 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>~20-28 g</t>
+          <t>~1-2 g</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>Kerala style; oil and coconut carry most of the calories</t>
+          <t>Often cream or butter based - the variable in a bowl like this</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Grilled chicken quarter (skin on)</t>
+          <t>Honest Bowl - Tofu Delight Bowl</t>
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>250</v>
+        <v>420</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>320</v>
+        <v>560</v>
       </c>
       <c r="D22" s="8">
         <f>AVERAGE(B22:C22)</f>
@@ -3039,26 +3171,26 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>~28-33 g</t>
+          <t>~20 g</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>Skin adds ~12-15 g fat over breast</t>
+          <t>Menu states 20 g; jasmine rice + cajun tofu + grilled eggplant. Half the protein of the chicken bowl at the same price</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Garlic sauce / toum (1 tbsp)</t>
+          <t>Chicken curry (1 takeaway container)</t>
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>90</v>
+        <v>280</v>
       </c>
       <c r="C23" s="7" t="n">
-        <v>110</v>
+        <v>420</v>
       </c>
       <c r="D23" s="8">
         <f>AVERAGE(B23:C23)</f>
@@ -3066,26 +3198,26 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>0 g</t>
+          <t>~20-28 g</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>Essentially emulsified oil - the hidden cost at a grill</t>
+          <t>Kerala style; oil and coconut carry most of the calories</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Khubz / pita (1 large)</t>
+          <t>Grilled chicken quarter (skin on)</t>
         </is>
       </c>
       <c r="B24" s="7" t="n">
         <v>250</v>
       </c>
       <c r="C24" s="7" t="n">
-        <v>300</v>
+        <v>320</v>
       </c>
       <c r="D24" s="8">
         <f>AVERAGE(B24:C24)</f>
@@ -3093,22 +3225,26 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>~8-9 g</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr"/>
+          <t>~28-33 g</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>Skin adds ~12-15 g fat over breast</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Barik/basmati rice (half container cooked)</t>
+          <t>Garlic sauce / toum (1 tbsp)</t>
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>200</v>
+        <v>90</v>
       </c>
       <c r="C25" s="7" t="n">
-        <v>280</v>
+        <v>110</v>
       </c>
       <c r="D25" s="8">
         <f>AVERAGE(B25:C25)</f>
@@ -3116,22 +3252,26 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>~4-5 g</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr"/>
+          <t>0 g</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>Essentially emulsified oil - the hidden cost at a grill</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Fresh pineapple juice (350-450 ml)</t>
+          <t>Khubz / pita (1 large)</t>
         </is>
       </c>
       <c r="B26" s="7" t="n">
-        <v>175</v>
+        <v>250</v>
       </c>
       <c r="C26" s="7" t="n">
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="D26" s="8">
         <f>AVERAGE(B26:C26)</f>
@@ -3139,26 +3279,22 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>~1-2 g</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>No added sugar but ~35-45 g natural sugar; no fibre; almost no protein</t>
-        </is>
-      </c>
+          <t>~8-9 g</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Fresh orange juice (350-450 ml)</t>
+          <t>Barik/basmati rice (half container cooked)</t>
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>155</v>
+        <v>200</v>
       </c>
       <c r="C27" s="7" t="n">
-        <v>205</v>
+        <v>280</v>
       </c>
       <c r="D27" s="8">
         <f>AVERAGE(B27:C27)</f>
@@ -3166,26 +3302,22 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>~2-3 g</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>No added sugar but ~32-40 g natural sugar; no fibre</t>
-        </is>
-      </c>
+          <t>~4-5 g</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in water)</t>
+          <t>Fresh pineapple juice (350-450 ml)</t>
         </is>
       </c>
       <c r="B28" s="7" t="n">
-        <v>100</v>
+        <v>175</v>
       </c>
       <c r="C28" s="7" t="n">
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="D28" s="8">
         <f>AVERAGE(B28:C28)</f>
@@ -3193,22 +3325,26 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr"/>
+          <t>~1-2 g</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>No added sugar but ~35-45 g natural sugar; no fibre; almost no protein</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Greek yogurt (200 g plain low-fat)</t>
+          <t>Fresh orange juice (350-450 ml)</t>
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>120</v>
+        <v>155</v>
       </c>
       <c r="C29" s="7" t="n">
-        <v>140</v>
+        <v>205</v>
       </c>
       <c r="D29" s="8">
         <f>AVERAGE(B29:C29)</f>
@@ -3216,26 +3352,26 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>~18-20 g</t>
+          <t>~2-3 g</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>Casein - digests slowly; good overnight</t>
+          <t>No added sugar but ~32-40 g natural sugar; no fibre</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Boiled egg (1 large)</t>
+          <t>Whey scoop (in water)</t>
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="C30" s="7" t="n">
-        <v>78</v>
+        <v>120</v>
       </c>
       <c r="D30" s="8">
         <f>AVERAGE(B30:C30)</f>
@@ -3243,26 +3379,22 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>~6-6.5 g</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>~5 g fat each</t>
-        </is>
-      </c>
+          <t>~20-25 g</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Paneer (50 g full-fat)</t>
+          <t>Greek yogurt (200 g plain low-fat)</t>
         </is>
       </c>
       <c r="B31" s="7" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="C31" s="7" t="n">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="D31" s="8">
         <f>AVERAGE(B31:C31)</f>
@@ -3270,26 +3402,26 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>~8-9 g</t>
+          <t>~18-20 g</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>Fat-dense for the protein it gives</t>
+          <t>Casein - digests slowly; good overnight</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Cucumber (1 medium)</t>
+          <t>Boiled egg (1 large)</t>
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>25</v>
+        <v>70</v>
       </c>
       <c r="C32" s="7" t="n">
-        <v>30</v>
+        <v>78</v>
       </c>
       <c r="D32" s="8">
         <f>AVERAGE(B32:C32)</f>
@@ -3297,26 +3429,26 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>~1.5 g</t>
+          <t>~6-6.5 g</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>Volume with almost no calories</t>
+          <t>~5 g fat each</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in black coffee no sugar)</t>
+          <t>Paneer (50 g full-fat)</t>
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="C33" s="7" t="n">
-        <v>130</v>
+        <v>150</v>
       </c>
       <c r="D33" s="8">
         <f>AVERAGE(B33:C33)</f>
@@ -3324,22 +3456,26 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="inlineStr"/>
+          <t>~8-9 g</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>Fat-dense for the protein it gives</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Cashew/almond biscuit (1)</t>
+          <t>Cucumber (1 medium)</t>
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="C34" s="7" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="D34" s="8">
         <f>AVERAGE(B34:C34)</f>
@@ -3347,22 +3483,26 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>~0.5 g</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="inlineStr"/>
+          <t>~1.5 g</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>Volume with almost no calories</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (~50g standard)</t>
+          <t>Whey scoop (in black coffee no sugar)</t>
         </is>
       </c>
       <c r="B35" s="7" t="n">
-        <v>245</v>
+        <v>100</v>
       </c>
       <c r="C35" s="7" t="n">
-        <v>250</v>
+        <v>130</v>
       </c>
       <c r="D35" s="8">
         <f>AVERAGE(B35:C35)</f>
@@ -3370,7 +3510,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>~4 g</t>
+          <t>~20-25 g</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr"/>
@@ -3378,14 +3518,14 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (70g king-size)</t>
+          <t>Cashew/almond biscuit (1)</t>
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>335</v>
+        <v>38</v>
       </c>
       <c r="C36" s="7" t="n">
-        <v>335</v>
+        <v>38</v>
       </c>
       <c r="D36" s="8">
         <f>AVERAGE(B36:C36)</f>
@@ -3393,7 +3533,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>~6 g</t>
+          <t>~0.5 g</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr"/>
@@ -3401,14 +3541,14 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Pre-workout scoop</t>
+          <t>Chocolate bar (~50g standard)</t>
         </is>
       </c>
       <c r="B37" s="7" t="n">
-        <v>5</v>
+        <v>245</v>
       </c>
       <c r="C37" s="7" t="n">
-        <v>15</v>
+        <v>250</v>
       </c>
       <c r="D37" s="8">
         <f>AVERAGE(B37:C37)</f>
@@ -3416,10 +3556,56 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
+          <t>~4 g</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>Chocolate bar (70g king-size)</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="n">
+        <v>335</v>
+      </c>
+      <c r="C38" s="7" t="n">
+        <v>335</v>
+      </c>
+      <c r="D38" s="8">
+        <f>AVERAGE(B38:C38)</f>
+        <v/>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>~6 g</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>Pre-workout scoop</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C39" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D39" s="8">
+        <f>AVERAGE(B39:C39)</f>
+        <v/>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
           <t>0 g</t>
         </is>
       </c>
-      <c r="F37" s="6" t="inlineStr">
+      <c r="F39" s="6" t="inlineStr">
         <is>
           <t>Negligible</t>
         </is>

</xml_diff>

<commit_message>
Log Day 4 whey shaker
Black coffee + 1 whey scoop: 100-130 kcal, 20-25 g protein. Day 4 stands at
490-650 kcal (mid 570), 32 g protein, 16 g fat, leaving 1,436 kcal and 98 g
of protein for lunch and dinner.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -537,7 +537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N22"/>
+  <dimension ref="A1:N23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1599,6 +1599,57 @@
           <t>Lightest breakfast in the log by calories; fourth straight breakfast under 20 g protein</t>
         </is>
       </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Black coffee + 1 whey scoop</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E23" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="F23" s="8">
+        <f>AVERAGE(D23:E23)</f>
+        <v/>
+      </c>
+      <c r="G23" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="H23" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="I23" s="10">
+        <f>AVERAGE(G23:H23)</f>
+        <v/>
+      </c>
+      <c r="J23" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K23" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="L23" s="10">
+        <f>AVERAGE(J23:K23)</f>
+        <v/>
+      </c>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N23" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1718,11 +1769,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$22,Meals!$A$5:$A$22,$A5,Meals!$M$5:$M$22,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$23,Meals!$A$5:$A$23,$A5,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$22,Meals!$A$5:$A$22,$A5,Meals!$M$5:$M$22,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$23,Meals!$A$5:$A$23,$A5,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -1730,11 +1781,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$22,Meals!$A$5:$A$22,$A5,Meals!$M$5:$M$22,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$23,Meals!$A$5:$A$23,$A5,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$22,Meals!$A$5:$A$22,$A5,Meals!$M$5:$M$22,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$23,Meals!$A$5:$A$23,$A5,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -1742,11 +1793,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$22,Meals!$A$5:$A$22,$A5,Meals!$M$5:$M$22,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$23,Meals!$A$5:$A$23,$A5,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$22,Meals!$A$5:$A$22,$A5,Meals!$M$5:$M$22,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$23,Meals!$A$5:$A$23,$A5,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -1754,11 +1805,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$22,$A5,Meals!$M$5:$M$22,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$23,$A5,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$22,$A5,Meals!$M$5:$M$22,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$23,$A5,Meals!$M$5:$M$23,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -1771,11 +1822,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$22,Meals!$A$5:$A$22,$A6,Meals!$M$5:$M$22,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$23,Meals!$A$5:$A$23,$A6,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$22,Meals!$A$5:$A$22,$A6,Meals!$M$5:$M$22,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$23,Meals!$A$5:$A$23,$A6,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -1783,11 +1834,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$22,Meals!$A$5:$A$22,$A6,Meals!$M$5:$M$22,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$23,Meals!$A$5:$A$23,$A6,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$22,Meals!$A$5:$A$22,$A6,Meals!$M$5:$M$22,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$23,Meals!$A$5:$A$23,$A6,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -1795,11 +1846,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$22,Meals!$A$5:$A$22,$A6,Meals!$M$5:$M$22,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$23,Meals!$A$5:$A$23,$A6,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$22,Meals!$A$5:$A$22,$A6,Meals!$M$5:$M$22,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$23,Meals!$A$5:$A$23,$A6,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -1807,11 +1858,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$22,$A6,Meals!$M$5:$M$22,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$23,$A6,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$22,$A6,Meals!$M$5:$M$22,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$23,$A6,Meals!$M$5:$M$23,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -1824,11 +1875,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$22,Meals!$A$5:$A$22,$A7,Meals!$M$5:$M$22,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$23,Meals!$A$5:$A$23,$A7,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$22,Meals!$A$5:$A$22,$A7,Meals!$M$5:$M$22,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$23,Meals!$A$5:$A$23,$A7,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -1836,11 +1887,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$22,Meals!$A$5:$A$22,$A7,Meals!$M$5:$M$22,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$23,Meals!$A$5:$A$23,$A7,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$22,Meals!$A$5:$A$22,$A7,Meals!$M$5:$M$22,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$23,Meals!$A$5:$A$23,$A7,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -1848,11 +1899,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$22,Meals!$A$5:$A$22,$A7,Meals!$M$5:$M$22,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$23,Meals!$A$5:$A$23,$A7,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$22,Meals!$A$5:$A$22,$A7,Meals!$M$5:$M$22,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$23,Meals!$A$5:$A$23,$A7,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -1860,11 +1911,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$22,$A7,Meals!$M$5:$M$22,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$23,$A7,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$22,$A7,Meals!$M$5:$M$22,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$23,$A7,Meals!$M$5:$M$23,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -1877,11 +1928,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$22,Meals!$A$5:$A$22,$A8,Meals!$M$5:$M$22,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$23,Meals!$A$5:$A$23,$A8,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$22,Meals!$A$5:$A$22,$A8,Meals!$M$5:$M$22,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$23,Meals!$A$5:$A$23,$A8,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -1889,11 +1940,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$22,Meals!$A$5:$A$22,$A8,Meals!$M$5:$M$22,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$23,Meals!$A$5:$A$23,$A8,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$22,Meals!$A$5:$A$22,$A8,Meals!$M$5:$M$22,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$23,Meals!$A$5:$A$23,$A8,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -1901,11 +1952,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$22,Meals!$A$5:$A$22,$A8,Meals!$M$5:$M$22,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$23,Meals!$A$5:$A$23,$A8,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$22,Meals!$A$5:$A$22,$A8,Meals!$M$5:$M$22,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$23,Meals!$A$5:$A$23,$A8,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -1913,11 +1964,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$22,$A8,Meals!$M$5:$M$22,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$23,$A8,Meals!$M$5:$M$23,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$22,$A8,Meals!$M$5:$M$22,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$23,$A8,Meals!$M$5:$M$23,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">

</xml_diff>

<commit_message>
Add the mess menu and a portion-control plan sheet
Food comes from a fixed Grill Spot mess subscription, so meal choice is not
a lever - only portion control and added protein are. Costed the full weekly
menu into mess_menu.csv and added a Mess Plan sheet that applies per-day
portion cuts and works out how many whey scoops fit in the calories freed.

The finding: as served the mess averages 1,904 kcal and 59.9 g protein, or
3.1 g per 100 kcal. It fills 95% of the calorie target while delivering
under half the protein floor, leaving ~100 kcal of room - less than one
scoop. Portion control is the precondition for hitting protein at all.

Thursday is the weakest day at 38 g as served; Wednesday and Saturday are
tightest on room. Noted that 115-125 g is the realistic operating band under
this constraint, with 130 kept as the aim.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -10,9 +10,10 @@
     <sheet name="Meals" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Daily" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Weights" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Trends" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Targets" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Reference" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Mess Plan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Trends" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Targets" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Reference" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -126,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -165,11 +166,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -2115,6 +2119,600 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:M24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Grill Spot mess - weekly plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>The menu is fixed, so the levers are portion control and added protein. Set how many bread items to skip and whether to halve the rice, per day, in the yellow columns; the sheet works out the calories that frees and how many whey scoops fit inside the target.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="28" t="inlineStr">
+        <is>
+          <t>Assumptions</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="29" t="inlineStr">
+        <is>
+          <t>Bread item - kcal</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="n">
+        <v>205</v>
+      </c>
+      <c r="C5" s="27" t="inlineStr">
+        <is>
+          <t>1 porotta/poori. The worst protein-per-calorie item on the menu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t>Bread item - protein (g)</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="29" t="inlineStr">
+        <is>
+          <t>Halving rice - kcal saved</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="C7" s="27" t="inlineStr">
+        <is>
+          <t>Applies to a full 'Meals' or ghee-rice plate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="29" t="inlineStr">
+        <is>
+          <t>Halving rice - protein (g)</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>Whey scoop - kcal</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>115</v>
+      </c>
+      <c r="C9" s="27" t="inlineStr">
+        <is>
+          <t>19.6 g protein per 100 kcal, vs 3.1 for the mess.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="29" t="inlineStr">
+        <is>
+          <t>Whey scoop - protein (g)</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="n">
+        <v>22.5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Morning</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Dinner</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Kcal as served</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Protein as served</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Bread items to skip</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Halve rice? (1/0)</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Kcal after cuts</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>Protein after cuts</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>Room to target</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>Scoops that fit</t>
+        </is>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>Protein with scoops</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="30" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B14" s="30" t="inlineStr">
+        <is>
+          <t>Poori, baji</t>
+        </is>
+      </c>
+      <c r="C14" s="30" t="inlineStr">
+        <is>
+          <t>Meals (barik/mota rice)</t>
+        </is>
+      </c>
+      <c r="D14" s="30" t="inlineStr">
+        <is>
+          <t>Chicken curry + bread items</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>1865</v>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>59.5</v>
+      </c>
+      <c r="G14" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" s="8">
+        <f>E14-G14*$B$5-H14*$B$7</f>
+        <v/>
+      </c>
+      <c r="J14" s="10">
+        <f>F14-G14*$B$6-H14*$B$8</f>
+        <v/>
+      </c>
+      <c r="K14" s="8">
+        <f>Targets!$B$16-I14</f>
+        <v/>
+      </c>
+      <c r="L14" s="18">
+        <f>MAX(0,ROUNDDOWN(K14/$B$9,0))</f>
+        <v/>
+      </c>
+      <c r="M14" s="10">
+        <f>J14+L14*$B$10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="30" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B15" s="30" t="inlineStr">
+        <is>
+          <t>Masala dosa</t>
+        </is>
+      </c>
+      <c r="C15" s="30" t="inlineStr">
+        <is>
+          <t>Ghee rice + chicken curry</t>
+        </is>
+      </c>
+      <c r="D15" s="30" t="inlineStr">
+        <is>
+          <t>Green peas + bread items</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>1745</v>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="G15" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="8">
+        <f>E15-G15*$B$5-H15*$B$7</f>
+        <v/>
+      </c>
+      <c r="J15" s="10">
+        <f>F15-G15*$B$6-H15*$B$8</f>
+        <v/>
+      </c>
+      <c r="K15" s="8">
+        <f>Targets!$B$16-I15</f>
+        <v/>
+      </c>
+      <c r="L15" s="18">
+        <f>MAX(0,ROUNDDOWN(K15/$B$9,0))</f>
+        <v/>
+      </c>
+      <c r="M15" s="10">
+        <f>J15+L15*$B$10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="30" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="B16" s="30" t="inlineStr">
+        <is>
+          <t>Poratta + egg roast</t>
+        </is>
+      </c>
+      <c r="C16" s="30" t="inlineStr">
+        <is>
+          <t>Meals (barik/mota rice)</t>
+        </is>
+      </c>
+      <c r="D16" s="30" t="inlineStr">
+        <is>
+          <t>Chicken traditional curry + bread</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>2140</v>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>75.5</v>
+      </c>
+      <c r="G16" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="8">
+        <f>E16-G16*$B$5-H16*$B$7</f>
+        <v/>
+      </c>
+      <c r="J16" s="10">
+        <f>F16-G16*$B$6-H16*$B$8</f>
+        <v/>
+      </c>
+      <c r="K16" s="8">
+        <f>Targets!$B$16-I16</f>
+        <v/>
+      </c>
+      <c r="L16" s="18">
+        <f>MAX(0,ROUNDDOWN(K16/$B$9,0))</f>
+        <v/>
+      </c>
+      <c r="M16" s="10">
+        <f>J16+L16*$B$10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="30" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B17" s="30" t="inlineStr">
+        <is>
+          <t>Ghee roast</t>
+        </is>
+      </c>
+      <c r="C17" s="30" t="inlineStr">
+        <is>
+          <t>Meals (barik/mota rice)</t>
+        </is>
+      </c>
+      <c r="D17" s="30" t="inlineStr">
+        <is>
+          <t>Gobbi chilly + bread items</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>1810</v>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>38</v>
+      </c>
+      <c r="G17" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="8">
+        <f>E17-G17*$B$5-H17*$B$7</f>
+        <v/>
+      </c>
+      <c r="J17" s="10">
+        <f>F17-G17*$B$6-H17*$B$8</f>
+        <v/>
+      </c>
+      <c r="K17" s="8">
+        <f>Targets!$B$16-I17</f>
+        <v/>
+      </c>
+      <c r="L17" s="18">
+        <f>MAX(0,ROUNDDOWN(K17/$B$9,0))</f>
+        <v/>
+      </c>
+      <c r="M17" s="10">
+        <f>J17+L17*$B$10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="30" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B18" s="30" t="inlineStr">
+        <is>
+          <t>Idly set</t>
+        </is>
+      </c>
+      <c r="C18" s="30" t="inlineStr">
+        <is>
+          <t>Chicken biriyani</t>
+        </is>
+      </c>
+      <c r="D18" s="30" t="inlineStr">
+        <is>
+          <t>Kadala curry + bread items</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>1635</v>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>61</v>
+      </c>
+      <c r="G18" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="8">
+        <f>E18-G18*$B$5-H18*$B$7</f>
+        <v/>
+      </c>
+      <c r="J18" s="10">
+        <f>F18-G18*$B$6-H18*$B$8</f>
+        <v/>
+      </c>
+      <c r="K18" s="8">
+        <f>Targets!$B$16-I18</f>
+        <v/>
+      </c>
+      <c r="L18" s="18">
+        <f>MAX(0,ROUNDDOWN(K18/$B$9,0))</f>
+        <v/>
+      </c>
+      <c r="M18" s="10">
+        <f>J18+L18*$B$10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="30" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="B19" s="30" t="inlineStr">
+        <is>
+          <t>Dosa set</t>
+        </is>
+      </c>
+      <c r="C19" s="30" t="inlineStr">
+        <is>
+          <t>Meals (barik/mota rice)</t>
+        </is>
+      </c>
+      <c r="D19" s="30" t="inlineStr">
+        <is>
+          <t>Chicken varutharachathu + bread</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>2080</v>
+      </c>
+      <c r="F19" s="9" t="n">
+        <v>62</v>
+      </c>
+      <c r="G19" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="8">
+        <f>E19-G19*$B$5-H19*$B$7</f>
+        <v/>
+      </c>
+      <c r="J19" s="10">
+        <f>F19-G19*$B$6-H19*$B$8</f>
+        <v/>
+      </c>
+      <c r="K19" s="8">
+        <f>Targets!$B$16-I19</f>
+        <v/>
+      </c>
+      <c r="L19" s="18">
+        <f>MAX(0,ROUNDDOWN(K19/$B$9,0))</f>
+        <v/>
+      </c>
+      <c r="M19" s="10">
+        <f>J19+L19*$B$10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="30" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>Kadala curry + poratta</t>
+        </is>
+      </c>
+      <c r="C20" s="30" t="inlineStr">
+        <is>
+          <t>Ghee rice + chicken curry</t>
+        </is>
+      </c>
+      <c r="D20" s="30" t="inlineStr">
+        <is>
+          <t>Egg roast + bread items</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>2055</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>69</v>
+      </c>
+      <c r="G20" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="8">
+        <f>E20-G20*$B$5-H20*$B$7</f>
+        <v/>
+      </c>
+      <c r="J20" s="10">
+        <f>F20-G20*$B$6-H20*$B$8</f>
+        <v/>
+      </c>
+      <c r="K20" s="8">
+        <f>Targets!$B$16-I20</f>
+        <v/>
+      </c>
+      <c r="L20" s="18">
+        <f>MAX(0,ROUNDDOWN(K20/$B$9,0))</f>
+        <v/>
+      </c>
+      <c r="M20" s="10">
+        <f>J20+L20*$B$10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="27" t="inlineStr">
+        <is>
+          <t>As served the mess averages ~1,904 kcal and ~60 g of protein - 3.1 g per 100 kcal. It fills 95% of the calorie target while delivering under half the protein floor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="27" t="inlineStr">
+        <is>
+          <t>That is why portion control is not optional here: without cutting, there is only ~100 kcal of room left for protein, which is less than one scoop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="27" t="inlineStr">
+        <is>
+          <t>Bread items are the cheapest cut - ~205 kcal for ~5 g of protein each.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:M2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2408,7 +3006,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2449,11 +3047,11 @@
           <t>Weight (kg)</t>
         </is>
       </c>
-      <c r="B5" s="30">
+      <c r="B5" s="32">
         <f>INDEX(Weights!$B$5:$B$500,COUNT(Weights!$B$5:$B$500))</f>
         <v/>
       </c>
-      <c r="C5" s="31" t="inlineStr">
+      <c r="C5" s="33" t="inlineStr">
         <is>
           <t>Latest entry on the Weights sheet - add a weigh-in there and everything below re-derives. Do not type over it.</t>
         </is>
@@ -2468,7 +3066,7 @@
       <c r="B6" s="16" t="n">
         <v>162.5</v>
       </c>
-      <c r="C6" s="31" t="inlineStr">
+      <c r="C6" s="33" t="inlineStr">
         <is>
           <t>Source: stated by user.</t>
         </is>
@@ -2480,10 +3078,10 @@
           <t>Age (years)</t>
         </is>
       </c>
-      <c r="B7" s="32" t="n">
+      <c r="B7" s="31" t="n">
         <v>33</v>
       </c>
-      <c r="C7" s="31" t="inlineStr">
+      <c r="C7" s="33" t="inlineStr">
         <is>
           <t>Source: stated by user (turns 33 on 2026-09-15).</t>
         </is>
@@ -2495,10 +3093,10 @@
           <t>Sex constant</t>
         </is>
       </c>
-      <c r="B8" s="32" t="n">
+      <c r="B8" s="31" t="n">
         <v>5</v>
       </c>
-      <c r="C8" s="31" t="inlineStr">
+      <c r="C8" s="33" t="inlineStr">
         <is>
           <t>Mifflin-St Jeor term: +5 male, -161 female.</t>
         </is>
@@ -2510,10 +3108,10 @@
           <t>Activity multiplier</t>
         </is>
       </c>
-      <c r="B9" s="33" t="n">
+      <c r="B9" s="34" t="n">
         <v>1.45</v>
       </c>
-      <c r="C9" s="31" t="inlineStr">
+      <c r="C9" s="33" t="inlineStr">
         <is>
           <t>1.45 = desk job plus 6 lifting sessions/week. Lifting burns less than cardio-based charts assume; raise it only if the scale says so.</t>
         </is>
@@ -2528,7 +3126,7 @@
       <c r="B10" s="14" t="n">
         <v>550</v>
       </c>
-      <c r="C10" s="31" t="inlineStr">
+      <c r="C10" s="33" t="inlineStr">
         <is>
           <t>550/day = 0.5 kg/week. Assumption, not a measurement.</t>
         </is>
@@ -2543,7 +3141,7 @@
       <c r="B11" s="14" t="n">
         <v>7700</v>
       </c>
-      <c r="C11" s="31" t="inlineStr">
+      <c r="C11" s="33" t="inlineStr">
         <is>
           <t>Standard 7,700 kcal/kg conversion.</t>
         </is>
@@ -2566,7 +3164,7 @@
         <f>10*B5+6.25*B6-5*B7+B8</f>
         <v/>
       </c>
-      <c r="C14" s="31" t="inlineStr">
+      <c r="C14" s="33" t="inlineStr">
         <is>
           <t>Resting burn: what the body uses doing nothing.</t>
         </is>
@@ -2582,7 +3180,7 @@
         <f>B14*B9</f>
         <v/>
       </c>
-      <c r="C15" s="31" t="inlineStr">
+      <c r="C15" s="33" t="inlineStr">
         <is>
           <t>Estimate. The scale over 2-3 weeks is the real measurement.</t>
         </is>
@@ -2594,11 +3192,11 @@
           <t>CALORIE TARGET</t>
         </is>
       </c>
-      <c r="B16" s="34">
+      <c r="B16" s="35">
         <f>B15-B10</f>
         <v/>
       </c>
-      <c r="C16" s="31" t="inlineStr">
+      <c r="C16" s="33" t="inlineStr">
         <is>
           <t>The number to eat.</t>
         </is>
@@ -2625,7 +3223,7 @@
         <f>B5/(B6/100)^2</f>
         <v/>
       </c>
-      <c r="C18" s="31" t="inlineStr">
+      <c r="C18" s="33" t="inlineStr">
         <is>
           <t>Worth a GP or dietitian check alongside this plan.</t>
         </is>
@@ -2644,10 +3242,10 @@
           <t>Protein target low (g)</t>
         </is>
       </c>
-      <c r="B21" s="32" t="n">
+      <c r="B21" s="31" t="n">
         <v>130</v>
       </c>
-      <c r="C21" s="31" t="inlineStr">
+      <c r="C21" s="33" t="inlineStr">
         <is>
           <t>~2.1 g/kg of estimated lean mass - the level that protects muscle in a deficit while training 6 days.</t>
         </is>
@@ -2659,7 +3257,7 @@
           <t>Protein target high (g)</t>
         </is>
       </c>
-      <c r="B22" s="32" t="n">
+      <c r="B22" s="31" t="n">
         <v>145</v>
       </c>
     </row>
@@ -2669,10 +3267,10 @@
           <t>Fat floor (g)</t>
         </is>
       </c>
-      <c r="B23" s="32" t="n">
+      <c r="B23" s="31" t="n">
         <v>55</v>
       </c>
-      <c r="C23" s="31" t="inlineStr">
+      <c r="C23" s="33" t="inlineStr">
         <is>
           <t>~0.6 g/kg. A floor for hormone health, not a goal to hit.</t>
         </is>
@@ -2688,7 +3286,7 @@
         <f>(B16-B21*4-B23*9)/4</f>
         <v/>
       </c>
-      <c r="C24" s="31" t="inlineStr">
+      <c r="C24" s="33" t="inlineStr">
         <is>
           <t>Whatever is left once protein and the fat floor are paid for. Fuels the PPL work.</t>
         </is>
@@ -2702,7 +3300,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Log sweet melon wedge on Day 4
35-55 kcal, 0.5-1 g protein. Day 4 stands at 615 kcal, 32.75 g protein.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N23"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1654,6 +1654,61 @@
         </is>
       </c>
       <c r="N23" s="6" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Sweet melon (1 wedge)</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="E24" s="7" t="n">
+        <v>55</v>
+      </c>
+      <c r="F24" s="8">
+        <f>AVERAGE(D24:E24)</f>
+        <v/>
+      </c>
+      <c r="G24" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H24" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" s="10">
+        <f>AVERAGE(G24:H24)</f>
+        <v/>
+      </c>
+      <c r="J24" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L24" s="10">
+        <f>AVERAGE(J24:K24)</f>
+        <v/>
+      </c>
+      <c r="M24" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N24" s="6" t="inlineStr">
+        <is>
+          <t>Whole fruit - fibre intact</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1773,11 +1828,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$23,Meals!$A$5:$A$23,$A5,Meals!$M$5:$M$23,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$24,Meals!$A$5:$A$24,$A5,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$23,Meals!$A$5:$A$23,$A5,Meals!$M$5:$M$23,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$24,Meals!$A$5:$A$24,$A5,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -1785,11 +1840,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$23,Meals!$A$5:$A$23,$A5,Meals!$M$5:$M$23,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$24,Meals!$A$5:$A$24,$A5,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$23,Meals!$A$5:$A$23,$A5,Meals!$M$5:$M$23,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$24,Meals!$A$5:$A$24,$A5,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -1797,11 +1852,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$23,Meals!$A$5:$A$23,$A5,Meals!$M$5:$M$23,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$24,Meals!$A$5:$A$24,$A5,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$23,Meals!$A$5:$A$23,$A5,Meals!$M$5:$M$23,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$24,Meals!$A$5:$A$24,$A5,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -1809,11 +1864,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$23,$A5,Meals!$M$5:$M$23,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$24,$A5,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$23,$A5,Meals!$M$5:$M$23,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$24,$A5,Meals!$M$5:$M$24,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -1826,11 +1881,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$23,Meals!$A$5:$A$23,$A6,Meals!$M$5:$M$23,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$24,Meals!$A$5:$A$24,$A6,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$23,Meals!$A$5:$A$23,$A6,Meals!$M$5:$M$23,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$24,Meals!$A$5:$A$24,$A6,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -1838,11 +1893,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$23,Meals!$A$5:$A$23,$A6,Meals!$M$5:$M$23,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$24,Meals!$A$5:$A$24,$A6,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$23,Meals!$A$5:$A$23,$A6,Meals!$M$5:$M$23,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$24,Meals!$A$5:$A$24,$A6,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -1850,11 +1905,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$23,Meals!$A$5:$A$23,$A6,Meals!$M$5:$M$23,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$24,Meals!$A$5:$A$24,$A6,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$23,Meals!$A$5:$A$23,$A6,Meals!$M$5:$M$23,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$24,Meals!$A$5:$A$24,$A6,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -1862,11 +1917,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$23,$A6,Meals!$M$5:$M$23,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$24,$A6,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$23,$A6,Meals!$M$5:$M$23,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$24,$A6,Meals!$M$5:$M$24,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -1879,11 +1934,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$23,Meals!$A$5:$A$23,$A7,Meals!$M$5:$M$23,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$24,Meals!$A$5:$A$24,$A7,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$23,Meals!$A$5:$A$23,$A7,Meals!$M$5:$M$23,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$24,Meals!$A$5:$A$24,$A7,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -1891,11 +1946,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$23,Meals!$A$5:$A$23,$A7,Meals!$M$5:$M$23,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$24,Meals!$A$5:$A$24,$A7,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$23,Meals!$A$5:$A$23,$A7,Meals!$M$5:$M$23,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$24,Meals!$A$5:$A$24,$A7,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -1903,11 +1958,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$23,Meals!$A$5:$A$23,$A7,Meals!$M$5:$M$23,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$24,Meals!$A$5:$A$24,$A7,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$23,Meals!$A$5:$A$23,$A7,Meals!$M$5:$M$23,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$24,Meals!$A$5:$A$24,$A7,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -1915,11 +1970,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$23,$A7,Meals!$M$5:$M$23,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$24,$A7,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$23,$A7,Meals!$M$5:$M$23,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$24,$A7,Meals!$M$5:$M$24,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -1932,11 +1987,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$23,Meals!$A$5:$A$23,$A8,Meals!$M$5:$M$23,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$24,Meals!$A$5:$A$24,$A8,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$23,Meals!$A$5:$A$23,$A8,Meals!$M$5:$M$23,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$24,Meals!$A$5:$A$24,$A8,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -1944,11 +1999,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$23,Meals!$A$5:$A$23,$A8,Meals!$M$5:$M$23,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$24,Meals!$A$5:$A$24,$A8,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$23,Meals!$A$5:$A$23,$A8,Meals!$M$5:$M$23,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$24,Meals!$A$5:$A$24,$A8,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -1956,11 +2011,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$23,Meals!$A$5:$A$23,$A8,Meals!$M$5:$M$23,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$24,Meals!$A$5:$A$24,$A8,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$23,Meals!$A$5:$A$23,$A8,Meals!$M$5:$M$23,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$24,Meals!$A$5:$A$24,$A8,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -1968,11 +2023,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$23,$A8,Meals!$M$5:$M$23,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$24,$A8,Meals!$M$5:$M$24,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$23,$A8,Meals!$M$5:$M$23,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$24,$A8,Meals!$M$5:$M$24,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -3306,7 +3361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4144,14 +4199,14 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in black coffee no sugar)</t>
+          <t>Sweet melon / cantaloupe (1 wedge ~100-150 g)</t>
         </is>
       </c>
       <c r="B35" s="7" t="n">
-        <v>100</v>
+        <v>35</v>
       </c>
       <c r="C35" s="7" t="n">
-        <v>130</v>
+        <v>55</v>
       </c>
       <c r="D35" s="8">
         <f>AVERAGE(B35:C35)</f>
@@ -4159,22 +4214,26 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="inlineStr"/>
+          <t>~0.5-1 g</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>Whole fruit - fibre and water intact; ~1/4 the calories of the same fruit juiced</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Cashew/almond biscuit (1)</t>
+          <t>Whey scoop (in black coffee no sugar)</t>
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C36" s="7" t="n">
-        <v>38</v>
+        <v>130</v>
       </c>
       <c r="D36" s="8">
         <f>AVERAGE(B36:C36)</f>
@@ -4182,7 +4241,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>~0.5 g</t>
+          <t>~20-25 g</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr"/>
@@ -4190,14 +4249,14 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (~50g standard)</t>
+          <t>Cashew/almond biscuit (1)</t>
         </is>
       </c>
       <c r="B37" s="7" t="n">
-        <v>245</v>
+        <v>38</v>
       </c>
       <c r="C37" s="7" t="n">
-        <v>250</v>
+        <v>38</v>
       </c>
       <c r="D37" s="8">
         <f>AVERAGE(B37:C37)</f>
@@ -4205,7 +4264,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>~4 g</t>
+          <t>~0.5 g</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr"/>
@@ -4213,14 +4272,14 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (70g king-size)</t>
+          <t>Chocolate bar (~50g standard)</t>
         </is>
       </c>
       <c r="B38" s="7" t="n">
-        <v>335</v>
+        <v>245</v>
       </c>
       <c r="C38" s="7" t="n">
-        <v>335</v>
+        <v>250</v>
       </c>
       <c r="D38" s="8">
         <f>AVERAGE(B38:C38)</f>
@@ -4228,7 +4287,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>~6 g</t>
+          <t>~4 g</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr"/>
@@ -4236,14 +4295,14 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>Pre-workout scoop</t>
+          <t>Chocolate bar (70g king-size)</t>
         </is>
       </c>
       <c r="B39" s="7" t="n">
-        <v>5</v>
+        <v>335</v>
       </c>
       <c r="C39" s="7" t="n">
-        <v>15</v>
+        <v>335</v>
       </c>
       <c r="D39" s="8">
         <f>AVERAGE(B39:C39)</f>
@@ -4251,10 +4310,33 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
+          <t>~6 g</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>Pre-workout scoop</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C40" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D40" s="8">
+        <f>AVERAGE(B40:C40)</f>
+        <v/>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
           <t>0 g</t>
         </is>
       </c>
-      <c r="F39" s="6" t="inlineStr">
+      <c r="F40" s="6" t="inlineStr">
         <is>
           <t>Negligible</t>
         </is>

</xml_diff>

<commit_message>
Update Day 4 melon to 2 wedges
70-110 kcal, 1-2 g protein. Day 4 stands at 660 kcal, 33.5 g protein.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -1666,24 +1666,24 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Sweet melon (1 wedge)</t>
+          <t>Sweet melon (2 wedges)</t>
         </is>
       </c>
       <c r="D24" s="7" t="n">
-        <v>35</v>
+        <v>70</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>55</v>
+        <v>110</v>
       </c>
       <c r="F24" s="8">
         <f>AVERAGE(D24:E24)</f>
         <v/>
       </c>
       <c r="G24" s="9" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I24" s="10">
         <f>AVERAGE(G24:H24)</f>
@@ -1693,7 +1693,7 @@
         <v>0</v>
       </c>
       <c r="K24" s="9" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L24" s="10">
         <f>AVERAGE(J24:K24)</f>
@@ -1706,7 +1706,7 @@
       </c>
       <c r="N24" s="6" t="inlineStr">
         <is>
-          <t>Whole fruit - fibre intact</t>
+          <t>Whole fruit - fibre intact; second wedge added</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log Monday mess lunch with added eggs
880-1,250 kcal (mid 1,065), 39-54 g protein (mid 46.5), 31-51 g fat. Two
boiled eggs added to the standard meals plate make this the highest-protein
single meal in the log, above the Honest Bowl.

Rice was not halved, so the day stands at 1,725 kcal with only 282 kcal of
room before dinner. Day 4 protein is at 80 g.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N24"/>
+  <dimension ref="A1:N25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1610,39 +1610,39 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Snack</t>
+          <t>Lunch</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Black coffee + 1 whey scoop</t>
+          <t>Mess meals plate: rice, 2 boiled eggs, 1 fried fish, sambar, green peas, buttermilk, veg curry, fish curry</t>
         </is>
       </c>
       <c r="D23" s="7" t="n">
-        <v>100</v>
+        <v>880</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>130</v>
+        <v>1250</v>
       </c>
       <c r="F23" s="8">
         <f>AVERAGE(D23:E23)</f>
         <v/>
       </c>
       <c r="G23" s="9" t="n">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="H23" s="9" t="n">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="I23" s="10">
         <f>AVERAGE(G23:H23)</f>
         <v/>
       </c>
       <c r="J23" s="9" t="n">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="K23" s="9" t="n">
-        <v>3</v>
+        <v>51</v>
       </c>
       <c r="L23" s="10">
         <f>AVERAGE(J23:K23)</f>
@@ -1653,7 +1653,11 @@
           <t>logged</t>
         </is>
       </c>
-      <c r="N23" s="6" t="inlineStr"/>
+      <c r="N23" s="6" t="inlineStr">
+        <is>
+          <t>Eggs added by user - highest-protein single meal in the log. Rice portion looks full rather than halved</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
@@ -1666,34 +1670,34 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Sweet melon (2 wedges)</t>
+          <t>Black coffee + 1 whey scoop</t>
         </is>
       </c>
       <c r="D24" s="7" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="F24" s="8">
         <f>AVERAGE(D24:E24)</f>
         <v/>
       </c>
       <c r="G24" s="9" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="I24" s="10">
         <f>AVERAGE(G24:H24)</f>
         <v/>
       </c>
       <c r="J24" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K24" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L24" s="10">
         <f>AVERAGE(J24:K24)</f>
@@ -1704,7 +1708,58 @@
           <t>logged</t>
         </is>
       </c>
-      <c r="N24" s="6" t="inlineStr">
+      <c r="N24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Sweet melon (2 wedges)</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>110</v>
+      </c>
+      <c r="F25" s="8">
+        <f>AVERAGE(D25:E25)</f>
+        <v/>
+      </c>
+      <c r="G25" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I25" s="10">
+        <f>AVERAGE(G25:H25)</f>
+        <v/>
+      </c>
+      <c r="J25" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="L25" s="10">
+        <f>AVERAGE(J25:K25)</f>
+        <v/>
+      </c>
+      <c r="M25" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N25" s="6" t="inlineStr">
         <is>
           <t>Whole fruit - fibre intact; second wedge added</t>
         </is>
@@ -1828,11 +1883,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$24,Meals!$A$5:$A$24,$A5,Meals!$M$5:$M$24,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$25,Meals!$A$5:$A$25,$A5,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$24,Meals!$A$5:$A$24,$A5,Meals!$M$5:$M$24,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$25,Meals!$A$5:$A$25,$A5,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -1840,11 +1895,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$24,Meals!$A$5:$A$24,$A5,Meals!$M$5:$M$24,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$25,Meals!$A$5:$A$25,$A5,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$24,Meals!$A$5:$A$24,$A5,Meals!$M$5:$M$24,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$25,Meals!$A$5:$A$25,$A5,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -1852,11 +1907,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$24,Meals!$A$5:$A$24,$A5,Meals!$M$5:$M$24,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$25,Meals!$A$5:$A$25,$A5,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$24,Meals!$A$5:$A$24,$A5,Meals!$M$5:$M$24,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$25,Meals!$A$5:$A$25,$A5,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -1864,11 +1919,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$24,$A5,Meals!$M$5:$M$24,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$25,$A5,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$24,$A5,Meals!$M$5:$M$24,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$25,$A5,Meals!$M$5:$M$25,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -1881,11 +1936,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$24,Meals!$A$5:$A$24,$A6,Meals!$M$5:$M$24,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$25,Meals!$A$5:$A$25,$A6,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$24,Meals!$A$5:$A$24,$A6,Meals!$M$5:$M$24,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$25,Meals!$A$5:$A$25,$A6,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -1893,11 +1948,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$24,Meals!$A$5:$A$24,$A6,Meals!$M$5:$M$24,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$25,Meals!$A$5:$A$25,$A6,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$24,Meals!$A$5:$A$24,$A6,Meals!$M$5:$M$24,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$25,Meals!$A$5:$A$25,$A6,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -1905,11 +1960,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$24,Meals!$A$5:$A$24,$A6,Meals!$M$5:$M$24,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$25,Meals!$A$5:$A$25,$A6,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$24,Meals!$A$5:$A$24,$A6,Meals!$M$5:$M$24,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$25,Meals!$A$5:$A$25,$A6,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -1917,11 +1972,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$24,$A6,Meals!$M$5:$M$24,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$25,$A6,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$24,$A6,Meals!$M$5:$M$24,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$25,$A6,Meals!$M$5:$M$25,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -1934,11 +1989,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$24,Meals!$A$5:$A$24,$A7,Meals!$M$5:$M$24,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$25,Meals!$A$5:$A$25,$A7,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$24,Meals!$A$5:$A$24,$A7,Meals!$M$5:$M$24,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$25,Meals!$A$5:$A$25,$A7,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -1946,11 +2001,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$24,Meals!$A$5:$A$24,$A7,Meals!$M$5:$M$24,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$25,Meals!$A$5:$A$25,$A7,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$24,Meals!$A$5:$A$24,$A7,Meals!$M$5:$M$24,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$25,Meals!$A$5:$A$25,$A7,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -1958,11 +2013,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$24,Meals!$A$5:$A$24,$A7,Meals!$M$5:$M$24,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$25,Meals!$A$5:$A$25,$A7,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$24,Meals!$A$5:$A$24,$A7,Meals!$M$5:$M$24,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$25,Meals!$A$5:$A$25,$A7,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -1970,11 +2025,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$24,$A7,Meals!$M$5:$M$24,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$25,$A7,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$24,$A7,Meals!$M$5:$M$24,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$25,$A7,Meals!$M$5:$M$25,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -1987,11 +2042,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$24,Meals!$A$5:$A$24,$A8,Meals!$M$5:$M$24,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$25,Meals!$A$5:$A$25,$A8,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$24,Meals!$A$5:$A$24,$A8,Meals!$M$5:$M$24,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$25,Meals!$A$5:$A$25,$A8,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -1999,11 +2054,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$24,Meals!$A$5:$A$24,$A8,Meals!$M$5:$M$24,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$25,Meals!$A$5:$A$25,$A8,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$24,Meals!$A$5:$A$24,$A8,Meals!$M$5:$M$24,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$25,Meals!$A$5:$A$25,$A8,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -2011,11 +2066,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$24,Meals!$A$5:$A$24,$A8,Meals!$M$5:$M$24,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$25,Meals!$A$5:$A$25,$A8,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$24,Meals!$A$5:$A$24,$A8,Meals!$M$5:$M$24,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$25,Meals!$A$5:$A$25,$A8,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -2023,11 +2078,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$24,$A8,Meals!$M$5:$M$24,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$25,$A8,Meals!$M$5:$M$25,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$24,$A8,Meals!$M$5:$M$24,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$25,$A8,Meals!$M$5:$M$25,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">

</xml_diff>

<commit_message>
Correct Monday lunch: rice was already halved
Revised to 790-1,100 kcal (mid 945), 37-51 g protein, 28-48 g fat. Both
levers were pulled - eggs added and rice halved - so Day 4 stands at
1,605 kcal and 77.5 g protein with 402 kcal of room for dinner.

The photographed plate also shows the mess "Meals" lunch is larger and
higher in protein than the model assumed (~950 kcal and ~33 g, not 750 and
18) because it carries fish, dal and a legume side. Updated mess_menu.csv,
which moves Monday, Wednesday, Thursday and Saturday up.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -1615,34 +1615,34 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Mess meals plate: rice, 2 boiled eggs, 1 fried fish, sambar, green peas, buttermilk, veg curry, fish curry</t>
+          <t>Mess meals plate (rice halved): rice, 2 boiled eggs, 1 fried fish, sambar, green peas, buttermilk, veg curry, fish curry</t>
         </is>
       </c>
       <c r="D23" s="7" t="n">
-        <v>880</v>
+        <v>790</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>1250</v>
+        <v>1100</v>
       </c>
       <c r="F23" s="8">
         <f>AVERAGE(D23:E23)</f>
         <v/>
       </c>
       <c r="G23" s="9" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="H23" s="9" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="I23" s="10">
         <f>AVERAGE(G23:H23)</f>
         <v/>
       </c>
       <c r="J23" s="9" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="K23" s="9" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="L23" s="10">
         <f>AVERAGE(J23:K23)</f>
@@ -1655,7 +1655,7 @@
       </c>
       <c r="N23" s="6" t="inlineStr">
         <is>
-          <t>Eggs added by user - highest-protein single meal in the log. Rice portion looks full rather than halved</t>
+          <t>Rice was already the half portion - both levers pulled. Highest-protein single meal in the log</t>
         </is>
       </c>
     </row>
@@ -2432,10 +2432,10 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>1865</v>
+        <v>2065</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>59.5</v>
+        <v>74.5</v>
       </c>
       <c r="G14" s="31" t="n">
         <v>1</v>
@@ -2540,10 +2540,10 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>2140</v>
+        <v>2340</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>75.5</v>
+        <v>90.5</v>
       </c>
       <c r="G16" s="31" t="n">
         <v>1</v>
@@ -2594,10 +2594,10 @@
         </is>
       </c>
       <c r="E17" s="7" t="n">
-        <v>1810</v>
+        <v>2010</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="G17" s="31" t="n">
         <v>1</v>
@@ -2702,10 +2702,10 @@
         </is>
       </c>
       <c r="E19" s="7" t="n">
-        <v>2080</v>
+        <v>2280</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="G19" s="31" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Log second egg serving on Day 4
2 boiled eggs at 5pm: 140-156 kcal, 12-13 g protein. Day 4 reaches 90 g of
protein before dinner, the best mid-day position in the log, at 1,753 kcal.
Fat is at 65 g against a 55 g floor.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:N26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1762,6 +1762,61 @@
       <c r="N25" s="6" t="inlineStr">
         <is>
           <t>Whole fruit - fibre intact; second wedge added</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>2 boiled eggs (5pm)</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="n">
+        <v>140</v>
+      </c>
+      <c r="E26" s="7" t="n">
+        <v>156</v>
+      </c>
+      <c r="F26" s="8">
+        <f>AVERAGE(D26:E26)</f>
+        <v/>
+      </c>
+      <c r="G26" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="H26" s="9" t="n">
+        <v>13</v>
+      </c>
+      <c r="I26" s="10">
+        <f>AVERAGE(G26:H26)</f>
+        <v/>
+      </c>
+      <c r="J26" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="K26" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="L26" s="10">
+        <f>AVERAGE(J26:K26)</f>
+        <v/>
+      </c>
+      <c r="M26" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N26" s="6" t="inlineStr">
+        <is>
+          <t>Second egg serving of the day - four eggs total</t>
         </is>
       </c>
     </row>
@@ -1883,11 +1938,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$25,Meals!$A$5:$A$25,$A5,Meals!$M$5:$M$25,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$26,Meals!$A$5:$A$26,$A5,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$25,Meals!$A$5:$A$25,$A5,Meals!$M$5:$M$25,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$26,Meals!$A$5:$A$26,$A5,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -1895,11 +1950,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$25,Meals!$A$5:$A$25,$A5,Meals!$M$5:$M$25,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$26,Meals!$A$5:$A$26,$A5,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$25,Meals!$A$5:$A$25,$A5,Meals!$M$5:$M$25,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$26,Meals!$A$5:$A$26,$A5,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -1907,11 +1962,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$25,Meals!$A$5:$A$25,$A5,Meals!$M$5:$M$25,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$26,Meals!$A$5:$A$26,$A5,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$25,Meals!$A$5:$A$25,$A5,Meals!$M$5:$M$25,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$26,Meals!$A$5:$A$26,$A5,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -1919,11 +1974,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$25,$A5,Meals!$M$5:$M$25,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$26,$A5,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$25,$A5,Meals!$M$5:$M$25,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$26,$A5,Meals!$M$5:$M$26,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -1936,11 +1991,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$25,Meals!$A$5:$A$25,$A6,Meals!$M$5:$M$25,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$26,Meals!$A$5:$A$26,$A6,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$25,Meals!$A$5:$A$25,$A6,Meals!$M$5:$M$25,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$26,Meals!$A$5:$A$26,$A6,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -1948,11 +2003,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$25,Meals!$A$5:$A$25,$A6,Meals!$M$5:$M$25,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$26,Meals!$A$5:$A$26,$A6,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$25,Meals!$A$5:$A$25,$A6,Meals!$M$5:$M$25,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$26,Meals!$A$5:$A$26,$A6,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -1960,11 +2015,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$25,Meals!$A$5:$A$25,$A6,Meals!$M$5:$M$25,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$26,Meals!$A$5:$A$26,$A6,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$25,Meals!$A$5:$A$25,$A6,Meals!$M$5:$M$25,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$26,Meals!$A$5:$A$26,$A6,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -1972,11 +2027,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$25,$A6,Meals!$M$5:$M$25,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$26,$A6,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$25,$A6,Meals!$M$5:$M$25,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$26,$A6,Meals!$M$5:$M$26,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -1989,11 +2044,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$25,Meals!$A$5:$A$25,$A7,Meals!$M$5:$M$25,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$26,Meals!$A$5:$A$26,$A7,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$25,Meals!$A$5:$A$25,$A7,Meals!$M$5:$M$25,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$26,Meals!$A$5:$A$26,$A7,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -2001,11 +2056,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$25,Meals!$A$5:$A$25,$A7,Meals!$M$5:$M$25,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$26,Meals!$A$5:$A$26,$A7,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$25,Meals!$A$5:$A$25,$A7,Meals!$M$5:$M$25,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$26,Meals!$A$5:$A$26,$A7,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -2013,11 +2068,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$25,Meals!$A$5:$A$25,$A7,Meals!$M$5:$M$25,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$26,Meals!$A$5:$A$26,$A7,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$25,Meals!$A$5:$A$25,$A7,Meals!$M$5:$M$25,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$26,Meals!$A$5:$A$26,$A7,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -2025,11 +2080,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$25,$A7,Meals!$M$5:$M$25,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$26,$A7,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$25,$A7,Meals!$M$5:$M$25,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$26,$A7,Meals!$M$5:$M$26,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -2042,11 +2097,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$25,Meals!$A$5:$A$25,$A8,Meals!$M$5:$M$25,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$26,Meals!$A$5:$A$26,$A8,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$25,Meals!$A$5:$A$25,$A8,Meals!$M$5:$M$25,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$26,Meals!$A$5:$A$26,$A8,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -2054,11 +2109,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$25,Meals!$A$5:$A$25,$A8,Meals!$M$5:$M$25,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$26,Meals!$A$5:$A$26,$A8,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$25,Meals!$A$5:$A$25,$A8,Meals!$M$5:$M$25,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$26,Meals!$A$5:$A$26,$A8,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -2066,11 +2121,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$25,Meals!$A$5:$A$25,$A8,Meals!$M$5:$M$25,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$26,Meals!$A$5:$A$26,$A8,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$25,Meals!$A$5:$A$25,$A8,Meals!$M$5:$M$25,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$26,Meals!$A$5:$A$26,$A8,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -2078,11 +2133,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$25,$A8,Meals!$M$5:$M$25,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$26,$A8,Meals!$M$5:$M$26,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$25,$A8,Meals!$M$5:$M$25,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$26,$A8,Meals!$M$5:$M$26,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">

</xml_diff>

<commit_message>
Show how training is counted in maintenance
Adds a breakdown on the Targets sheet: sedentary baseline (BMR x 1.2),
the training allowance that makes up the rest of the multiplier, and the
implied kcal per session against a sessions-per-week input.

At 1.45 the gym is credited 441 kcal/day, or ~514 per session across the
6-day split - right for a 75-90 minute session at 91 kg, generous for a
shorter one. Makes the assumption inspectable instead of buried in a
single multiplier.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -3177,7 +3177,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3454,6 +3454,76 @@
       <c r="C24" s="33" t="inlineStr">
         <is>
           <t>Whatever is left once protein and the fat floor are paid for. Fuels the PPL work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="28" t="inlineStr">
+        <is>
+          <t>Where maintenance comes from</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="29" t="inlineStr">
+        <is>
+          <t>Sedentary baseline (BMR x 1.2)</t>
+        </is>
+      </c>
+      <c r="B27" s="8">
+        <f>B14*1.2</f>
+        <v/>
+      </c>
+      <c r="C27" s="33" t="inlineStr">
+        <is>
+          <t>Living, digestion, fidgeting, walking about - no training.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="29" t="inlineStr">
+        <is>
+          <t>Training allowance</t>
+        </is>
+      </c>
+      <c r="B28" s="8">
+        <f>B15-B27</f>
+        <v/>
+      </c>
+      <c r="C28" s="33" t="inlineStr">
+        <is>
+          <t>The part of the multiplier that is the gym.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="29" t="inlineStr">
+        <is>
+          <t>Sessions per week</t>
+        </is>
+      </c>
+      <c r="B29" s="31" t="n">
+        <v>6</v>
+      </c>
+      <c r="C29" s="33" t="inlineStr">
+        <is>
+          <t>6-day PPL split.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="29" t="inlineStr">
+        <is>
+          <t>Implied kcal per session</t>
+        </is>
+      </c>
+      <c r="B30" s="8">
+        <f>B28*7/B29</f>
+        <v/>
+      </c>
+      <c r="C30" s="33" t="inlineStr">
+        <is>
+          <t>Sanity check: resistance training runs ~5-7 kcal/min, so 45-90 min at this bodyweight is ~225-630 kcal. If sessions are short, this allowance is generous and the multiplier should come down - but let the scale decide, not this cell.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Model walking and calisthenics without crediting them to the target
3 km daily walk plus 60 push-ups and 36 pull-ups comes to ~203 kcal/day
(136 walk, 67 calisthenics), moving maintenance from 2,557 to ~2,760 and
the implied multiplier from 1.45 to 1.57.

Added as a separate block on the Targets sheet that deliberately does not
feed the calorie target: activity credited in advance is how a deficit
disappears. At the unchanged target it implies a 753 kcal/day deficit and
~0.68 kg/week rather than 0.50.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -3177,7 +3177,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3525,6 +3525,123 @@
         <is>
           <t>Sanity check: resistance training runs ~5-7 kcal/min, so 45-90 min at this bodyweight is ~225-630 kcal. If sessions are short, this allowance is generous and the multiplier should come down - but let the scale decide, not this cell.</t>
         </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="28" t="inlineStr">
+        <is>
+          <t>Optional extra activity - modelled but NOT in the target above</t>
+        </is>
+      </c>
+      <c r="C32" s="27" t="inlineStr">
+        <is>
+          <t>Deliberately excluded from the calorie target. Activity credited in advance is the commonest way a deficit quietly disappears; let the scale confirm it first, then decide whether to eat it back.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="29" t="inlineStr">
+        <is>
+          <t>Daily walk (km)</t>
+        </is>
+      </c>
+      <c r="B33" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C33" s="33" t="inlineStr">
+        <is>
+          <t>~30-35 min at a normal pace.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="29" t="inlineStr">
+        <is>
+          <t>Net kcal per kg per km</t>
+        </is>
+      </c>
+      <c r="B34" s="34" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C34" s="33" t="inlineStr">
+        <is>
+          <t>Net of what would have been burned sitting. Gross is ~0.65.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="29" t="inlineStr">
+        <is>
+          <t>Calisthenics (kcal/day)</t>
+        </is>
+      </c>
+      <c r="B35" s="14" t="n">
+        <v>67</v>
+      </c>
+      <c r="C35" s="33" t="inlineStr">
+        <is>
+          <t>60 push-ups ~24 kcal, 36 pull-ups ~43. Real training stimulus, small calorie cost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="29" t="inlineStr">
+        <is>
+          <t>Extra burn</t>
+        </is>
+      </c>
+      <c r="B36" s="8">
+        <f>B33*B34*B5+B35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="29" t="inlineStr">
+        <is>
+          <t>Adjusted maintenance</t>
+        </is>
+      </c>
+      <c r="B37" s="8">
+        <f>B15+B36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="29" t="inlineStr">
+        <is>
+          <t>Implied multiplier</t>
+        </is>
+      </c>
+      <c r="B38" s="26">
+        <f>B37/B14</f>
+        <v/>
+      </c>
+      <c r="C38" s="33" t="inlineStr">
+        <is>
+          <t>Against the 1.45 used above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="29" t="inlineStr">
+        <is>
+          <t>Deficit at the current target</t>
+        </is>
+      </c>
+      <c r="B39" s="8">
+        <f>B37-B16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="29" t="inlineStr">
+        <is>
+          <t>Implied loss (kg/week)</t>
+        </is>
+      </c>
+      <c r="B40" s="26">
+        <f>B39*7/B11</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add grapes to the reference estimates
~60-75 kcal per 100 g (15-20 grapes), roughly twice the calorie density of
melon. Not logged - asked about, not eaten.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -3658,7 +3658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4523,14 +4523,14 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in black coffee no sugar)</t>
+          <t>Grapes (~100 g / 15-20 grapes)</t>
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="C36" s="7" t="n">
-        <v>130</v>
+        <v>75</v>
       </c>
       <c r="D36" s="8">
         <f>AVERAGE(B36:C36)</f>
@@ -4538,22 +4538,26 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="inlineStr"/>
+          <t>~0.6 g</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>Twice the calorie density of melon; easy to eat a large handful without noticing</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Cashew/almond biscuit (1)</t>
+          <t>Whey scoop (in black coffee no sugar)</t>
         </is>
       </c>
       <c r="B37" s="7" t="n">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C37" s="7" t="n">
-        <v>38</v>
+        <v>130</v>
       </c>
       <c r="D37" s="8">
         <f>AVERAGE(B37:C37)</f>
@@ -4561,7 +4565,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>~0.5 g</t>
+          <t>~20-25 g</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr"/>
@@ -4569,14 +4573,14 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (~50g standard)</t>
+          <t>Cashew/almond biscuit (1)</t>
         </is>
       </c>
       <c r="B38" s="7" t="n">
-        <v>245</v>
+        <v>38</v>
       </c>
       <c r="C38" s="7" t="n">
-        <v>250</v>
+        <v>38</v>
       </c>
       <c r="D38" s="8">
         <f>AVERAGE(B38:C38)</f>
@@ -4584,7 +4588,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>~4 g</t>
+          <t>~0.5 g</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr"/>
@@ -4592,14 +4596,14 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (70g king-size)</t>
+          <t>Chocolate bar (~50g standard)</t>
         </is>
       </c>
       <c r="B39" s="7" t="n">
-        <v>335</v>
+        <v>245</v>
       </c>
       <c r="C39" s="7" t="n">
-        <v>335</v>
+        <v>250</v>
       </c>
       <c r="D39" s="8">
         <f>AVERAGE(B39:C39)</f>
@@ -4607,7 +4611,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>~6 g</t>
+          <t>~4 g</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr"/>
@@ -4615,14 +4619,14 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>Pre-workout scoop</t>
+          <t>Chocolate bar (70g king-size)</t>
         </is>
       </c>
       <c r="B40" s="7" t="n">
-        <v>5</v>
+        <v>335</v>
       </c>
       <c r="C40" s="7" t="n">
-        <v>15</v>
+        <v>335</v>
       </c>
       <c r="D40" s="8">
         <f>AVERAGE(B40:C40)</f>
@@ -4630,10 +4634,33 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
+          <t>~6 g</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>Pre-workout scoop</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C41" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D41" s="8">
+        <f>AVERAGE(B41:C41)</f>
+        <v/>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
           <t>0 g</t>
         </is>
       </c>
-      <c r="F40" s="6" t="inlineStr">
+      <c r="F41" s="6" t="inlineStr">
         <is>
           <t>Negligible</t>
         </is>

</xml_diff>

<commit_message>
Log ~100 g red grapes on Day 4
60-75 kcal, 0.5-0.7 g protein. Day 4 stands at 1,820.5 kcal and 90.6 g of
protein before dinner.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N26"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1817,6 +1817,61 @@
       <c r="N26" s="6" t="inlineStr">
         <is>
           <t>Second egg serving of the day - four eggs total</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Red grapes (~100 g)</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="F27" s="8">
+        <f>AVERAGE(D27:E27)</f>
+        <v/>
+      </c>
+      <c r="G27" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H27" s="9" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I27" s="10">
+        <f>AVERAGE(G27:H27)</f>
+        <v/>
+      </c>
+      <c r="J27" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L27" s="10">
+        <f>AVERAGE(J27:K27)</f>
+        <v/>
+      </c>
+      <c r="M27" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N27" s="6" t="inlineStr">
+        <is>
+          <t>Portioned into a box rather than eaten from the bunch; some left over</t>
         </is>
       </c>
     </row>
@@ -1938,11 +1993,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$26,Meals!$A$5:$A$26,$A5,Meals!$M$5:$M$26,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$27,Meals!$A$5:$A$27,$A5,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$26,Meals!$A$5:$A$26,$A5,Meals!$M$5:$M$26,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$27,Meals!$A$5:$A$27,$A5,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -1950,11 +2005,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$26,Meals!$A$5:$A$26,$A5,Meals!$M$5:$M$26,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$27,Meals!$A$5:$A$27,$A5,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$26,Meals!$A$5:$A$26,$A5,Meals!$M$5:$M$26,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$27,Meals!$A$5:$A$27,$A5,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -1962,11 +2017,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$26,Meals!$A$5:$A$26,$A5,Meals!$M$5:$M$26,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$27,Meals!$A$5:$A$27,$A5,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$26,Meals!$A$5:$A$26,$A5,Meals!$M$5:$M$26,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$27,Meals!$A$5:$A$27,$A5,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -1974,11 +2029,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$26,$A5,Meals!$M$5:$M$26,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$27,$A5,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$26,$A5,Meals!$M$5:$M$26,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$27,$A5,Meals!$M$5:$M$27,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -1991,11 +2046,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$26,Meals!$A$5:$A$26,$A6,Meals!$M$5:$M$26,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$27,Meals!$A$5:$A$27,$A6,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$26,Meals!$A$5:$A$26,$A6,Meals!$M$5:$M$26,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$27,Meals!$A$5:$A$27,$A6,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -2003,11 +2058,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$26,Meals!$A$5:$A$26,$A6,Meals!$M$5:$M$26,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$27,Meals!$A$5:$A$27,$A6,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$26,Meals!$A$5:$A$26,$A6,Meals!$M$5:$M$26,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$27,Meals!$A$5:$A$27,$A6,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -2015,11 +2070,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$26,Meals!$A$5:$A$26,$A6,Meals!$M$5:$M$26,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$27,Meals!$A$5:$A$27,$A6,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$26,Meals!$A$5:$A$26,$A6,Meals!$M$5:$M$26,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$27,Meals!$A$5:$A$27,$A6,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -2027,11 +2082,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$26,$A6,Meals!$M$5:$M$26,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$27,$A6,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$26,$A6,Meals!$M$5:$M$26,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$27,$A6,Meals!$M$5:$M$27,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -2044,11 +2099,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$26,Meals!$A$5:$A$26,$A7,Meals!$M$5:$M$26,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$27,Meals!$A$5:$A$27,$A7,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$26,Meals!$A$5:$A$26,$A7,Meals!$M$5:$M$26,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$27,Meals!$A$5:$A$27,$A7,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -2056,11 +2111,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$26,Meals!$A$5:$A$26,$A7,Meals!$M$5:$M$26,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$27,Meals!$A$5:$A$27,$A7,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$26,Meals!$A$5:$A$26,$A7,Meals!$M$5:$M$26,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$27,Meals!$A$5:$A$27,$A7,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -2068,11 +2123,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$26,Meals!$A$5:$A$26,$A7,Meals!$M$5:$M$26,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$27,Meals!$A$5:$A$27,$A7,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$26,Meals!$A$5:$A$26,$A7,Meals!$M$5:$M$26,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$27,Meals!$A$5:$A$27,$A7,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -2080,11 +2135,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$26,$A7,Meals!$M$5:$M$26,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$27,$A7,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$26,$A7,Meals!$M$5:$M$26,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$27,$A7,Meals!$M$5:$M$27,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -2097,11 +2152,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$26,Meals!$A$5:$A$26,$A8,Meals!$M$5:$M$26,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$27,Meals!$A$5:$A$27,$A8,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$26,Meals!$A$5:$A$26,$A8,Meals!$M$5:$M$26,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$27,Meals!$A$5:$A$27,$A8,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -2109,11 +2164,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$26,Meals!$A$5:$A$26,$A8,Meals!$M$5:$M$26,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$27,Meals!$A$5:$A$27,$A8,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$26,Meals!$A$5:$A$26,$A8,Meals!$M$5:$M$26,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$27,Meals!$A$5:$A$27,$A8,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -2121,11 +2176,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$26,Meals!$A$5:$A$26,$A8,Meals!$M$5:$M$26,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$27,Meals!$A$5:$A$27,$A8,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$26,Meals!$A$5:$A$26,$A8,Meals!$M$5:$M$26,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$27,Meals!$A$5:$A$27,$A8,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -2133,11 +2188,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$26,$A8,Meals!$M$5:$M$26,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$27,$A8,Meals!$M$5:$M$27,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$26,$A8,Meals!$M$5:$M$26,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$27,$A8,Meals!$M$5:$M$27,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">

</xml_diff>

<commit_message>
Correct the mess model: dinner bread is chapati, not porotta
Chapati is ~115 kcal and ~3 g fat against ~205 kcal and ~11 g for a porotta,
so every dinner in the model was overstated. Reworked all seven dinners in
mess_menu.csv and reset the Mess Plan bread assumption.

The week now averages 1,839 kcal and 67.8 g protein (3.7 g per 100 kcal,
up from 3.1). This reverses the earlier advice to skip a bread item: chapati
is good value and both should be kept. Rice is the lever instead.

Wednesday and Saturday are now the tight days at 2,160 and 2,100 kcal as
served, loaded by the poratta and dosa-set breakfasts. Friday is the best at
1,455 kcal and 47.5 g fat.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -2385,11 +2385,11 @@
         </is>
       </c>
       <c r="B5" s="14" t="n">
-        <v>205</v>
+        <v>115</v>
       </c>
       <c r="C5" s="27" t="inlineStr">
         <is>
-          <t>1 porotta/poori. The worst protein-per-calorie item on the menu.</t>
+          <t>Dinner bread is chapati, not porotta - roughly half the calories and a third of the fat.</t>
         </is>
       </c>
     </row>
@@ -2400,7 +2400,7 @@
         </is>
       </c>
       <c r="B6" s="16" t="n">
-        <v>5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="7">
@@ -2538,17 +2538,17 @@
       </c>
       <c r="D14" s="30" t="inlineStr">
         <is>
-          <t>Chicken curry + bread items</t>
+          <t>Chicken curry + 2 chapati</t>
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>2065</v>
+        <v>1885</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>74.5</v>
+        <v>72.5</v>
       </c>
       <c r="G14" s="31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H14" s="31" t="n">
         <v>1</v>
@@ -2592,17 +2592,17 @@
       </c>
       <c r="D15" s="30" t="inlineStr">
         <is>
-          <t>Green peas + bread items</t>
+          <t>Green peas + 2 chapati</t>
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>1745</v>
+        <v>1565</v>
       </c>
       <c r="F15" s="9" t="n">
         <v>54.5</v>
       </c>
       <c r="G15" s="31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H15" s="31" t="n">
         <v>1</v>
@@ -2646,17 +2646,17 @@
       </c>
       <c r="D16" s="30" t="inlineStr">
         <is>
-          <t>Chicken traditional curry + bread</t>
+          <t>Chicken traditional curry + 2 chapati</t>
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>2340</v>
+        <v>2160</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>90.5</v>
+        <v>88.5</v>
       </c>
       <c r="G16" s="31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H16" s="31" t="n">
         <v>1</v>
@@ -2700,17 +2700,17 @@
       </c>
       <c r="D17" s="30" t="inlineStr">
         <is>
-          <t>Gobbi chilly + bread items</t>
+          <t>Gobbi chilly + 2 chapati</t>
         </is>
       </c>
       <c r="E17" s="7" t="n">
-        <v>2010</v>
+        <v>1830</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G17" s="31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H17" s="31" t="n">
         <v>1</v>
@@ -2754,17 +2754,17 @@
       </c>
       <c r="D18" s="30" t="inlineStr">
         <is>
-          <t>Kadala curry + bread items</t>
+          <t>Kadala curry + 2 chapati</t>
         </is>
       </c>
       <c r="E18" s="7" t="n">
-        <v>1635</v>
+        <v>1455</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="G18" s="31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H18" s="31" t="n">
         <v>0</v>
@@ -2808,17 +2808,17 @@
       </c>
       <c r="D19" s="30" t="inlineStr">
         <is>
-          <t>Chicken varutharachathu + bread</t>
+          <t>Chicken varutharachathu + 2 chapati</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
-        <v>2280</v>
+        <v>2100</v>
       </c>
       <c r="F19" s="9" t="n">
         <v>77</v>
       </c>
       <c r="G19" s="31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H19" s="31" t="n">
         <v>1</v>
@@ -2862,17 +2862,17 @@
       </c>
       <c r="D20" s="30" t="inlineStr">
         <is>
-          <t>Egg roast + bread items</t>
+          <t>Egg roast + 2 chapati</t>
         </is>
       </c>
       <c r="E20" s="7" t="n">
-        <v>2055</v>
+        <v>1875</v>
       </c>
       <c r="F20" s="9" t="n">
         <v>69</v>
       </c>
       <c r="G20" s="31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H20" s="31" t="n">
         <v>1</v>
@@ -3713,7 +3713,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4035,14 +4035,14 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Uzhunnu vada / medu vada (1)</t>
+          <t>Chapati (1)</t>
         </is>
       </c>
       <c r="B15" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>130</v>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>180</v>
       </c>
       <c r="D15" s="8">
         <f>AVERAGE(B15:C15)</f>
@@ -4050,26 +4050,26 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>~3.5-5 g each</t>
+          <t>~3-4 g each</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>Deep-fried urad dal - protein-bearing but fat-dense</t>
+          <t>Whole wheat with little or no oil - about half a porotta's calories and a third of its fat</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Kadala curry (1 container)</t>
+          <t>Uzhunnu vada / medu vada (1)</t>
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>200</v>
+        <v>130</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>300</v>
+        <v>180</v>
       </c>
       <c r="D16" s="8">
         <f>AVERAGE(B16:C16)</f>
@@ -4077,22 +4077,26 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>~8-10 g</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr"/>
+          <t>~3.5-5 g each</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Deep-fried urad dal - protein-bearing but fat-dense</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Fish fry (1 piece pan-fried)</t>
+          <t>Kadala curry (1 container)</t>
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="C17" s="7" t="n">
-        <v>220</v>
+        <v>300</v>
       </c>
       <c r="D17" s="8">
         <f>AVERAGE(B17:C17)</f>
@@ -4100,7 +4104,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>~15-20 g</t>
+          <t>~8-10 g</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr"/>
@@ -4108,14 +4112,14 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Grilled chicken breast (100 g skinless)</t>
+          <t>Fish fry (1 piece pan-fried)</t>
         </is>
       </c>
       <c r="B18" s="7" t="n">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>180</v>
+        <v>220</v>
       </c>
       <c r="D18" s="8">
         <f>AVERAGE(B18:C18)</f>
@@ -4123,26 +4127,22 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>~30-32 g</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>Best protein-per-calorie item in this list</t>
-        </is>
-      </c>
+          <t>~15-20 g</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Grilled chicken breast (150 g skinless)</t>
+          <t>Grilled chicken breast (100 g skinless)</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>240</v>
+        <v>160</v>
       </c>
       <c r="C19" s="7" t="n">
-        <v>270</v>
+        <v>180</v>
       </c>
       <c r="D19" s="8">
         <f>AVERAGE(B19:C19)</f>
@@ -4150,22 +4150,26 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>~45-48 g</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr"/>
+          <t>~30-32 g</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>Best protein-per-calorie item in this list</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Honest Bowl - Grilled Chicken and Rice Bowl</t>
+          <t>Grilled chicken breast (150 g skinless)</t>
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>550</v>
+        <v>240</v>
       </c>
       <c r="C20" s="7" t="n">
-        <v>710</v>
+        <v>270</v>
       </c>
       <c r="D20" s="8">
         <f>AVERAGE(B20:C20)</f>
@@ -4173,26 +4177,22 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>42-48 g</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>Menu states 42 g protein; chicken + jasmine rice + sweet potato. Sauce served separately</t>
-        </is>
-      </c>
+          <t>~45-48 g</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Brown/mushroom sauce (side pot)</t>
+          <t>Honest Bowl - Grilled Chicken and Rice Bowl</t>
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>50</v>
+        <v>550</v>
       </c>
       <c r="C21" s="7" t="n">
-        <v>120</v>
+        <v>710</v>
       </c>
       <c r="D21" s="8">
         <f>AVERAGE(B21:C21)</f>
@@ -4200,26 +4200,26 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>~1-2 g</t>
+          <t>42-48 g</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>Often cream or butter based - the variable in a bowl like this</t>
+          <t>Menu states 42 g protein; chicken + jasmine rice + sweet potato. Sauce served separately</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Honest Bowl - Tofu Delight Bowl</t>
+          <t>Brown/mushroom sauce (side pot)</t>
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>420</v>
+        <v>50</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>560</v>
+        <v>120</v>
       </c>
       <c r="D22" s="8">
         <f>AVERAGE(B22:C22)</f>
@@ -4227,26 +4227,26 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>~20 g</t>
+          <t>~1-2 g</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>Menu states 20 g; jasmine rice + cajun tofu + grilled eggplant. Half the protein of the chicken bowl at the same price</t>
+          <t>Often cream or butter based - the variable in a bowl like this</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Chicken curry (1 takeaway container)</t>
+          <t>Honest Bowl - Tofu Delight Bowl</t>
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>280</v>
+        <v>420</v>
       </c>
       <c r="C23" s="7" t="n">
-        <v>420</v>
+        <v>560</v>
       </c>
       <c r="D23" s="8">
         <f>AVERAGE(B23:C23)</f>
@@ -4254,26 +4254,26 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>~20-28 g</t>
+          <t>~20 g</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>Kerala style; oil and coconut carry most of the calories</t>
+          <t>Menu states 20 g; jasmine rice + cajun tofu + grilled eggplant. Half the protein of the chicken bowl at the same price</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Grilled chicken quarter (skin on)</t>
+          <t>Chicken curry (1 takeaway container)</t>
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>250</v>
+        <v>280</v>
       </c>
       <c r="C24" s="7" t="n">
-        <v>320</v>
+        <v>420</v>
       </c>
       <c r="D24" s="8">
         <f>AVERAGE(B24:C24)</f>
@@ -4281,26 +4281,26 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>~28-33 g</t>
+          <t>~20-28 g</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>Skin adds ~12-15 g fat over breast</t>
+          <t>Kerala style; oil and coconut carry most of the calories</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Garlic sauce / toum (1 tbsp)</t>
+          <t>Grilled chicken quarter (skin on)</t>
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>90</v>
+        <v>250</v>
       </c>
       <c r="C25" s="7" t="n">
-        <v>110</v>
+        <v>320</v>
       </c>
       <c r="D25" s="8">
         <f>AVERAGE(B25:C25)</f>
@@ -4308,26 +4308,26 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>0 g</t>
+          <t>~28-33 g</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>Essentially emulsified oil - the hidden cost at a grill</t>
+          <t>Skin adds ~12-15 g fat over breast</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Khubz / pita (1 large)</t>
+          <t>Garlic sauce / toum (1 tbsp)</t>
         </is>
       </c>
       <c r="B26" s="7" t="n">
-        <v>250</v>
+        <v>90</v>
       </c>
       <c r="C26" s="7" t="n">
-        <v>300</v>
+        <v>110</v>
       </c>
       <c r="D26" s="8">
         <f>AVERAGE(B26:C26)</f>
@@ -4335,22 +4335,26 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>~8-9 g</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr"/>
+          <t>0 g</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>Essentially emulsified oil - the hidden cost at a grill</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Barik/basmati rice (half container cooked)</t>
+          <t>Khubz / pita (1 large)</t>
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="C27" s="7" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="D27" s="8">
         <f>AVERAGE(B27:C27)</f>
@@ -4358,7 +4362,7 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>~4-5 g</t>
+          <t>~8-9 g</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr"/>
@@ -4366,14 +4370,14 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Fresh pineapple juice (350-450 ml)</t>
+          <t>Barik/basmati rice (half container cooked)</t>
         </is>
       </c>
       <c r="B28" s="7" t="n">
-        <v>175</v>
+        <v>200</v>
       </c>
       <c r="C28" s="7" t="n">
-        <v>240</v>
+        <v>280</v>
       </c>
       <c r="D28" s="8">
         <f>AVERAGE(B28:C28)</f>
@@ -4381,26 +4385,22 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>~1-2 g</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>No added sugar but ~35-45 g natural sugar; no fibre; almost no protein</t>
-        </is>
-      </c>
+          <t>~4-5 g</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Fresh orange juice (350-450 ml)</t>
+          <t>Fresh pineapple juice (350-450 ml)</t>
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>155</v>
+        <v>175</v>
       </c>
       <c r="C29" s="7" t="n">
-        <v>205</v>
+        <v>240</v>
       </c>
       <c r="D29" s="8">
         <f>AVERAGE(B29:C29)</f>
@@ -4408,26 +4408,26 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>~2-3 g</t>
+          <t>~1-2 g</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>No added sugar but ~32-40 g natural sugar; no fibre</t>
+          <t>No added sugar but ~35-45 g natural sugar; no fibre; almost no protein</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in water)</t>
+          <t>Fresh orange juice (350-450 ml)</t>
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>100</v>
+        <v>155</v>
       </c>
       <c r="C30" s="7" t="n">
-        <v>120</v>
+        <v>205</v>
       </c>
       <c r="D30" s="8">
         <f>AVERAGE(B30:C30)</f>
@@ -4435,22 +4435,26 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="inlineStr"/>
+          <t>~2-3 g</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>No added sugar but ~32-40 g natural sugar; no fibre</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Greek yogurt (200 g plain low-fat)</t>
+          <t>Whey scoop (in water)</t>
         </is>
       </c>
       <c r="B31" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C31" s="7" t="n">
         <v>120</v>
-      </c>
-      <c r="C31" s="7" t="n">
-        <v>140</v>
       </c>
       <c r="D31" s="8">
         <f>AVERAGE(B31:C31)</f>
@@ -4458,26 +4462,22 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>~18-20 g</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="inlineStr">
-        <is>
-          <t>Casein - digests slowly; good overnight</t>
-        </is>
-      </c>
+          <t>~20-25 g</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Boiled egg (1 large)</t>
+          <t>Greek yogurt (200 g plain low-fat)</t>
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>70</v>
+        <v>120</v>
       </c>
       <c r="C32" s="7" t="n">
-        <v>78</v>
+        <v>140</v>
       </c>
       <c r="D32" s="8">
         <f>AVERAGE(B32:C32)</f>
@@ -4485,26 +4485,26 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>~6-6.5 g</t>
+          <t>~18-20 g</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>~5 g fat each</t>
+          <t>Casein - digests slowly; good overnight</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Paneer (50 g full-fat)</t>
+          <t>Boiled egg (1 large)</t>
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>130</v>
+        <v>70</v>
       </c>
       <c r="C33" s="7" t="n">
-        <v>150</v>
+        <v>78</v>
       </c>
       <c r="D33" s="8">
         <f>AVERAGE(B33:C33)</f>
@@ -4512,26 +4512,26 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>~8-9 g</t>
+          <t>~6-6.5 g</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>Fat-dense for the protein it gives</t>
+          <t>~5 g fat each</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Cucumber (1 medium)</t>
+          <t>Paneer (50 g full-fat)</t>
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>25</v>
+        <v>130</v>
       </c>
       <c r="C34" s="7" t="n">
-        <v>30</v>
+        <v>150</v>
       </c>
       <c r="D34" s="8">
         <f>AVERAGE(B34:C34)</f>
@@ -4539,26 +4539,26 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>~1.5 g</t>
+          <t>~8-9 g</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>Volume with almost no calories</t>
+          <t>Fat-dense for the protein it gives</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Sweet melon / cantaloupe (1 wedge ~100-150 g)</t>
+          <t>Cucumber (1 medium)</t>
         </is>
       </c>
       <c r="B35" s="7" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="C35" s="7" t="n">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="D35" s="8">
         <f>AVERAGE(B35:C35)</f>
@@ -4566,26 +4566,26 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>~0.5-1 g</t>
+          <t>~1.5 g</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>Whole fruit - fibre and water intact; ~1/4 the calories of the same fruit juiced</t>
+          <t>Volume with almost no calories</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Grapes (~100 g / 15-20 grapes)</t>
+          <t>Sweet melon / cantaloupe (1 wedge ~100-150 g)</t>
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="C36" s="7" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="D36" s="8">
         <f>AVERAGE(B36:C36)</f>
@@ -4593,26 +4593,26 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>~0.6 g</t>
+          <t>~0.5-1 g</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>Twice the calorie density of melon; easy to eat a large handful without noticing</t>
+          <t>Whole fruit - fibre and water intact; ~1/4 the calories of the same fruit juiced</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in black coffee no sugar)</t>
+          <t>Grapes (~100 g / 15-20 grapes)</t>
         </is>
       </c>
       <c r="B37" s="7" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="C37" s="7" t="n">
-        <v>130</v>
+        <v>75</v>
       </c>
       <c r="D37" s="8">
         <f>AVERAGE(B37:C37)</f>
@@ -4620,22 +4620,26 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F37" s="6" t="inlineStr"/>
+          <t>~0.6 g</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>Twice the calorie density of melon; easy to eat a large handful without noticing</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>Cashew/almond biscuit (1)</t>
+          <t>Whey scoop (in black coffee no sugar)</t>
         </is>
       </c>
       <c r="B38" s="7" t="n">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C38" s="7" t="n">
-        <v>38</v>
+        <v>130</v>
       </c>
       <c r="D38" s="8">
         <f>AVERAGE(B38:C38)</f>
@@ -4643,7 +4647,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>~0.5 g</t>
+          <t>~20-25 g</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr"/>
@@ -4651,14 +4655,14 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (~50g standard)</t>
+          <t>Cashew/almond biscuit (1)</t>
         </is>
       </c>
       <c r="B39" s="7" t="n">
-        <v>245</v>
+        <v>38</v>
       </c>
       <c r="C39" s="7" t="n">
-        <v>250</v>
+        <v>38</v>
       </c>
       <c r="D39" s="8">
         <f>AVERAGE(B39:C39)</f>
@@ -4666,7 +4670,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>~4 g</t>
+          <t>~0.5 g</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr"/>
@@ -4674,14 +4678,14 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (70g king-size)</t>
+          <t>Chocolate bar (~50g standard)</t>
         </is>
       </c>
       <c r="B40" s="7" t="n">
-        <v>335</v>
+        <v>245</v>
       </c>
       <c r="C40" s="7" t="n">
-        <v>335</v>
+        <v>250</v>
       </c>
       <c r="D40" s="8">
         <f>AVERAGE(B40:C40)</f>
@@ -4689,7 +4693,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>~6 g</t>
+          <t>~4 g</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr"/>
@@ -4697,14 +4701,14 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>Pre-workout scoop</t>
+          <t>Chocolate bar (70g king-size)</t>
         </is>
       </c>
       <c r="B41" s="7" t="n">
-        <v>5</v>
+        <v>335</v>
       </c>
       <c r="C41" s="7" t="n">
-        <v>15</v>
+        <v>335</v>
       </c>
       <c r="D41" s="8">
         <f>AVERAGE(B41:C41)</f>
@@ -4712,10 +4716,33 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
+          <t>~6 g</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>Pre-workout scoop</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C42" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D42" s="8">
+        <f>AVERAGE(B42:C42)</f>
+        <v/>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
           <t>0 g</t>
         </is>
       </c>
-      <c r="F41" s="6" t="inlineStr">
+      <c r="F42" s="6" t="inlineStr">
         <is>
           <t>Negligible</t>
         </is>

</xml_diff>

<commit_message>
Log chatti pathiri chicken on Day 4
1 slice at 230-320 kcal, 10-14 g protein, 12-18 g fat. Day 4 reaches
2,095.5 kcal and 80.25 g of fat before dinner, so dinner drops to curry
with at most one chapati.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N27"/>
+  <dimension ref="A1:N28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1872,6 +1872,61 @@
       <c r="N27" s="6" t="inlineStr">
         <is>
           <t>Portioned into a box rather than eaten from the bunch; some left over</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>Chatti pathiri chicken (1 slice)</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>230</v>
+      </c>
+      <c r="E28" s="7" t="n">
+        <v>320</v>
+      </c>
+      <c r="F28" s="8">
+        <f>AVERAGE(D28:E28)</f>
+        <v/>
+      </c>
+      <c r="G28" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="H28" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="I28" s="10">
+        <f>AVERAGE(G28:H28)</f>
+        <v/>
+      </c>
+      <c r="J28" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="K28" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="L28" s="10">
+        <f>AVERAGE(J28:K28)</f>
+        <v/>
+      </c>
+      <c r="M28" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N28" s="6" t="inlineStr">
+        <is>
+          <t>Before dinner. Slice count assumed 1 - double if it was 2</t>
         </is>
       </c>
     </row>
@@ -1993,11 +2048,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$27,Meals!$A$5:$A$27,$A5,Meals!$M$5:$M$27,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$28,Meals!$A$5:$A$28,$A5,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$27,Meals!$A$5:$A$27,$A5,Meals!$M$5:$M$27,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$28,Meals!$A$5:$A$28,$A5,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -2005,11 +2060,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$27,Meals!$A$5:$A$27,$A5,Meals!$M$5:$M$27,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$28,Meals!$A$5:$A$28,$A5,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$27,Meals!$A$5:$A$27,$A5,Meals!$M$5:$M$27,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$28,Meals!$A$5:$A$28,$A5,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -2017,11 +2072,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$27,Meals!$A$5:$A$27,$A5,Meals!$M$5:$M$27,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$28,Meals!$A$5:$A$28,$A5,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$27,Meals!$A$5:$A$27,$A5,Meals!$M$5:$M$27,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$28,Meals!$A$5:$A$28,$A5,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -2029,11 +2084,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$27,$A5,Meals!$M$5:$M$27,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$28,$A5,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$27,$A5,Meals!$M$5:$M$27,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$28,$A5,Meals!$M$5:$M$28,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -2046,11 +2101,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$27,Meals!$A$5:$A$27,$A6,Meals!$M$5:$M$27,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$28,Meals!$A$5:$A$28,$A6,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$27,Meals!$A$5:$A$27,$A6,Meals!$M$5:$M$27,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$28,Meals!$A$5:$A$28,$A6,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -2058,11 +2113,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$27,Meals!$A$5:$A$27,$A6,Meals!$M$5:$M$27,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$28,Meals!$A$5:$A$28,$A6,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$27,Meals!$A$5:$A$27,$A6,Meals!$M$5:$M$27,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$28,Meals!$A$5:$A$28,$A6,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -2070,11 +2125,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$27,Meals!$A$5:$A$27,$A6,Meals!$M$5:$M$27,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$28,Meals!$A$5:$A$28,$A6,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$27,Meals!$A$5:$A$27,$A6,Meals!$M$5:$M$27,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$28,Meals!$A$5:$A$28,$A6,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -2082,11 +2137,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$27,$A6,Meals!$M$5:$M$27,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$28,$A6,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$27,$A6,Meals!$M$5:$M$27,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$28,$A6,Meals!$M$5:$M$28,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -2099,11 +2154,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$27,Meals!$A$5:$A$27,$A7,Meals!$M$5:$M$27,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$28,Meals!$A$5:$A$28,$A7,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$27,Meals!$A$5:$A$27,$A7,Meals!$M$5:$M$27,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$28,Meals!$A$5:$A$28,$A7,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -2111,11 +2166,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$27,Meals!$A$5:$A$27,$A7,Meals!$M$5:$M$27,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$28,Meals!$A$5:$A$28,$A7,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$27,Meals!$A$5:$A$27,$A7,Meals!$M$5:$M$27,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$28,Meals!$A$5:$A$28,$A7,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -2123,11 +2178,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$27,Meals!$A$5:$A$27,$A7,Meals!$M$5:$M$27,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$28,Meals!$A$5:$A$28,$A7,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$27,Meals!$A$5:$A$27,$A7,Meals!$M$5:$M$27,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$28,Meals!$A$5:$A$28,$A7,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -2135,11 +2190,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$27,$A7,Meals!$M$5:$M$27,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$28,$A7,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$27,$A7,Meals!$M$5:$M$27,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$28,$A7,Meals!$M$5:$M$28,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -2152,11 +2207,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$27,Meals!$A$5:$A$27,$A8,Meals!$M$5:$M$27,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$28,Meals!$A$5:$A$28,$A8,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$27,Meals!$A$5:$A$27,$A8,Meals!$M$5:$M$27,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$28,Meals!$A$5:$A$28,$A8,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -2164,11 +2219,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$27,Meals!$A$5:$A$27,$A8,Meals!$M$5:$M$27,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$28,Meals!$A$5:$A$28,$A8,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$27,Meals!$A$5:$A$27,$A8,Meals!$M$5:$M$27,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$28,Meals!$A$5:$A$28,$A8,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -2176,11 +2231,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$27,Meals!$A$5:$A$27,$A8,Meals!$M$5:$M$27,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$28,Meals!$A$5:$A$28,$A8,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$27,Meals!$A$5:$A$27,$A8,Meals!$M$5:$M$27,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$28,Meals!$A$5:$A$28,$A8,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -2188,11 +2243,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$27,$A8,Meals!$M$5:$M$27,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$28,$A8,Meals!$M$5:$M$28,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$27,$A8,Meals!$M$5:$M$27,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$28,$A8,Meals!$M$5:$M$28,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -3713,7 +3768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4062,14 +4117,14 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Uzhunnu vada / medu vada (1)</t>
+          <t>Chatti pathiri chicken (1 slice ~100-120 g)</t>
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>130</v>
+        <v>230</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>180</v>
+        <v>320</v>
       </c>
       <c r="D16" s="8">
         <f>AVERAGE(B16:C16)</f>
@@ -4077,26 +4132,26 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>~3.5-5 g each</t>
+          <t>~10-14 g</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>Deep-fried urad dal - protein-bearing but fat-dense</t>
+          <t>Layered maida pathiri with chicken masala and an egg-milk binder; ghee-rich</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Kadala curry (1 container)</t>
+          <t>Uzhunnu vada / medu vada (1)</t>
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>200</v>
+        <v>130</v>
       </c>
       <c r="C17" s="7" t="n">
-        <v>300</v>
+        <v>180</v>
       </c>
       <c r="D17" s="8">
         <f>AVERAGE(B17:C17)</f>
@@ -4104,22 +4159,26 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>~8-10 g</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr"/>
+          <t>~3.5-5 g each</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Deep-fried urad dal - protein-bearing but fat-dense</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Fish fry (1 piece pan-fried)</t>
+          <t>Kadala curry (1 container)</t>
         </is>
       </c>
       <c r="B18" s="7" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>220</v>
+        <v>300</v>
       </c>
       <c r="D18" s="8">
         <f>AVERAGE(B18:C18)</f>
@@ -4127,7 +4186,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>~15-20 g</t>
+          <t>~8-10 g</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr"/>
@@ -4135,14 +4194,14 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Grilled chicken breast (100 g skinless)</t>
+          <t>Fish fry (1 piece pan-fried)</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="C19" s="7" t="n">
-        <v>180</v>
+        <v>220</v>
       </c>
       <c r="D19" s="8">
         <f>AVERAGE(B19:C19)</f>
@@ -4150,26 +4209,22 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>~30-32 g</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>Best protein-per-calorie item in this list</t>
-        </is>
-      </c>
+          <t>~15-20 g</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Grilled chicken breast (150 g skinless)</t>
+          <t>Grilled chicken breast (100 g skinless)</t>
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>240</v>
+        <v>160</v>
       </c>
       <c r="C20" s="7" t="n">
-        <v>270</v>
+        <v>180</v>
       </c>
       <c r="D20" s="8">
         <f>AVERAGE(B20:C20)</f>
@@ -4177,22 +4232,26 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>~45-48 g</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr"/>
+          <t>~30-32 g</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Best protein-per-calorie item in this list</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Honest Bowl - Grilled Chicken and Rice Bowl</t>
+          <t>Grilled chicken breast (150 g skinless)</t>
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>550</v>
+        <v>240</v>
       </c>
       <c r="C21" s="7" t="n">
-        <v>710</v>
+        <v>270</v>
       </c>
       <c r="D21" s="8">
         <f>AVERAGE(B21:C21)</f>
@@ -4200,26 +4259,22 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>42-48 g</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>Menu states 42 g protein; chicken + jasmine rice + sweet potato. Sauce served separately</t>
-        </is>
-      </c>
+          <t>~45-48 g</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Brown/mushroom sauce (side pot)</t>
+          <t>Honest Bowl - Grilled Chicken and Rice Bowl</t>
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>50</v>
+        <v>550</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>120</v>
+        <v>710</v>
       </c>
       <c r="D22" s="8">
         <f>AVERAGE(B22:C22)</f>
@@ -4227,26 +4282,26 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>~1-2 g</t>
+          <t>42-48 g</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>Often cream or butter based - the variable in a bowl like this</t>
+          <t>Menu states 42 g protein; chicken + jasmine rice + sweet potato. Sauce served separately</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Honest Bowl - Tofu Delight Bowl</t>
+          <t>Brown/mushroom sauce (side pot)</t>
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>420</v>
+        <v>50</v>
       </c>
       <c r="C23" s="7" t="n">
-        <v>560</v>
+        <v>120</v>
       </c>
       <c r="D23" s="8">
         <f>AVERAGE(B23:C23)</f>
@@ -4254,26 +4309,26 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>~20 g</t>
+          <t>~1-2 g</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>Menu states 20 g; jasmine rice + cajun tofu + grilled eggplant. Half the protein of the chicken bowl at the same price</t>
+          <t>Often cream or butter based - the variable in a bowl like this</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Chicken curry (1 takeaway container)</t>
+          <t>Honest Bowl - Tofu Delight Bowl</t>
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>280</v>
+        <v>420</v>
       </c>
       <c r="C24" s="7" t="n">
-        <v>420</v>
+        <v>560</v>
       </c>
       <c r="D24" s="8">
         <f>AVERAGE(B24:C24)</f>
@@ -4281,26 +4336,26 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>~20-28 g</t>
+          <t>~20 g</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>Kerala style; oil and coconut carry most of the calories</t>
+          <t>Menu states 20 g; jasmine rice + cajun tofu + grilled eggplant. Half the protein of the chicken bowl at the same price</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Grilled chicken quarter (skin on)</t>
+          <t>Chicken curry (1 takeaway container)</t>
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>250</v>
+        <v>280</v>
       </c>
       <c r="C25" s="7" t="n">
-        <v>320</v>
+        <v>420</v>
       </c>
       <c r="D25" s="8">
         <f>AVERAGE(B25:C25)</f>
@@ -4308,26 +4363,26 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>~28-33 g</t>
+          <t>~20-28 g</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>Skin adds ~12-15 g fat over breast</t>
+          <t>Kerala style; oil and coconut carry most of the calories</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Garlic sauce / toum (1 tbsp)</t>
+          <t>Grilled chicken quarter (skin on)</t>
         </is>
       </c>
       <c r="B26" s="7" t="n">
-        <v>90</v>
+        <v>250</v>
       </c>
       <c r="C26" s="7" t="n">
-        <v>110</v>
+        <v>320</v>
       </c>
       <c r="D26" s="8">
         <f>AVERAGE(B26:C26)</f>
@@ -4335,26 +4390,26 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>0 g</t>
+          <t>~28-33 g</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>Essentially emulsified oil - the hidden cost at a grill</t>
+          <t>Skin adds ~12-15 g fat over breast</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Khubz / pita (1 large)</t>
+          <t>Garlic sauce / toum (1 tbsp)</t>
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>250</v>
+        <v>90</v>
       </c>
       <c r="C27" s="7" t="n">
-        <v>300</v>
+        <v>110</v>
       </c>
       <c r="D27" s="8">
         <f>AVERAGE(B27:C27)</f>
@@ -4362,22 +4417,26 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>~8-9 g</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr"/>
+          <t>0 g</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>Essentially emulsified oil - the hidden cost at a grill</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Barik/basmati rice (half container cooked)</t>
+          <t>Khubz / pita (1 large)</t>
         </is>
       </c>
       <c r="B28" s="7" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="C28" s="7" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="D28" s="8">
         <f>AVERAGE(B28:C28)</f>
@@ -4385,7 +4444,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>~4-5 g</t>
+          <t>~8-9 g</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr"/>
@@ -4393,14 +4452,14 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Fresh pineapple juice (350-450 ml)</t>
+          <t>Barik/basmati rice (half container cooked)</t>
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>175</v>
+        <v>200</v>
       </c>
       <c r="C29" s="7" t="n">
-        <v>240</v>
+        <v>280</v>
       </c>
       <c r="D29" s="8">
         <f>AVERAGE(B29:C29)</f>
@@ -4408,26 +4467,22 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>~1-2 g</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="inlineStr">
-        <is>
-          <t>No added sugar but ~35-45 g natural sugar; no fibre; almost no protein</t>
-        </is>
-      </c>
+          <t>~4-5 g</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Fresh orange juice (350-450 ml)</t>
+          <t>Fresh pineapple juice (350-450 ml)</t>
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>155</v>
+        <v>175</v>
       </c>
       <c r="C30" s="7" t="n">
-        <v>205</v>
+        <v>240</v>
       </c>
       <c r="D30" s="8">
         <f>AVERAGE(B30:C30)</f>
@@ -4435,26 +4490,26 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>~2-3 g</t>
+          <t>~1-2 g</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>No added sugar but ~32-40 g natural sugar; no fibre</t>
+          <t>No added sugar but ~35-45 g natural sugar; no fibre; almost no protein</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in water)</t>
+          <t>Fresh orange juice (350-450 ml)</t>
         </is>
       </c>
       <c r="B31" s="7" t="n">
-        <v>100</v>
+        <v>155</v>
       </c>
       <c r="C31" s="7" t="n">
-        <v>120</v>
+        <v>205</v>
       </c>
       <c r="D31" s="8">
         <f>AVERAGE(B31:C31)</f>
@@ -4462,22 +4517,26 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="inlineStr"/>
+          <t>~2-3 g</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>No added sugar but ~32-40 g natural sugar; no fibre</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Greek yogurt (200 g plain low-fat)</t>
+          <t>Whey scoop (in water)</t>
         </is>
       </c>
       <c r="B32" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C32" s="7" t="n">
         <v>120</v>
-      </c>
-      <c r="C32" s="7" t="n">
-        <v>140</v>
       </c>
       <c r="D32" s="8">
         <f>AVERAGE(B32:C32)</f>
@@ -4485,26 +4544,22 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>~18-20 g</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="inlineStr">
-        <is>
-          <t>Casein - digests slowly; good overnight</t>
-        </is>
-      </c>
+          <t>~20-25 g</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Boiled egg (1 large)</t>
+          <t>Greek yogurt (200 g plain low-fat)</t>
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>70</v>
+        <v>120</v>
       </c>
       <c r="C33" s="7" t="n">
-        <v>78</v>
+        <v>140</v>
       </c>
       <c r="D33" s="8">
         <f>AVERAGE(B33:C33)</f>
@@ -4512,26 +4567,26 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>~6-6.5 g</t>
+          <t>~18-20 g</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>~5 g fat each</t>
+          <t>Casein - digests slowly; good overnight</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Paneer (50 g full-fat)</t>
+          <t>Boiled egg (1 large)</t>
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>130</v>
+        <v>70</v>
       </c>
       <c r="C34" s="7" t="n">
-        <v>150</v>
+        <v>78</v>
       </c>
       <c r="D34" s="8">
         <f>AVERAGE(B34:C34)</f>
@@ -4539,26 +4594,26 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>~8-9 g</t>
+          <t>~6-6.5 g</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>Fat-dense for the protein it gives</t>
+          <t>~5 g fat each</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Cucumber (1 medium)</t>
+          <t>Paneer (50 g full-fat)</t>
         </is>
       </c>
       <c r="B35" s="7" t="n">
-        <v>25</v>
+        <v>130</v>
       </c>
       <c r="C35" s="7" t="n">
-        <v>30</v>
+        <v>150</v>
       </c>
       <c r="D35" s="8">
         <f>AVERAGE(B35:C35)</f>
@@ -4566,26 +4621,26 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>~1.5 g</t>
+          <t>~8-9 g</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>Volume with almost no calories</t>
+          <t>Fat-dense for the protein it gives</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Sweet melon / cantaloupe (1 wedge ~100-150 g)</t>
+          <t>Cucumber (1 medium)</t>
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="C36" s="7" t="n">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="D36" s="8">
         <f>AVERAGE(B36:C36)</f>
@@ -4593,26 +4648,26 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>~0.5-1 g</t>
+          <t>~1.5 g</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>Whole fruit - fibre and water intact; ~1/4 the calories of the same fruit juiced</t>
+          <t>Volume with almost no calories</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Grapes (~100 g / 15-20 grapes)</t>
+          <t>Sweet melon / cantaloupe (1 wedge ~100-150 g)</t>
         </is>
       </c>
       <c r="B37" s="7" t="n">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="C37" s="7" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="D37" s="8">
         <f>AVERAGE(B37:C37)</f>
@@ -4620,26 +4675,26 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>~0.6 g</t>
+          <t>~0.5-1 g</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>Twice the calorie density of melon; easy to eat a large handful without noticing</t>
+          <t>Whole fruit - fibre and water intact; ~1/4 the calories of the same fruit juiced</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in black coffee no sugar)</t>
+          <t>Grapes (~100 g / 15-20 grapes)</t>
         </is>
       </c>
       <c r="B38" s="7" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="C38" s="7" t="n">
-        <v>130</v>
+        <v>75</v>
       </c>
       <c r="D38" s="8">
         <f>AVERAGE(B38:C38)</f>
@@ -4647,22 +4702,26 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F38" s="6" t="inlineStr"/>
+          <t>~0.6 g</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>Twice the calorie density of melon; easy to eat a large handful without noticing</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>Cashew/almond biscuit (1)</t>
+          <t>Whey scoop (in black coffee no sugar)</t>
         </is>
       </c>
       <c r="B39" s="7" t="n">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C39" s="7" t="n">
-        <v>38</v>
+        <v>130</v>
       </c>
       <c r="D39" s="8">
         <f>AVERAGE(B39:C39)</f>
@@ -4670,7 +4729,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>~0.5 g</t>
+          <t>~20-25 g</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr"/>
@@ -4678,14 +4737,14 @@
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (~50g standard)</t>
+          <t>Cashew/almond biscuit (1)</t>
         </is>
       </c>
       <c r="B40" s="7" t="n">
-        <v>245</v>
+        <v>38</v>
       </c>
       <c r="C40" s="7" t="n">
-        <v>250</v>
+        <v>38</v>
       </c>
       <c r="D40" s="8">
         <f>AVERAGE(B40:C40)</f>
@@ -4693,7 +4752,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>~4 g</t>
+          <t>~0.5 g</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr"/>
@@ -4701,14 +4760,14 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (70g king-size)</t>
+          <t>Chocolate bar (~50g standard)</t>
         </is>
       </c>
       <c r="B41" s="7" t="n">
-        <v>335</v>
+        <v>245</v>
       </c>
       <c r="C41" s="7" t="n">
-        <v>335</v>
+        <v>250</v>
       </c>
       <c r="D41" s="8">
         <f>AVERAGE(B41:C41)</f>
@@ -4716,7 +4775,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>~6 g</t>
+          <t>~4 g</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr"/>
@@ -4724,14 +4783,14 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Pre-workout scoop</t>
+          <t>Chocolate bar (70g king-size)</t>
         </is>
       </c>
       <c r="B42" s="7" t="n">
-        <v>5</v>
+        <v>335</v>
       </c>
       <c r="C42" s="7" t="n">
-        <v>15</v>
+        <v>335</v>
       </c>
       <c r="D42" s="8">
         <f>AVERAGE(B42:C42)</f>
@@ -4739,10 +4798,33 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
+          <t>~6 g</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>Pre-workout scoop</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C43" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D43" s="8">
+        <f>AVERAGE(B43:C43)</f>
+        <v/>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
           <t>0 g</t>
         </is>
       </c>
-      <c r="F42" s="6" t="inlineStr">
+      <c r="F43" s="6" t="inlineStr">
         <is>
           <t>Negligible</t>
         </is>

</xml_diff>

<commit_message>
Record 5 km walked on Day 4
First entry in activity.csv. At 90.75 kg, 5 km nets ~227 kcal against the
136 modelled for 3 km, putting today's maintenance at ~2,784. Updated the
Targets extra-activity block to 5 km; the calorie target is still not fed
from it.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -3656,11 +3656,11 @@
         </is>
       </c>
       <c r="B33" s="16" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C33" s="33" t="inlineStr">
         <is>
-          <t>~30-35 min at a normal pace.</t>
+          <t>Reported 5 km on 2026-09-07. ~50-60 min at a normal pace.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close Day 4: protein floor cleared, deficit nearly erased
Dinner of chicken curry with one chapati brings Day 4 to 2,560.5 kcal,
130.1 g protein and 104.25 g fat - the first day over the 130 g floor, and
also the first day at base maintenance rather than under it.

Rewrote the trends section on four complete days. Protein has improved
every day (78.5 -> 130.1) but calories are up 42% and fat up 55% over the
same four days, so the four-day average deficit is 342/day, 0.31 kg/week
rather than 0.50. Protein was bought by adding food rather than replacing
it; next week's job is the swap.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N28"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1610,39 +1610,39 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Lunch</t>
+          <t>Dinner</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Mess meals plate (rice halved): rice, 2 boiled eggs, 1 fried fish, sambar, green peas, buttermilk, veg curry, fish curry</t>
+          <t>Chicken curry + 1 chapati</t>
         </is>
       </c>
       <c r="D23" s="7" t="n">
-        <v>790</v>
+        <v>380</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>1100</v>
+        <v>550</v>
       </c>
       <c r="F23" s="8">
         <f>AVERAGE(D23:E23)</f>
         <v/>
       </c>
       <c r="G23" s="9" t="n">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="H23" s="9" t="n">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="I23" s="10">
         <f>AVERAGE(G23:H23)</f>
         <v/>
       </c>
       <c r="J23" s="9" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="K23" s="9" t="n">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="L23" s="10">
         <f>AVERAGE(J23:K23)</f>
@@ -1655,7 +1655,7 @@
       </c>
       <c r="N23" s="6" t="inlineStr">
         <is>
-          <t>Rice was already the half portion - both levers pulled. Highest-protein single meal in the log</t>
+          <t>Mess Monday dinner; took one chapati rather than two</t>
         </is>
       </c>
     </row>
@@ -1665,39 +1665,39 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Snack</t>
+          <t>Lunch</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Black coffee + 1 whey scoop</t>
+          <t>Mess meals plate (rice halved): rice, 2 boiled eggs, 1 fried fish, sambar, green peas, buttermilk, veg curry, fish curry</t>
         </is>
       </c>
       <c r="D24" s="7" t="n">
-        <v>100</v>
+        <v>790</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>130</v>
+        <v>1100</v>
       </c>
       <c r="F24" s="8">
         <f>AVERAGE(D24:E24)</f>
         <v/>
       </c>
       <c r="G24" s="9" t="n">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="I24" s="10">
         <f>AVERAGE(G24:H24)</f>
         <v/>
       </c>
       <c r="J24" s="9" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="K24" s="9" t="n">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="L24" s="10">
         <f>AVERAGE(J24:K24)</f>
@@ -1708,7 +1708,11 @@
           <t>logged</t>
         </is>
       </c>
-      <c r="N24" s="6" t="inlineStr"/>
+      <c r="N24" s="6" t="inlineStr">
+        <is>
+          <t>Rice was already the half portion - both levers pulled. Highest-protein single meal in the log</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
@@ -1721,34 +1725,34 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Sweet melon (2 wedges)</t>
+          <t>Black coffee + 1 whey scoop</t>
         </is>
       </c>
       <c r="D25" s="7" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="F25" s="8">
         <f>AVERAGE(D25:E25)</f>
         <v/>
       </c>
       <c r="G25" s="9" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="I25" s="10">
         <f>AVERAGE(G25:H25)</f>
         <v/>
       </c>
       <c r="J25" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K25" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L25" s="10">
         <f>AVERAGE(J25:K25)</f>
@@ -1759,11 +1763,7 @@
           <t>logged</t>
         </is>
       </c>
-      <c r="N25" s="6" t="inlineStr">
-        <is>
-          <t>Whole fruit - fibre intact; second wedge added</t>
-        </is>
-      </c>
+      <c r="N25" s="6" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
@@ -1776,34 +1776,34 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>2 boiled eggs (5pm)</t>
+          <t>Sweet melon (2 wedges)</t>
         </is>
       </c>
       <c r="D26" s="7" t="n">
-        <v>140</v>
+        <v>70</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>156</v>
+        <v>110</v>
       </c>
       <c r="F26" s="8">
         <f>AVERAGE(D26:E26)</f>
         <v/>
       </c>
       <c r="G26" s="9" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="I26" s="10">
         <f>AVERAGE(G26:H26)</f>
         <v/>
       </c>
       <c r="J26" s="9" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K26" s="9" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="L26" s="10">
         <f>AVERAGE(J26:K26)</f>
@@ -1816,7 +1816,7 @@
       </c>
       <c r="N26" s="6" t="inlineStr">
         <is>
-          <t>Second egg serving of the day - four eggs total</t>
+          <t>Whole fruit - fibre intact; second wedge added</t>
         </is>
       </c>
     </row>
@@ -1831,34 +1831,34 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Red grapes (~100 g)</t>
+          <t>2 boiled eggs (5pm)</t>
         </is>
       </c>
       <c r="D27" s="7" t="n">
-        <v>60</v>
+        <v>140</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>75</v>
+        <v>156</v>
       </c>
       <c r="F27" s="8">
         <f>AVERAGE(D27:E27)</f>
         <v/>
       </c>
       <c r="G27" s="9" t="n">
-        <v>0.5</v>
+        <v>12</v>
       </c>
       <c r="H27" s="9" t="n">
-        <v>0.7</v>
+        <v>13</v>
       </c>
       <c r="I27" s="10">
         <f>AVERAGE(G27:H27)</f>
         <v/>
       </c>
       <c r="J27" s="9" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K27" s="9" t="n">
-        <v>0.5</v>
+        <v>11</v>
       </c>
       <c r="L27" s="10">
         <f>AVERAGE(J27:K27)</f>
@@ -1871,7 +1871,7 @@
       </c>
       <c r="N27" s="6" t="inlineStr">
         <is>
-          <t>Portioned into a box rather than eaten from the bunch; some left over</t>
+          <t>Second egg serving of the day - four eggs total</t>
         </is>
       </c>
     </row>
@@ -1886,34 +1886,34 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Chatti pathiri chicken (1 slice)</t>
+          <t>Red grapes (~100 g)</t>
         </is>
       </c>
       <c r="D28" s="7" t="n">
-        <v>230</v>
+        <v>60</v>
       </c>
       <c r="E28" s="7" t="n">
-        <v>320</v>
+        <v>75</v>
       </c>
       <c r="F28" s="8">
         <f>AVERAGE(D28:E28)</f>
         <v/>
       </c>
       <c r="G28" s="9" t="n">
-        <v>10</v>
+        <v>0.5</v>
       </c>
       <c r="H28" s="9" t="n">
-        <v>14</v>
+        <v>0.7</v>
       </c>
       <c r="I28" s="10">
         <f>AVERAGE(G28:H28)</f>
         <v/>
       </c>
       <c r="J28" s="9" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="K28" s="9" t="n">
-        <v>18</v>
+        <v>0.5</v>
       </c>
       <c r="L28" s="10">
         <f>AVERAGE(J28:K28)</f>
@@ -1925,6 +1925,61 @@
         </is>
       </c>
       <c r="N28" s="6" t="inlineStr">
+        <is>
+          <t>Portioned into a box rather than eaten from the bunch; some left over</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Chatti pathiri chicken (1 slice)</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="n">
+        <v>230</v>
+      </c>
+      <c r="E29" s="7" t="n">
+        <v>320</v>
+      </c>
+      <c r="F29" s="8">
+        <f>AVERAGE(D29:E29)</f>
+        <v/>
+      </c>
+      <c r="G29" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="H29" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="I29" s="10">
+        <f>AVERAGE(G29:H29)</f>
+        <v/>
+      </c>
+      <c r="J29" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="K29" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="L29" s="10">
+        <f>AVERAGE(J29:K29)</f>
+        <v/>
+      </c>
+      <c r="M29" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N29" s="6" t="inlineStr">
         <is>
           <t>Before dinner. Slice count assumed 1 - double if it was 2</t>
         </is>
@@ -2048,11 +2103,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$28,Meals!$A$5:$A$28,$A5,Meals!$M$5:$M$28,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$29,Meals!$A$5:$A$29,$A5,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$28,Meals!$A$5:$A$28,$A5,Meals!$M$5:$M$28,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$29,Meals!$A$5:$A$29,$A5,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -2060,11 +2115,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$28,Meals!$A$5:$A$28,$A5,Meals!$M$5:$M$28,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$29,Meals!$A$5:$A$29,$A5,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$28,Meals!$A$5:$A$28,$A5,Meals!$M$5:$M$28,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$29,Meals!$A$5:$A$29,$A5,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -2072,11 +2127,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$28,Meals!$A$5:$A$28,$A5,Meals!$M$5:$M$28,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$29,Meals!$A$5:$A$29,$A5,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$28,Meals!$A$5:$A$28,$A5,Meals!$M$5:$M$28,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$29,Meals!$A$5:$A$29,$A5,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -2084,11 +2139,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$28,$A5,Meals!$M$5:$M$28,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$29,$A5,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$28,$A5,Meals!$M$5:$M$28,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$29,$A5,Meals!$M$5:$M$29,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -2101,11 +2156,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$28,Meals!$A$5:$A$28,$A6,Meals!$M$5:$M$28,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$29,Meals!$A$5:$A$29,$A6,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$28,Meals!$A$5:$A$28,$A6,Meals!$M$5:$M$28,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$29,Meals!$A$5:$A$29,$A6,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -2113,11 +2168,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$28,Meals!$A$5:$A$28,$A6,Meals!$M$5:$M$28,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$29,Meals!$A$5:$A$29,$A6,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$28,Meals!$A$5:$A$28,$A6,Meals!$M$5:$M$28,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$29,Meals!$A$5:$A$29,$A6,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -2125,11 +2180,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$28,Meals!$A$5:$A$28,$A6,Meals!$M$5:$M$28,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$29,Meals!$A$5:$A$29,$A6,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$28,Meals!$A$5:$A$28,$A6,Meals!$M$5:$M$28,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$29,Meals!$A$5:$A$29,$A6,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -2137,11 +2192,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$28,$A6,Meals!$M$5:$M$28,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$29,$A6,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$28,$A6,Meals!$M$5:$M$28,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$29,$A6,Meals!$M$5:$M$29,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -2154,11 +2209,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$28,Meals!$A$5:$A$28,$A7,Meals!$M$5:$M$28,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$29,Meals!$A$5:$A$29,$A7,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$28,Meals!$A$5:$A$28,$A7,Meals!$M$5:$M$28,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$29,Meals!$A$5:$A$29,$A7,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -2166,11 +2221,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$28,Meals!$A$5:$A$28,$A7,Meals!$M$5:$M$28,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$29,Meals!$A$5:$A$29,$A7,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$28,Meals!$A$5:$A$28,$A7,Meals!$M$5:$M$28,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$29,Meals!$A$5:$A$29,$A7,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -2178,11 +2233,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$28,Meals!$A$5:$A$28,$A7,Meals!$M$5:$M$28,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$29,Meals!$A$5:$A$29,$A7,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$28,Meals!$A$5:$A$28,$A7,Meals!$M$5:$M$28,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$29,Meals!$A$5:$A$29,$A7,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -2190,11 +2245,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$28,$A7,Meals!$M$5:$M$28,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$29,$A7,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$28,$A7,Meals!$M$5:$M$28,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$29,$A7,Meals!$M$5:$M$29,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -2207,11 +2262,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$28,Meals!$A$5:$A$28,$A8,Meals!$M$5:$M$28,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$29,Meals!$A$5:$A$29,$A8,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$28,Meals!$A$5:$A$28,$A8,Meals!$M$5:$M$28,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$29,Meals!$A$5:$A$29,$A8,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -2219,11 +2274,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$28,Meals!$A$5:$A$28,$A8,Meals!$M$5:$M$28,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$29,Meals!$A$5:$A$29,$A8,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$28,Meals!$A$5:$A$28,$A8,Meals!$M$5:$M$28,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$29,Meals!$A$5:$A$29,$A8,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -2231,11 +2286,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$28,Meals!$A$5:$A$28,$A8,Meals!$M$5:$M$28,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$29,Meals!$A$5:$A$29,$A8,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$28,Meals!$A$5:$A$28,$A8,Meals!$M$5:$M$28,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$29,Meals!$A$5:$A$29,$A8,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -2243,11 +2298,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$28,$A8,Meals!$M$5:$M$28,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$29,$A8,Meals!$M$5:$M$29,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$28,$A8,Meals!$M$5:$M$28,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$29,$A8,Meals!$M$5:$M$29,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">

</xml_diff>

<commit_message>
Log Day 5 breakfast: puttu with kadala curry
420-600 kcal (mid 510), 12-16 g protein, 12-19 g fat. Puttu is steamed with
no frying oil and the kadala carries protein, so 14 g is the second-best
breakfast protein in the log.

Adds a plan for the rest of the day: halved ghee rice at lunch, the light
green-peas dinner and 3 whey scoops lands 1,870 kcal and 126.5 g protein,
686 under maintenance - which would break the four-day rise in calories
and fat.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N29"/>
+  <dimension ref="A1:N30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1985,6 +1985,61 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="4" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Breakfast</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Puttu + kadala curry</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>420</v>
+      </c>
+      <c r="E30" s="7" t="n">
+        <v>600</v>
+      </c>
+      <c r="F30" s="8">
+        <f>AVERAGE(D30:E30)</f>
+        <v/>
+      </c>
+      <c r="G30" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="H30" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="I30" s="10">
+        <f>AVERAGE(G30:H30)</f>
+        <v/>
+      </c>
+      <c r="J30" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="K30" s="9" t="n">
+        <v>19</v>
+      </c>
+      <c r="L30" s="10">
+        <f>AVERAGE(J30:K30)</f>
+        <v/>
+      </c>
+      <c r="M30" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N30" s="6" t="inlineStr">
+        <is>
+          <t>Mess served puttu rather than the Tuesday masala dosa on the menu</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:N2"/>
@@ -1999,7 +2054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2103,11 +2158,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$29,Meals!$A$5:$A$29,$A5,Meals!$M$5:$M$29,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$30,Meals!$A$5:$A$30,$A5,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$29,Meals!$A$5:$A$29,$A5,Meals!$M$5:$M$29,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$30,Meals!$A$5:$A$30,$A5,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -2115,11 +2170,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$29,Meals!$A$5:$A$29,$A5,Meals!$M$5:$M$29,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$30,Meals!$A$5:$A$30,$A5,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$29,Meals!$A$5:$A$29,$A5,Meals!$M$5:$M$29,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$30,Meals!$A$5:$A$30,$A5,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -2127,11 +2182,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$29,Meals!$A$5:$A$29,$A5,Meals!$M$5:$M$29,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$30,Meals!$A$5:$A$30,$A5,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$29,Meals!$A$5:$A$29,$A5,Meals!$M$5:$M$29,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$30,Meals!$A$5:$A$30,$A5,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -2139,11 +2194,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$29,$A5,Meals!$M$5:$M$29,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$30,$A5,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$29,$A5,Meals!$M$5:$M$29,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$30,$A5,Meals!$M$5:$M$30,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -2156,11 +2211,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$29,Meals!$A$5:$A$29,$A6,Meals!$M$5:$M$29,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$30,Meals!$A$5:$A$30,$A6,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$29,Meals!$A$5:$A$29,$A6,Meals!$M$5:$M$29,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$30,Meals!$A$5:$A$30,$A6,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -2168,11 +2223,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$29,Meals!$A$5:$A$29,$A6,Meals!$M$5:$M$29,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$30,Meals!$A$5:$A$30,$A6,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$29,Meals!$A$5:$A$29,$A6,Meals!$M$5:$M$29,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$30,Meals!$A$5:$A$30,$A6,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -2180,11 +2235,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$29,Meals!$A$5:$A$29,$A6,Meals!$M$5:$M$29,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$30,Meals!$A$5:$A$30,$A6,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$29,Meals!$A$5:$A$29,$A6,Meals!$M$5:$M$29,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$30,Meals!$A$5:$A$30,$A6,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -2192,11 +2247,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$29,$A6,Meals!$M$5:$M$29,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$30,$A6,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$29,$A6,Meals!$M$5:$M$29,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$30,$A6,Meals!$M$5:$M$30,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -2209,11 +2264,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$29,Meals!$A$5:$A$29,$A7,Meals!$M$5:$M$29,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$30,Meals!$A$5:$A$30,$A7,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$29,Meals!$A$5:$A$29,$A7,Meals!$M$5:$M$29,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$30,Meals!$A$5:$A$30,$A7,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -2221,11 +2276,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$29,Meals!$A$5:$A$29,$A7,Meals!$M$5:$M$29,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$30,Meals!$A$5:$A$30,$A7,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$29,Meals!$A$5:$A$29,$A7,Meals!$M$5:$M$29,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$30,Meals!$A$5:$A$30,$A7,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -2233,11 +2288,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$29,Meals!$A$5:$A$29,$A7,Meals!$M$5:$M$29,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$30,Meals!$A$5:$A$30,$A7,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$29,Meals!$A$5:$A$29,$A7,Meals!$M$5:$M$29,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$30,Meals!$A$5:$A$30,$A7,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -2245,11 +2300,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$29,$A7,Meals!$M$5:$M$29,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$30,$A7,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$29,$A7,Meals!$M$5:$M$29,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$30,$A7,Meals!$M$5:$M$30,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -2262,11 +2317,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$29,Meals!$A$5:$A$29,$A8,Meals!$M$5:$M$29,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$30,Meals!$A$5:$A$30,$A8,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$29,Meals!$A$5:$A$29,$A8,Meals!$M$5:$M$29,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$30,Meals!$A$5:$A$30,$A8,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -2274,11 +2329,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$29,Meals!$A$5:$A$29,$A8,Meals!$M$5:$M$29,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$30,Meals!$A$5:$A$30,$A8,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$29,Meals!$A$5:$A$29,$A8,Meals!$M$5:$M$29,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$30,Meals!$A$5:$A$30,$A8,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -2286,11 +2341,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$29,Meals!$A$5:$A$29,$A8,Meals!$M$5:$M$29,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$30,Meals!$A$5:$A$30,$A8,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$29,Meals!$A$5:$A$29,$A8,Meals!$M$5:$M$29,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$30,Meals!$A$5:$A$30,$A8,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -2298,15 +2353,68 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$29,$A8,Meals!$M$5:$M$29,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$30,$A8,Meals!$M$5:$M$30,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$29,$A8,Meals!$M$5:$M$29,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$30,$A8,Meals!$M$5:$M$30,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
         <f>D8-Targets!$B$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="18" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B9" s="8">
+        <f>SUMIFS(Meals!$D$5:$D$30,Meals!$A$5:$A$30,$A9,Meals!$M$5:$M$30,"logged")</f>
+        <v/>
+      </c>
+      <c r="C9" s="8">
+        <f>SUMIFS(Meals!$E$5:$E$30,Meals!$A$5:$A$30,$A9,Meals!$M$5:$M$30,"logged")</f>
+        <v/>
+      </c>
+      <c r="D9" s="8">
+        <f>AVERAGE(B9:C9)</f>
+        <v/>
+      </c>
+      <c r="E9" s="10">
+        <f>SUMIFS(Meals!$G$5:$G$30,Meals!$A$5:$A$30,$A9,Meals!$M$5:$M$30,"logged")</f>
+        <v/>
+      </c>
+      <c r="F9" s="10">
+        <f>SUMIFS(Meals!$H$5:$H$30,Meals!$A$5:$A$30,$A9,Meals!$M$5:$M$30,"logged")</f>
+        <v/>
+      </c>
+      <c r="G9" s="10">
+        <f>AVERAGE(E9:F9)</f>
+        <v/>
+      </c>
+      <c r="H9" s="10">
+        <f>SUMIFS(Meals!$J$5:$J$30,Meals!$A$5:$A$30,$A9,Meals!$M$5:$M$30,"logged")</f>
+        <v/>
+      </c>
+      <c r="I9" s="10">
+        <f>SUMIFS(Meals!$K$5:$K$30,Meals!$A$5:$A$30,$A9,Meals!$M$5:$M$30,"logged")</f>
+        <v/>
+      </c>
+      <c r="J9" s="10">
+        <f>AVERAGE(H9:I9)</f>
+        <v/>
+      </c>
+      <c r="K9" s="18">
+        <f>COUNTIFS(Meals!$A$5:$A$30,$A9,Meals!$M$5:$M$30,"logged")</f>
+        <v/>
+      </c>
+      <c r="L9" s="18">
+        <f>COUNTIFS(Meals!$A$5:$A$30,$A9,Meals!$M$5:$M$30,"pending")</f>
+        <v/>
+      </c>
+      <c r="M9" s="19">
+        <f>D9-Targets!$B$16</f>
         <v/>
       </c>
     </row>
@@ -3082,7 +3190,7 @@
         </is>
       </c>
       <c r="B5" s="18">
-        <f>COUNT(Daily!$A$5:$A$8)</f>
+        <f>COUNT(Daily!$A$5:$A$9)</f>
         <v/>
       </c>
     </row>
@@ -3093,7 +3201,7 @@
         </is>
       </c>
       <c r="B6" s="8">
-        <f>IFERROR(AVERAGE(Daily!$D$5:$D$8),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$D$5:$D$9),0)</f>
         <v/>
       </c>
     </row>
@@ -3104,7 +3212,7 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>IFERROR(AVERAGE(Daily!$G$5:$G$8),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$G$5:$G$9),0)</f>
         <v/>
       </c>
     </row>
@@ -3115,7 +3223,7 @@
         </is>
       </c>
       <c r="B8" s="10">
-        <f>IFERROR(AVERAGE(Daily!$J$5:$J$8),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$J$5:$J$9),0)</f>
         <v/>
       </c>
     </row>
@@ -3159,7 +3267,7 @@
         </is>
       </c>
       <c r="B12" s="18">
-        <f>COUNTIFS(Daily!$G$5:$G$8,"&gt;="&amp;Targets!$B$20)</f>
+        <f>COUNTIFS(Daily!$G$5:$G$9,"&gt;="&amp;Targets!$B$20)</f>
         <v/>
       </c>
     </row>
@@ -3170,7 +3278,7 @@
         </is>
       </c>
       <c r="B13" s="18">
-        <f>SUM(Daily!$L$5:$L$8)</f>
+        <f>SUM(Daily!$L$5:$L$9)</f>
         <v/>
       </c>
     </row>
@@ -3221,19 +3329,19 @@
         <v>46271</v>
       </c>
       <c r="C17" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$8,"&gt;="&amp;$A17,Daily!$A$5:$A$8,"&lt;="&amp;$B17)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$9,"&gt;="&amp;$A17,Daily!$A$5:$A$9,"&lt;="&amp;$B17)</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$8,Daily!$A$5:$A$8,"&gt;="&amp;$A17,Daily!$A$5:$A$8,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$9,Daily!$A$5:$A$9,"&gt;="&amp;$A17,Daily!$A$5:$A$9,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$8,Daily!$A$5:$A$8,"&gt;="&amp;$A17,Daily!$A$5:$A$8,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$9,Daily!$A$5:$A$9,"&gt;="&amp;$A17,Daily!$A$5:$A$9,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$8,Daily!$A$5:$A$8,"&gt;="&amp;$A17,Daily!$A$5:$A$8,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$9,Daily!$A$5:$A$9,"&gt;="&amp;$A17,Daily!$A$5:$A$9,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
     </row>
@@ -3245,19 +3353,19 @@
         <v>46278</v>
       </c>
       <c r="C18" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$8,"&gt;="&amp;$A18,Daily!$A$5:$A$8,"&lt;="&amp;$B18)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$9,"&gt;="&amp;$A18,Daily!$A$5:$A$9,"&lt;="&amp;$B18)</f>
         <v/>
       </c>
       <c r="D18" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$8,Daily!$A$5:$A$8,"&gt;="&amp;$A18,Daily!$A$5:$A$8,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$9,Daily!$A$5:$A$9,"&gt;="&amp;$A18,Daily!$A$5:$A$9,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="E18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$8,Daily!$A$5:$A$8,"&gt;="&amp;$A18,Daily!$A$5:$A$8,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$9,Daily!$A$5:$A$9,"&gt;="&amp;$A18,Daily!$A$5:$A$9,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="F18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$8,Daily!$A$5:$A$8,"&gt;="&amp;$A18,Daily!$A$5:$A$8,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$9,Daily!$A$5:$A$9,"&gt;="&amp;$A18,Daily!$A$5:$A$9,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
     </row>
@@ -3308,19 +3416,19 @@
         <v>46295</v>
       </c>
       <c r="C22" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$8,"&gt;="&amp;$A22,Daily!$A$5:$A$8,"&lt;="&amp;$B22)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$9,"&gt;="&amp;$A22,Daily!$A$5:$A$9,"&lt;="&amp;$B22)</f>
         <v/>
       </c>
       <c r="D22" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$8,Daily!$A$5:$A$8,"&gt;="&amp;$A22,Daily!$A$5:$A$8,"&lt;="&amp;$B22),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$9,Daily!$A$5:$A$9,"&gt;="&amp;$A22,Daily!$A$5:$A$9,"&lt;="&amp;$B22),0)</f>
         <v/>
       </c>
       <c r="E22" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$8,Daily!$A$5:$A$8,"&gt;="&amp;$A22,Daily!$A$5:$A$8,"&lt;="&amp;$B22),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$9,Daily!$A$5:$A$9,"&gt;="&amp;$A22,Daily!$A$5:$A$9,"&lt;="&amp;$B22),0)</f>
         <v/>
       </c>
       <c r="F22" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$8,Daily!$A$5:$A$8,"&gt;="&amp;$A22,Daily!$A$5:$A$8,"&lt;="&amp;$B22),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$9,Daily!$A$5:$A$9,"&gt;="&amp;$A22,Daily!$A$5:$A$9,"&lt;="&amp;$B22),0)</f>
         <v/>
       </c>
     </row>
@@ -3823,7 +3931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -3964,14 +4072,14 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Potato bhaji / curry (small bowl)</t>
+          <t>Puttu (1 cylinder ~180-220 g)</t>
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>150</v>
+        <v>220</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>220</v>
+        <v>300</v>
       </c>
       <c r="D8" s="8">
         <f>AVERAGE(B8:C8)</f>
@@ -3979,26 +4087,26 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>~3-4 g</t>
+          <t>~4-6 g</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Kerala style; oil and coconut milk carry the calories</t>
+          <t>Steamed rice flour and coconut - no frying oil at all</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Sambar (with veg)</t>
+          <t>Potato bhaji / curry (small bowl)</t>
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>130</v>
+        <v>150</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>160</v>
+        <v>220</v>
       </c>
       <c r="D9" s="8">
         <f>AVERAGE(B9:C9)</f>
@@ -4006,26 +4114,26 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>~4-6 g</t>
+          <t>~3-4 g</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>Per serving</t>
+          <t>Kerala style; oil and coconut milk carry the calories</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Coconut chutney (~2 tbsp)</t>
+          <t>Sambar (with veg)</t>
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>90</v>
+        <v>130</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>110</v>
+        <v>160</v>
       </c>
       <c r="D10" s="8">
         <f>AVERAGE(B10:C10)</f>
@@ -4033,26 +4141,26 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>~1-2 g</t>
+          <t>~4-6 g</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>Fat-dense - the usual thing to cut</t>
+          <t>Per serving</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Red/tomato chutney (~2 tbsp)</t>
+          <t>Coconut chutney (~2 tbsp)</t>
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="C11" s="7" t="n">
-        <v>70</v>
+        <v>110</v>
       </c>
       <c r="D11" s="8">
         <f>AVERAGE(B11:C11)</f>
@@ -4060,22 +4168,26 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>~1 g</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr"/>
+          <t>~1-2 g</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Fat-dense - the usual thing to cut</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Chicken biryani (half plate)</t>
+          <t>Red/tomato chutney (~2 tbsp)</t>
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>450</v>
+        <v>40</v>
       </c>
       <c r="C12" s="7" t="n">
-        <v>600</v>
+        <v>70</v>
       </c>
       <c r="D12" s="8">
         <f>AVERAGE(B12:C12)</f>
@@ -4083,26 +4195,22 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>~22-30 g</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>Rice + 2 pieces</t>
-        </is>
-      </c>
+          <t>~1 g</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Raita (small)</t>
+          <t>Chicken biryani (half plate)</t>
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>50</v>
+        <v>450</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>80</v>
+        <v>600</v>
       </c>
       <c r="D13" s="8">
         <f>AVERAGE(B13:C13)</f>
@@ -4110,22 +4218,26 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>~2-4 g</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr"/>
+          <t>~22-30 g</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>Rice + 2 pieces</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Maida porotta</t>
+          <t>Raita (small)</t>
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>160</v>
+        <v>50</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>250</v>
+        <v>80</v>
       </c>
       <c r="D14" s="8">
         <f>AVERAGE(B14:C14)</f>
@@ -4133,26 +4245,22 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>~4-6 g each</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>Refined flour + layered oil/ghee</t>
-        </is>
-      </c>
+          <t>~2-4 g</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Chapati (1)</t>
+          <t>Maida porotta</t>
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>100</v>
+        <v>160</v>
       </c>
       <c r="C15" s="7" t="n">
-        <v>130</v>
+        <v>250</v>
       </c>
       <c r="D15" s="8">
         <f>AVERAGE(B15:C15)</f>
@@ -4160,26 +4268,26 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>~3-4 g each</t>
+          <t>~4-6 g each</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>Whole wheat with little or no oil - about half a porotta's calories and a third of its fat</t>
+          <t>Refined flour + layered oil/ghee</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Chatti pathiri chicken (1 slice ~100-120 g)</t>
+          <t>Chapati (1)</t>
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>230</v>
+        <v>100</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>320</v>
+        <v>130</v>
       </c>
       <c r="D16" s="8">
         <f>AVERAGE(B16:C16)</f>
@@ -4187,26 +4295,26 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>~10-14 g</t>
+          <t>~3-4 g each</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>Layered maida pathiri with chicken masala and an egg-milk binder; ghee-rich</t>
+          <t>Whole wheat with little or no oil - about half a porotta's calories and a third of its fat</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Uzhunnu vada / medu vada (1)</t>
+          <t>Chatti pathiri chicken (1 slice ~100-120 g)</t>
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>130</v>
+        <v>230</v>
       </c>
       <c r="C17" s="7" t="n">
-        <v>180</v>
+        <v>320</v>
       </c>
       <c r="D17" s="8">
         <f>AVERAGE(B17:C17)</f>
@@ -4214,26 +4322,26 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>~3.5-5 g each</t>
+          <t>~10-14 g</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>Deep-fried urad dal - protein-bearing but fat-dense</t>
+          <t>Layered maida pathiri with chicken masala and an egg-milk binder; ghee-rich</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Kadala curry (1 container)</t>
+          <t>Uzhunnu vada / medu vada (1)</t>
         </is>
       </c>
       <c r="B18" s="7" t="n">
-        <v>200</v>
+        <v>130</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>300</v>
+        <v>180</v>
       </c>
       <c r="D18" s="8">
         <f>AVERAGE(B18:C18)</f>
@@ -4241,22 +4349,26 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>~8-10 g</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr"/>
+          <t>~3.5-5 g each</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Deep-fried urad dal - protein-bearing but fat-dense</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Fish fry (1 piece pan-fried)</t>
+          <t>Kadala curry (1 container)</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="C19" s="7" t="n">
-        <v>220</v>
+        <v>300</v>
       </c>
       <c r="D19" s="8">
         <f>AVERAGE(B19:C19)</f>
@@ -4264,7 +4376,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>~15-20 g</t>
+          <t>~8-10 g</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr"/>
@@ -4272,14 +4384,14 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Grilled chicken breast (100 g skinless)</t>
+          <t>Fish fry (1 piece pan-fried)</t>
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="C20" s="7" t="n">
-        <v>180</v>
+        <v>220</v>
       </c>
       <c r="D20" s="8">
         <f>AVERAGE(B20:C20)</f>
@@ -4287,26 +4399,22 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>~30-32 g</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>Best protein-per-calorie item in this list</t>
-        </is>
-      </c>
+          <t>~15-20 g</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Grilled chicken breast (150 g skinless)</t>
+          <t>Grilled chicken breast (100 g skinless)</t>
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>240</v>
+        <v>160</v>
       </c>
       <c r="C21" s="7" t="n">
-        <v>270</v>
+        <v>180</v>
       </c>
       <c r="D21" s="8">
         <f>AVERAGE(B21:C21)</f>
@@ -4314,22 +4422,26 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>~45-48 g</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr"/>
+          <t>~30-32 g</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>Best protein-per-calorie item in this list</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Honest Bowl - Grilled Chicken and Rice Bowl</t>
+          <t>Grilled chicken breast (150 g skinless)</t>
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>550</v>
+        <v>240</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>710</v>
+        <v>270</v>
       </c>
       <c r="D22" s="8">
         <f>AVERAGE(B22:C22)</f>
@@ -4337,26 +4449,22 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>42-48 g</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>Menu states 42 g protein; chicken + jasmine rice + sweet potato. Sauce served separately</t>
-        </is>
-      </c>
+          <t>~45-48 g</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Brown/mushroom sauce (side pot)</t>
+          <t>Honest Bowl - Grilled Chicken and Rice Bowl</t>
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>50</v>
+        <v>550</v>
       </c>
       <c r="C23" s="7" t="n">
-        <v>120</v>
+        <v>710</v>
       </c>
       <c r="D23" s="8">
         <f>AVERAGE(B23:C23)</f>
@@ -4364,26 +4472,26 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>~1-2 g</t>
+          <t>42-48 g</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>Often cream or butter based - the variable in a bowl like this</t>
+          <t>Menu states 42 g protein; chicken + jasmine rice + sweet potato. Sauce served separately</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Honest Bowl - Tofu Delight Bowl</t>
+          <t>Brown/mushroom sauce (side pot)</t>
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>420</v>
+        <v>50</v>
       </c>
       <c r="C24" s="7" t="n">
-        <v>560</v>
+        <v>120</v>
       </c>
       <c r="D24" s="8">
         <f>AVERAGE(B24:C24)</f>
@@ -4391,26 +4499,26 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>~20 g</t>
+          <t>~1-2 g</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>Menu states 20 g; jasmine rice + cajun tofu + grilled eggplant. Half the protein of the chicken bowl at the same price</t>
+          <t>Often cream or butter based - the variable in a bowl like this</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Chicken curry (1 takeaway container)</t>
+          <t>Honest Bowl - Tofu Delight Bowl</t>
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>280</v>
+        <v>420</v>
       </c>
       <c r="C25" s="7" t="n">
-        <v>420</v>
+        <v>560</v>
       </c>
       <c r="D25" s="8">
         <f>AVERAGE(B25:C25)</f>
@@ -4418,26 +4526,26 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>~20-28 g</t>
+          <t>~20 g</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>Kerala style; oil and coconut carry most of the calories</t>
+          <t>Menu states 20 g; jasmine rice + cajun tofu + grilled eggplant. Half the protein of the chicken bowl at the same price</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Grilled chicken quarter (skin on)</t>
+          <t>Chicken curry (1 takeaway container)</t>
         </is>
       </c>
       <c r="B26" s="7" t="n">
-        <v>250</v>
+        <v>280</v>
       </c>
       <c r="C26" s="7" t="n">
-        <v>320</v>
+        <v>420</v>
       </c>
       <c r="D26" s="8">
         <f>AVERAGE(B26:C26)</f>
@@ -4445,26 +4553,26 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>~28-33 g</t>
+          <t>~20-28 g</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>Skin adds ~12-15 g fat over breast</t>
+          <t>Kerala style; oil and coconut carry most of the calories</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Garlic sauce / toum (1 tbsp)</t>
+          <t>Grilled chicken quarter (skin on)</t>
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>90</v>
+        <v>250</v>
       </c>
       <c r="C27" s="7" t="n">
-        <v>110</v>
+        <v>320</v>
       </c>
       <c r="D27" s="8">
         <f>AVERAGE(B27:C27)</f>
@@ -4472,26 +4580,26 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>0 g</t>
+          <t>~28-33 g</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>Essentially emulsified oil - the hidden cost at a grill</t>
+          <t>Skin adds ~12-15 g fat over breast</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Khubz / pita (1 large)</t>
+          <t>Garlic sauce / toum (1 tbsp)</t>
         </is>
       </c>
       <c r="B28" s="7" t="n">
-        <v>250</v>
+        <v>90</v>
       </c>
       <c r="C28" s="7" t="n">
-        <v>300</v>
+        <v>110</v>
       </c>
       <c r="D28" s="8">
         <f>AVERAGE(B28:C28)</f>
@@ -4499,22 +4607,26 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>~8-9 g</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr"/>
+          <t>0 g</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>Essentially emulsified oil - the hidden cost at a grill</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Barik/basmati rice (half container cooked)</t>
+          <t>Khubz / pita (1 large)</t>
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="C29" s="7" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="D29" s="8">
         <f>AVERAGE(B29:C29)</f>
@@ -4522,7 +4634,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>~4-5 g</t>
+          <t>~8-9 g</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr"/>
@@ -4530,14 +4642,14 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Fresh pineapple juice (350-450 ml)</t>
+          <t>Barik/basmati rice (half container cooked)</t>
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>175</v>
+        <v>200</v>
       </c>
       <c r="C30" s="7" t="n">
-        <v>240</v>
+        <v>280</v>
       </c>
       <c r="D30" s="8">
         <f>AVERAGE(B30:C30)</f>
@@ -4545,26 +4657,22 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>~1-2 g</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>No added sugar but ~35-45 g natural sugar; no fibre; almost no protein</t>
-        </is>
-      </c>
+          <t>~4-5 g</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Fresh orange juice (350-450 ml)</t>
+          <t>Fresh pineapple juice (350-450 ml)</t>
         </is>
       </c>
       <c r="B31" s="7" t="n">
-        <v>155</v>
+        <v>175</v>
       </c>
       <c r="C31" s="7" t="n">
-        <v>205</v>
+        <v>240</v>
       </c>
       <c r="D31" s="8">
         <f>AVERAGE(B31:C31)</f>
@@ -4572,26 +4680,26 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>~2-3 g</t>
+          <t>~1-2 g</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>No added sugar but ~32-40 g natural sugar; no fibre</t>
+          <t>No added sugar but ~35-45 g natural sugar; no fibre; almost no protein</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in water)</t>
+          <t>Fresh orange juice (350-450 ml)</t>
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>100</v>
+        <v>155</v>
       </c>
       <c r="C32" s="7" t="n">
-        <v>120</v>
+        <v>205</v>
       </c>
       <c r="D32" s="8">
         <f>AVERAGE(B32:C32)</f>
@@ -4599,22 +4707,26 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="inlineStr"/>
+          <t>~2-3 g</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>No added sugar but ~32-40 g natural sugar; no fibre</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Greek yogurt (200 g plain low-fat)</t>
+          <t>Whey scoop (in water)</t>
         </is>
       </c>
       <c r="B33" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C33" s="7" t="n">
         <v>120</v>
-      </c>
-      <c r="C33" s="7" t="n">
-        <v>140</v>
       </c>
       <c r="D33" s="8">
         <f>AVERAGE(B33:C33)</f>
@@ -4622,26 +4734,22 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>~18-20 g</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="inlineStr">
-        <is>
-          <t>Casein - digests slowly; good overnight</t>
-        </is>
-      </c>
+          <t>~20-25 g</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Boiled egg (1 large)</t>
+          <t>Greek yogurt (200 g plain low-fat)</t>
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>70</v>
+        <v>120</v>
       </c>
       <c r="C34" s="7" t="n">
-        <v>78</v>
+        <v>140</v>
       </c>
       <c r="D34" s="8">
         <f>AVERAGE(B34:C34)</f>
@@ -4649,26 +4757,26 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>~6-6.5 g</t>
+          <t>~18-20 g</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>~5 g fat each</t>
+          <t>Casein - digests slowly; good overnight</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Paneer (50 g full-fat)</t>
+          <t>Boiled egg (1 large)</t>
         </is>
       </c>
       <c r="B35" s="7" t="n">
-        <v>130</v>
+        <v>70</v>
       </c>
       <c r="C35" s="7" t="n">
-        <v>150</v>
+        <v>78</v>
       </c>
       <c r="D35" s="8">
         <f>AVERAGE(B35:C35)</f>
@@ -4676,26 +4784,26 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>~8-9 g</t>
+          <t>~6-6.5 g</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>Fat-dense for the protein it gives</t>
+          <t>~5 g fat each</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Cucumber (1 medium)</t>
+          <t>Paneer (50 g full-fat)</t>
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>25</v>
+        <v>130</v>
       </c>
       <c r="C36" s="7" t="n">
-        <v>30</v>
+        <v>150</v>
       </c>
       <c r="D36" s="8">
         <f>AVERAGE(B36:C36)</f>
@@ -4703,26 +4811,26 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>~1.5 g</t>
+          <t>~8-9 g</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>Volume with almost no calories</t>
+          <t>Fat-dense for the protein it gives</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Sweet melon / cantaloupe (1 wedge ~100-150 g)</t>
+          <t>Cucumber (1 medium)</t>
         </is>
       </c>
       <c r="B37" s="7" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="C37" s="7" t="n">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="D37" s="8">
         <f>AVERAGE(B37:C37)</f>
@@ -4730,26 +4838,26 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>~0.5-1 g</t>
+          <t>~1.5 g</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>Whole fruit - fibre and water intact; ~1/4 the calories of the same fruit juiced</t>
+          <t>Volume with almost no calories</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>Grapes (~100 g / 15-20 grapes)</t>
+          <t>Sweet melon / cantaloupe (1 wedge ~100-150 g)</t>
         </is>
       </c>
       <c r="B38" s="7" t="n">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="C38" s="7" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="D38" s="8">
         <f>AVERAGE(B38:C38)</f>
@@ -4757,26 +4865,26 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>~0.6 g</t>
+          <t>~0.5-1 g</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>Twice the calorie density of melon; easy to eat a large handful without noticing</t>
+          <t>Whole fruit - fibre and water intact; ~1/4 the calories of the same fruit juiced</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in black coffee no sugar)</t>
+          <t>Grapes (~100 g / 15-20 grapes)</t>
         </is>
       </c>
       <c r="B39" s="7" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="C39" s="7" t="n">
-        <v>130</v>
+        <v>75</v>
       </c>
       <c r="D39" s="8">
         <f>AVERAGE(B39:C39)</f>
@@ -4784,22 +4892,26 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="inlineStr"/>
+          <t>~0.6 g</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>Twice the calorie density of melon; easy to eat a large handful without noticing</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>Cashew/almond biscuit (1)</t>
+          <t>Whey scoop (in black coffee no sugar)</t>
         </is>
       </c>
       <c r="B40" s="7" t="n">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C40" s="7" t="n">
-        <v>38</v>
+        <v>130</v>
       </c>
       <c r="D40" s="8">
         <f>AVERAGE(B40:C40)</f>
@@ -4807,7 +4919,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>~0.5 g</t>
+          <t>~20-25 g</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr"/>
@@ -4815,14 +4927,14 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (~50g standard)</t>
+          <t>Cashew/almond biscuit (1)</t>
         </is>
       </c>
       <c r="B41" s="7" t="n">
-        <v>245</v>
+        <v>38</v>
       </c>
       <c r="C41" s="7" t="n">
-        <v>250</v>
+        <v>38</v>
       </c>
       <c r="D41" s="8">
         <f>AVERAGE(B41:C41)</f>
@@ -4830,7 +4942,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>~4 g</t>
+          <t>~0.5 g</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr"/>
@@ -4838,14 +4950,14 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (70g king-size)</t>
+          <t>Chocolate bar (~50g standard)</t>
         </is>
       </c>
       <c r="B42" s="7" t="n">
-        <v>335</v>
+        <v>245</v>
       </c>
       <c r="C42" s="7" t="n">
-        <v>335</v>
+        <v>250</v>
       </c>
       <c r="D42" s="8">
         <f>AVERAGE(B42:C42)</f>
@@ -4853,7 +4965,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>~6 g</t>
+          <t>~4 g</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr"/>
@@ -4861,14 +4973,14 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>Pre-workout scoop</t>
+          <t>Chocolate bar (70g king-size)</t>
         </is>
       </c>
       <c r="B43" s="7" t="n">
-        <v>5</v>
+        <v>335</v>
       </c>
       <c r="C43" s="7" t="n">
-        <v>15</v>
+        <v>335</v>
       </c>
       <c r="D43" s="8">
         <f>AVERAGE(B43:C43)</f>
@@ -4876,10 +4988,33 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
+          <t>~6 g</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>Pre-workout scoop</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C44" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D44" s="8">
+        <f>AVERAGE(B44:C44)</f>
+        <v/>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
           <t>0 g</t>
         </is>
       </c>
-      <c r="F43" s="6" t="inlineStr">
+      <c r="F44" s="6" t="inlineStr">
         <is>
           <t>Negligible</t>
         </is>

</xml_diff>

<commit_message>
Fix malformed reference row and a rounding drift in the log
The dry-fried egg row carried an unquoted comma, which split the CSV and
broke the build. Renamed it. Also corrected Day 5's midpoint in log.md from
1,186 to 1,185.5, which verify_tracker.py caught.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N30"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2037,6 +2037,61 @@
       <c r="N30" s="6" t="inlineStr">
         <is>
           <t>Mess served puttu rather than the Tuesday masala dosa on the menu</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>2 eggs fried without oil + half container ghee rice + small container chicken curry + curd salad</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="n">
+        <v>565</v>
+      </c>
+      <c r="E31" s="7" t="n">
+        <v>786</v>
+      </c>
+      <c r="F31" s="8">
+        <f>AVERAGE(D31:E31)</f>
+        <v/>
+      </c>
+      <c r="G31" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="H31" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I31" s="10">
+        <f>AVERAGE(G31:H31)</f>
+        <v/>
+      </c>
+      <c r="J31" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="K31" s="9" t="n">
+        <v>44</v>
+      </c>
+      <c r="L31" s="10">
+        <f>AVERAGE(J31:K31)</f>
+        <v/>
+      </c>
+      <c r="M31" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N31" s="6" t="inlineStr">
+        <is>
+          <t>Eggs dry-fried with pepper and salt; rice halved by the user</t>
         </is>
       </c>
     </row>
@@ -2158,11 +2213,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$30,Meals!$A$5:$A$30,$A5,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$31,Meals!$A$5:$A$31,$A5,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$30,Meals!$A$5:$A$30,$A5,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$31,Meals!$A$5:$A$31,$A5,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -2170,11 +2225,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$30,Meals!$A$5:$A$30,$A5,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$31,Meals!$A$5:$A$31,$A5,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$30,Meals!$A$5:$A$30,$A5,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$31,Meals!$A$5:$A$31,$A5,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -2182,11 +2237,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$30,Meals!$A$5:$A$30,$A5,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$31,Meals!$A$5:$A$31,$A5,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$30,Meals!$A$5:$A$30,$A5,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$31,Meals!$A$5:$A$31,$A5,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -2194,11 +2249,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$30,$A5,Meals!$M$5:$M$30,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$31,$A5,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$30,$A5,Meals!$M$5:$M$30,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$31,$A5,Meals!$M$5:$M$31,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -2211,11 +2266,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$30,Meals!$A$5:$A$30,$A6,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$31,Meals!$A$5:$A$31,$A6,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$30,Meals!$A$5:$A$30,$A6,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$31,Meals!$A$5:$A$31,$A6,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -2223,11 +2278,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$30,Meals!$A$5:$A$30,$A6,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$31,Meals!$A$5:$A$31,$A6,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$30,Meals!$A$5:$A$30,$A6,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$31,Meals!$A$5:$A$31,$A6,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -2235,11 +2290,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$30,Meals!$A$5:$A$30,$A6,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$31,Meals!$A$5:$A$31,$A6,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$30,Meals!$A$5:$A$30,$A6,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$31,Meals!$A$5:$A$31,$A6,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -2247,11 +2302,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$30,$A6,Meals!$M$5:$M$30,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$31,$A6,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$30,$A6,Meals!$M$5:$M$30,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$31,$A6,Meals!$M$5:$M$31,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -2264,11 +2319,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$30,Meals!$A$5:$A$30,$A7,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$31,Meals!$A$5:$A$31,$A7,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$30,Meals!$A$5:$A$30,$A7,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$31,Meals!$A$5:$A$31,$A7,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -2276,11 +2331,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$30,Meals!$A$5:$A$30,$A7,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$31,Meals!$A$5:$A$31,$A7,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$30,Meals!$A$5:$A$30,$A7,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$31,Meals!$A$5:$A$31,$A7,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -2288,11 +2343,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$30,Meals!$A$5:$A$30,$A7,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$31,Meals!$A$5:$A$31,$A7,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$30,Meals!$A$5:$A$30,$A7,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$31,Meals!$A$5:$A$31,$A7,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -2300,11 +2355,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$30,$A7,Meals!$M$5:$M$30,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$31,$A7,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$30,$A7,Meals!$M$5:$M$30,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$31,$A7,Meals!$M$5:$M$31,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -2317,11 +2372,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$30,Meals!$A$5:$A$30,$A8,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$31,Meals!$A$5:$A$31,$A8,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$30,Meals!$A$5:$A$30,$A8,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$31,Meals!$A$5:$A$31,$A8,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -2329,11 +2384,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$30,Meals!$A$5:$A$30,$A8,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$31,Meals!$A$5:$A$31,$A8,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$30,Meals!$A$5:$A$30,$A8,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$31,Meals!$A$5:$A$31,$A8,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -2341,11 +2396,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$30,Meals!$A$5:$A$30,$A8,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$31,Meals!$A$5:$A$31,$A8,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$30,Meals!$A$5:$A$30,$A8,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$31,Meals!$A$5:$A$31,$A8,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -2353,11 +2408,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$30,$A8,Meals!$M$5:$M$30,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$31,$A8,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$30,$A8,Meals!$M$5:$M$30,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$31,$A8,Meals!$M$5:$M$31,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -2370,11 +2425,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$30,Meals!$A$5:$A$30,$A9,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$31,Meals!$A$5:$A$31,$A9,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$30,Meals!$A$5:$A$30,$A9,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$31,Meals!$A$5:$A$31,$A9,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -2382,11 +2437,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$30,Meals!$A$5:$A$30,$A9,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$31,Meals!$A$5:$A$31,$A9,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$30,Meals!$A$5:$A$30,$A9,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$31,Meals!$A$5:$A$31,$A9,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -2394,11 +2449,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$30,Meals!$A$5:$A$30,$A9,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$31,Meals!$A$5:$A$31,$A9,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$30,Meals!$A$5:$A$30,$A9,Meals!$M$5:$M$30,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$31,Meals!$A$5:$A$31,$A9,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -2406,11 +2461,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$30,$A9,Meals!$M$5:$M$30,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$31,$A9,Meals!$M$5:$M$31,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$30,$A9,Meals!$M$5:$M$30,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$31,$A9,Meals!$M$5:$M$31,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -3931,7 +3986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4796,14 +4851,14 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Paneer (50 g full-fat)</t>
+          <t>Egg fried dry with no oil (1)</t>
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>130</v>
+        <v>70</v>
       </c>
       <c r="C36" s="7" t="n">
-        <v>150</v>
+        <v>78</v>
       </c>
       <c r="D36" s="8">
         <f>AVERAGE(B36:C36)</f>
@@ -4811,26 +4866,26 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>~8-9 g</t>
+          <t>~6-6.5 g</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>Fat-dense for the protein it gives</t>
+          <t>Same as boiled - dry-frying saves the ~20-25 kcal per egg that pan oil adds</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Cucumber (1 medium)</t>
+          <t>Paneer (50 g full-fat)</t>
         </is>
       </c>
       <c r="B37" s="7" t="n">
-        <v>25</v>
+        <v>130</v>
       </c>
       <c r="C37" s="7" t="n">
-        <v>30</v>
+        <v>150</v>
       </c>
       <c r="D37" s="8">
         <f>AVERAGE(B37:C37)</f>
@@ -4838,26 +4893,26 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>~1.5 g</t>
+          <t>~8-9 g</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>Volume with almost no calories</t>
+          <t>Fat-dense for the protein it gives</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>Sweet melon / cantaloupe (1 wedge ~100-150 g)</t>
+          <t>Cucumber (1 medium)</t>
         </is>
       </c>
       <c r="B38" s="7" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="C38" s="7" t="n">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="D38" s="8">
         <f>AVERAGE(B38:C38)</f>
@@ -4865,26 +4920,26 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>~0.5-1 g</t>
+          <t>~1.5 g</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>Whole fruit - fibre and water intact; ~1/4 the calories of the same fruit juiced</t>
+          <t>Volume with almost no calories</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>Grapes (~100 g / 15-20 grapes)</t>
+          <t>Sweet melon / cantaloupe (1 wedge ~100-150 g)</t>
         </is>
       </c>
       <c r="B39" s="7" t="n">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="C39" s="7" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="D39" s="8">
         <f>AVERAGE(B39:C39)</f>
@@ -4892,26 +4947,26 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>~0.6 g</t>
+          <t>~0.5-1 g</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
         <is>
-          <t>Twice the calorie density of melon; easy to eat a large handful without noticing</t>
+          <t>Whole fruit - fibre and water intact; ~1/4 the calories of the same fruit juiced</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in black coffee no sugar)</t>
+          <t>Grapes (~100 g / 15-20 grapes)</t>
         </is>
       </c>
       <c r="B40" s="7" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="C40" s="7" t="n">
-        <v>130</v>
+        <v>75</v>
       </c>
       <c r="D40" s="8">
         <f>AVERAGE(B40:C40)</f>
@@ -4919,22 +4974,26 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="inlineStr"/>
+          <t>~0.6 g</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>Twice the calorie density of melon; easy to eat a large handful without noticing</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>Cashew/almond biscuit (1)</t>
+          <t>Whey scoop (in black coffee no sugar)</t>
         </is>
       </c>
       <c r="B41" s="7" t="n">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C41" s="7" t="n">
-        <v>38</v>
+        <v>130</v>
       </c>
       <c r="D41" s="8">
         <f>AVERAGE(B41:C41)</f>
@@ -4942,7 +5001,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>~0.5 g</t>
+          <t>~20-25 g</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr"/>
@@ -4950,14 +5009,14 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (~50g standard)</t>
+          <t>Cashew/almond biscuit (1)</t>
         </is>
       </c>
       <c r="B42" s="7" t="n">
-        <v>245</v>
+        <v>38</v>
       </c>
       <c r="C42" s="7" t="n">
-        <v>250</v>
+        <v>38</v>
       </c>
       <c r="D42" s="8">
         <f>AVERAGE(B42:C42)</f>
@@ -4965,7 +5024,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>~4 g</t>
+          <t>~0.5 g</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr"/>
@@ -4973,14 +5032,14 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (70g king-size)</t>
+          <t>Chocolate bar (~50g standard)</t>
         </is>
       </c>
       <c r="B43" s="7" t="n">
-        <v>335</v>
+        <v>245</v>
       </c>
       <c r="C43" s="7" t="n">
-        <v>335</v>
+        <v>250</v>
       </c>
       <c r="D43" s="8">
         <f>AVERAGE(B43:C43)</f>
@@ -4988,7 +5047,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>~6 g</t>
+          <t>~4 g</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr"/>
@@ -4996,14 +5055,14 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>Pre-workout scoop</t>
+          <t>Chocolate bar (70g king-size)</t>
         </is>
       </c>
       <c r="B44" s="7" t="n">
-        <v>5</v>
+        <v>335</v>
       </c>
       <c r="C44" s="7" t="n">
-        <v>15</v>
+        <v>335</v>
       </c>
       <c r="D44" s="8">
         <f>AVERAGE(B44:C44)</f>
@@ -5011,10 +5070,33 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
+          <t>~6 g</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>Pre-workout scoop</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C45" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D45" s="8">
+        <f>AVERAGE(B45:C45)</f>
+        <v/>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
           <t>0 g</t>
         </is>
       </c>
-      <c r="F44" s="6" t="inlineStr">
+      <c r="F45" s="6" t="inlineStr">
         <is>
           <t>Negligible</t>
         </is>

</xml_diff>

<commit_message>
Log first whey scoop of Day 5
100-130 kcal, 20-25 g protein. Day 5 stands at 1,300.5 kcal and 76.5 g of
protein, with dinner and two more scoops to come.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N31"/>
+  <dimension ref="A1:N32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2092,6 +2092,61 @@
       <c r="N31" s="6" t="inlineStr">
         <is>
           <t>Eggs dry-fried with pepper and salt; rice halved by the user</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Black coffee + 1 whey scoop</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E32" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="F32" s="8">
+        <f>AVERAGE(D32:E32)</f>
+        <v/>
+      </c>
+      <c r="G32" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="H32" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="I32" s="10">
+        <f>AVERAGE(G32:H32)</f>
+        <v/>
+      </c>
+      <c r="J32" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K32" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="L32" s="10">
+        <f>AVERAGE(J32:K32)</f>
+        <v/>
+      </c>
+      <c r="M32" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N32" s="6" t="inlineStr">
+        <is>
+          <t>Scoop 1 of the 3 planned for today</t>
         </is>
       </c>
     </row>
@@ -2213,11 +2268,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$31,Meals!$A$5:$A$31,$A5,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$32,Meals!$A$5:$A$32,$A5,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$31,Meals!$A$5:$A$31,$A5,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$32,Meals!$A$5:$A$32,$A5,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -2225,11 +2280,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$31,Meals!$A$5:$A$31,$A5,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$32,Meals!$A$5:$A$32,$A5,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$31,Meals!$A$5:$A$31,$A5,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$32,Meals!$A$5:$A$32,$A5,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -2237,11 +2292,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$31,Meals!$A$5:$A$31,$A5,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$32,Meals!$A$5:$A$32,$A5,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$31,Meals!$A$5:$A$31,$A5,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$32,Meals!$A$5:$A$32,$A5,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -2249,11 +2304,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$31,$A5,Meals!$M$5:$M$31,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$32,$A5,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$31,$A5,Meals!$M$5:$M$31,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$32,$A5,Meals!$M$5:$M$32,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -2266,11 +2321,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$31,Meals!$A$5:$A$31,$A6,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$32,Meals!$A$5:$A$32,$A6,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$31,Meals!$A$5:$A$31,$A6,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$32,Meals!$A$5:$A$32,$A6,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -2278,11 +2333,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$31,Meals!$A$5:$A$31,$A6,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$32,Meals!$A$5:$A$32,$A6,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$31,Meals!$A$5:$A$31,$A6,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$32,Meals!$A$5:$A$32,$A6,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -2290,11 +2345,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$31,Meals!$A$5:$A$31,$A6,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$32,Meals!$A$5:$A$32,$A6,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$31,Meals!$A$5:$A$31,$A6,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$32,Meals!$A$5:$A$32,$A6,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -2302,11 +2357,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$31,$A6,Meals!$M$5:$M$31,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$32,$A6,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$31,$A6,Meals!$M$5:$M$31,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$32,$A6,Meals!$M$5:$M$32,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -2319,11 +2374,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$31,Meals!$A$5:$A$31,$A7,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$32,Meals!$A$5:$A$32,$A7,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$31,Meals!$A$5:$A$31,$A7,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$32,Meals!$A$5:$A$32,$A7,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -2331,11 +2386,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$31,Meals!$A$5:$A$31,$A7,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$32,Meals!$A$5:$A$32,$A7,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$31,Meals!$A$5:$A$31,$A7,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$32,Meals!$A$5:$A$32,$A7,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -2343,11 +2398,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$31,Meals!$A$5:$A$31,$A7,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$32,Meals!$A$5:$A$32,$A7,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$31,Meals!$A$5:$A$31,$A7,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$32,Meals!$A$5:$A$32,$A7,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -2355,11 +2410,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$31,$A7,Meals!$M$5:$M$31,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$32,$A7,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$31,$A7,Meals!$M$5:$M$31,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$32,$A7,Meals!$M$5:$M$32,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -2372,11 +2427,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$31,Meals!$A$5:$A$31,$A8,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$32,Meals!$A$5:$A$32,$A8,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$31,Meals!$A$5:$A$31,$A8,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$32,Meals!$A$5:$A$32,$A8,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -2384,11 +2439,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$31,Meals!$A$5:$A$31,$A8,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$32,Meals!$A$5:$A$32,$A8,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$31,Meals!$A$5:$A$31,$A8,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$32,Meals!$A$5:$A$32,$A8,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -2396,11 +2451,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$31,Meals!$A$5:$A$31,$A8,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$32,Meals!$A$5:$A$32,$A8,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$31,Meals!$A$5:$A$31,$A8,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$32,Meals!$A$5:$A$32,$A8,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -2408,11 +2463,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$31,$A8,Meals!$M$5:$M$31,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$32,$A8,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$31,$A8,Meals!$M$5:$M$31,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$32,$A8,Meals!$M$5:$M$32,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -2425,11 +2480,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$31,Meals!$A$5:$A$31,$A9,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$32,Meals!$A$5:$A$32,$A9,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$31,Meals!$A$5:$A$31,$A9,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$32,Meals!$A$5:$A$32,$A9,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -2437,11 +2492,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$31,Meals!$A$5:$A$31,$A9,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$32,Meals!$A$5:$A$32,$A9,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$31,Meals!$A$5:$A$31,$A9,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$32,Meals!$A$5:$A$32,$A9,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -2449,11 +2504,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$31,Meals!$A$5:$A$31,$A9,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$32,Meals!$A$5:$A$32,$A9,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$31,Meals!$A$5:$A$31,$A9,Meals!$M$5:$M$31,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$32,Meals!$A$5:$A$32,$A9,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -2461,11 +2516,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$31,$A9,Meals!$M$5:$M$31,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$32,$A9,Meals!$M$5:$M$32,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$31,$A9,Meals!$M$5:$M$31,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$32,$A9,Meals!$M$5:$M$32,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">

</xml_diff>

<commit_message>
Log Day 5 dinner: chapati, green peas and 2 boiled eggs
520-676 kcal (mid 598), 26-33 g protein, 22-33 g fat. Eggs added to the
mess dinner take it to 29.5 g of protein against the 17 g it would
otherwise give.

Day 5 stands at 1,898.5 kcal, 106 g protein, 81.5 g fat. One more scoop
closes it at 2,013.5 kcal and 128.5 g - 7 over target and 543 under
maintenance.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N32"/>
+  <dimension ref="A1:N33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2046,39 +2046,39 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Lunch</t>
+          <t>Dinner</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>2 eggs fried without oil + half container ghee rice + small container chicken curry + curd salad</t>
+          <t>2 chapati + green peas curry + 2 boiled eggs</t>
         </is>
       </c>
       <c r="D31" s="7" t="n">
-        <v>565</v>
+        <v>520</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>786</v>
+        <v>676</v>
       </c>
       <c r="F31" s="8">
         <f>AVERAGE(D31:E31)</f>
         <v/>
       </c>
       <c r="G31" s="9" t="n">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="H31" s="9" t="n">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="I31" s="10">
         <f>AVERAGE(G31:H31)</f>
         <v/>
       </c>
       <c r="J31" s="9" t="n">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="K31" s="9" t="n">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="L31" s="10">
         <f>AVERAGE(J31:K31)</f>
@@ -2091,7 +2091,7 @@
       </c>
       <c r="N31" s="6" t="inlineStr">
         <is>
-          <t>Eggs dry-fried with pepper and salt; rice halved by the user</t>
+          <t>Eggs added to the mess dinner as the protein anchor</t>
         </is>
       </c>
     </row>
@@ -2101,39 +2101,39 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Snack</t>
+          <t>Lunch</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Black coffee + 1 whey scoop</t>
+          <t>2 eggs fried without oil + half container ghee rice + small container chicken curry + curd salad</t>
         </is>
       </c>
       <c r="D32" s="7" t="n">
-        <v>100</v>
+        <v>565</v>
       </c>
       <c r="E32" s="7" t="n">
-        <v>130</v>
+        <v>786</v>
       </c>
       <c r="F32" s="8">
         <f>AVERAGE(D32:E32)</f>
         <v/>
       </c>
       <c r="G32" s="9" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="H32" s="9" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="I32" s="10">
         <f>AVERAGE(G32:H32)</f>
         <v/>
       </c>
       <c r="J32" s="9" t="n">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="K32" s="9" t="n">
-        <v>3</v>
+        <v>44</v>
       </c>
       <c r="L32" s="10">
         <f>AVERAGE(J32:K32)</f>
@@ -2145,6 +2145,61 @@
         </is>
       </c>
       <c r="N32" s="6" t="inlineStr">
+        <is>
+          <t>Eggs dry-fried with pepper and salt; rice halved by the user</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Black coffee + 1 whey scoop</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E33" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="F33" s="8">
+        <f>AVERAGE(D33:E33)</f>
+        <v/>
+      </c>
+      <c r="G33" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="H33" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="I33" s="10">
+        <f>AVERAGE(G33:H33)</f>
+        <v/>
+      </c>
+      <c r="J33" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K33" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="L33" s="10">
+        <f>AVERAGE(J33:K33)</f>
+        <v/>
+      </c>
+      <c r="M33" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N33" s="6" t="inlineStr">
         <is>
           <t>Scoop 1 of the 3 planned for today</t>
         </is>
@@ -2268,11 +2323,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$32,Meals!$A$5:$A$32,$A5,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$33,Meals!$A$5:$A$33,$A5,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$32,Meals!$A$5:$A$32,$A5,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$33,Meals!$A$5:$A$33,$A5,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -2280,11 +2335,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$32,Meals!$A$5:$A$32,$A5,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$33,Meals!$A$5:$A$33,$A5,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$32,Meals!$A$5:$A$32,$A5,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$33,Meals!$A$5:$A$33,$A5,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -2292,11 +2347,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$32,Meals!$A$5:$A$32,$A5,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$33,Meals!$A$5:$A$33,$A5,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$32,Meals!$A$5:$A$32,$A5,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$33,Meals!$A$5:$A$33,$A5,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -2304,11 +2359,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$32,$A5,Meals!$M$5:$M$32,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$33,$A5,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$32,$A5,Meals!$M$5:$M$32,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$33,$A5,Meals!$M$5:$M$33,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -2321,11 +2376,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$32,Meals!$A$5:$A$32,$A6,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$33,Meals!$A$5:$A$33,$A6,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$32,Meals!$A$5:$A$32,$A6,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$33,Meals!$A$5:$A$33,$A6,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -2333,11 +2388,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$32,Meals!$A$5:$A$32,$A6,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$33,Meals!$A$5:$A$33,$A6,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$32,Meals!$A$5:$A$32,$A6,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$33,Meals!$A$5:$A$33,$A6,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -2345,11 +2400,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$32,Meals!$A$5:$A$32,$A6,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$33,Meals!$A$5:$A$33,$A6,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$32,Meals!$A$5:$A$32,$A6,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$33,Meals!$A$5:$A$33,$A6,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -2357,11 +2412,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$32,$A6,Meals!$M$5:$M$32,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$33,$A6,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$32,$A6,Meals!$M$5:$M$32,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$33,$A6,Meals!$M$5:$M$33,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -2374,11 +2429,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$32,Meals!$A$5:$A$32,$A7,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$33,Meals!$A$5:$A$33,$A7,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$32,Meals!$A$5:$A$32,$A7,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$33,Meals!$A$5:$A$33,$A7,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -2386,11 +2441,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$32,Meals!$A$5:$A$32,$A7,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$33,Meals!$A$5:$A$33,$A7,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$32,Meals!$A$5:$A$32,$A7,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$33,Meals!$A$5:$A$33,$A7,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -2398,11 +2453,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$32,Meals!$A$5:$A$32,$A7,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$33,Meals!$A$5:$A$33,$A7,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$32,Meals!$A$5:$A$32,$A7,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$33,Meals!$A$5:$A$33,$A7,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -2410,11 +2465,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$32,$A7,Meals!$M$5:$M$32,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$33,$A7,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$32,$A7,Meals!$M$5:$M$32,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$33,$A7,Meals!$M$5:$M$33,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -2427,11 +2482,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$32,Meals!$A$5:$A$32,$A8,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$33,Meals!$A$5:$A$33,$A8,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$32,Meals!$A$5:$A$32,$A8,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$33,Meals!$A$5:$A$33,$A8,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -2439,11 +2494,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$32,Meals!$A$5:$A$32,$A8,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$33,Meals!$A$5:$A$33,$A8,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$32,Meals!$A$5:$A$32,$A8,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$33,Meals!$A$5:$A$33,$A8,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -2451,11 +2506,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$32,Meals!$A$5:$A$32,$A8,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$33,Meals!$A$5:$A$33,$A8,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$32,Meals!$A$5:$A$32,$A8,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$33,Meals!$A$5:$A$33,$A8,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -2463,11 +2518,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$32,$A8,Meals!$M$5:$M$32,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$33,$A8,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$32,$A8,Meals!$M$5:$M$32,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$33,$A8,Meals!$M$5:$M$33,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -2480,11 +2535,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$32,Meals!$A$5:$A$32,$A9,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$33,Meals!$A$5:$A$33,$A9,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$32,Meals!$A$5:$A$32,$A9,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$33,Meals!$A$5:$A$33,$A9,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -2492,11 +2547,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$32,Meals!$A$5:$A$32,$A9,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$33,Meals!$A$5:$A$33,$A9,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$32,Meals!$A$5:$A$32,$A9,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$33,Meals!$A$5:$A$33,$A9,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -2504,11 +2559,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$32,Meals!$A$5:$A$32,$A9,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$33,Meals!$A$5:$A$33,$A9,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$32,Meals!$A$5:$A$32,$A9,Meals!$M$5:$M$32,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$33,Meals!$A$5:$A$33,$A9,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -2516,11 +2571,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$32,$A9,Meals!$M$5:$M$32,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$33,$A9,Meals!$M$5:$M$33,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$32,$A9,Meals!$M$5:$M$32,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$33,$A9,Meals!$M$5:$M$33,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">

</xml_diff>

<commit_message>
Log Coca-Cola Zero on Day 5
0-2 kcal. Day 5 stands at 1,899.5 kcal, 106 g protein, 81.5 g fat, with one
scoop still to come.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N33"/>
+  <dimension ref="A1:N34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2202,6 +2202,61 @@
       <c r="N33" s="6" t="inlineStr">
         <is>
           <t>Scoop 1 of the 3 planned for today</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>Coca-Cola Zero Sugar (245 ml)</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F34" s="8">
+        <f>AVERAGE(D34:E34)</f>
+        <v/>
+      </c>
+      <c r="G34" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="10">
+        <f>AVERAGE(G34:H34)</f>
+        <v/>
+      </c>
+      <c r="J34" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" s="10">
+        <f>AVERAGE(J34:K34)</f>
+        <v/>
+      </c>
+      <c r="M34" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N34" s="6" t="inlineStr">
+        <is>
+          <t>Genuinely zero calorie</t>
         </is>
       </c>
     </row>
@@ -2323,11 +2378,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$33,Meals!$A$5:$A$33,$A5,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$34,Meals!$A$5:$A$34,$A5,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$33,Meals!$A$5:$A$33,$A5,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$34,Meals!$A$5:$A$34,$A5,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -2335,11 +2390,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$33,Meals!$A$5:$A$33,$A5,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$34,Meals!$A$5:$A$34,$A5,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$33,Meals!$A$5:$A$33,$A5,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$34,Meals!$A$5:$A$34,$A5,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -2347,11 +2402,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$33,Meals!$A$5:$A$33,$A5,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$34,Meals!$A$5:$A$34,$A5,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$33,Meals!$A$5:$A$33,$A5,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$34,Meals!$A$5:$A$34,$A5,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -2359,11 +2414,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$33,$A5,Meals!$M$5:$M$33,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$34,$A5,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$33,$A5,Meals!$M$5:$M$33,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$34,$A5,Meals!$M$5:$M$34,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -2376,11 +2431,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$33,Meals!$A$5:$A$33,$A6,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$34,Meals!$A$5:$A$34,$A6,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$33,Meals!$A$5:$A$33,$A6,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$34,Meals!$A$5:$A$34,$A6,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -2388,11 +2443,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$33,Meals!$A$5:$A$33,$A6,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$34,Meals!$A$5:$A$34,$A6,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$33,Meals!$A$5:$A$33,$A6,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$34,Meals!$A$5:$A$34,$A6,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -2400,11 +2455,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$33,Meals!$A$5:$A$33,$A6,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$34,Meals!$A$5:$A$34,$A6,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$33,Meals!$A$5:$A$33,$A6,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$34,Meals!$A$5:$A$34,$A6,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -2412,11 +2467,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$33,$A6,Meals!$M$5:$M$33,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$34,$A6,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$33,$A6,Meals!$M$5:$M$33,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$34,$A6,Meals!$M$5:$M$34,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -2429,11 +2484,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$33,Meals!$A$5:$A$33,$A7,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$34,Meals!$A$5:$A$34,$A7,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$33,Meals!$A$5:$A$33,$A7,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$34,Meals!$A$5:$A$34,$A7,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -2441,11 +2496,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$33,Meals!$A$5:$A$33,$A7,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$34,Meals!$A$5:$A$34,$A7,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$33,Meals!$A$5:$A$33,$A7,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$34,Meals!$A$5:$A$34,$A7,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -2453,11 +2508,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$33,Meals!$A$5:$A$33,$A7,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$34,Meals!$A$5:$A$34,$A7,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$33,Meals!$A$5:$A$33,$A7,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$34,Meals!$A$5:$A$34,$A7,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -2465,11 +2520,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$33,$A7,Meals!$M$5:$M$33,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$34,$A7,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$33,$A7,Meals!$M$5:$M$33,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$34,$A7,Meals!$M$5:$M$34,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -2482,11 +2537,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$33,Meals!$A$5:$A$33,$A8,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$34,Meals!$A$5:$A$34,$A8,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$33,Meals!$A$5:$A$33,$A8,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$34,Meals!$A$5:$A$34,$A8,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -2494,11 +2549,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$33,Meals!$A$5:$A$33,$A8,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$34,Meals!$A$5:$A$34,$A8,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$33,Meals!$A$5:$A$33,$A8,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$34,Meals!$A$5:$A$34,$A8,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -2506,11 +2561,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$33,Meals!$A$5:$A$33,$A8,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$34,Meals!$A$5:$A$34,$A8,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$33,Meals!$A$5:$A$33,$A8,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$34,Meals!$A$5:$A$34,$A8,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -2518,11 +2573,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$33,$A8,Meals!$M$5:$M$33,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$34,$A8,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$33,$A8,Meals!$M$5:$M$33,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$34,$A8,Meals!$M$5:$M$34,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -2535,11 +2590,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$33,Meals!$A$5:$A$33,$A9,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$34,Meals!$A$5:$A$34,$A9,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$33,Meals!$A$5:$A$33,$A9,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$34,Meals!$A$5:$A$34,$A9,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -2547,11 +2602,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$33,Meals!$A$5:$A$33,$A9,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$34,Meals!$A$5:$A$34,$A9,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$33,Meals!$A$5:$A$33,$A9,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$34,Meals!$A$5:$A$34,$A9,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -2559,11 +2614,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$33,Meals!$A$5:$A$33,$A9,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$34,Meals!$A$5:$A$34,$A9,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$33,Meals!$A$5:$A$33,$A9,Meals!$M$5:$M$33,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$34,Meals!$A$5:$A$34,$A9,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -2571,11 +2626,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$33,$A9,Meals!$M$5:$M$33,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$34,$A9,Meals!$M$5:$M$34,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$33,$A9,Meals!$M$5:$M$33,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$34,$A9,Meals!$M$5:$M$34,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -4096,7 +4151,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5096,14 +5151,14 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in black coffee no sugar)</t>
+          <t>Diet/zero-sugar soft drink (330 ml)</t>
         </is>
       </c>
       <c r="B41" s="7" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="C41" s="7" t="n">
-        <v>130</v>
+        <v>2</v>
       </c>
       <c r="D41" s="8">
         <f>AVERAGE(B41:C41)</f>
@@ -5111,22 +5166,26 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="inlineStr"/>
+          <t>0 g</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>Genuinely zero - unlike fruit juice sold as no added sugar</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Cashew/almond biscuit (1)</t>
+          <t>Whey scoop (in black coffee no sugar)</t>
         </is>
       </c>
       <c r="B42" s="7" t="n">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C42" s="7" t="n">
-        <v>38</v>
+        <v>130</v>
       </c>
       <c r="D42" s="8">
         <f>AVERAGE(B42:C42)</f>
@@ -5134,7 +5193,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>~0.5 g</t>
+          <t>~20-25 g</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr"/>
@@ -5142,14 +5201,14 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (~50g standard)</t>
+          <t>Cashew/almond biscuit (1)</t>
         </is>
       </c>
       <c r="B43" s="7" t="n">
-        <v>245</v>
+        <v>38</v>
       </c>
       <c r="C43" s="7" t="n">
-        <v>250</v>
+        <v>38</v>
       </c>
       <c r="D43" s="8">
         <f>AVERAGE(B43:C43)</f>
@@ -5157,7 +5216,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>~4 g</t>
+          <t>~0.5 g</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr"/>
@@ -5165,14 +5224,14 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (70g king-size)</t>
+          <t>Chocolate bar (~50g standard)</t>
         </is>
       </c>
       <c r="B44" s="7" t="n">
-        <v>335</v>
+        <v>245</v>
       </c>
       <c r="C44" s="7" t="n">
-        <v>335</v>
+        <v>250</v>
       </c>
       <c r="D44" s="8">
         <f>AVERAGE(B44:C44)</f>
@@ -5180,7 +5239,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>~6 g</t>
+          <t>~4 g</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr"/>
@@ -5188,14 +5247,14 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Pre-workout scoop</t>
+          <t>Chocolate bar (70g king-size)</t>
         </is>
       </c>
       <c r="B45" s="7" t="n">
-        <v>5</v>
+        <v>335</v>
       </c>
       <c r="C45" s="7" t="n">
-        <v>15</v>
+        <v>335</v>
       </c>
       <c r="D45" s="8">
         <f>AVERAGE(B45:C45)</f>
@@ -5203,10 +5262,33 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
+          <t>~6 g</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>Pre-workout scoop</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C46" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D46" s="8">
+        <f>AVERAGE(B46:C46)</f>
+        <v/>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
           <t>0 g</t>
         </is>
       </c>
-      <c r="F45" s="6" t="inlineStr">
+      <c r="F46" s="6" t="inlineStr">
         <is>
           <t>Negligible</t>
         </is>

</xml_diff>

<commit_message>
Close Day 5: the four-day rise in calories and fat breaks
Final scoop brings Day 5 to 2,009.5 kcal, 128.5 g protein, 83 g fat -
3 above target and 547 under maintenance, against Day 4's 2,560 kcal,
104 g fat and no deficit at all.

Rewrote the trends section on five complete days. The average is now
2,173 kcal, 110.8 g protein, 83.7 g fat: a 383/day deficit, 0.35 kg/week.
Protein is solved, the calorie rise is broken, fat has turned but is still
28 g above the floor.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N34"/>
+  <dimension ref="A1:N35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2258,6 +2258,61 @@
       <c r="N34" s="6" t="inlineStr">
         <is>
           <t>Genuinely zero calorie</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>1 whey scoop + water</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E35" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="F35" s="8">
+        <f>AVERAGE(D35:E35)</f>
+        <v/>
+      </c>
+      <c r="G35" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="H35" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="I35" s="10">
+        <f>AVERAGE(G35:H35)</f>
+        <v/>
+      </c>
+      <c r="J35" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K35" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="L35" s="10">
+        <f>AVERAGE(J35:K35)</f>
+        <v/>
+      </c>
+      <c r="M35" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N35" s="6" t="inlineStr">
+        <is>
+          <t>Closing scoop for the day</t>
         </is>
       </c>
     </row>
@@ -2379,11 +2434,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$34,Meals!$A$5:$A$34,$A5,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$35,Meals!$A$5:$A$35,$A5,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$34,Meals!$A$5:$A$34,$A5,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$35,Meals!$A$5:$A$35,$A5,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -2391,11 +2446,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$34,Meals!$A$5:$A$34,$A5,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$35,Meals!$A$5:$A$35,$A5,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$34,Meals!$A$5:$A$34,$A5,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$35,Meals!$A$5:$A$35,$A5,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -2403,11 +2458,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$34,Meals!$A$5:$A$34,$A5,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$35,Meals!$A$5:$A$35,$A5,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$34,Meals!$A$5:$A$34,$A5,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$35,Meals!$A$5:$A$35,$A5,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -2415,11 +2470,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$34,$A5,Meals!$M$5:$M$34,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$35,$A5,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$34,$A5,Meals!$M$5:$M$34,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$35,$A5,Meals!$M$5:$M$35,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -2432,11 +2487,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$34,Meals!$A$5:$A$34,$A6,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$35,Meals!$A$5:$A$35,$A6,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$34,Meals!$A$5:$A$34,$A6,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$35,Meals!$A$5:$A$35,$A6,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -2444,11 +2499,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$34,Meals!$A$5:$A$34,$A6,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$35,Meals!$A$5:$A$35,$A6,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$34,Meals!$A$5:$A$34,$A6,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$35,Meals!$A$5:$A$35,$A6,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -2456,11 +2511,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$34,Meals!$A$5:$A$34,$A6,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$35,Meals!$A$5:$A$35,$A6,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$34,Meals!$A$5:$A$34,$A6,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$35,Meals!$A$5:$A$35,$A6,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -2468,11 +2523,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$34,$A6,Meals!$M$5:$M$34,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$35,$A6,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$34,$A6,Meals!$M$5:$M$34,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$35,$A6,Meals!$M$5:$M$35,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -2485,11 +2540,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$34,Meals!$A$5:$A$34,$A7,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$35,Meals!$A$5:$A$35,$A7,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$34,Meals!$A$5:$A$34,$A7,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$35,Meals!$A$5:$A$35,$A7,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -2497,11 +2552,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$34,Meals!$A$5:$A$34,$A7,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$35,Meals!$A$5:$A$35,$A7,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$34,Meals!$A$5:$A$34,$A7,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$35,Meals!$A$5:$A$35,$A7,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -2509,11 +2564,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$34,Meals!$A$5:$A$34,$A7,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$35,Meals!$A$5:$A$35,$A7,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$34,Meals!$A$5:$A$34,$A7,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$35,Meals!$A$5:$A$35,$A7,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -2521,11 +2576,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$34,$A7,Meals!$M$5:$M$34,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$35,$A7,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$34,$A7,Meals!$M$5:$M$34,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$35,$A7,Meals!$M$5:$M$35,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -2538,11 +2593,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$34,Meals!$A$5:$A$34,$A8,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$35,Meals!$A$5:$A$35,$A8,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$34,Meals!$A$5:$A$34,$A8,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$35,Meals!$A$5:$A$35,$A8,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -2550,11 +2605,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$34,Meals!$A$5:$A$34,$A8,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$35,Meals!$A$5:$A$35,$A8,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$34,Meals!$A$5:$A$34,$A8,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$35,Meals!$A$5:$A$35,$A8,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -2562,11 +2617,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$34,Meals!$A$5:$A$34,$A8,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$35,Meals!$A$5:$A$35,$A8,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$34,Meals!$A$5:$A$34,$A8,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$35,Meals!$A$5:$A$35,$A8,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -2574,11 +2629,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$34,$A8,Meals!$M$5:$M$34,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$35,$A8,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$34,$A8,Meals!$M$5:$M$34,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$35,$A8,Meals!$M$5:$M$35,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -2591,11 +2646,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$34,Meals!$A$5:$A$34,$A9,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$35,Meals!$A$5:$A$35,$A9,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$34,Meals!$A$5:$A$34,$A9,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$35,Meals!$A$5:$A$35,$A9,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -2603,11 +2658,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$34,Meals!$A$5:$A$34,$A9,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$35,Meals!$A$5:$A$35,$A9,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$34,Meals!$A$5:$A$34,$A9,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$35,Meals!$A$5:$A$35,$A9,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -2615,11 +2670,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$34,Meals!$A$5:$A$34,$A9,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$35,Meals!$A$5:$A$35,$A9,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$34,Meals!$A$5:$A$34,$A9,Meals!$M$5:$M$34,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$35,Meals!$A$5:$A$35,$A9,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -2627,11 +2682,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$34,$A9,Meals!$M$5:$M$34,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$35,$A9,Meals!$M$5:$M$35,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$34,$A9,Meals!$M$5:$M$34,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$35,$A9,Meals!$M$5:$M$35,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">

</xml_diff>

<commit_message>
Log 90.3 kg weigh-in and add calf to measurements
Third weigh-in: 91.50 -> 90.75 -> 90.30 kg, down 1.20 kg in four days with
a trailing average of 90.85. The logged deficit over those days accounts for
0.15 kg of fat, so ~87% of the drop is still water and glycogen.

At 90.3 kg the targets re-derive to BMR 1,759, maintenance 2,550 and a
2,000 kcal target. BMI 34.2.

Added a calf column to measurements.csv and the Measurements sheet.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -2708,7 +2708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2812,8 +2812,33 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="27" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B7" s="24" t="n">
+        <v>90.3</v>
+      </c>
+      <c r="C7" s="25">
+        <f>B7-B6</f>
+        <v/>
+      </c>
+      <c r="D7" s="25">
+        <f>B7-$B$5</f>
+        <v/>
+      </c>
+      <c r="E7" s="26">
+        <f>AVERAGE(B5:B7)</f>
+        <v/>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Morning weigh-in</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="27" t="inlineStr">
         <is>
           <t>A drop in the first week is mostly water and glycogen, not fat. Judge the trend over 2-3 weeks, and change the activity multiplier on Targets only then.</t>
         </is>
@@ -2833,7 +2858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2843,9 +2868,10 @@
     <col width="9" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2900,15 +2926,20 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
+          <t>Calf</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
           <t>Waist change</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Arm change</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
@@ -2923,7 +2954,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A2:K2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Log Day 6 breakfast: dosa with egg roast
360-490 kcal (mid 425), 10-14 g protein, 17-28 g fat. A dosa in place of the
menu's poratta saves ~205 kcal on the heaviest breakfast of the week, which
is where Wednesday's cut belonged.

Sets out the two ways to spend the remaining 1,575 kcal: both land at
1,985 kcal, but trading one chapati for one scoop at dinner is worth 19 g
more protein at identical calories.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N35"/>
+  <dimension ref="A1:N36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2316,6 +2316,61 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="4" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Breakfast</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>1 dosa + egg roast (1 whole egg)</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="n">
+        <v>360</v>
+      </c>
+      <c r="E36" s="7" t="n">
+        <v>490</v>
+      </c>
+      <c r="F36" s="8">
+        <f>AVERAGE(D36:E36)</f>
+        <v/>
+      </c>
+      <c r="G36" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="H36" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="I36" s="10">
+        <f>AVERAGE(G36:H36)</f>
+        <v/>
+      </c>
+      <c r="J36" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="K36" s="9" t="n">
+        <v>28</v>
+      </c>
+      <c r="L36" s="10">
+        <f>AVERAGE(J36:K36)</f>
+        <v/>
+      </c>
+      <c r="M36" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N36" s="6" t="inlineStr">
+        <is>
+          <t>Took a dosa instead of the menu's poratta - the Wednesday cut</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:N2"/>
@@ -2330,7 +2385,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2434,11 +2489,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$35,Meals!$A$5:$A$35,$A5,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$36,Meals!$A$5:$A$36,$A5,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$35,Meals!$A$5:$A$35,$A5,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$36,Meals!$A$5:$A$36,$A5,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -2446,11 +2501,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$35,Meals!$A$5:$A$35,$A5,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$36,Meals!$A$5:$A$36,$A5,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$35,Meals!$A$5:$A$35,$A5,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$36,Meals!$A$5:$A$36,$A5,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -2458,11 +2513,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$35,Meals!$A$5:$A$35,$A5,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$36,Meals!$A$5:$A$36,$A5,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$35,Meals!$A$5:$A$35,$A5,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$36,Meals!$A$5:$A$36,$A5,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -2470,11 +2525,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$35,$A5,Meals!$M$5:$M$35,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$36,$A5,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$35,$A5,Meals!$M$5:$M$35,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$36,$A5,Meals!$M$5:$M$36,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -2487,11 +2542,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$35,Meals!$A$5:$A$35,$A6,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$36,Meals!$A$5:$A$36,$A6,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$35,Meals!$A$5:$A$35,$A6,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$36,Meals!$A$5:$A$36,$A6,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -2499,11 +2554,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$35,Meals!$A$5:$A$35,$A6,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$36,Meals!$A$5:$A$36,$A6,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$35,Meals!$A$5:$A$35,$A6,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$36,Meals!$A$5:$A$36,$A6,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -2511,11 +2566,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$35,Meals!$A$5:$A$35,$A6,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$36,Meals!$A$5:$A$36,$A6,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$35,Meals!$A$5:$A$35,$A6,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$36,Meals!$A$5:$A$36,$A6,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -2523,11 +2578,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$35,$A6,Meals!$M$5:$M$35,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$36,$A6,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$35,$A6,Meals!$M$5:$M$35,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$36,$A6,Meals!$M$5:$M$36,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -2540,11 +2595,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$35,Meals!$A$5:$A$35,$A7,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$36,Meals!$A$5:$A$36,$A7,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$35,Meals!$A$5:$A$35,$A7,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$36,Meals!$A$5:$A$36,$A7,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -2552,11 +2607,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$35,Meals!$A$5:$A$35,$A7,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$36,Meals!$A$5:$A$36,$A7,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$35,Meals!$A$5:$A$35,$A7,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$36,Meals!$A$5:$A$36,$A7,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -2564,11 +2619,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$35,Meals!$A$5:$A$35,$A7,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$36,Meals!$A$5:$A$36,$A7,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$35,Meals!$A$5:$A$35,$A7,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$36,Meals!$A$5:$A$36,$A7,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -2576,11 +2631,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$35,$A7,Meals!$M$5:$M$35,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$36,$A7,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$35,$A7,Meals!$M$5:$M$35,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$36,$A7,Meals!$M$5:$M$36,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -2593,11 +2648,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$35,Meals!$A$5:$A$35,$A8,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$36,Meals!$A$5:$A$36,$A8,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$35,Meals!$A$5:$A$35,$A8,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$36,Meals!$A$5:$A$36,$A8,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -2605,11 +2660,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$35,Meals!$A$5:$A$35,$A8,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$36,Meals!$A$5:$A$36,$A8,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$35,Meals!$A$5:$A$35,$A8,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$36,Meals!$A$5:$A$36,$A8,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -2617,11 +2672,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$35,Meals!$A$5:$A$35,$A8,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$36,Meals!$A$5:$A$36,$A8,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$35,Meals!$A$5:$A$35,$A8,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$36,Meals!$A$5:$A$36,$A8,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -2629,11 +2684,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$35,$A8,Meals!$M$5:$M$35,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$36,$A8,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$35,$A8,Meals!$M$5:$M$35,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$36,$A8,Meals!$M$5:$M$36,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -2646,11 +2701,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$35,Meals!$A$5:$A$35,$A9,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$36,Meals!$A$5:$A$36,$A9,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$35,Meals!$A$5:$A$35,$A9,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$36,Meals!$A$5:$A$36,$A9,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -2658,11 +2713,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$35,Meals!$A$5:$A$35,$A9,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$36,Meals!$A$5:$A$36,$A9,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$35,Meals!$A$5:$A$35,$A9,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$36,Meals!$A$5:$A$36,$A9,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -2670,11 +2725,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$35,Meals!$A$5:$A$35,$A9,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$36,Meals!$A$5:$A$36,$A9,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$35,Meals!$A$5:$A$35,$A9,Meals!$M$5:$M$35,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$36,Meals!$A$5:$A$36,$A9,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -2682,15 +2737,68 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$35,$A9,Meals!$M$5:$M$35,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$36,$A9,Meals!$M$5:$M$36,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$35,$A9,Meals!$M$5:$M$35,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$36,$A9,Meals!$M$5:$M$36,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
         <f>D9-Targets!$B$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B10" s="21">
+        <f>SUMIFS(Meals!$D$5:$D$36,Meals!$A$5:$A$36,$A10,Meals!$M$5:$M$36,"logged")</f>
+        <v/>
+      </c>
+      <c r="C10" s="21">
+        <f>SUMIFS(Meals!$E$5:$E$36,Meals!$A$5:$A$36,$A10,Meals!$M$5:$M$36,"logged")</f>
+        <v/>
+      </c>
+      <c r="D10" s="21">
+        <f>AVERAGE(B10:C10)</f>
+        <v/>
+      </c>
+      <c r="E10" s="22">
+        <f>SUMIFS(Meals!$G$5:$G$36,Meals!$A$5:$A$36,$A10,Meals!$M$5:$M$36,"logged")</f>
+        <v/>
+      </c>
+      <c r="F10" s="22">
+        <f>SUMIFS(Meals!$H$5:$H$36,Meals!$A$5:$A$36,$A10,Meals!$M$5:$M$36,"logged")</f>
+        <v/>
+      </c>
+      <c r="G10" s="22">
+        <f>AVERAGE(E10:F10)</f>
+        <v/>
+      </c>
+      <c r="H10" s="22">
+        <f>SUMIFS(Meals!$J$5:$J$36,Meals!$A$5:$A$36,$A10,Meals!$M$5:$M$36,"logged")</f>
+        <v/>
+      </c>
+      <c r="I10" s="22">
+        <f>SUMIFS(Meals!$K$5:$K$36,Meals!$A$5:$A$36,$A10,Meals!$M$5:$M$36,"logged")</f>
+        <v/>
+      </c>
+      <c r="J10" s="22">
+        <f>AVERAGE(H10:I10)</f>
+        <v/>
+      </c>
+      <c r="K10" s="20">
+        <f>COUNTIFS(Meals!$A$5:$A$36,$A10,Meals!$M$5:$M$36,"logged")</f>
+        <v/>
+      </c>
+      <c r="L10" s="20">
+        <f>COUNTIFS(Meals!$A$5:$A$36,$A10,Meals!$M$5:$M$36,"pending")</f>
+        <v/>
+      </c>
+      <c r="M10" s="23">
+        <f>D10-Targets!$B$16</f>
         <v/>
       </c>
     </row>
@@ -3599,7 +3707,7 @@
         </is>
       </c>
       <c r="B5" s="18">
-        <f>COUNT(Daily!$A$5:$A$9)</f>
+        <f>COUNT(Daily!$A$5:$A$10)</f>
         <v/>
       </c>
     </row>
@@ -3610,7 +3718,7 @@
         </is>
       </c>
       <c r="B6" s="8">
-        <f>IFERROR(AVERAGE(Daily!$D$5:$D$9),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$D$5:$D$10),0)</f>
         <v/>
       </c>
     </row>
@@ -3621,7 +3729,7 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>IFERROR(AVERAGE(Daily!$G$5:$G$9),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$G$5:$G$10),0)</f>
         <v/>
       </c>
     </row>
@@ -3632,7 +3740,7 @@
         </is>
       </c>
       <c r="B8" s="10">
-        <f>IFERROR(AVERAGE(Daily!$J$5:$J$9),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$J$5:$J$10),0)</f>
         <v/>
       </c>
     </row>
@@ -3676,7 +3784,7 @@
         </is>
       </c>
       <c r="B12" s="18">
-        <f>COUNTIFS(Daily!$G$5:$G$9,"&gt;="&amp;Targets!$B$20)</f>
+        <f>COUNTIFS(Daily!$G$5:$G$10,"&gt;="&amp;Targets!$B$20)</f>
         <v/>
       </c>
     </row>
@@ -3687,7 +3795,7 @@
         </is>
       </c>
       <c r="B13" s="18">
-        <f>SUM(Daily!$L$5:$L$9)</f>
+        <f>SUM(Daily!$L$5:$L$10)</f>
         <v/>
       </c>
     </row>
@@ -3738,19 +3846,19 @@
         <v>46271</v>
       </c>
       <c r="C17" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$9,"&gt;="&amp;$A17,Daily!$A$5:$A$9,"&lt;="&amp;$B17)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$10,"&gt;="&amp;$A17,Daily!$A$5:$A$10,"&lt;="&amp;$B17)</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$9,Daily!$A$5:$A$9,"&gt;="&amp;$A17,Daily!$A$5:$A$9,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$10,Daily!$A$5:$A$10,"&gt;="&amp;$A17,Daily!$A$5:$A$10,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$9,Daily!$A$5:$A$9,"&gt;="&amp;$A17,Daily!$A$5:$A$9,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$10,Daily!$A$5:$A$10,"&gt;="&amp;$A17,Daily!$A$5:$A$10,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$9,Daily!$A$5:$A$9,"&gt;="&amp;$A17,Daily!$A$5:$A$9,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$10,Daily!$A$5:$A$10,"&gt;="&amp;$A17,Daily!$A$5:$A$10,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
     </row>
@@ -3762,19 +3870,19 @@
         <v>46278</v>
       </c>
       <c r="C18" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$9,"&gt;="&amp;$A18,Daily!$A$5:$A$9,"&lt;="&amp;$B18)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$10,"&gt;="&amp;$A18,Daily!$A$5:$A$10,"&lt;="&amp;$B18)</f>
         <v/>
       </c>
       <c r="D18" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$9,Daily!$A$5:$A$9,"&gt;="&amp;$A18,Daily!$A$5:$A$9,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$10,Daily!$A$5:$A$10,"&gt;="&amp;$A18,Daily!$A$5:$A$10,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="E18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$9,Daily!$A$5:$A$9,"&gt;="&amp;$A18,Daily!$A$5:$A$9,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$10,Daily!$A$5:$A$10,"&gt;="&amp;$A18,Daily!$A$5:$A$10,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="F18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$9,Daily!$A$5:$A$9,"&gt;="&amp;$A18,Daily!$A$5:$A$9,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$10,Daily!$A$5:$A$10,"&gt;="&amp;$A18,Daily!$A$5:$A$10,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
     </row>
@@ -3825,19 +3933,19 @@
         <v>46295</v>
       </c>
       <c r="C22" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$9,"&gt;="&amp;$A22,Daily!$A$5:$A$9,"&lt;="&amp;$B22)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$10,"&gt;="&amp;$A22,Daily!$A$5:$A$10,"&lt;="&amp;$B22)</f>
         <v/>
       </c>
       <c r="D22" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$9,Daily!$A$5:$A$9,"&gt;="&amp;$A22,Daily!$A$5:$A$9,"&lt;="&amp;$B22),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$10,Daily!$A$5:$A$10,"&gt;="&amp;$A22,Daily!$A$5:$A$10,"&lt;="&amp;$B22),0)</f>
         <v/>
       </c>
       <c r="E22" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$9,Daily!$A$5:$A$9,"&gt;="&amp;$A22,Daily!$A$5:$A$9,"&lt;="&amp;$B22),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$10,Daily!$A$5:$A$10,"&gt;="&amp;$A22,Daily!$A$5:$A$10,"&lt;="&amp;$B22),0)</f>
         <v/>
       </c>
       <c r="F22" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$9,Daily!$A$5:$A$9,"&gt;="&amp;$A22,Daily!$A$5:$A$9,"&lt;="&amp;$B22),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$10,Daily!$A$5:$A$10,"&gt;="&amp;$A22,Daily!$A$5:$A$10,"&lt;="&amp;$B22),0)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Log first whey scoop of Day 6
100-130 kcal, 20-25 g protein. Day 6 stands at 540 kcal and 34.5 g protein
with 1,460 kcal and 95.5 g still to place.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N36"/>
+  <dimension ref="A1:N37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2368,6 +2368,61 @@
       <c r="N36" s="6" t="inlineStr">
         <is>
           <t>Took a dosa instead of the menu's poratta - the Wednesday cut</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>Black coffee + 1 whey scoop</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E37" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="F37" s="8">
+        <f>AVERAGE(D37:E37)</f>
+        <v/>
+      </c>
+      <c r="G37" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="H37" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="I37" s="10">
+        <f>AVERAGE(G37:H37)</f>
+        <v/>
+      </c>
+      <c r="J37" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K37" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="L37" s="10">
+        <f>AVERAGE(J37:K37)</f>
+        <v/>
+      </c>
+      <c r="M37" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N37" s="6" t="inlineStr">
+        <is>
+          <t>Scoop 1 of the 3 planned for today</t>
         </is>
       </c>
     </row>
@@ -2489,11 +2544,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$36,Meals!$A$5:$A$36,$A5,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$37,Meals!$A$5:$A$37,$A5,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$36,Meals!$A$5:$A$36,$A5,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$37,Meals!$A$5:$A$37,$A5,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -2501,11 +2556,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$36,Meals!$A$5:$A$36,$A5,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$37,Meals!$A$5:$A$37,$A5,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$36,Meals!$A$5:$A$36,$A5,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$37,Meals!$A$5:$A$37,$A5,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -2513,11 +2568,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$36,Meals!$A$5:$A$36,$A5,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$37,Meals!$A$5:$A$37,$A5,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$36,Meals!$A$5:$A$36,$A5,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$37,Meals!$A$5:$A$37,$A5,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -2525,11 +2580,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$36,$A5,Meals!$M$5:$M$36,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$37,$A5,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$36,$A5,Meals!$M$5:$M$36,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$37,$A5,Meals!$M$5:$M$37,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -2542,11 +2597,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$36,Meals!$A$5:$A$36,$A6,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$37,Meals!$A$5:$A$37,$A6,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$36,Meals!$A$5:$A$36,$A6,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$37,Meals!$A$5:$A$37,$A6,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -2554,11 +2609,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$36,Meals!$A$5:$A$36,$A6,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$37,Meals!$A$5:$A$37,$A6,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$36,Meals!$A$5:$A$36,$A6,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$37,Meals!$A$5:$A$37,$A6,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -2566,11 +2621,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$36,Meals!$A$5:$A$36,$A6,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$37,Meals!$A$5:$A$37,$A6,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$36,Meals!$A$5:$A$36,$A6,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$37,Meals!$A$5:$A$37,$A6,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -2578,11 +2633,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$36,$A6,Meals!$M$5:$M$36,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$37,$A6,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$36,$A6,Meals!$M$5:$M$36,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$37,$A6,Meals!$M$5:$M$37,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -2595,11 +2650,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$36,Meals!$A$5:$A$36,$A7,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$37,Meals!$A$5:$A$37,$A7,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$36,Meals!$A$5:$A$36,$A7,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$37,Meals!$A$5:$A$37,$A7,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -2607,11 +2662,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$36,Meals!$A$5:$A$36,$A7,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$37,Meals!$A$5:$A$37,$A7,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$36,Meals!$A$5:$A$36,$A7,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$37,Meals!$A$5:$A$37,$A7,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -2619,11 +2674,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$36,Meals!$A$5:$A$36,$A7,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$37,Meals!$A$5:$A$37,$A7,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$36,Meals!$A$5:$A$36,$A7,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$37,Meals!$A$5:$A$37,$A7,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -2631,11 +2686,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$36,$A7,Meals!$M$5:$M$36,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$37,$A7,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$36,$A7,Meals!$M$5:$M$36,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$37,$A7,Meals!$M$5:$M$37,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -2648,11 +2703,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$36,Meals!$A$5:$A$36,$A8,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$37,Meals!$A$5:$A$37,$A8,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$36,Meals!$A$5:$A$36,$A8,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$37,Meals!$A$5:$A$37,$A8,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -2660,11 +2715,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$36,Meals!$A$5:$A$36,$A8,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$37,Meals!$A$5:$A$37,$A8,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$36,Meals!$A$5:$A$36,$A8,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$37,Meals!$A$5:$A$37,$A8,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -2672,11 +2727,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$36,Meals!$A$5:$A$36,$A8,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$37,Meals!$A$5:$A$37,$A8,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$36,Meals!$A$5:$A$36,$A8,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$37,Meals!$A$5:$A$37,$A8,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -2684,11 +2739,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$36,$A8,Meals!$M$5:$M$36,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$37,$A8,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$36,$A8,Meals!$M$5:$M$36,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$37,$A8,Meals!$M$5:$M$37,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -2701,11 +2756,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$36,Meals!$A$5:$A$36,$A9,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$37,Meals!$A$5:$A$37,$A9,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$36,Meals!$A$5:$A$36,$A9,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$37,Meals!$A$5:$A$37,$A9,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -2713,11 +2768,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$36,Meals!$A$5:$A$36,$A9,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$37,Meals!$A$5:$A$37,$A9,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$36,Meals!$A$5:$A$36,$A9,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$37,Meals!$A$5:$A$37,$A9,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -2725,11 +2780,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$36,Meals!$A$5:$A$36,$A9,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$37,Meals!$A$5:$A$37,$A9,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$36,Meals!$A$5:$A$36,$A9,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$37,Meals!$A$5:$A$37,$A9,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -2737,11 +2792,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$36,$A9,Meals!$M$5:$M$36,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$37,$A9,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$36,$A9,Meals!$M$5:$M$36,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$37,$A9,Meals!$M$5:$M$37,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -2754,11 +2809,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$36,Meals!$A$5:$A$36,$A10,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$37,Meals!$A$5:$A$37,$A10,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$36,Meals!$A$5:$A$36,$A10,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$37,Meals!$A$5:$A$37,$A10,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -2766,11 +2821,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$36,Meals!$A$5:$A$36,$A10,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$37,Meals!$A$5:$A$37,$A10,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$36,Meals!$A$5:$A$36,$A10,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$37,Meals!$A$5:$A$37,$A10,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -2778,11 +2833,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$36,Meals!$A$5:$A$36,$A10,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$37,Meals!$A$5:$A$37,$A10,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$36,Meals!$A$5:$A$36,$A10,Meals!$M$5:$M$36,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$37,Meals!$A$5:$A$37,$A10,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -2790,11 +2845,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$36,$A10,Meals!$M$5:$M$36,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$37,$A10,Meals!$M$5:$M$37,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$36,$A10,Meals!$M$5:$M$36,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$37,$A10,Meals!$M$5:$M$37,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">

</xml_diff>

<commit_message>
Log Wednesday lunch: halved rice with three eggs
760-1,060 kcal (mid 910), 32-44 g protein, 29-46 g fat. Rice halved and
2 boiled eggs plus a 1-egg omelette added - both levers for a third day.
4.2 g of protein per 100 kcal against the mess baseline of 3.7.

Day 6 stands at 1,450 kcal, 72.5 g protein, 62 g fat. Lunch ran ~160 kcal
above plan because three eggs cost more than the model's fish, so the
dinner options are recosted.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N37"/>
+  <dimension ref="A1:N38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2377,39 +2377,39 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Snack</t>
+          <t>Lunch</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Black coffee + 1 whey scoop</t>
+          <t>Mess meals plate (rice halved) + 2 boiled eggs + 1-egg omelette + sambar, curd, veg curries, pickle</t>
         </is>
       </c>
       <c r="D37" s="7" t="n">
-        <v>100</v>
+        <v>760</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>130</v>
+        <v>1060</v>
       </c>
       <c r="F37" s="8">
         <f>AVERAGE(D37:E37)</f>
         <v/>
       </c>
       <c r="G37" s="9" t="n">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="H37" s="9" t="n">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="I37" s="10">
         <f>AVERAGE(G37:H37)</f>
         <v/>
       </c>
       <c r="J37" s="9" t="n">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="K37" s="9" t="n">
-        <v>3</v>
+        <v>46</v>
       </c>
       <c r="L37" s="10">
         <f>AVERAGE(J37:K37)</f>
@@ -2421,6 +2421,61 @@
         </is>
       </c>
       <c r="N37" s="6" t="inlineStr">
+        <is>
+          <t>Both levers again - rice halved and three eggs' worth of protein added</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Black coffee + 1 whey scoop</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E38" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="F38" s="8">
+        <f>AVERAGE(D38:E38)</f>
+        <v/>
+      </c>
+      <c r="G38" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="H38" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="I38" s="10">
+        <f>AVERAGE(G38:H38)</f>
+        <v/>
+      </c>
+      <c r="J38" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K38" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="L38" s="10">
+        <f>AVERAGE(J38:K38)</f>
+        <v/>
+      </c>
+      <c r="M38" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N38" s="6" t="inlineStr">
         <is>
           <t>Scoop 1 of the 3 planned for today</t>
         </is>
@@ -2544,11 +2599,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$37,Meals!$A$5:$A$37,$A5,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$38,Meals!$A$5:$A$38,$A5,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$37,Meals!$A$5:$A$37,$A5,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$38,Meals!$A$5:$A$38,$A5,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -2556,11 +2611,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$37,Meals!$A$5:$A$37,$A5,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$38,Meals!$A$5:$A$38,$A5,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$37,Meals!$A$5:$A$37,$A5,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$38,Meals!$A$5:$A$38,$A5,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -2568,11 +2623,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$37,Meals!$A$5:$A$37,$A5,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$38,Meals!$A$5:$A$38,$A5,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$37,Meals!$A$5:$A$37,$A5,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$38,Meals!$A$5:$A$38,$A5,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -2580,11 +2635,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$37,$A5,Meals!$M$5:$M$37,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$38,$A5,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$37,$A5,Meals!$M$5:$M$37,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$38,$A5,Meals!$M$5:$M$38,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -2597,11 +2652,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$37,Meals!$A$5:$A$37,$A6,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$38,Meals!$A$5:$A$38,$A6,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$37,Meals!$A$5:$A$37,$A6,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$38,Meals!$A$5:$A$38,$A6,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -2609,11 +2664,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$37,Meals!$A$5:$A$37,$A6,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$38,Meals!$A$5:$A$38,$A6,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$37,Meals!$A$5:$A$37,$A6,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$38,Meals!$A$5:$A$38,$A6,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -2621,11 +2676,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$37,Meals!$A$5:$A$37,$A6,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$38,Meals!$A$5:$A$38,$A6,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$37,Meals!$A$5:$A$37,$A6,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$38,Meals!$A$5:$A$38,$A6,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -2633,11 +2688,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$37,$A6,Meals!$M$5:$M$37,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$38,$A6,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$37,$A6,Meals!$M$5:$M$37,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$38,$A6,Meals!$M$5:$M$38,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -2650,11 +2705,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$37,Meals!$A$5:$A$37,$A7,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$38,Meals!$A$5:$A$38,$A7,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$37,Meals!$A$5:$A$37,$A7,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$38,Meals!$A$5:$A$38,$A7,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -2662,11 +2717,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$37,Meals!$A$5:$A$37,$A7,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$38,Meals!$A$5:$A$38,$A7,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$37,Meals!$A$5:$A$37,$A7,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$38,Meals!$A$5:$A$38,$A7,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -2674,11 +2729,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$37,Meals!$A$5:$A$37,$A7,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$38,Meals!$A$5:$A$38,$A7,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$37,Meals!$A$5:$A$37,$A7,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$38,Meals!$A$5:$A$38,$A7,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -2686,11 +2741,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$37,$A7,Meals!$M$5:$M$37,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$38,$A7,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$37,$A7,Meals!$M$5:$M$37,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$38,$A7,Meals!$M$5:$M$38,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -2703,11 +2758,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$37,Meals!$A$5:$A$37,$A8,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$38,Meals!$A$5:$A$38,$A8,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$37,Meals!$A$5:$A$37,$A8,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$38,Meals!$A$5:$A$38,$A8,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -2715,11 +2770,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$37,Meals!$A$5:$A$37,$A8,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$38,Meals!$A$5:$A$38,$A8,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$37,Meals!$A$5:$A$37,$A8,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$38,Meals!$A$5:$A$38,$A8,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -2727,11 +2782,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$37,Meals!$A$5:$A$37,$A8,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$38,Meals!$A$5:$A$38,$A8,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$37,Meals!$A$5:$A$37,$A8,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$38,Meals!$A$5:$A$38,$A8,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -2739,11 +2794,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$37,$A8,Meals!$M$5:$M$37,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$38,$A8,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$37,$A8,Meals!$M$5:$M$37,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$38,$A8,Meals!$M$5:$M$38,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -2756,11 +2811,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$37,Meals!$A$5:$A$37,$A9,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$38,Meals!$A$5:$A$38,$A9,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$37,Meals!$A$5:$A$37,$A9,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$38,Meals!$A$5:$A$38,$A9,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -2768,11 +2823,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$37,Meals!$A$5:$A$37,$A9,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$38,Meals!$A$5:$A$38,$A9,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$37,Meals!$A$5:$A$37,$A9,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$38,Meals!$A$5:$A$38,$A9,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -2780,11 +2835,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$37,Meals!$A$5:$A$37,$A9,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$38,Meals!$A$5:$A$38,$A9,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$37,Meals!$A$5:$A$37,$A9,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$38,Meals!$A$5:$A$38,$A9,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -2792,11 +2847,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$37,$A9,Meals!$M$5:$M$37,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$38,$A9,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$37,$A9,Meals!$M$5:$M$37,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$38,$A9,Meals!$M$5:$M$38,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -2809,11 +2864,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$37,Meals!$A$5:$A$37,$A10,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$38,Meals!$A$5:$A$38,$A10,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$37,Meals!$A$5:$A$37,$A10,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$38,Meals!$A$5:$A$38,$A10,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -2821,11 +2876,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$37,Meals!$A$5:$A$37,$A10,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$38,Meals!$A$5:$A$38,$A10,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$37,Meals!$A$5:$A$37,$A10,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$38,Meals!$A$5:$A$38,$A10,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -2833,11 +2888,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$37,Meals!$A$5:$A$37,$A10,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$38,Meals!$A$5:$A$38,$A10,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$37,Meals!$A$5:$A$37,$A10,Meals!$M$5:$M$37,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$38,Meals!$A$5:$A$38,$A10,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -2845,11 +2900,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$37,$A10,Meals!$M$5:$M$37,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$38,$A10,Meals!$M$5:$M$38,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$37,$A10,Meals!$M$5:$M$37,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$38,$A10,Meals!$M$5:$M$38,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">

</xml_diff>

<commit_message>
Refine Wednesday lunch from a clearer photo
Calories unchanged at 760-1,060. Protein low edged to 33 g for the visible
kadala in the veg side, and fat to 31-48 for the coconut thoran. Day 6 fat
moves 62 -> 64 g; the dinner options are otherwise unchanged.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -2382,7 +2382,7 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Mess meals plate (rice halved) + 2 boiled eggs + 1-egg omelette + sambar, curd, veg curries, pickle</t>
+          <t>Mess meals plate (rice halved) + 2 boiled eggs + 1-egg omelette + veg curry, coconut thoran, kadala-veg thoran, chutney</t>
         </is>
       </c>
       <c r="D37" s="7" t="n">
@@ -2396,7 +2396,7 @@
         <v/>
       </c>
       <c r="G37" s="9" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H37" s="9" t="n">
         <v>44</v>
@@ -2406,10 +2406,10 @@
         <v/>
       </c>
       <c r="J37" s="9" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="K37" s="9" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="L37" s="10">
         <f>AVERAGE(J37:K37)</f>
@@ -2422,7 +2422,7 @@
       </c>
       <c r="N37" s="6" t="inlineStr">
         <is>
-          <t>Both levers again - rice halved and three eggs' worth of protein added</t>
+          <t>Both levers again - rice halved and three eggs' worth of protein added. Fat nudged up for the coconut thoran after a clearer photo</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log second scoop and two more eggs on Day 6
Day 6 reaches 1,713 kcal and 108 g of protein before dinner, the best
pre-dinner position in the log - the third scoop is no longer needed.

Six eggs today come to ~444 kcal, ~38 g protein and ~31 g fat; the same
protein from whey would be ~195 kcal and ~2.5 g fat. Noted in the log:
protein is solved, fat is the remaining line and eggs are most of it.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N38"/>
+  <dimension ref="A1:N40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2478,6 +2478,116 @@
       <c r="N38" s="6" t="inlineStr">
         <is>
           <t>Scoop 1 of the 3 planned for today</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>Black coffee + 1 whey scoop</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E39" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="F39" s="8">
+        <f>AVERAGE(D39:E39)</f>
+        <v/>
+      </c>
+      <c r="G39" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="H39" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="I39" s="10">
+        <f>AVERAGE(G39:H39)</f>
+        <v/>
+      </c>
+      <c r="J39" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K39" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="L39" s="10">
+        <f>AVERAGE(J39:K39)</f>
+        <v/>
+      </c>
+      <c r="M39" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N39" s="6" t="inlineStr">
+        <is>
+          <t>Scoop 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>2 boiled eggs</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="n">
+        <v>140</v>
+      </c>
+      <c r="E40" s="7" t="n">
+        <v>156</v>
+      </c>
+      <c r="F40" s="8">
+        <f>AVERAGE(D40:E40)</f>
+        <v/>
+      </c>
+      <c r="G40" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="H40" s="9" t="n">
+        <v>13</v>
+      </c>
+      <c r="I40" s="10">
+        <f>AVERAGE(G40:H40)</f>
+        <v/>
+      </c>
+      <c r="J40" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="K40" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="L40" s="10">
+        <f>AVERAGE(J40:K40)</f>
+        <v/>
+      </c>
+      <c r="M40" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N40" s="6" t="inlineStr">
+        <is>
+          <t>Eggs 5 and 6 of the day</t>
         </is>
       </c>
     </row>
@@ -2599,11 +2709,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$38,Meals!$A$5:$A$38,$A5,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$40,Meals!$A$5:$A$40,$A5,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$38,Meals!$A$5:$A$38,$A5,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$40,Meals!$A$5:$A$40,$A5,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -2611,11 +2721,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$38,Meals!$A$5:$A$38,$A5,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$40,Meals!$A$5:$A$40,$A5,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$38,Meals!$A$5:$A$38,$A5,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$40,Meals!$A$5:$A$40,$A5,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -2623,11 +2733,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$38,Meals!$A$5:$A$38,$A5,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$40,Meals!$A$5:$A$40,$A5,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$38,Meals!$A$5:$A$38,$A5,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$40,Meals!$A$5:$A$40,$A5,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -2635,11 +2745,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$38,$A5,Meals!$M$5:$M$38,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$40,$A5,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$38,$A5,Meals!$M$5:$M$38,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$40,$A5,Meals!$M$5:$M$40,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -2652,11 +2762,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$38,Meals!$A$5:$A$38,$A6,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$40,Meals!$A$5:$A$40,$A6,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$38,Meals!$A$5:$A$38,$A6,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$40,Meals!$A$5:$A$40,$A6,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -2664,11 +2774,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$38,Meals!$A$5:$A$38,$A6,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$40,Meals!$A$5:$A$40,$A6,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$38,Meals!$A$5:$A$38,$A6,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$40,Meals!$A$5:$A$40,$A6,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -2676,11 +2786,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$38,Meals!$A$5:$A$38,$A6,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$40,Meals!$A$5:$A$40,$A6,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$38,Meals!$A$5:$A$38,$A6,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$40,Meals!$A$5:$A$40,$A6,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -2688,11 +2798,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$38,$A6,Meals!$M$5:$M$38,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$40,$A6,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$38,$A6,Meals!$M$5:$M$38,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$40,$A6,Meals!$M$5:$M$40,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -2705,11 +2815,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$38,Meals!$A$5:$A$38,$A7,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$40,Meals!$A$5:$A$40,$A7,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$38,Meals!$A$5:$A$38,$A7,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$40,Meals!$A$5:$A$40,$A7,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -2717,11 +2827,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$38,Meals!$A$5:$A$38,$A7,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$40,Meals!$A$5:$A$40,$A7,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$38,Meals!$A$5:$A$38,$A7,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$40,Meals!$A$5:$A$40,$A7,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -2729,11 +2839,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$38,Meals!$A$5:$A$38,$A7,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$40,Meals!$A$5:$A$40,$A7,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$38,Meals!$A$5:$A$38,$A7,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$40,Meals!$A$5:$A$40,$A7,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -2741,11 +2851,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$38,$A7,Meals!$M$5:$M$38,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$40,$A7,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$38,$A7,Meals!$M$5:$M$38,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$40,$A7,Meals!$M$5:$M$40,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -2758,11 +2868,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$38,Meals!$A$5:$A$38,$A8,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$40,Meals!$A$5:$A$40,$A8,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$38,Meals!$A$5:$A$38,$A8,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$40,Meals!$A$5:$A$40,$A8,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -2770,11 +2880,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$38,Meals!$A$5:$A$38,$A8,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$40,Meals!$A$5:$A$40,$A8,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$38,Meals!$A$5:$A$38,$A8,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$40,Meals!$A$5:$A$40,$A8,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -2782,11 +2892,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$38,Meals!$A$5:$A$38,$A8,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$40,Meals!$A$5:$A$40,$A8,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$38,Meals!$A$5:$A$38,$A8,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$40,Meals!$A$5:$A$40,$A8,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -2794,11 +2904,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$38,$A8,Meals!$M$5:$M$38,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$40,$A8,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$38,$A8,Meals!$M$5:$M$38,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$40,$A8,Meals!$M$5:$M$40,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -2811,11 +2921,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$38,Meals!$A$5:$A$38,$A9,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$40,Meals!$A$5:$A$40,$A9,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$38,Meals!$A$5:$A$38,$A9,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$40,Meals!$A$5:$A$40,$A9,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -2823,11 +2933,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$38,Meals!$A$5:$A$38,$A9,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$40,Meals!$A$5:$A$40,$A9,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$38,Meals!$A$5:$A$38,$A9,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$40,Meals!$A$5:$A$40,$A9,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -2835,11 +2945,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$38,Meals!$A$5:$A$38,$A9,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$40,Meals!$A$5:$A$40,$A9,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$38,Meals!$A$5:$A$38,$A9,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$40,Meals!$A$5:$A$40,$A9,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -2847,11 +2957,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$38,$A9,Meals!$M$5:$M$38,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$40,$A9,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$38,$A9,Meals!$M$5:$M$38,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$40,$A9,Meals!$M$5:$M$40,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -2864,11 +2974,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$38,Meals!$A$5:$A$38,$A10,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$40,Meals!$A$5:$A$40,$A10,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$38,Meals!$A$5:$A$38,$A10,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$40,Meals!$A$5:$A$40,$A10,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -2876,11 +2986,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$38,Meals!$A$5:$A$38,$A10,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$40,Meals!$A$5:$A$40,$A10,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$38,Meals!$A$5:$A$38,$A10,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$40,Meals!$A$5:$A$40,$A10,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -2888,11 +2998,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$38,Meals!$A$5:$A$38,$A10,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$40,Meals!$A$5:$A$40,$A10,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$38,Meals!$A$5:$A$38,$A10,Meals!$M$5:$M$38,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$40,Meals!$A$5:$A$40,$A10,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -2900,11 +3010,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$38,$A10,Meals!$M$5:$M$38,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$40,$A10,Meals!$M$5:$M$40,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$38,$A10,Meals!$M$5:$M$38,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$40,$A10,Meals!$M$5:$M$40,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">

</xml_diff>

<commit_message>
Close Day 6 and rewrite trends on six days
Dinner of 2 chapati with chicken curry brings Day 6 to 2,294 kcal, 139 g
protein and 103.5 g fat - the best protein day and second-highest fat.

The day's meals came to 1,916 kcal, under target on their own; the 378 kcal
snack layer took it 294 over. Dropping the 5pm eggs alone would have given
2,146 kcal and 126.5 g protein.

Six-day average is now 2,193 kcal, 115.5 g protein, 87 g fat - a 357/day
deficit, 0.32 kg/week. Protein is solved three days running; calories show
no trend and fat remains the wrong line, and both trace to the snack layer
rather than the mess plates.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N40"/>
+  <dimension ref="A1:N42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2377,39 +2377,39 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Lunch</t>
+          <t>Dinner</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Mess meals plate (rice halved) + 2 boiled eggs + 1-egg omelette + veg curry, coconut thoran, kadala-veg thoran, chutney</t>
+          <t>2 chapati + chicken curry</t>
         </is>
       </c>
       <c r="D37" s="7" t="n">
-        <v>760</v>
+        <v>480</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>1060</v>
+        <v>680</v>
       </c>
       <c r="F37" s="8">
         <f>AVERAGE(D37:E37)</f>
         <v/>
       </c>
       <c r="G37" s="9" t="n">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="H37" s="9" t="n">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="I37" s="10">
         <f>AVERAGE(G37:H37)</f>
         <v/>
       </c>
       <c r="J37" s="9" t="n">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="K37" s="9" t="n">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="L37" s="10">
         <f>AVERAGE(J37:K37)</f>
@@ -2422,7 +2422,7 @@
       </c>
       <c r="N37" s="6" t="inlineStr">
         <is>
-          <t>Both levers again - rice halved and three eggs' worth of protein added. Fat nudged up for the coconut thoran after a clearer photo</t>
+          <t>Mess Wednesday dinner</t>
         </is>
       </c>
     </row>
@@ -2432,39 +2432,39 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Snack</t>
+          <t>Drink</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Black coffee + 1 whey scoop</t>
+          <t>Coca-Cola Zero Sugar (245 ml)</t>
         </is>
       </c>
       <c r="D38" s="7" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E38" s="7" t="n">
-        <v>130</v>
+        <v>2</v>
       </c>
       <c r="F38" s="8">
         <f>AVERAGE(D38:E38)</f>
         <v/>
       </c>
       <c r="G38" s="9" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H38" s="9" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I38" s="10">
         <f>AVERAGE(G38:H38)</f>
         <v/>
       </c>
       <c r="J38" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K38" s="9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L38" s="10">
         <f>AVERAGE(J38:K38)</f>
@@ -2477,7 +2477,7 @@
       </c>
       <c r="N38" s="6" t="inlineStr">
         <is>
-          <t>Scoop 1 of the 3 planned for today</t>
+          <t>Genuinely zero calorie</t>
         </is>
       </c>
     </row>
@@ -2487,39 +2487,39 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Snack</t>
+          <t>Lunch</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Black coffee + 1 whey scoop</t>
+          <t>Mess meals plate (rice halved) + 2 boiled eggs + 1-egg omelette + veg curry, coconut thoran, kadala-veg thoran, chutney</t>
         </is>
       </c>
       <c r="D39" s="7" t="n">
-        <v>100</v>
+        <v>760</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>130</v>
+        <v>1060</v>
       </c>
       <c r="F39" s="8">
         <f>AVERAGE(D39:E39)</f>
         <v/>
       </c>
       <c r="G39" s="9" t="n">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="H39" s="9" t="n">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="I39" s="10">
         <f>AVERAGE(G39:H39)</f>
         <v/>
       </c>
       <c r="J39" s="9" t="n">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="K39" s="9" t="n">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="L39" s="10">
         <f>AVERAGE(J39:K39)</f>
@@ -2532,7 +2532,7 @@
       </c>
       <c r="N39" s="6" t="inlineStr">
         <is>
-          <t>Scoop 2</t>
+          <t>Both levers again - rice halved and three eggs' worth of protein added. Fat nudged up for the coconut thoran after a clearer photo</t>
         </is>
       </c>
     </row>
@@ -2547,34 +2547,34 @@
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>2 boiled eggs</t>
+          <t>Black coffee + 1 whey scoop</t>
         </is>
       </c>
       <c r="D40" s="7" t="n">
-        <v>140</v>
+        <v>100</v>
       </c>
       <c r="E40" s="7" t="n">
-        <v>156</v>
+        <v>130</v>
       </c>
       <c r="F40" s="8">
         <f>AVERAGE(D40:E40)</f>
         <v/>
       </c>
       <c r="G40" s="9" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H40" s="9" t="n">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="I40" s="10">
         <f>AVERAGE(G40:H40)</f>
         <v/>
       </c>
       <c r="J40" s="9" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K40" s="9" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="L40" s="10">
         <f>AVERAGE(J40:K40)</f>
@@ -2586,6 +2586,116 @@
         </is>
       </c>
       <c r="N40" s="6" t="inlineStr">
+        <is>
+          <t>Scoop 1 of the 3 planned for today</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Black coffee + 1 whey scoop</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E41" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="F41" s="8">
+        <f>AVERAGE(D41:E41)</f>
+        <v/>
+      </c>
+      <c r="G41" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="H41" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="I41" s="10">
+        <f>AVERAGE(G41:H41)</f>
+        <v/>
+      </c>
+      <c r="J41" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K41" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="L41" s="10">
+        <f>AVERAGE(J41:K41)</f>
+        <v/>
+      </c>
+      <c r="M41" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N41" s="6" t="inlineStr">
+        <is>
+          <t>Scoop 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>2 boiled eggs</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="n">
+        <v>140</v>
+      </c>
+      <c r="E42" s="7" t="n">
+        <v>156</v>
+      </c>
+      <c r="F42" s="8">
+        <f>AVERAGE(D42:E42)</f>
+        <v/>
+      </c>
+      <c r="G42" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="H42" s="9" t="n">
+        <v>13</v>
+      </c>
+      <c r="I42" s="10">
+        <f>AVERAGE(G42:H42)</f>
+        <v/>
+      </c>
+      <c r="J42" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="K42" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="L42" s="10">
+        <f>AVERAGE(J42:K42)</f>
+        <v/>
+      </c>
+      <c r="M42" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N42" s="6" t="inlineStr">
         <is>
           <t>Eggs 5 and 6 of the day</t>
         </is>
@@ -2709,11 +2819,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$40,Meals!$A$5:$A$40,$A5,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$42,Meals!$A$5:$A$42,$A5,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$40,Meals!$A$5:$A$40,$A5,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$42,Meals!$A$5:$A$42,$A5,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -2721,11 +2831,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$40,Meals!$A$5:$A$40,$A5,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$42,Meals!$A$5:$A$42,$A5,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$40,Meals!$A$5:$A$40,$A5,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$42,Meals!$A$5:$A$42,$A5,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -2733,11 +2843,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$40,Meals!$A$5:$A$40,$A5,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$42,Meals!$A$5:$A$42,$A5,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$40,Meals!$A$5:$A$40,$A5,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$42,Meals!$A$5:$A$42,$A5,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -2745,11 +2855,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$40,$A5,Meals!$M$5:$M$40,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$42,$A5,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$40,$A5,Meals!$M$5:$M$40,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$42,$A5,Meals!$M$5:$M$42,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -2762,11 +2872,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$40,Meals!$A$5:$A$40,$A6,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$42,Meals!$A$5:$A$42,$A6,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$40,Meals!$A$5:$A$40,$A6,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$42,Meals!$A$5:$A$42,$A6,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -2774,11 +2884,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$40,Meals!$A$5:$A$40,$A6,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$42,Meals!$A$5:$A$42,$A6,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$40,Meals!$A$5:$A$40,$A6,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$42,Meals!$A$5:$A$42,$A6,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -2786,11 +2896,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$40,Meals!$A$5:$A$40,$A6,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$42,Meals!$A$5:$A$42,$A6,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$40,Meals!$A$5:$A$40,$A6,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$42,Meals!$A$5:$A$42,$A6,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -2798,11 +2908,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$40,$A6,Meals!$M$5:$M$40,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$42,$A6,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$40,$A6,Meals!$M$5:$M$40,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$42,$A6,Meals!$M$5:$M$42,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -2815,11 +2925,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$40,Meals!$A$5:$A$40,$A7,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$42,Meals!$A$5:$A$42,$A7,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$40,Meals!$A$5:$A$40,$A7,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$42,Meals!$A$5:$A$42,$A7,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -2827,11 +2937,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$40,Meals!$A$5:$A$40,$A7,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$42,Meals!$A$5:$A$42,$A7,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$40,Meals!$A$5:$A$40,$A7,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$42,Meals!$A$5:$A$42,$A7,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -2839,11 +2949,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$40,Meals!$A$5:$A$40,$A7,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$42,Meals!$A$5:$A$42,$A7,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$40,Meals!$A$5:$A$40,$A7,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$42,Meals!$A$5:$A$42,$A7,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -2851,11 +2961,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$40,$A7,Meals!$M$5:$M$40,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$42,$A7,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$40,$A7,Meals!$M$5:$M$40,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$42,$A7,Meals!$M$5:$M$42,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -2868,11 +2978,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$40,Meals!$A$5:$A$40,$A8,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$42,Meals!$A$5:$A$42,$A8,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$40,Meals!$A$5:$A$40,$A8,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$42,Meals!$A$5:$A$42,$A8,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -2880,11 +2990,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$40,Meals!$A$5:$A$40,$A8,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$42,Meals!$A$5:$A$42,$A8,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$40,Meals!$A$5:$A$40,$A8,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$42,Meals!$A$5:$A$42,$A8,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -2892,11 +3002,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$40,Meals!$A$5:$A$40,$A8,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$42,Meals!$A$5:$A$42,$A8,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$40,Meals!$A$5:$A$40,$A8,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$42,Meals!$A$5:$A$42,$A8,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -2904,11 +3014,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$40,$A8,Meals!$M$5:$M$40,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$42,$A8,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$40,$A8,Meals!$M$5:$M$40,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$42,$A8,Meals!$M$5:$M$42,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -2921,11 +3031,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$40,Meals!$A$5:$A$40,$A9,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$42,Meals!$A$5:$A$42,$A9,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$40,Meals!$A$5:$A$40,$A9,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$42,Meals!$A$5:$A$42,$A9,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -2933,11 +3043,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$40,Meals!$A$5:$A$40,$A9,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$42,Meals!$A$5:$A$42,$A9,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$40,Meals!$A$5:$A$40,$A9,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$42,Meals!$A$5:$A$42,$A9,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -2945,11 +3055,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$40,Meals!$A$5:$A$40,$A9,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$42,Meals!$A$5:$A$42,$A9,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$40,Meals!$A$5:$A$40,$A9,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$42,Meals!$A$5:$A$42,$A9,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -2957,11 +3067,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$40,$A9,Meals!$M$5:$M$40,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$42,$A9,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$40,$A9,Meals!$M$5:$M$40,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$42,$A9,Meals!$M$5:$M$42,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -2974,11 +3084,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$40,Meals!$A$5:$A$40,$A10,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$42,Meals!$A$5:$A$42,$A10,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$40,Meals!$A$5:$A$40,$A10,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$42,Meals!$A$5:$A$42,$A10,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -2986,11 +3096,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$40,Meals!$A$5:$A$40,$A10,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$42,Meals!$A$5:$A$42,$A10,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$40,Meals!$A$5:$A$40,$A10,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$42,Meals!$A$5:$A$42,$A10,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -2998,11 +3108,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$40,Meals!$A$5:$A$40,$A10,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$42,Meals!$A$5:$A$42,$A10,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$40,Meals!$A$5:$A$40,$A10,Meals!$M$5:$M$40,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$42,Meals!$A$5:$A$42,$A10,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -3010,11 +3120,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$40,$A10,Meals!$M$5:$M$40,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$42,$A10,Meals!$M$5:$M$42,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$40,$A10,Meals!$M$5:$M$40,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$42,$A10,Meals!$M$5:$M$42,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -4668,7 +4778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5668,14 +5778,14 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>Diet/zero-sugar soft drink (330 ml)</t>
+          <t>Mango misiri (1 whole ~450-600 g)</t>
         </is>
       </c>
       <c r="B41" s="7" t="n">
-        <v>0</v>
+        <v>170</v>
       </c>
       <c r="C41" s="7" t="n">
-        <v>2</v>
+        <v>230</v>
       </c>
       <c r="D41" s="8">
         <f>AVERAGE(B41:C41)</f>
@@ -5683,26 +5793,26 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>0 g</t>
+          <t>~2-2.5 g</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
-          <t>Genuinely zero - unlike fruit juice sold as no added sugar</t>
+          <t>~60-65% is edible flesh; ~35-50 g sugar but fibre intact</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in black coffee no sugar)</t>
+          <t>Diet/zero-sugar soft drink (330 ml)</t>
         </is>
       </c>
       <c r="B42" s="7" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="C42" s="7" t="n">
-        <v>130</v>
+        <v>2</v>
       </c>
       <c r="D42" s="8">
         <f>AVERAGE(B42:C42)</f>
@@ -5710,22 +5820,26 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="inlineStr"/>
+          <t>0 g</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>Genuinely zero - unlike fruit juice sold as no added sugar</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>Cashew/almond biscuit (1)</t>
+          <t>Whey scoop (in black coffee no sugar)</t>
         </is>
       </c>
       <c r="B43" s="7" t="n">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C43" s="7" t="n">
-        <v>38</v>
+        <v>130</v>
       </c>
       <c r="D43" s="8">
         <f>AVERAGE(B43:C43)</f>
@@ -5733,7 +5847,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>~0.5 g</t>
+          <t>~20-25 g</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr"/>
@@ -5741,14 +5855,14 @@
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (~50g standard)</t>
+          <t>Cashew/almond biscuit (1)</t>
         </is>
       </c>
       <c r="B44" s="7" t="n">
-        <v>245</v>
+        <v>38</v>
       </c>
       <c r="C44" s="7" t="n">
-        <v>250</v>
+        <v>38</v>
       </c>
       <c r="D44" s="8">
         <f>AVERAGE(B44:C44)</f>
@@ -5756,7 +5870,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>~4 g</t>
+          <t>~0.5 g</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr"/>
@@ -5764,14 +5878,14 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (70g king-size)</t>
+          <t>Chocolate bar (~50g standard)</t>
         </is>
       </c>
       <c r="B45" s="7" t="n">
-        <v>335</v>
+        <v>245</v>
       </c>
       <c r="C45" s="7" t="n">
-        <v>335</v>
+        <v>250</v>
       </c>
       <c r="D45" s="8">
         <f>AVERAGE(B45:C45)</f>
@@ -5779,7 +5893,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>~6 g</t>
+          <t>~4 g</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr"/>
@@ -5787,14 +5901,14 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>Pre-workout scoop</t>
+          <t>Chocolate bar (70g king-size)</t>
         </is>
       </c>
       <c r="B46" s="7" t="n">
-        <v>5</v>
+        <v>335</v>
       </c>
       <c r="C46" s="7" t="n">
-        <v>15</v>
+        <v>335</v>
       </c>
       <c r="D46" s="8">
         <f>AVERAGE(B46:C46)</f>
@@ -5802,10 +5916,33 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
+          <t>~6 g</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>Pre-workout scoop</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C47" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D47" s="8">
+        <f>AVERAGE(B47:C47)</f>
+        <v/>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
           <t>0 g</t>
         </is>
       </c>
-      <c r="F46" s="6" t="inlineStr">
+      <c r="F47" s="6" t="inlineStr">
         <is>
           <t>Negligible</t>
         </is>

</xml_diff>

<commit_message>
Add grilled sea bream to the reference estimates
250-400 kcal for a whole 300-400 g fish, ~35-50 g protein. Not logged -
asked about, not eaten.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -4778,7 +4778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5254,14 +5254,14 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Grilled chicken breast (100 g skinless)</t>
+          <t>Grilled sea bream (1 whole ~300-400 g)</t>
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>160</v>
+        <v>250</v>
       </c>
       <c r="C21" s="7" t="n">
-        <v>180</v>
+        <v>400</v>
       </c>
       <c r="D21" s="8">
         <f>AVERAGE(B21:C21)</f>
@@ -5269,26 +5269,26 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>~30-32 g</t>
+          <t>~35-50 g</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>Best protein-per-calorie item in this list</t>
+          <t>Lean white fish; best protein-per-calorie item available. Most fat is the grill oil</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Grilled chicken breast (150 g skinless)</t>
+          <t>Grilled chicken breast (100 g skinless)</t>
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>240</v>
+        <v>160</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>270</v>
+        <v>180</v>
       </c>
       <c r="D22" s="8">
         <f>AVERAGE(B22:C22)</f>
@@ -5296,22 +5296,26 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>~45-48 g</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr"/>
+          <t>~30-32 g</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>Best protein-per-calorie item in this list</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Honest Bowl - Grilled Chicken and Rice Bowl</t>
+          <t>Grilled chicken breast (150 g skinless)</t>
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>550</v>
+        <v>240</v>
       </c>
       <c r="C23" s="7" t="n">
-        <v>710</v>
+        <v>270</v>
       </c>
       <c r="D23" s="8">
         <f>AVERAGE(B23:C23)</f>
@@ -5319,26 +5323,22 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>42-48 g</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="inlineStr">
-        <is>
-          <t>Menu states 42 g protein; chicken + jasmine rice + sweet potato. Sauce served separately</t>
-        </is>
-      </c>
+          <t>~45-48 g</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Brown/mushroom sauce (side pot)</t>
+          <t>Honest Bowl - Grilled Chicken and Rice Bowl</t>
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>50</v>
+        <v>550</v>
       </c>
       <c r="C24" s="7" t="n">
-        <v>120</v>
+        <v>710</v>
       </c>
       <c r="D24" s="8">
         <f>AVERAGE(B24:C24)</f>
@@ -5346,26 +5346,26 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>~1-2 g</t>
+          <t>42-48 g</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>Often cream or butter based - the variable in a bowl like this</t>
+          <t>Menu states 42 g protein; chicken + jasmine rice + sweet potato. Sauce served separately</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Honest Bowl - Tofu Delight Bowl</t>
+          <t>Brown/mushroom sauce (side pot)</t>
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>420</v>
+        <v>50</v>
       </c>
       <c r="C25" s="7" t="n">
-        <v>560</v>
+        <v>120</v>
       </c>
       <c r="D25" s="8">
         <f>AVERAGE(B25:C25)</f>
@@ -5373,26 +5373,26 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>~20 g</t>
+          <t>~1-2 g</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>Menu states 20 g; jasmine rice + cajun tofu + grilled eggplant. Half the protein of the chicken bowl at the same price</t>
+          <t>Often cream or butter based - the variable in a bowl like this</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Chicken curry (1 takeaway container)</t>
+          <t>Honest Bowl - Tofu Delight Bowl</t>
         </is>
       </c>
       <c r="B26" s="7" t="n">
-        <v>280</v>
+        <v>420</v>
       </c>
       <c r="C26" s="7" t="n">
-        <v>420</v>
+        <v>560</v>
       </c>
       <c r="D26" s="8">
         <f>AVERAGE(B26:C26)</f>
@@ -5400,26 +5400,26 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>~20-28 g</t>
+          <t>~20 g</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>Kerala style; oil and coconut carry most of the calories</t>
+          <t>Menu states 20 g; jasmine rice + cajun tofu + grilled eggplant. Half the protein of the chicken bowl at the same price</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Grilled chicken quarter (skin on)</t>
+          <t>Chicken curry (1 takeaway container)</t>
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>250</v>
+        <v>280</v>
       </c>
       <c r="C27" s="7" t="n">
-        <v>320</v>
+        <v>420</v>
       </c>
       <c r="D27" s="8">
         <f>AVERAGE(B27:C27)</f>
@@ -5427,26 +5427,26 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>~28-33 g</t>
+          <t>~20-28 g</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>Skin adds ~12-15 g fat over breast</t>
+          <t>Kerala style; oil and coconut carry most of the calories</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Garlic sauce / toum (1 tbsp)</t>
+          <t>Grilled chicken quarter (skin on)</t>
         </is>
       </c>
       <c r="B28" s="7" t="n">
-        <v>90</v>
+        <v>250</v>
       </c>
       <c r="C28" s="7" t="n">
-        <v>110</v>
+        <v>320</v>
       </c>
       <c r="D28" s="8">
         <f>AVERAGE(B28:C28)</f>
@@ -5454,26 +5454,26 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>0 g</t>
+          <t>~28-33 g</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>Essentially emulsified oil - the hidden cost at a grill</t>
+          <t>Skin adds ~12-15 g fat over breast</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Khubz / pita (1 large)</t>
+          <t>Garlic sauce / toum (1 tbsp)</t>
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>250</v>
+        <v>90</v>
       </c>
       <c r="C29" s="7" t="n">
-        <v>300</v>
+        <v>110</v>
       </c>
       <c r="D29" s="8">
         <f>AVERAGE(B29:C29)</f>
@@ -5481,22 +5481,26 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>~8-9 g</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="inlineStr"/>
+          <t>0 g</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>Essentially emulsified oil - the hidden cost at a grill</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Barik/basmati rice (half container cooked)</t>
+          <t>Khubz / pita (1 large)</t>
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="C30" s="7" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="D30" s="8">
         <f>AVERAGE(B30:C30)</f>
@@ -5504,7 +5508,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>~4-5 g</t>
+          <t>~8-9 g</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr"/>
@@ -5512,14 +5516,14 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Fresh pineapple juice (350-450 ml)</t>
+          <t>Barik/basmati rice (half container cooked)</t>
         </is>
       </c>
       <c r="B31" s="7" t="n">
-        <v>175</v>
+        <v>200</v>
       </c>
       <c r="C31" s="7" t="n">
-        <v>240</v>
+        <v>280</v>
       </c>
       <c r="D31" s="8">
         <f>AVERAGE(B31:C31)</f>
@@ -5527,26 +5531,22 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>~1-2 g</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="inlineStr">
-        <is>
-          <t>No added sugar but ~35-45 g natural sugar; no fibre; almost no protein</t>
-        </is>
-      </c>
+          <t>~4-5 g</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Fresh orange juice (350-450 ml)</t>
+          <t>Fresh pineapple juice (350-450 ml)</t>
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>155</v>
+        <v>175</v>
       </c>
       <c r="C32" s="7" t="n">
-        <v>205</v>
+        <v>240</v>
       </c>
       <c r="D32" s="8">
         <f>AVERAGE(B32:C32)</f>
@@ -5554,26 +5554,26 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>~2-3 g</t>
+          <t>~1-2 g</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>No added sugar but ~32-40 g natural sugar; no fibre</t>
+          <t>No added sugar but ~35-45 g natural sugar; no fibre; almost no protein</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in water)</t>
+          <t>Fresh orange juice (350-450 ml)</t>
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>100</v>
+        <v>155</v>
       </c>
       <c r="C33" s="7" t="n">
-        <v>120</v>
+        <v>205</v>
       </c>
       <c r="D33" s="8">
         <f>AVERAGE(B33:C33)</f>
@@ -5581,22 +5581,26 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="inlineStr"/>
+          <t>~2-3 g</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>No added sugar but ~32-40 g natural sugar; no fibre</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Greek yogurt (200 g plain low-fat)</t>
+          <t>Whey scoop (in water)</t>
         </is>
       </c>
       <c r="B34" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C34" s="7" t="n">
         <v>120</v>
-      </c>
-      <c r="C34" s="7" t="n">
-        <v>140</v>
       </c>
       <c r="D34" s="8">
         <f>AVERAGE(B34:C34)</f>
@@ -5604,26 +5608,22 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>~18-20 g</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="inlineStr">
-        <is>
-          <t>Casein - digests slowly; good overnight</t>
-        </is>
-      </c>
+          <t>~20-25 g</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Boiled egg (1 large)</t>
+          <t>Greek yogurt (200 g plain low-fat)</t>
         </is>
       </c>
       <c r="B35" s="7" t="n">
-        <v>70</v>
+        <v>120</v>
       </c>
       <c r="C35" s="7" t="n">
-        <v>78</v>
+        <v>140</v>
       </c>
       <c r="D35" s="8">
         <f>AVERAGE(B35:C35)</f>
@@ -5631,19 +5631,19 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>~6-6.5 g</t>
+          <t>~18-20 g</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>~5 g fat each</t>
+          <t>Casein - digests slowly; good overnight</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Egg fried dry with no oil (1)</t>
+          <t>Boiled egg (1 large)</t>
         </is>
       </c>
       <c r="B36" s="7" t="n">
@@ -5663,21 +5663,21 @@
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>Same as boiled - dry-frying saves the ~20-25 kcal per egg that pan oil adds</t>
+          <t>~5 g fat each</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Paneer (50 g full-fat)</t>
+          <t>Egg fried dry with no oil (1)</t>
         </is>
       </c>
       <c r="B37" s="7" t="n">
-        <v>130</v>
+        <v>70</v>
       </c>
       <c r="C37" s="7" t="n">
-        <v>150</v>
+        <v>78</v>
       </c>
       <c r="D37" s="8">
         <f>AVERAGE(B37:C37)</f>
@@ -5685,26 +5685,26 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>~8-9 g</t>
+          <t>~6-6.5 g</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>Fat-dense for the protein it gives</t>
+          <t>Same as boiled - dry-frying saves the ~20-25 kcal per egg that pan oil adds</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>Cucumber (1 medium)</t>
+          <t>Paneer (50 g full-fat)</t>
         </is>
       </c>
       <c r="B38" s="7" t="n">
-        <v>25</v>
+        <v>130</v>
       </c>
       <c r="C38" s="7" t="n">
-        <v>30</v>
+        <v>150</v>
       </c>
       <c r="D38" s="8">
         <f>AVERAGE(B38:C38)</f>
@@ -5712,26 +5712,26 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>~1.5 g</t>
+          <t>~8-9 g</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>Volume with almost no calories</t>
+          <t>Fat-dense for the protein it gives</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>Sweet melon / cantaloupe (1 wedge ~100-150 g)</t>
+          <t>Cucumber (1 medium)</t>
         </is>
       </c>
       <c r="B39" s="7" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="C39" s="7" t="n">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="D39" s="8">
         <f>AVERAGE(B39:C39)</f>
@@ -5739,26 +5739,26 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>~0.5-1 g</t>
+          <t>~1.5 g</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
         <is>
-          <t>Whole fruit - fibre and water intact; ~1/4 the calories of the same fruit juiced</t>
+          <t>Volume with almost no calories</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>Grapes (~100 g / 15-20 grapes)</t>
+          <t>Sweet melon / cantaloupe (1 wedge ~100-150 g)</t>
         </is>
       </c>
       <c r="B40" s="7" t="n">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="C40" s="7" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="D40" s="8">
         <f>AVERAGE(B40:C40)</f>
@@ -5766,26 +5766,26 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>~0.6 g</t>
+          <t>~0.5-1 g</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>Twice the calorie density of melon; easy to eat a large handful without noticing</t>
+          <t>Whole fruit - fibre and water intact; ~1/4 the calories of the same fruit juiced</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>Mango misiri (1 whole ~450-600 g)</t>
+          <t>Grapes (~100 g / 15-20 grapes)</t>
         </is>
       </c>
       <c r="B41" s="7" t="n">
-        <v>170</v>
+        <v>60</v>
       </c>
       <c r="C41" s="7" t="n">
-        <v>230</v>
+        <v>75</v>
       </c>
       <c r="D41" s="8">
         <f>AVERAGE(B41:C41)</f>
@@ -5793,26 +5793,26 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>~2-2.5 g</t>
+          <t>~0.6 g</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
-          <t>~60-65% is edible flesh; ~35-50 g sugar but fibre intact</t>
+          <t>Twice the calorie density of melon; easy to eat a large handful without noticing</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Diet/zero-sugar soft drink (330 ml)</t>
+          <t>Mango misiri (1 whole ~450-600 g)</t>
         </is>
       </c>
       <c r="B42" s="7" t="n">
-        <v>0</v>
+        <v>170</v>
       </c>
       <c r="C42" s="7" t="n">
-        <v>2</v>
+        <v>230</v>
       </c>
       <c r="D42" s="8">
         <f>AVERAGE(B42:C42)</f>
@@ -5820,26 +5820,26 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>0 g</t>
+          <t>~2-2.5 g</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>Genuinely zero - unlike fruit juice sold as no added sugar</t>
+          <t>~60-65% is edible flesh; ~35-50 g sugar but fibre intact</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in black coffee no sugar)</t>
+          <t>Diet/zero-sugar soft drink (330 ml)</t>
         </is>
       </c>
       <c r="B43" s="7" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="C43" s="7" t="n">
-        <v>130</v>
+        <v>2</v>
       </c>
       <c r="D43" s="8">
         <f>AVERAGE(B43:C43)</f>
@@ -5847,22 +5847,26 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="inlineStr"/>
+          <t>0 g</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>Genuinely zero - unlike fruit juice sold as no added sugar</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>Cashew/almond biscuit (1)</t>
+          <t>Whey scoop (in black coffee no sugar)</t>
         </is>
       </c>
       <c r="B44" s="7" t="n">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C44" s="7" t="n">
-        <v>38</v>
+        <v>130</v>
       </c>
       <c r="D44" s="8">
         <f>AVERAGE(B44:C44)</f>
@@ -5870,7 +5874,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>~0.5 g</t>
+          <t>~20-25 g</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr"/>
@@ -5878,14 +5882,14 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (~50g standard)</t>
+          <t>Cashew/almond biscuit (1)</t>
         </is>
       </c>
       <c r="B45" s="7" t="n">
-        <v>245</v>
+        <v>38</v>
       </c>
       <c r="C45" s="7" t="n">
-        <v>250</v>
+        <v>38</v>
       </c>
       <c r="D45" s="8">
         <f>AVERAGE(B45:C45)</f>
@@ -5893,7 +5897,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>~4 g</t>
+          <t>~0.5 g</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr"/>
@@ -5901,14 +5905,14 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (70g king-size)</t>
+          <t>Chocolate bar (~50g standard)</t>
         </is>
       </c>
       <c r="B46" s="7" t="n">
-        <v>335</v>
+        <v>245</v>
       </c>
       <c r="C46" s="7" t="n">
-        <v>335</v>
+        <v>250</v>
       </c>
       <c r="D46" s="8">
         <f>AVERAGE(B46:C46)</f>
@@ -5916,7 +5920,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>~6 g</t>
+          <t>~4 g</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr"/>
@@ -5924,14 +5928,14 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>Pre-workout scoop</t>
+          <t>Chocolate bar (70g king-size)</t>
         </is>
       </c>
       <c r="B47" s="7" t="n">
-        <v>5</v>
+        <v>335</v>
       </c>
       <c r="C47" s="7" t="n">
-        <v>15</v>
+        <v>335</v>
       </c>
       <c r="D47" s="8">
         <f>AVERAGE(B47:C47)</f>
@@ -5939,10 +5943,33 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
+          <t>~6 g</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>Pre-workout scoop</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C48" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D48" s="8">
+        <f>AVERAGE(B48:C48)</f>
+        <v/>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
           <t>0 g</t>
         </is>
       </c>
-      <c r="F47" s="6" t="inlineStr">
+      <c r="F48" s="6" t="inlineStr">
         <is>
           <t>Negligible</t>
         </is>

</xml_diff>

<commit_message>
Log Day 7 breakfast and plan the protein desert
1 dosa with sambar and red chutney, coconut chutney skipped: 350-480 kcal
(mid 415), 8-12 g protein, 12-25 g fat.

Thursday carries no meat on the menu at all - 54 g as served, the lowest of
the week. Sets out three paths for the remaining 1,585 kcal; the grilled sea
bream that would have erased yesterday's deficit creates a 715 kcal one
today.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N42"/>
+  <dimension ref="A1:N43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2701,6 +2701,61 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="4" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Breakfast</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>1 dosa + sambar + red chutney (coconut chutney skipped)</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="n">
+        <v>350</v>
+      </c>
+      <c r="E43" s="7" t="n">
+        <v>480</v>
+      </c>
+      <c r="F43" s="8">
+        <f>AVERAGE(D43:E43)</f>
+        <v/>
+      </c>
+      <c r="G43" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="H43" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="I43" s="10">
+        <f>AVERAGE(G43:H43)</f>
+        <v/>
+      </c>
+      <c r="J43" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="K43" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="L43" s="10">
+        <f>AVERAGE(J43:K43)</f>
+        <v/>
+      </c>
+      <c r="M43" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N43" s="6" t="inlineStr">
+        <is>
+          <t>Coconut chutney skipped again - saves ~100 kcal and ~9 g fat</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:N2"/>
@@ -2715,7 +2770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2819,11 +2874,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$42,Meals!$A$5:$A$42,$A5,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$43,Meals!$A$5:$A$43,$A5,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$42,Meals!$A$5:$A$42,$A5,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$43,Meals!$A$5:$A$43,$A5,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -2831,11 +2886,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$42,Meals!$A$5:$A$42,$A5,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$43,Meals!$A$5:$A$43,$A5,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$42,Meals!$A$5:$A$42,$A5,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$43,Meals!$A$5:$A$43,$A5,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -2843,11 +2898,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$42,Meals!$A$5:$A$42,$A5,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$43,Meals!$A$5:$A$43,$A5,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$42,Meals!$A$5:$A$42,$A5,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$43,Meals!$A$5:$A$43,$A5,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -2855,11 +2910,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$42,$A5,Meals!$M$5:$M$42,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$43,$A5,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$42,$A5,Meals!$M$5:$M$42,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$43,$A5,Meals!$M$5:$M$43,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -2872,11 +2927,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$42,Meals!$A$5:$A$42,$A6,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$43,Meals!$A$5:$A$43,$A6,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$42,Meals!$A$5:$A$42,$A6,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$43,Meals!$A$5:$A$43,$A6,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -2884,11 +2939,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$42,Meals!$A$5:$A$42,$A6,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$43,Meals!$A$5:$A$43,$A6,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$42,Meals!$A$5:$A$42,$A6,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$43,Meals!$A$5:$A$43,$A6,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -2896,11 +2951,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$42,Meals!$A$5:$A$42,$A6,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$43,Meals!$A$5:$A$43,$A6,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$42,Meals!$A$5:$A$42,$A6,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$43,Meals!$A$5:$A$43,$A6,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -2908,11 +2963,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$42,$A6,Meals!$M$5:$M$42,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$43,$A6,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$42,$A6,Meals!$M$5:$M$42,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$43,$A6,Meals!$M$5:$M$43,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -2925,11 +2980,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$42,Meals!$A$5:$A$42,$A7,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$43,Meals!$A$5:$A$43,$A7,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$42,Meals!$A$5:$A$42,$A7,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$43,Meals!$A$5:$A$43,$A7,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -2937,11 +2992,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$42,Meals!$A$5:$A$42,$A7,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$43,Meals!$A$5:$A$43,$A7,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$42,Meals!$A$5:$A$42,$A7,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$43,Meals!$A$5:$A$43,$A7,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -2949,11 +3004,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$42,Meals!$A$5:$A$42,$A7,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$43,Meals!$A$5:$A$43,$A7,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$42,Meals!$A$5:$A$42,$A7,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$43,Meals!$A$5:$A$43,$A7,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -2961,11 +3016,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$42,$A7,Meals!$M$5:$M$42,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$43,$A7,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$42,$A7,Meals!$M$5:$M$42,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$43,$A7,Meals!$M$5:$M$43,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -2978,11 +3033,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$42,Meals!$A$5:$A$42,$A8,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$43,Meals!$A$5:$A$43,$A8,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$42,Meals!$A$5:$A$42,$A8,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$43,Meals!$A$5:$A$43,$A8,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -2990,11 +3045,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$42,Meals!$A$5:$A$42,$A8,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$43,Meals!$A$5:$A$43,$A8,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$42,Meals!$A$5:$A$42,$A8,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$43,Meals!$A$5:$A$43,$A8,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -3002,11 +3057,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$42,Meals!$A$5:$A$42,$A8,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$43,Meals!$A$5:$A$43,$A8,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$42,Meals!$A$5:$A$42,$A8,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$43,Meals!$A$5:$A$43,$A8,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -3014,11 +3069,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$42,$A8,Meals!$M$5:$M$42,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$43,$A8,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$42,$A8,Meals!$M$5:$M$42,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$43,$A8,Meals!$M$5:$M$43,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -3031,11 +3086,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$42,Meals!$A$5:$A$42,$A9,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$43,Meals!$A$5:$A$43,$A9,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$42,Meals!$A$5:$A$42,$A9,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$43,Meals!$A$5:$A$43,$A9,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -3043,11 +3098,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$42,Meals!$A$5:$A$42,$A9,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$43,Meals!$A$5:$A$43,$A9,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$42,Meals!$A$5:$A$42,$A9,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$43,Meals!$A$5:$A$43,$A9,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -3055,11 +3110,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$42,Meals!$A$5:$A$42,$A9,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$43,Meals!$A$5:$A$43,$A9,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$42,Meals!$A$5:$A$42,$A9,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$43,Meals!$A$5:$A$43,$A9,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -3067,11 +3122,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$42,$A9,Meals!$M$5:$M$42,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$43,$A9,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$42,$A9,Meals!$M$5:$M$42,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$43,$A9,Meals!$M$5:$M$43,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -3084,11 +3139,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$42,Meals!$A$5:$A$42,$A10,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$43,Meals!$A$5:$A$43,$A10,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$42,Meals!$A$5:$A$42,$A10,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$43,Meals!$A$5:$A$43,$A10,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -3096,11 +3151,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$42,Meals!$A$5:$A$42,$A10,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$43,Meals!$A$5:$A$43,$A10,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$42,Meals!$A$5:$A$42,$A10,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$43,Meals!$A$5:$A$43,$A10,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -3108,11 +3163,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$42,Meals!$A$5:$A$42,$A10,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$43,Meals!$A$5:$A$43,$A10,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$42,Meals!$A$5:$A$42,$A10,Meals!$M$5:$M$42,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$43,Meals!$A$5:$A$43,$A10,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -3120,15 +3175,68 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$42,$A10,Meals!$M$5:$M$42,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$43,$A10,Meals!$M$5:$M$43,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$42,$A10,Meals!$M$5:$M$42,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$43,$A10,Meals!$M$5:$M$43,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
         <f>D10-Targets!$B$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="18" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B11" s="8">
+        <f>SUMIFS(Meals!$D$5:$D$43,Meals!$A$5:$A$43,$A11,Meals!$M$5:$M$43,"logged")</f>
+        <v/>
+      </c>
+      <c r="C11" s="8">
+        <f>SUMIFS(Meals!$E$5:$E$43,Meals!$A$5:$A$43,$A11,Meals!$M$5:$M$43,"logged")</f>
+        <v/>
+      </c>
+      <c r="D11" s="8">
+        <f>AVERAGE(B11:C11)</f>
+        <v/>
+      </c>
+      <c r="E11" s="10">
+        <f>SUMIFS(Meals!$G$5:$G$43,Meals!$A$5:$A$43,$A11,Meals!$M$5:$M$43,"logged")</f>
+        <v/>
+      </c>
+      <c r="F11" s="10">
+        <f>SUMIFS(Meals!$H$5:$H$43,Meals!$A$5:$A$43,$A11,Meals!$M$5:$M$43,"logged")</f>
+        <v/>
+      </c>
+      <c r="G11" s="10">
+        <f>AVERAGE(E11:F11)</f>
+        <v/>
+      </c>
+      <c r="H11" s="10">
+        <f>SUMIFS(Meals!$J$5:$J$43,Meals!$A$5:$A$43,$A11,Meals!$M$5:$M$43,"logged")</f>
+        <v/>
+      </c>
+      <c r="I11" s="10">
+        <f>SUMIFS(Meals!$K$5:$K$43,Meals!$A$5:$A$43,$A11,Meals!$M$5:$M$43,"logged")</f>
+        <v/>
+      </c>
+      <c r="J11" s="10">
+        <f>AVERAGE(H11:I11)</f>
+        <v/>
+      </c>
+      <c r="K11" s="18">
+        <f>COUNTIFS(Meals!$A$5:$A$43,$A11,Meals!$M$5:$M$43,"logged")</f>
+        <v/>
+      </c>
+      <c r="L11" s="18">
+        <f>COUNTIFS(Meals!$A$5:$A$43,$A11,Meals!$M$5:$M$43,"pending")</f>
+        <v/>
+      </c>
+      <c r="M11" s="19">
+        <f>D11-Targets!$B$16</f>
         <v/>
       </c>
     </row>
@@ -4037,7 +4145,7 @@
         </is>
       </c>
       <c r="B5" s="18">
-        <f>COUNT(Daily!$A$5:$A$10)</f>
+        <f>COUNT(Daily!$A$5:$A$11)</f>
         <v/>
       </c>
     </row>
@@ -4048,7 +4156,7 @@
         </is>
       </c>
       <c r="B6" s="8">
-        <f>IFERROR(AVERAGE(Daily!$D$5:$D$10),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$D$5:$D$11),0)</f>
         <v/>
       </c>
     </row>
@@ -4059,7 +4167,7 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>IFERROR(AVERAGE(Daily!$G$5:$G$10),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$G$5:$G$11),0)</f>
         <v/>
       </c>
     </row>
@@ -4070,7 +4178,7 @@
         </is>
       </c>
       <c r="B8" s="10">
-        <f>IFERROR(AVERAGE(Daily!$J$5:$J$10),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$J$5:$J$11),0)</f>
         <v/>
       </c>
     </row>
@@ -4114,7 +4222,7 @@
         </is>
       </c>
       <c r="B12" s="18">
-        <f>COUNTIFS(Daily!$G$5:$G$10,"&gt;="&amp;Targets!$B$20)</f>
+        <f>COUNTIFS(Daily!$G$5:$G$11,"&gt;="&amp;Targets!$B$20)</f>
         <v/>
       </c>
     </row>
@@ -4125,7 +4233,7 @@
         </is>
       </c>
       <c r="B13" s="18">
-        <f>SUM(Daily!$L$5:$L$10)</f>
+        <f>SUM(Daily!$L$5:$L$11)</f>
         <v/>
       </c>
     </row>
@@ -4176,19 +4284,19 @@
         <v>46271</v>
       </c>
       <c r="C17" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$10,"&gt;="&amp;$A17,Daily!$A$5:$A$10,"&lt;="&amp;$B17)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$11,"&gt;="&amp;$A17,Daily!$A$5:$A$11,"&lt;="&amp;$B17)</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$10,Daily!$A$5:$A$10,"&gt;="&amp;$A17,Daily!$A$5:$A$10,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$11,Daily!$A$5:$A$11,"&gt;="&amp;$A17,Daily!$A$5:$A$11,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$10,Daily!$A$5:$A$10,"&gt;="&amp;$A17,Daily!$A$5:$A$10,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$11,Daily!$A$5:$A$11,"&gt;="&amp;$A17,Daily!$A$5:$A$11,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$10,Daily!$A$5:$A$10,"&gt;="&amp;$A17,Daily!$A$5:$A$10,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$11,Daily!$A$5:$A$11,"&gt;="&amp;$A17,Daily!$A$5:$A$11,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
     </row>
@@ -4200,19 +4308,19 @@
         <v>46278</v>
       </c>
       <c r="C18" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$10,"&gt;="&amp;$A18,Daily!$A$5:$A$10,"&lt;="&amp;$B18)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$11,"&gt;="&amp;$A18,Daily!$A$5:$A$11,"&lt;="&amp;$B18)</f>
         <v/>
       </c>
       <c r="D18" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$10,Daily!$A$5:$A$10,"&gt;="&amp;$A18,Daily!$A$5:$A$10,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$11,Daily!$A$5:$A$11,"&gt;="&amp;$A18,Daily!$A$5:$A$11,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="E18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$10,Daily!$A$5:$A$10,"&gt;="&amp;$A18,Daily!$A$5:$A$10,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$11,Daily!$A$5:$A$11,"&gt;="&amp;$A18,Daily!$A$5:$A$11,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="F18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$10,Daily!$A$5:$A$10,"&gt;="&amp;$A18,Daily!$A$5:$A$10,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$11,Daily!$A$5:$A$11,"&gt;="&amp;$A18,Daily!$A$5:$A$11,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
     </row>
@@ -4263,19 +4371,19 @@
         <v>46295</v>
       </c>
       <c r="C22" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$10,"&gt;="&amp;$A22,Daily!$A$5:$A$10,"&lt;="&amp;$B22)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$11,"&gt;="&amp;$A22,Daily!$A$5:$A$11,"&lt;="&amp;$B22)</f>
         <v/>
       </c>
       <c r="D22" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$10,Daily!$A$5:$A$10,"&gt;="&amp;$A22,Daily!$A$5:$A$10,"&lt;="&amp;$B22),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$11,Daily!$A$5:$A$11,"&gt;="&amp;$A22,Daily!$A$5:$A$11,"&lt;="&amp;$B22),0)</f>
         <v/>
       </c>
       <c r="E22" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$10,Daily!$A$5:$A$10,"&gt;="&amp;$A22,Daily!$A$5:$A$10,"&lt;="&amp;$B22),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$11,Daily!$A$5:$A$11,"&gt;="&amp;$A22,Daily!$A$5:$A$11,"&lt;="&amp;$B22),0)</f>
         <v/>
       </c>
       <c r="F22" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$10,Daily!$A$5:$A$10,"&gt;="&amp;$A22,Daily!$A$5:$A$10,"&lt;="&amp;$B22),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$11,Daily!$A$5:$A$11,"&gt;="&amp;$A22,Daily!$A$5:$A$11,"&lt;="&amp;$B22),0)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Log Thursday lunch: halved rice with matthi taken out of its gravy
740-1,130 kcal (mid 935), 39-57 g protein, 27-52 g fat. Lifting the fish
out and leaving the oily gravy keeps ~22 g of protein while dropping about
100 kcal and 10 g of fat - 5.1 g of protein per 100 kcal, the best mess
lunch in the log.

Day 7 stands at 1,350 kcal and 58 g protein, already above the 54 g the
whole Thursday menu provides as served.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N43"/>
+  <dimension ref="A1:N44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2753,6 +2753,61 @@
       <c r="N43" s="6" t="inlineStr">
         <is>
           <t>Coconut chutney skipped again - saves ~100 kcal and ~9 g fat</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>Mess meals plate (rice halved) + matthi taken without the gravy + chicken piece + coconut chammanthi, thoran, veg curries</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="n">
+        <v>740</v>
+      </c>
+      <c r="E44" s="7" t="n">
+        <v>1130</v>
+      </c>
+      <c r="F44" s="8">
+        <f>AVERAGE(D44:E44)</f>
+        <v/>
+      </c>
+      <c r="G44" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="H44" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="I44" s="10">
+        <f>AVERAGE(G44:H44)</f>
+        <v/>
+      </c>
+      <c r="J44" s="9" t="n">
+        <v>27</v>
+      </c>
+      <c r="K44" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="L44" s="10">
+        <f>AVERAGE(J44:K44)</f>
+        <v/>
+      </c>
+      <c r="M44" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N44" s="6" t="inlineStr">
+        <is>
+          <t>Fish lifted out of the curry and the oily gravy left behind</t>
         </is>
       </c>
     </row>
@@ -2874,11 +2929,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$43,Meals!$A$5:$A$43,$A5,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$44,Meals!$A$5:$A$44,$A5,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$43,Meals!$A$5:$A$43,$A5,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$44,Meals!$A$5:$A$44,$A5,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -2886,11 +2941,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$43,Meals!$A$5:$A$43,$A5,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$44,Meals!$A$5:$A$44,$A5,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$43,Meals!$A$5:$A$43,$A5,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$44,Meals!$A$5:$A$44,$A5,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -2898,11 +2953,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$43,Meals!$A$5:$A$43,$A5,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$44,Meals!$A$5:$A$44,$A5,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$43,Meals!$A$5:$A$43,$A5,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$44,Meals!$A$5:$A$44,$A5,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -2910,11 +2965,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$43,$A5,Meals!$M$5:$M$43,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$44,$A5,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$43,$A5,Meals!$M$5:$M$43,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$44,$A5,Meals!$M$5:$M$44,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -2927,11 +2982,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$43,Meals!$A$5:$A$43,$A6,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$44,Meals!$A$5:$A$44,$A6,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$43,Meals!$A$5:$A$43,$A6,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$44,Meals!$A$5:$A$44,$A6,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -2939,11 +2994,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$43,Meals!$A$5:$A$43,$A6,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$44,Meals!$A$5:$A$44,$A6,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$43,Meals!$A$5:$A$43,$A6,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$44,Meals!$A$5:$A$44,$A6,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -2951,11 +3006,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$43,Meals!$A$5:$A$43,$A6,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$44,Meals!$A$5:$A$44,$A6,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$43,Meals!$A$5:$A$43,$A6,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$44,Meals!$A$5:$A$44,$A6,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -2963,11 +3018,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$43,$A6,Meals!$M$5:$M$43,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$44,$A6,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$43,$A6,Meals!$M$5:$M$43,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$44,$A6,Meals!$M$5:$M$44,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -2980,11 +3035,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$43,Meals!$A$5:$A$43,$A7,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$44,Meals!$A$5:$A$44,$A7,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$43,Meals!$A$5:$A$43,$A7,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$44,Meals!$A$5:$A$44,$A7,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -2992,11 +3047,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$43,Meals!$A$5:$A$43,$A7,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$44,Meals!$A$5:$A$44,$A7,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$43,Meals!$A$5:$A$43,$A7,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$44,Meals!$A$5:$A$44,$A7,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -3004,11 +3059,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$43,Meals!$A$5:$A$43,$A7,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$44,Meals!$A$5:$A$44,$A7,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$43,Meals!$A$5:$A$43,$A7,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$44,Meals!$A$5:$A$44,$A7,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -3016,11 +3071,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$43,$A7,Meals!$M$5:$M$43,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$44,$A7,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$43,$A7,Meals!$M$5:$M$43,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$44,$A7,Meals!$M$5:$M$44,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -3033,11 +3088,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$43,Meals!$A$5:$A$43,$A8,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$44,Meals!$A$5:$A$44,$A8,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$43,Meals!$A$5:$A$43,$A8,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$44,Meals!$A$5:$A$44,$A8,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -3045,11 +3100,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$43,Meals!$A$5:$A$43,$A8,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$44,Meals!$A$5:$A$44,$A8,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$43,Meals!$A$5:$A$43,$A8,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$44,Meals!$A$5:$A$44,$A8,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -3057,11 +3112,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$43,Meals!$A$5:$A$43,$A8,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$44,Meals!$A$5:$A$44,$A8,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$43,Meals!$A$5:$A$43,$A8,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$44,Meals!$A$5:$A$44,$A8,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -3069,11 +3124,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$43,$A8,Meals!$M$5:$M$43,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$44,$A8,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$43,$A8,Meals!$M$5:$M$43,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$44,$A8,Meals!$M$5:$M$44,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -3086,11 +3141,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$43,Meals!$A$5:$A$43,$A9,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$44,Meals!$A$5:$A$44,$A9,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$43,Meals!$A$5:$A$43,$A9,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$44,Meals!$A$5:$A$44,$A9,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -3098,11 +3153,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$43,Meals!$A$5:$A$43,$A9,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$44,Meals!$A$5:$A$44,$A9,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$43,Meals!$A$5:$A$43,$A9,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$44,Meals!$A$5:$A$44,$A9,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -3110,11 +3165,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$43,Meals!$A$5:$A$43,$A9,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$44,Meals!$A$5:$A$44,$A9,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$43,Meals!$A$5:$A$43,$A9,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$44,Meals!$A$5:$A$44,$A9,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -3122,11 +3177,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$43,$A9,Meals!$M$5:$M$43,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$44,$A9,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$43,$A9,Meals!$M$5:$M$43,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$44,$A9,Meals!$M$5:$M$44,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -3139,11 +3194,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$43,Meals!$A$5:$A$43,$A10,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$44,Meals!$A$5:$A$44,$A10,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$43,Meals!$A$5:$A$43,$A10,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$44,Meals!$A$5:$A$44,$A10,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -3151,11 +3206,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$43,Meals!$A$5:$A$43,$A10,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$44,Meals!$A$5:$A$44,$A10,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$43,Meals!$A$5:$A$43,$A10,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$44,Meals!$A$5:$A$44,$A10,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -3163,11 +3218,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$43,Meals!$A$5:$A$43,$A10,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$44,Meals!$A$5:$A$44,$A10,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$43,Meals!$A$5:$A$43,$A10,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$44,Meals!$A$5:$A$44,$A10,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -3175,11 +3230,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$43,$A10,Meals!$M$5:$M$43,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$44,$A10,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$43,$A10,Meals!$M$5:$M$43,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$44,$A10,Meals!$M$5:$M$44,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -3192,11 +3247,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$43,Meals!$A$5:$A$43,$A11,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$44,Meals!$A$5:$A$44,$A11,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$43,Meals!$A$5:$A$43,$A11,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$44,Meals!$A$5:$A$44,$A11,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -3204,11 +3259,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$43,Meals!$A$5:$A$43,$A11,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$44,Meals!$A$5:$A$44,$A11,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$43,Meals!$A$5:$A$43,$A11,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$44,Meals!$A$5:$A$44,$A11,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -3216,11 +3271,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$43,Meals!$A$5:$A$43,$A11,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$44,Meals!$A$5:$A$44,$A11,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$43,Meals!$A$5:$A$43,$A11,Meals!$M$5:$M$43,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$44,Meals!$A$5:$A$44,$A11,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -3228,11 +3283,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$43,$A11,Meals!$M$5:$M$43,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$44,$A11,Meals!$M$5:$M$44,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$43,$A11,Meals!$M$5:$M$43,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$44,$A11,Meals!$M$5:$M$44,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -4886,7 +4941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5389,14 +5444,14 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Grilled chicken breast (100 g skinless)</t>
+          <t>Matthi / sardine (2-3 fish taken without gravy)</t>
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>180</v>
+        <v>230</v>
       </c>
       <c r="D22" s="8">
         <f>AVERAGE(B22:C22)</f>
@@ -5404,26 +5459,26 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>~30-32 g</t>
+          <t>~18-26 g</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>Best protein-per-calorie item in this list</t>
+          <t>Oily fish - denser than white fish but excellent protein. Leaving the gravy saves ~100 kcal and ~10 g fat</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Grilled chicken breast (150 g skinless)</t>
+          <t>Grilled chicken breast (100 g skinless)</t>
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>240</v>
+        <v>160</v>
       </c>
       <c r="C23" s="7" t="n">
-        <v>270</v>
+        <v>180</v>
       </c>
       <c r="D23" s="8">
         <f>AVERAGE(B23:C23)</f>
@@ -5431,22 +5486,26 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>~45-48 g</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="inlineStr"/>
+          <t>~30-32 g</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>Best protein-per-calorie item in this list</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Honest Bowl - Grilled Chicken and Rice Bowl</t>
+          <t>Grilled chicken breast (150 g skinless)</t>
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>550</v>
+        <v>240</v>
       </c>
       <c r="C24" s="7" t="n">
-        <v>710</v>
+        <v>270</v>
       </c>
       <c r="D24" s="8">
         <f>AVERAGE(B24:C24)</f>
@@ -5454,26 +5513,22 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>42-48 g</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>Menu states 42 g protein; chicken + jasmine rice + sweet potato. Sauce served separately</t>
-        </is>
-      </c>
+          <t>~45-48 g</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Brown/mushroom sauce (side pot)</t>
+          <t>Honest Bowl - Grilled Chicken and Rice Bowl</t>
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>50</v>
+        <v>550</v>
       </c>
       <c r="C25" s="7" t="n">
-        <v>120</v>
+        <v>710</v>
       </c>
       <c r="D25" s="8">
         <f>AVERAGE(B25:C25)</f>
@@ -5481,26 +5536,26 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>~1-2 g</t>
+          <t>42-48 g</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>Often cream or butter based - the variable in a bowl like this</t>
+          <t>Menu states 42 g protein; chicken + jasmine rice + sweet potato. Sauce served separately</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Honest Bowl - Tofu Delight Bowl</t>
+          <t>Brown/mushroom sauce (side pot)</t>
         </is>
       </c>
       <c r="B26" s="7" t="n">
-        <v>420</v>
+        <v>50</v>
       </c>
       <c r="C26" s="7" t="n">
-        <v>560</v>
+        <v>120</v>
       </c>
       <c r="D26" s="8">
         <f>AVERAGE(B26:C26)</f>
@@ -5508,26 +5563,26 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>~20 g</t>
+          <t>~1-2 g</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>Menu states 20 g; jasmine rice + cajun tofu + grilled eggplant. Half the protein of the chicken bowl at the same price</t>
+          <t>Often cream or butter based - the variable in a bowl like this</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Chicken curry (1 takeaway container)</t>
+          <t>Honest Bowl - Tofu Delight Bowl</t>
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>280</v>
+        <v>420</v>
       </c>
       <c r="C27" s="7" t="n">
-        <v>420</v>
+        <v>560</v>
       </c>
       <c r="D27" s="8">
         <f>AVERAGE(B27:C27)</f>
@@ -5535,26 +5590,26 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>~20-28 g</t>
+          <t>~20 g</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>Kerala style; oil and coconut carry most of the calories</t>
+          <t>Menu states 20 g; jasmine rice + cajun tofu + grilled eggplant. Half the protein of the chicken bowl at the same price</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Grilled chicken quarter (skin on)</t>
+          <t>Chicken curry (1 takeaway container)</t>
         </is>
       </c>
       <c r="B28" s="7" t="n">
-        <v>250</v>
+        <v>280</v>
       </c>
       <c r="C28" s="7" t="n">
-        <v>320</v>
+        <v>420</v>
       </c>
       <c r="D28" s="8">
         <f>AVERAGE(B28:C28)</f>
@@ -5562,26 +5617,26 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>~28-33 g</t>
+          <t>~20-28 g</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>Skin adds ~12-15 g fat over breast</t>
+          <t>Kerala style; oil and coconut carry most of the calories</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Garlic sauce / toum (1 tbsp)</t>
+          <t>Grilled chicken quarter (skin on)</t>
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>90</v>
+        <v>250</v>
       </c>
       <c r="C29" s="7" t="n">
-        <v>110</v>
+        <v>320</v>
       </c>
       <c r="D29" s="8">
         <f>AVERAGE(B29:C29)</f>
@@ -5589,26 +5644,26 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>0 g</t>
+          <t>~28-33 g</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>Essentially emulsified oil - the hidden cost at a grill</t>
+          <t>Skin adds ~12-15 g fat over breast</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Khubz / pita (1 large)</t>
+          <t>Garlic sauce / toum (1 tbsp)</t>
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>250</v>
+        <v>90</v>
       </c>
       <c r="C30" s="7" t="n">
-        <v>300</v>
+        <v>110</v>
       </c>
       <c r="D30" s="8">
         <f>AVERAGE(B30:C30)</f>
@@ -5616,22 +5671,26 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>~8-9 g</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="inlineStr"/>
+          <t>0 g</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>Essentially emulsified oil - the hidden cost at a grill</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Barik/basmati rice (half container cooked)</t>
+          <t>Khubz / pita (1 large)</t>
         </is>
       </c>
       <c r="B31" s="7" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="C31" s="7" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="D31" s="8">
         <f>AVERAGE(B31:C31)</f>
@@ -5639,7 +5698,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>~4-5 g</t>
+          <t>~8-9 g</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr"/>
@@ -5647,14 +5706,14 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Fresh pineapple juice (350-450 ml)</t>
+          <t>Barik/basmati rice (half container cooked)</t>
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>175</v>
+        <v>200</v>
       </c>
       <c r="C32" s="7" t="n">
-        <v>240</v>
+        <v>280</v>
       </c>
       <c r="D32" s="8">
         <f>AVERAGE(B32:C32)</f>
@@ -5662,26 +5721,22 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>~1-2 g</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="inlineStr">
-        <is>
-          <t>No added sugar but ~35-45 g natural sugar; no fibre; almost no protein</t>
-        </is>
-      </c>
+          <t>~4-5 g</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Fresh orange juice (350-450 ml)</t>
+          <t>Fresh pineapple juice (350-450 ml)</t>
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>155</v>
+        <v>175</v>
       </c>
       <c r="C33" s="7" t="n">
-        <v>205</v>
+        <v>240</v>
       </c>
       <c r="D33" s="8">
         <f>AVERAGE(B33:C33)</f>
@@ -5689,26 +5744,26 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>~2-3 g</t>
+          <t>~1-2 g</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>No added sugar but ~32-40 g natural sugar; no fibre</t>
+          <t>No added sugar but ~35-45 g natural sugar; no fibre; almost no protein</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in water)</t>
+          <t>Fresh orange juice (350-450 ml)</t>
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>100</v>
+        <v>155</v>
       </c>
       <c r="C34" s="7" t="n">
-        <v>120</v>
+        <v>205</v>
       </c>
       <c r="D34" s="8">
         <f>AVERAGE(B34:C34)</f>
@@ -5716,22 +5771,26 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="inlineStr"/>
+          <t>~2-3 g</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>No added sugar but ~32-40 g natural sugar; no fibre</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Greek yogurt (200 g plain low-fat)</t>
+          <t>Whey scoop (in water)</t>
         </is>
       </c>
       <c r="B35" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C35" s="7" t="n">
         <v>120</v>
-      </c>
-      <c r="C35" s="7" t="n">
-        <v>140</v>
       </c>
       <c r="D35" s="8">
         <f>AVERAGE(B35:C35)</f>
@@ -5739,26 +5798,22 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>~18-20 g</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="inlineStr">
-        <is>
-          <t>Casein - digests slowly; good overnight</t>
-        </is>
-      </c>
+          <t>~20-25 g</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Boiled egg (1 large)</t>
+          <t>Greek yogurt (200 g plain low-fat)</t>
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>70</v>
+        <v>120</v>
       </c>
       <c r="C36" s="7" t="n">
-        <v>78</v>
+        <v>140</v>
       </c>
       <c r="D36" s="8">
         <f>AVERAGE(B36:C36)</f>
@@ -5766,19 +5821,19 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>~6-6.5 g</t>
+          <t>~18-20 g</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>~5 g fat each</t>
+          <t>Casein - digests slowly; good overnight</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Egg fried dry with no oil (1)</t>
+          <t>Boiled egg (1 large)</t>
         </is>
       </c>
       <c r="B37" s="7" t="n">
@@ -5798,21 +5853,21 @@
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>Same as boiled - dry-frying saves the ~20-25 kcal per egg that pan oil adds</t>
+          <t>~5 g fat each</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>Paneer (50 g full-fat)</t>
+          <t>Egg fried dry with no oil (1)</t>
         </is>
       </c>
       <c r="B38" s="7" t="n">
-        <v>130</v>
+        <v>70</v>
       </c>
       <c r="C38" s="7" t="n">
-        <v>150</v>
+        <v>78</v>
       </c>
       <c r="D38" s="8">
         <f>AVERAGE(B38:C38)</f>
@@ -5820,26 +5875,26 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>~8-9 g</t>
+          <t>~6-6.5 g</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>Fat-dense for the protein it gives</t>
+          <t>Same as boiled - dry-frying saves the ~20-25 kcal per egg that pan oil adds</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>Cucumber (1 medium)</t>
+          <t>Paneer (50 g full-fat)</t>
         </is>
       </c>
       <c r="B39" s="7" t="n">
-        <v>25</v>
+        <v>130</v>
       </c>
       <c r="C39" s="7" t="n">
-        <v>30</v>
+        <v>150</v>
       </c>
       <c r="D39" s="8">
         <f>AVERAGE(B39:C39)</f>
@@ -5847,26 +5902,26 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>~1.5 g</t>
+          <t>~8-9 g</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
         <is>
-          <t>Volume with almost no calories</t>
+          <t>Fat-dense for the protein it gives</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>Sweet melon / cantaloupe (1 wedge ~100-150 g)</t>
+          <t>Cucumber (1 medium)</t>
         </is>
       </c>
       <c r="B40" s="7" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="C40" s="7" t="n">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="D40" s="8">
         <f>AVERAGE(B40:C40)</f>
@@ -5874,26 +5929,26 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>~0.5-1 g</t>
+          <t>~1.5 g</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>Whole fruit - fibre and water intact; ~1/4 the calories of the same fruit juiced</t>
+          <t>Volume with almost no calories</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>Grapes (~100 g / 15-20 grapes)</t>
+          <t>Sweet melon / cantaloupe (1 wedge ~100-150 g)</t>
         </is>
       </c>
       <c r="B41" s="7" t="n">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="C41" s="7" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="D41" s="8">
         <f>AVERAGE(B41:C41)</f>
@@ -5901,26 +5956,26 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>~0.6 g</t>
+          <t>~0.5-1 g</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
-          <t>Twice the calorie density of melon; easy to eat a large handful without noticing</t>
+          <t>Whole fruit - fibre and water intact; ~1/4 the calories of the same fruit juiced</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Mango misiri (1 whole ~450-600 g)</t>
+          <t>Grapes (~100 g / 15-20 grapes)</t>
         </is>
       </c>
       <c r="B42" s="7" t="n">
-        <v>170</v>
+        <v>60</v>
       </c>
       <c r="C42" s="7" t="n">
-        <v>230</v>
+        <v>75</v>
       </c>
       <c r="D42" s="8">
         <f>AVERAGE(B42:C42)</f>
@@ -5928,26 +5983,26 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>~2-2.5 g</t>
+          <t>~0.6 g</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>~60-65% is edible flesh; ~35-50 g sugar but fibre intact</t>
+          <t>Twice the calorie density of melon; easy to eat a large handful without noticing</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>Diet/zero-sugar soft drink (330 ml)</t>
+          <t>Mango misiri (1 whole ~450-600 g)</t>
         </is>
       </c>
       <c r="B43" s="7" t="n">
-        <v>0</v>
+        <v>170</v>
       </c>
       <c r="C43" s="7" t="n">
-        <v>2</v>
+        <v>230</v>
       </c>
       <c r="D43" s="8">
         <f>AVERAGE(B43:C43)</f>
@@ -5955,26 +6010,26 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>0 g</t>
+          <t>~2-2.5 g</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t>Genuinely zero - unlike fruit juice sold as no added sugar</t>
+          <t>~60-65% is edible flesh; ~35-50 g sugar but fibre intact</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in black coffee no sugar)</t>
+          <t>Diet/zero-sugar soft drink (330 ml)</t>
         </is>
       </c>
       <c r="B44" s="7" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="C44" s="7" t="n">
-        <v>130</v>
+        <v>2</v>
       </c>
       <c r="D44" s="8">
         <f>AVERAGE(B44:C44)</f>
@@ -5982,22 +6037,26 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F44" s="6" t="inlineStr"/>
+          <t>0 g</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>Genuinely zero - unlike fruit juice sold as no added sugar</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Cashew/almond biscuit (1)</t>
+          <t>Whey scoop (in black coffee no sugar)</t>
         </is>
       </c>
       <c r="B45" s="7" t="n">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C45" s="7" t="n">
-        <v>38</v>
+        <v>130</v>
       </c>
       <c r="D45" s="8">
         <f>AVERAGE(B45:C45)</f>
@@ -6005,7 +6064,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>~0.5 g</t>
+          <t>~20-25 g</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr"/>
@@ -6013,14 +6072,14 @@
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (~50g standard)</t>
+          <t>Cashew/almond biscuit (1)</t>
         </is>
       </c>
       <c r="B46" s="7" t="n">
-        <v>245</v>
+        <v>38</v>
       </c>
       <c r="C46" s="7" t="n">
-        <v>250</v>
+        <v>38</v>
       </c>
       <c r="D46" s="8">
         <f>AVERAGE(B46:C46)</f>
@@ -6028,7 +6087,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>~4 g</t>
+          <t>~0.5 g</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr"/>
@@ -6036,14 +6095,14 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (70g king-size)</t>
+          <t>Chocolate bar (~50g standard)</t>
         </is>
       </c>
       <c r="B47" s="7" t="n">
-        <v>335</v>
+        <v>245</v>
       </c>
       <c r="C47" s="7" t="n">
-        <v>335</v>
+        <v>250</v>
       </c>
       <c r="D47" s="8">
         <f>AVERAGE(B47:C47)</f>
@@ -6051,7 +6110,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>~6 g</t>
+          <t>~4 g</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr"/>
@@ -6059,14 +6118,14 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>Pre-workout scoop</t>
+          <t>Chocolate bar (70g king-size)</t>
         </is>
       </c>
       <c r="B48" s="7" t="n">
-        <v>5</v>
+        <v>335</v>
       </c>
       <c r="C48" s="7" t="n">
-        <v>15</v>
+        <v>335</v>
       </c>
       <c r="D48" s="8">
         <f>AVERAGE(B48:C48)</f>
@@ -6074,10 +6133,33 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
+          <t>~6 g</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>Pre-workout scoop</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C49" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D49" s="8">
+        <f>AVERAGE(B49:C49)</f>
+        <v/>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
           <t>0 g</t>
         </is>
       </c>
-      <c r="F48" s="6" t="inlineStr">
+      <c r="F49" s="6" t="inlineStr">
         <is>
           <t>Negligible</t>
         </is>

</xml_diff>

<commit_message>
Name the two fried chicken pieces in Thursday lunch
They were already counted, but the row said "chicken piece" singular.
Nudged the range up 20 kcal and 1 g fat for the frying: 760-1,150 kcal.
Day 7 moves to 1,370 kcal and 59 g fat; protein unchanged at 58 g.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -2767,14 +2767,14 @@
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>Mess meals plate (rice halved) + matthi taken without the gravy + chicken piece + coconut chammanthi, thoran, veg curries</t>
+          <t>Mess meals plate (rice halved) + matthi taken without the gravy + 2 small fried chicken pieces + coconut chammanthi, thoran, veg curries</t>
         </is>
       </c>
       <c r="D44" s="7" t="n">
-        <v>740</v>
+        <v>760</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>1130</v>
+        <v>1150</v>
       </c>
       <c r="F44" s="8">
         <f>AVERAGE(D44:E44)</f>
@@ -2791,10 +2791,10 @@
         <v/>
       </c>
       <c r="J44" s="9" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="K44" s="9" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="L44" s="10">
         <f>AVERAGE(J44:K44)</f>
@@ -2807,7 +2807,7 @@
       </c>
       <c r="N44" s="6" t="inlineStr">
         <is>
-          <t>Fish lifted out of the curry and the oily gravy left behind</t>
+          <t>Fish lifted out of the curry and the oily gravy left behind; 2 fried chicken pieces on the plate</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log first whey scoop of Day 7
100-130 kcal, 20-25 g protein. Day 7 stands at 1,485 kcal and 80.5 g of
protein with 515 kcal and 49.5 g still to place.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N44"/>
+  <dimension ref="A1:N45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2808,6 +2808,61 @@
       <c r="N44" s="6" t="inlineStr">
         <is>
           <t>Fish lifted out of the curry and the oily gravy left behind; 2 fried chicken pieces on the plate</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>Black coffee + 1 whey scoop</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E45" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="F45" s="8">
+        <f>AVERAGE(D45:E45)</f>
+        <v/>
+      </c>
+      <c r="G45" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="H45" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="I45" s="10">
+        <f>AVERAGE(G45:H45)</f>
+        <v/>
+      </c>
+      <c r="J45" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K45" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="L45" s="10">
+        <f>AVERAGE(J45:K45)</f>
+        <v/>
+      </c>
+      <c r="M45" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N45" s="6" t="inlineStr">
+        <is>
+          <t>Scoop 1</t>
         </is>
       </c>
     </row>
@@ -2929,11 +2984,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$44,Meals!$A$5:$A$44,$A5,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$45,Meals!$A$5:$A$45,$A5,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$44,Meals!$A$5:$A$44,$A5,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$45,Meals!$A$5:$A$45,$A5,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -2941,11 +2996,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$44,Meals!$A$5:$A$44,$A5,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$45,Meals!$A$5:$A$45,$A5,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$44,Meals!$A$5:$A$44,$A5,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$45,Meals!$A$5:$A$45,$A5,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -2953,11 +3008,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$44,Meals!$A$5:$A$44,$A5,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$45,Meals!$A$5:$A$45,$A5,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$44,Meals!$A$5:$A$44,$A5,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$45,Meals!$A$5:$A$45,$A5,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -2965,11 +3020,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$44,$A5,Meals!$M$5:$M$44,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$45,$A5,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$44,$A5,Meals!$M$5:$M$44,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$45,$A5,Meals!$M$5:$M$45,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -2982,11 +3037,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$44,Meals!$A$5:$A$44,$A6,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$45,Meals!$A$5:$A$45,$A6,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$44,Meals!$A$5:$A$44,$A6,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$45,Meals!$A$5:$A$45,$A6,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -2994,11 +3049,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$44,Meals!$A$5:$A$44,$A6,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$45,Meals!$A$5:$A$45,$A6,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$44,Meals!$A$5:$A$44,$A6,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$45,Meals!$A$5:$A$45,$A6,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -3006,11 +3061,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$44,Meals!$A$5:$A$44,$A6,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$45,Meals!$A$5:$A$45,$A6,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$44,Meals!$A$5:$A$44,$A6,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$45,Meals!$A$5:$A$45,$A6,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -3018,11 +3073,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$44,$A6,Meals!$M$5:$M$44,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$45,$A6,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$44,$A6,Meals!$M$5:$M$44,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$45,$A6,Meals!$M$5:$M$45,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -3035,11 +3090,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$44,Meals!$A$5:$A$44,$A7,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$45,Meals!$A$5:$A$45,$A7,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$44,Meals!$A$5:$A$44,$A7,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$45,Meals!$A$5:$A$45,$A7,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -3047,11 +3102,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$44,Meals!$A$5:$A$44,$A7,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$45,Meals!$A$5:$A$45,$A7,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$44,Meals!$A$5:$A$44,$A7,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$45,Meals!$A$5:$A$45,$A7,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -3059,11 +3114,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$44,Meals!$A$5:$A$44,$A7,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$45,Meals!$A$5:$A$45,$A7,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$44,Meals!$A$5:$A$44,$A7,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$45,Meals!$A$5:$A$45,$A7,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -3071,11 +3126,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$44,$A7,Meals!$M$5:$M$44,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$45,$A7,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$44,$A7,Meals!$M$5:$M$44,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$45,$A7,Meals!$M$5:$M$45,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -3088,11 +3143,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$44,Meals!$A$5:$A$44,$A8,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$45,Meals!$A$5:$A$45,$A8,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$44,Meals!$A$5:$A$44,$A8,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$45,Meals!$A$5:$A$45,$A8,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -3100,11 +3155,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$44,Meals!$A$5:$A$44,$A8,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$45,Meals!$A$5:$A$45,$A8,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$44,Meals!$A$5:$A$44,$A8,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$45,Meals!$A$5:$A$45,$A8,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -3112,11 +3167,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$44,Meals!$A$5:$A$44,$A8,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$45,Meals!$A$5:$A$45,$A8,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$44,Meals!$A$5:$A$44,$A8,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$45,Meals!$A$5:$A$45,$A8,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -3124,11 +3179,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$44,$A8,Meals!$M$5:$M$44,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$45,$A8,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$44,$A8,Meals!$M$5:$M$44,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$45,$A8,Meals!$M$5:$M$45,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -3141,11 +3196,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$44,Meals!$A$5:$A$44,$A9,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$45,Meals!$A$5:$A$45,$A9,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$44,Meals!$A$5:$A$44,$A9,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$45,Meals!$A$5:$A$45,$A9,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -3153,11 +3208,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$44,Meals!$A$5:$A$44,$A9,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$45,Meals!$A$5:$A$45,$A9,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$44,Meals!$A$5:$A$44,$A9,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$45,Meals!$A$5:$A$45,$A9,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -3165,11 +3220,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$44,Meals!$A$5:$A$44,$A9,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$45,Meals!$A$5:$A$45,$A9,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$44,Meals!$A$5:$A$44,$A9,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$45,Meals!$A$5:$A$45,$A9,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -3177,11 +3232,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$44,$A9,Meals!$M$5:$M$44,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$45,$A9,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$44,$A9,Meals!$M$5:$M$44,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$45,$A9,Meals!$M$5:$M$45,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -3194,11 +3249,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$44,Meals!$A$5:$A$44,$A10,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$45,Meals!$A$5:$A$45,$A10,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$44,Meals!$A$5:$A$44,$A10,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$45,Meals!$A$5:$A$45,$A10,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -3206,11 +3261,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$44,Meals!$A$5:$A$44,$A10,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$45,Meals!$A$5:$A$45,$A10,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$44,Meals!$A$5:$A$44,$A10,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$45,Meals!$A$5:$A$45,$A10,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -3218,11 +3273,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$44,Meals!$A$5:$A$44,$A10,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$45,Meals!$A$5:$A$45,$A10,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$44,Meals!$A$5:$A$44,$A10,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$45,Meals!$A$5:$A$45,$A10,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -3230,11 +3285,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$44,$A10,Meals!$M$5:$M$44,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$45,$A10,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$44,$A10,Meals!$M$5:$M$44,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$45,$A10,Meals!$M$5:$M$45,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -3247,11 +3302,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$44,Meals!$A$5:$A$44,$A11,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$45,Meals!$A$5:$A$45,$A11,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$44,Meals!$A$5:$A$44,$A11,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$45,Meals!$A$5:$A$45,$A11,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -3259,11 +3314,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$44,Meals!$A$5:$A$44,$A11,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$45,Meals!$A$5:$A$45,$A11,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$44,Meals!$A$5:$A$44,$A11,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$45,Meals!$A$5:$A$45,$A11,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -3271,11 +3326,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$44,Meals!$A$5:$A$44,$A11,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$45,Meals!$A$5:$A$45,$A11,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$44,Meals!$A$5:$A$44,$A11,Meals!$M$5:$M$44,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$45,Meals!$A$5:$A$45,$A11,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -3283,11 +3338,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$44,$A11,Meals!$M$5:$M$44,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$45,$A11,Meals!$M$5:$M$45,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$44,$A11,Meals!$M$5:$M$44,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$45,$A11,Meals!$M$5:$M$45,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">

</xml_diff>

<commit_message>
Revise the chicken roll down on inspection
It is a breadcrumbed deep-fried bread roll, not a paratha wrap: mostly bread
and absorbed oil with a thin filling. Protein revised from ~17 g to 12.5 g
and fat up to 19 g; calories unchanged at 290-400.

At 3.6 g of protein per 100 kcal it is barely above the mess baseline. Day 7
stands at 1,830 kcal, 93 g protein, 80 g fat.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N45"/>
+  <dimension ref="A1:N46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2863,6 +2863,61 @@
       <c r="N45" s="6" t="inlineStr">
         <is>
           <t>Scoop 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>Chicken roll (breadcrumbed and deep-fried)</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="n">
+        <v>290</v>
+      </c>
+      <c r="E46" s="7" t="n">
+        <v>400</v>
+      </c>
+      <c r="F46" s="8">
+        <f>AVERAGE(D46:E46)</f>
+        <v/>
+      </c>
+      <c r="G46" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="H46" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="I46" s="10">
+        <f>AVERAGE(G46:H46)</f>
+        <v/>
+      </c>
+      <c r="J46" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="K46" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="L46" s="10">
+        <f>AVERAGE(J46:K46)</f>
+        <v/>
+      </c>
+      <c r="M46" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N46" s="6" t="inlineStr">
+        <is>
+          <t>Revised down on inspection - mostly bread and frying oil</t>
         </is>
       </c>
     </row>
@@ -2984,11 +3039,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$45,Meals!$A$5:$A$45,$A5,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$46,Meals!$A$5:$A$46,$A5,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$45,Meals!$A$5:$A$45,$A5,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$46,Meals!$A$5:$A$46,$A5,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -2996,11 +3051,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$45,Meals!$A$5:$A$45,$A5,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$46,Meals!$A$5:$A$46,$A5,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$45,Meals!$A$5:$A$45,$A5,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$46,Meals!$A$5:$A$46,$A5,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -3008,11 +3063,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$45,Meals!$A$5:$A$45,$A5,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$46,Meals!$A$5:$A$46,$A5,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$45,Meals!$A$5:$A$45,$A5,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$46,Meals!$A$5:$A$46,$A5,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -3020,11 +3075,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$45,$A5,Meals!$M$5:$M$45,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$46,$A5,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$45,$A5,Meals!$M$5:$M$45,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$46,$A5,Meals!$M$5:$M$46,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -3037,11 +3092,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$45,Meals!$A$5:$A$45,$A6,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$46,Meals!$A$5:$A$46,$A6,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$45,Meals!$A$5:$A$45,$A6,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$46,Meals!$A$5:$A$46,$A6,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -3049,11 +3104,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$45,Meals!$A$5:$A$45,$A6,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$46,Meals!$A$5:$A$46,$A6,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$45,Meals!$A$5:$A$45,$A6,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$46,Meals!$A$5:$A$46,$A6,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -3061,11 +3116,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$45,Meals!$A$5:$A$45,$A6,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$46,Meals!$A$5:$A$46,$A6,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$45,Meals!$A$5:$A$45,$A6,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$46,Meals!$A$5:$A$46,$A6,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -3073,11 +3128,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$45,$A6,Meals!$M$5:$M$45,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$46,$A6,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$45,$A6,Meals!$M$5:$M$45,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$46,$A6,Meals!$M$5:$M$46,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -3090,11 +3145,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$45,Meals!$A$5:$A$45,$A7,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$46,Meals!$A$5:$A$46,$A7,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$45,Meals!$A$5:$A$45,$A7,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$46,Meals!$A$5:$A$46,$A7,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -3102,11 +3157,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$45,Meals!$A$5:$A$45,$A7,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$46,Meals!$A$5:$A$46,$A7,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$45,Meals!$A$5:$A$45,$A7,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$46,Meals!$A$5:$A$46,$A7,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -3114,11 +3169,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$45,Meals!$A$5:$A$45,$A7,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$46,Meals!$A$5:$A$46,$A7,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$45,Meals!$A$5:$A$45,$A7,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$46,Meals!$A$5:$A$46,$A7,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -3126,11 +3181,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$45,$A7,Meals!$M$5:$M$45,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$46,$A7,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$45,$A7,Meals!$M$5:$M$45,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$46,$A7,Meals!$M$5:$M$46,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -3143,11 +3198,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$45,Meals!$A$5:$A$45,$A8,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$46,Meals!$A$5:$A$46,$A8,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$45,Meals!$A$5:$A$45,$A8,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$46,Meals!$A$5:$A$46,$A8,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -3155,11 +3210,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$45,Meals!$A$5:$A$45,$A8,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$46,Meals!$A$5:$A$46,$A8,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$45,Meals!$A$5:$A$45,$A8,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$46,Meals!$A$5:$A$46,$A8,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -3167,11 +3222,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$45,Meals!$A$5:$A$45,$A8,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$46,Meals!$A$5:$A$46,$A8,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$45,Meals!$A$5:$A$45,$A8,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$46,Meals!$A$5:$A$46,$A8,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -3179,11 +3234,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$45,$A8,Meals!$M$5:$M$45,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$46,$A8,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$45,$A8,Meals!$M$5:$M$45,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$46,$A8,Meals!$M$5:$M$46,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -3196,11 +3251,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$45,Meals!$A$5:$A$45,$A9,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$46,Meals!$A$5:$A$46,$A9,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$45,Meals!$A$5:$A$45,$A9,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$46,Meals!$A$5:$A$46,$A9,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -3208,11 +3263,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$45,Meals!$A$5:$A$45,$A9,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$46,Meals!$A$5:$A$46,$A9,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$45,Meals!$A$5:$A$45,$A9,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$46,Meals!$A$5:$A$46,$A9,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -3220,11 +3275,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$45,Meals!$A$5:$A$45,$A9,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$46,Meals!$A$5:$A$46,$A9,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$45,Meals!$A$5:$A$45,$A9,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$46,Meals!$A$5:$A$46,$A9,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -3232,11 +3287,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$45,$A9,Meals!$M$5:$M$45,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$46,$A9,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$45,$A9,Meals!$M$5:$M$45,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$46,$A9,Meals!$M$5:$M$46,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -3249,11 +3304,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$45,Meals!$A$5:$A$45,$A10,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$46,Meals!$A$5:$A$46,$A10,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$45,Meals!$A$5:$A$45,$A10,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$46,Meals!$A$5:$A$46,$A10,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -3261,11 +3316,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$45,Meals!$A$5:$A$45,$A10,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$46,Meals!$A$5:$A$46,$A10,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$45,Meals!$A$5:$A$45,$A10,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$46,Meals!$A$5:$A$46,$A10,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -3273,11 +3328,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$45,Meals!$A$5:$A$45,$A10,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$46,Meals!$A$5:$A$46,$A10,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$45,Meals!$A$5:$A$45,$A10,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$46,Meals!$A$5:$A$46,$A10,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -3285,11 +3340,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$45,$A10,Meals!$M$5:$M$45,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$46,$A10,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$45,$A10,Meals!$M$5:$M$45,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$46,$A10,Meals!$M$5:$M$46,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -3302,11 +3357,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$45,Meals!$A$5:$A$45,$A11,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$46,Meals!$A$5:$A$46,$A11,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$45,Meals!$A$5:$A$45,$A11,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$46,Meals!$A$5:$A$46,$A11,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -3314,11 +3369,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$45,Meals!$A$5:$A$45,$A11,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$46,Meals!$A$5:$A$46,$A11,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$45,Meals!$A$5:$A$45,$A11,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$46,Meals!$A$5:$A$46,$A11,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -3326,11 +3381,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$45,Meals!$A$5:$A$45,$A11,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$46,Meals!$A$5:$A$46,$A11,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$45,Meals!$A$5:$A$45,$A11,Meals!$M$5:$M$45,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$46,Meals!$A$5:$A$46,$A11,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -3338,11 +3393,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$45,$A11,Meals!$M$5:$M$45,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$46,$A11,Meals!$M$5:$M$46,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$45,$A11,Meals!$M$5:$M$45,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$46,$A11,Meals!$M$5:$M$46,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -4996,7 +5051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -5372,14 +5427,14 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Chatti pathiri chicken (1 slice ~100-120 g)</t>
+          <t>Chicken roll - breadcrumbed and deep-fried (1)</t>
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>230</v>
+        <v>290</v>
       </c>
       <c r="C17" s="7" t="n">
-        <v>320</v>
+        <v>400</v>
       </c>
       <c r="D17" s="8">
         <f>AVERAGE(B17:C17)</f>
@@ -5387,26 +5442,26 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>~10-14 g</t>
+          <t>~10-15 g</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>Layered maida pathiri with chicken masala and an egg-milk binder; ghee-rich</t>
+          <t>Mostly bread and absorbed frying oil; the chicken filling is a thin layer. 3.6 g protein per 100 kcal</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Uzhunnu vada / medu vada (1)</t>
+          <t>Chatti pathiri chicken (1 slice ~100-120 g)</t>
         </is>
       </c>
       <c r="B18" s="7" t="n">
-        <v>130</v>
+        <v>230</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>180</v>
+        <v>320</v>
       </c>
       <c r="D18" s="8">
         <f>AVERAGE(B18:C18)</f>
@@ -5414,26 +5469,26 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>~3.5-5 g each</t>
+          <t>~10-14 g</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>Deep-fried urad dal - protein-bearing but fat-dense</t>
+          <t>Layered maida pathiri with chicken masala and an egg-milk binder; ghee-rich</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Kadala curry (1 container)</t>
+          <t>Uzhunnu vada / medu vada (1)</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>200</v>
+        <v>130</v>
       </c>
       <c r="C19" s="7" t="n">
-        <v>300</v>
+        <v>180</v>
       </c>
       <c r="D19" s="8">
         <f>AVERAGE(B19:C19)</f>
@@ -5441,22 +5496,26 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>~8-10 g</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr"/>
+          <t>~3.5-5 g each</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>Deep-fried urad dal - protein-bearing but fat-dense</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Fish fry (1 piece pan-fried)</t>
+          <t>Kadala curry (1 container)</t>
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="C20" s="7" t="n">
-        <v>220</v>
+        <v>300</v>
       </c>
       <c r="D20" s="8">
         <f>AVERAGE(B20:C20)</f>
@@ -5464,7 +5523,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>~15-20 g</t>
+          <t>~8-10 g</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr"/>
@@ -5472,14 +5531,14 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Grilled sea bream (1 whole ~300-400 g)</t>
+          <t>Fish fry (1 piece pan-fried)</t>
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="C21" s="7" t="n">
-        <v>400</v>
+        <v>220</v>
       </c>
       <c r="D21" s="8">
         <f>AVERAGE(B21:C21)</f>
@@ -5487,26 +5546,22 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>~35-50 g</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>Lean white fish; best protein-per-calorie item available. Most fat is the grill oil</t>
-        </is>
-      </c>
+          <t>~15-20 g</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Matthi / sardine (2-3 fish taken without gravy)</t>
+          <t>Grilled sea bream (1 whole ~300-400 g)</t>
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>230</v>
+        <v>400</v>
       </c>
       <c r="D22" s="8">
         <f>AVERAGE(B22:C22)</f>
@@ -5514,26 +5569,26 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>~18-26 g</t>
+          <t>~35-50 g</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>Oily fish - denser than white fish but excellent protein. Leaving the gravy saves ~100 kcal and ~10 g fat</t>
+          <t>Lean white fish; best protein-per-calorie item available. Most fat is the grill oil</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Grilled chicken breast (100 g skinless)</t>
+          <t>Matthi / sardine (2-3 fish taken without gravy)</t>
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="C23" s="7" t="n">
-        <v>180</v>
+        <v>230</v>
       </c>
       <c r="D23" s="8">
         <f>AVERAGE(B23:C23)</f>
@@ -5541,26 +5596,26 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>~30-32 g</t>
+          <t>~18-26 g</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>Best protein-per-calorie item in this list</t>
+          <t>Oily fish - denser than white fish but excellent protein. Leaving the gravy saves ~100 kcal and ~10 g fat</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Grilled chicken breast (150 g skinless)</t>
+          <t>Grilled chicken breast (100 g skinless)</t>
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>240</v>
+        <v>160</v>
       </c>
       <c r="C24" s="7" t="n">
-        <v>270</v>
+        <v>180</v>
       </c>
       <c r="D24" s="8">
         <f>AVERAGE(B24:C24)</f>
@@ -5568,22 +5623,26 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>~45-48 g</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr"/>
+          <t>~30-32 g</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>Best protein-per-calorie item in this list</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Honest Bowl - Grilled Chicken and Rice Bowl</t>
+          <t>Grilled chicken breast (150 g skinless)</t>
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>550</v>
+        <v>240</v>
       </c>
       <c r="C25" s="7" t="n">
-        <v>710</v>
+        <v>270</v>
       </c>
       <c r="D25" s="8">
         <f>AVERAGE(B25:C25)</f>
@@ -5591,26 +5650,22 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>42-48 g</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>Menu states 42 g protein; chicken + jasmine rice + sweet potato. Sauce served separately</t>
-        </is>
-      </c>
+          <t>~45-48 g</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Brown/mushroom sauce (side pot)</t>
+          <t>Honest Bowl - Grilled Chicken and Rice Bowl</t>
         </is>
       </c>
       <c r="B26" s="7" t="n">
-        <v>50</v>
+        <v>550</v>
       </c>
       <c r="C26" s="7" t="n">
-        <v>120</v>
+        <v>710</v>
       </c>
       <c r="D26" s="8">
         <f>AVERAGE(B26:C26)</f>
@@ -5618,26 +5673,26 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>~1-2 g</t>
+          <t>42-48 g</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>Often cream or butter based - the variable in a bowl like this</t>
+          <t>Menu states 42 g protein; chicken + jasmine rice + sweet potato. Sauce served separately</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Honest Bowl - Tofu Delight Bowl</t>
+          <t>Brown/mushroom sauce (side pot)</t>
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>420</v>
+        <v>50</v>
       </c>
       <c r="C27" s="7" t="n">
-        <v>560</v>
+        <v>120</v>
       </c>
       <c r="D27" s="8">
         <f>AVERAGE(B27:C27)</f>
@@ -5645,26 +5700,26 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>~20 g</t>
+          <t>~1-2 g</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>Menu states 20 g; jasmine rice + cajun tofu + grilled eggplant. Half the protein of the chicken bowl at the same price</t>
+          <t>Often cream or butter based - the variable in a bowl like this</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Chicken curry (1 takeaway container)</t>
+          <t>Honest Bowl - Tofu Delight Bowl</t>
         </is>
       </c>
       <c r="B28" s="7" t="n">
-        <v>280</v>
+        <v>420</v>
       </c>
       <c r="C28" s="7" t="n">
-        <v>420</v>
+        <v>560</v>
       </c>
       <c r="D28" s="8">
         <f>AVERAGE(B28:C28)</f>
@@ -5672,26 +5727,26 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>~20-28 g</t>
+          <t>~20 g</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>Kerala style; oil and coconut carry most of the calories</t>
+          <t>Menu states 20 g; jasmine rice + cajun tofu + grilled eggplant. Half the protein of the chicken bowl at the same price</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Grilled chicken quarter (skin on)</t>
+          <t>Chicken curry (1 takeaway container)</t>
         </is>
       </c>
       <c r="B29" s="7" t="n">
-        <v>250</v>
+        <v>280</v>
       </c>
       <c r="C29" s="7" t="n">
-        <v>320</v>
+        <v>420</v>
       </c>
       <c r="D29" s="8">
         <f>AVERAGE(B29:C29)</f>
@@ -5699,26 +5754,26 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>~28-33 g</t>
+          <t>~20-28 g</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>Skin adds ~12-15 g fat over breast</t>
+          <t>Kerala style; oil and coconut carry most of the calories</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Garlic sauce / toum (1 tbsp)</t>
+          <t>Grilled chicken quarter (skin on)</t>
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>90</v>
+        <v>250</v>
       </c>
       <c r="C30" s="7" t="n">
-        <v>110</v>
+        <v>320</v>
       </c>
       <c r="D30" s="8">
         <f>AVERAGE(B30:C30)</f>
@@ -5726,26 +5781,26 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>0 g</t>
+          <t>~28-33 g</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>Essentially emulsified oil - the hidden cost at a grill</t>
+          <t>Skin adds ~12-15 g fat over breast</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Khubz / pita (1 large)</t>
+          <t>Garlic sauce / toum (1 tbsp)</t>
         </is>
       </c>
       <c r="B31" s="7" t="n">
-        <v>250</v>
+        <v>90</v>
       </c>
       <c r="C31" s="7" t="n">
-        <v>300</v>
+        <v>110</v>
       </c>
       <c r="D31" s="8">
         <f>AVERAGE(B31:C31)</f>
@@ -5753,22 +5808,26 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>~8-9 g</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="inlineStr"/>
+          <t>0 g</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>Essentially emulsified oil - the hidden cost at a grill</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Barik/basmati rice (half container cooked)</t>
+          <t>Khubz / pita (1 large)</t>
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="C32" s="7" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="D32" s="8">
         <f>AVERAGE(B32:C32)</f>
@@ -5776,7 +5835,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>~4-5 g</t>
+          <t>~8-9 g</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr"/>
@@ -5784,14 +5843,14 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Fresh pineapple juice (350-450 ml)</t>
+          <t>Barik/basmati rice (half container cooked)</t>
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>175</v>
+        <v>200</v>
       </c>
       <c r="C33" s="7" t="n">
-        <v>240</v>
+        <v>280</v>
       </c>
       <c r="D33" s="8">
         <f>AVERAGE(B33:C33)</f>
@@ -5799,26 +5858,22 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>~1-2 g</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="inlineStr">
-        <is>
-          <t>No added sugar but ~35-45 g natural sugar; no fibre; almost no protein</t>
-        </is>
-      </c>
+          <t>~4-5 g</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Fresh orange juice (350-450 ml)</t>
+          <t>Fresh pineapple juice (350-450 ml)</t>
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>155</v>
+        <v>175</v>
       </c>
       <c r="C34" s="7" t="n">
-        <v>205</v>
+        <v>240</v>
       </c>
       <c r="D34" s="8">
         <f>AVERAGE(B34:C34)</f>
@@ -5826,26 +5881,26 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>~2-3 g</t>
+          <t>~1-2 g</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>No added sugar but ~32-40 g natural sugar; no fibre</t>
+          <t>No added sugar but ~35-45 g natural sugar; no fibre; almost no protein</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in water)</t>
+          <t>Fresh orange juice (350-450 ml)</t>
         </is>
       </c>
       <c r="B35" s="7" t="n">
-        <v>100</v>
+        <v>155</v>
       </c>
       <c r="C35" s="7" t="n">
-        <v>120</v>
+        <v>205</v>
       </c>
       <c r="D35" s="8">
         <f>AVERAGE(B35:C35)</f>
@@ -5853,22 +5908,26 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="inlineStr"/>
+          <t>~2-3 g</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>No added sugar but ~32-40 g natural sugar; no fibre</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Greek yogurt (200 g plain low-fat)</t>
+          <t>Whey scoop (in water)</t>
         </is>
       </c>
       <c r="B36" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C36" s="7" t="n">
         <v>120</v>
-      </c>
-      <c r="C36" s="7" t="n">
-        <v>140</v>
       </c>
       <c r="D36" s="8">
         <f>AVERAGE(B36:C36)</f>
@@ -5876,26 +5935,22 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>~18-20 g</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="inlineStr">
-        <is>
-          <t>Casein - digests slowly; good overnight</t>
-        </is>
-      </c>
+          <t>~20-25 g</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Boiled egg (1 large)</t>
+          <t>Greek yogurt (200 g plain low-fat)</t>
         </is>
       </c>
       <c r="B37" s="7" t="n">
-        <v>70</v>
+        <v>120</v>
       </c>
       <c r="C37" s="7" t="n">
-        <v>78</v>
+        <v>140</v>
       </c>
       <c r="D37" s="8">
         <f>AVERAGE(B37:C37)</f>
@@ -5903,19 +5958,19 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>~6-6.5 g</t>
+          <t>~18-20 g</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>~5 g fat each</t>
+          <t>Casein - digests slowly; good overnight</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>Egg fried dry with no oil (1)</t>
+          <t>Boiled egg (1 large)</t>
         </is>
       </c>
       <c r="B38" s="7" t="n">
@@ -5935,21 +5990,21 @@
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>Same as boiled - dry-frying saves the ~20-25 kcal per egg that pan oil adds</t>
+          <t>~5 g fat each</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>Paneer (50 g full-fat)</t>
+          <t>Egg fried dry with no oil (1)</t>
         </is>
       </c>
       <c r="B39" s="7" t="n">
-        <v>130</v>
+        <v>70</v>
       </c>
       <c r="C39" s="7" t="n">
-        <v>150</v>
+        <v>78</v>
       </c>
       <c r="D39" s="8">
         <f>AVERAGE(B39:C39)</f>
@@ -5957,26 +6012,26 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>~8-9 g</t>
+          <t>~6-6.5 g</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
         <is>
-          <t>Fat-dense for the protein it gives</t>
+          <t>Same as boiled - dry-frying saves the ~20-25 kcal per egg that pan oil adds</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>Cucumber (1 medium)</t>
+          <t>Paneer (50 g full-fat)</t>
         </is>
       </c>
       <c r="B40" s="7" t="n">
-        <v>25</v>
+        <v>130</v>
       </c>
       <c r="C40" s="7" t="n">
-        <v>30</v>
+        <v>150</v>
       </c>
       <c r="D40" s="8">
         <f>AVERAGE(B40:C40)</f>
@@ -5984,26 +6039,26 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>~1.5 g</t>
+          <t>~8-9 g</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>Volume with almost no calories</t>
+          <t>Fat-dense for the protein it gives</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>Sweet melon / cantaloupe (1 wedge ~100-150 g)</t>
+          <t>Cucumber (1 medium)</t>
         </is>
       </c>
       <c r="B41" s="7" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="C41" s="7" t="n">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="D41" s="8">
         <f>AVERAGE(B41:C41)</f>
@@ -6011,26 +6066,26 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>~0.5-1 g</t>
+          <t>~1.5 g</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
-          <t>Whole fruit - fibre and water intact; ~1/4 the calories of the same fruit juiced</t>
+          <t>Volume with almost no calories</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Grapes (~100 g / 15-20 grapes)</t>
+          <t>Sweet melon / cantaloupe (1 wedge ~100-150 g)</t>
         </is>
       </c>
       <c r="B42" s="7" t="n">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="C42" s="7" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="D42" s="8">
         <f>AVERAGE(B42:C42)</f>
@@ -6038,26 +6093,26 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>~0.6 g</t>
+          <t>~0.5-1 g</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>Twice the calorie density of melon; easy to eat a large handful without noticing</t>
+          <t>Whole fruit - fibre and water intact; ~1/4 the calories of the same fruit juiced</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>Mango misiri (1 whole ~450-600 g)</t>
+          <t>Grapes (~100 g / 15-20 grapes)</t>
         </is>
       </c>
       <c r="B43" s="7" t="n">
-        <v>170</v>
+        <v>60</v>
       </c>
       <c r="C43" s="7" t="n">
-        <v>230</v>
+        <v>75</v>
       </c>
       <c r="D43" s="8">
         <f>AVERAGE(B43:C43)</f>
@@ -6065,26 +6120,26 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>~2-2.5 g</t>
+          <t>~0.6 g</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t>~60-65% is edible flesh; ~35-50 g sugar but fibre intact</t>
+          <t>Twice the calorie density of melon; easy to eat a large handful without noticing</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>Diet/zero-sugar soft drink (330 ml)</t>
+          <t>Mango misiri (1 whole ~450-600 g)</t>
         </is>
       </c>
       <c r="B44" s="7" t="n">
-        <v>0</v>
+        <v>170</v>
       </c>
       <c r="C44" s="7" t="n">
-        <v>2</v>
+        <v>230</v>
       </c>
       <c r="D44" s="8">
         <f>AVERAGE(B44:C44)</f>
@@ -6092,26 +6147,26 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>0 g</t>
+          <t>~2-2.5 g</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t>Genuinely zero - unlike fruit juice sold as no added sugar</t>
+          <t>~60-65% is edible flesh; ~35-50 g sugar but fibre intact</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in black coffee no sugar)</t>
+          <t>Diet/zero-sugar soft drink (330 ml)</t>
         </is>
       </c>
       <c r="B45" s="7" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="C45" s="7" t="n">
-        <v>130</v>
+        <v>2</v>
       </c>
       <c r="D45" s="8">
         <f>AVERAGE(B45:C45)</f>
@@ -6119,22 +6174,26 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="inlineStr"/>
+          <t>0 g</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>Genuinely zero - unlike fruit juice sold as no added sugar</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>Cashew/almond biscuit (1)</t>
+          <t>Whey scoop (in black coffee no sugar)</t>
         </is>
       </c>
       <c r="B46" s="7" t="n">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C46" s="7" t="n">
-        <v>38</v>
+        <v>130</v>
       </c>
       <c r="D46" s="8">
         <f>AVERAGE(B46:C46)</f>
@@ -6142,7 +6201,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>~0.5 g</t>
+          <t>~20-25 g</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr"/>
@@ -6150,14 +6209,14 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (~50g standard)</t>
+          <t>Cashew/almond biscuit (1)</t>
         </is>
       </c>
       <c r="B47" s="7" t="n">
-        <v>245</v>
+        <v>38</v>
       </c>
       <c r="C47" s="7" t="n">
-        <v>250</v>
+        <v>38</v>
       </c>
       <c r="D47" s="8">
         <f>AVERAGE(B47:C47)</f>
@@ -6165,7 +6224,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>~4 g</t>
+          <t>~0.5 g</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr"/>
@@ -6173,14 +6232,14 @@
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (70g king-size)</t>
+          <t>Chocolate bar (~50g standard)</t>
         </is>
       </c>
       <c r="B48" s="7" t="n">
-        <v>335</v>
+        <v>245</v>
       </c>
       <c r="C48" s="7" t="n">
-        <v>335</v>
+        <v>250</v>
       </c>
       <c r="D48" s="8">
         <f>AVERAGE(B48:C48)</f>
@@ -6188,7 +6247,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>~6 g</t>
+          <t>~4 g</t>
         </is>
       </c>
       <c r="F48" s="6" t="inlineStr"/>
@@ -6196,14 +6255,14 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>Pre-workout scoop</t>
+          <t>Chocolate bar (70g king-size)</t>
         </is>
       </c>
       <c r="B49" s="7" t="n">
-        <v>5</v>
+        <v>335</v>
       </c>
       <c r="C49" s="7" t="n">
-        <v>15</v>
+        <v>335</v>
       </c>
       <c r="D49" s="8">
         <f>AVERAGE(B49:C49)</f>
@@ -6211,10 +6270,33 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
+          <t>~6 g</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>Pre-workout scoop</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C50" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D50" s="8">
+        <f>AVERAGE(B50:C50)</f>
+        <v/>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
           <t>0 g</t>
         </is>
       </c>
-      <c r="F49" s="6" t="inlineStr">
+      <c r="F50" s="6" t="inlineStr">
         <is>
           <t>Negligible</t>
         </is>

</xml_diff>

<commit_message>
Log Day 7 dinner: 2 chapati with gobi chilli
380-540 kcal (mid 460), 10-15 g protein, 14-26 g fat. Day 7 stands at
2,290 kcal, 105.5 g protein and 100 g fat with one scoop still to come.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N46"/>
+  <dimension ref="A1:N47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2762,39 +2762,39 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Lunch</t>
+          <t>Dinner</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>Mess meals plate (rice halved) + matthi taken without the gravy + 2 small fried chicken pieces + coconut chammanthi, thoran, veg curries</t>
+          <t>2 chapati + gobi chilli</t>
         </is>
       </c>
       <c r="D44" s="7" t="n">
-        <v>760</v>
+        <v>380</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>1150</v>
+        <v>540</v>
       </c>
       <c r="F44" s="8">
         <f>AVERAGE(D44:E44)</f>
         <v/>
       </c>
       <c r="G44" s="9" t="n">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>57</v>
+        <v>15</v>
       </c>
       <c r="I44" s="10">
         <f>AVERAGE(G44:H44)</f>
         <v/>
       </c>
       <c r="J44" s="9" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="K44" s="9" t="n">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="L44" s="10">
         <f>AVERAGE(J44:K44)</f>
@@ -2807,7 +2807,7 @@
       </c>
       <c r="N44" s="6" t="inlineStr">
         <is>
-          <t>Fish lifted out of the curry and the oily gravy left behind; 2 fried chicken pieces on the plate</t>
+          <t>Mess Thursday dinner; modest gobi portion</t>
         </is>
       </c>
     </row>
@@ -2817,39 +2817,39 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Snack</t>
+          <t>Lunch</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>Black coffee + 1 whey scoop</t>
+          <t>Mess meals plate (rice halved) + matthi taken without the gravy + 2 small fried chicken pieces + coconut chammanthi, thoran, veg curries</t>
         </is>
       </c>
       <c r="D45" s="7" t="n">
-        <v>100</v>
+        <v>760</v>
       </c>
       <c r="E45" s="7" t="n">
-        <v>130</v>
+        <v>1150</v>
       </c>
       <c r="F45" s="8">
         <f>AVERAGE(D45:E45)</f>
         <v/>
       </c>
       <c r="G45" s="9" t="n">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="H45" s="9" t="n">
-        <v>25</v>
+        <v>57</v>
       </c>
       <c r="I45" s="10">
         <f>AVERAGE(G45:H45)</f>
         <v/>
       </c>
       <c r="J45" s="9" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="K45" s="9" t="n">
-        <v>3</v>
+        <v>53</v>
       </c>
       <c r="L45" s="10">
         <f>AVERAGE(J45:K45)</f>
@@ -2862,7 +2862,7 @@
       </c>
       <c r="N45" s="6" t="inlineStr">
         <is>
-          <t>Scoop 1</t>
+          <t>Fish lifted out of the curry and the oily gravy left behind; 2 fried chicken pieces on the plate</t>
         </is>
       </c>
     </row>
@@ -2877,34 +2877,34 @@
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>Chicken roll (breadcrumbed and deep-fried)</t>
+          <t>Black coffee + 1 whey scoop</t>
         </is>
       </c>
       <c r="D46" s="7" t="n">
-        <v>290</v>
+        <v>100</v>
       </c>
       <c r="E46" s="7" t="n">
-        <v>400</v>
+        <v>130</v>
       </c>
       <c r="F46" s="8">
         <f>AVERAGE(D46:E46)</f>
         <v/>
       </c>
       <c r="G46" s="9" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="I46" s="10">
         <f>AVERAGE(G46:H46)</f>
         <v/>
       </c>
       <c r="J46" s="9" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="K46" s="9" t="n">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="L46" s="10">
         <f>AVERAGE(J46:K46)</f>
@@ -2916,6 +2916,61 @@
         </is>
       </c>
       <c r="N46" s="6" t="inlineStr">
+        <is>
+          <t>Scoop 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>Chicken roll (breadcrumbed and deep-fried)</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="n">
+        <v>290</v>
+      </c>
+      <c r="E47" s="7" t="n">
+        <v>400</v>
+      </c>
+      <c r="F47" s="8">
+        <f>AVERAGE(D47:E47)</f>
+        <v/>
+      </c>
+      <c r="G47" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="H47" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="I47" s="10">
+        <f>AVERAGE(G47:H47)</f>
+        <v/>
+      </c>
+      <c r="J47" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="K47" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="L47" s="10">
+        <f>AVERAGE(J47:K47)</f>
+        <v/>
+      </c>
+      <c r="M47" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N47" s="6" t="inlineStr">
         <is>
           <t>Revised down on inspection - mostly bread and frying oil</t>
         </is>
@@ -3039,11 +3094,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$46,Meals!$A$5:$A$46,$A5,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$47,Meals!$A$5:$A$47,$A5,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$46,Meals!$A$5:$A$46,$A5,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$47,Meals!$A$5:$A$47,$A5,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -3051,11 +3106,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$46,Meals!$A$5:$A$46,$A5,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$47,Meals!$A$5:$A$47,$A5,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$46,Meals!$A$5:$A$46,$A5,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$47,Meals!$A$5:$A$47,$A5,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -3063,11 +3118,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$46,Meals!$A$5:$A$46,$A5,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$47,Meals!$A$5:$A$47,$A5,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$46,Meals!$A$5:$A$46,$A5,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$47,Meals!$A$5:$A$47,$A5,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -3075,11 +3130,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$46,$A5,Meals!$M$5:$M$46,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$47,$A5,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$46,$A5,Meals!$M$5:$M$46,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$47,$A5,Meals!$M$5:$M$47,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -3092,11 +3147,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$46,Meals!$A$5:$A$46,$A6,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$47,Meals!$A$5:$A$47,$A6,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$46,Meals!$A$5:$A$46,$A6,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$47,Meals!$A$5:$A$47,$A6,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -3104,11 +3159,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$46,Meals!$A$5:$A$46,$A6,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$47,Meals!$A$5:$A$47,$A6,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$46,Meals!$A$5:$A$46,$A6,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$47,Meals!$A$5:$A$47,$A6,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -3116,11 +3171,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$46,Meals!$A$5:$A$46,$A6,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$47,Meals!$A$5:$A$47,$A6,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$46,Meals!$A$5:$A$46,$A6,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$47,Meals!$A$5:$A$47,$A6,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -3128,11 +3183,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$46,$A6,Meals!$M$5:$M$46,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$47,$A6,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$46,$A6,Meals!$M$5:$M$46,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$47,$A6,Meals!$M$5:$M$47,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -3145,11 +3200,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$46,Meals!$A$5:$A$46,$A7,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$47,Meals!$A$5:$A$47,$A7,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$46,Meals!$A$5:$A$46,$A7,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$47,Meals!$A$5:$A$47,$A7,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -3157,11 +3212,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$46,Meals!$A$5:$A$46,$A7,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$47,Meals!$A$5:$A$47,$A7,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$46,Meals!$A$5:$A$46,$A7,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$47,Meals!$A$5:$A$47,$A7,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -3169,11 +3224,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$46,Meals!$A$5:$A$46,$A7,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$47,Meals!$A$5:$A$47,$A7,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$46,Meals!$A$5:$A$46,$A7,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$47,Meals!$A$5:$A$47,$A7,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -3181,11 +3236,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$46,$A7,Meals!$M$5:$M$46,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$47,$A7,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$46,$A7,Meals!$M$5:$M$46,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$47,$A7,Meals!$M$5:$M$47,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -3198,11 +3253,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$46,Meals!$A$5:$A$46,$A8,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$47,Meals!$A$5:$A$47,$A8,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$46,Meals!$A$5:$A$46,$A8,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$47,Meals!$A$5:$A$47,$A8,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -3210,11 +3265,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$46,Meals!$A$5:$A$46,$A8,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$47,Meals!$A$5:$A$47,$A8,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$46,Meals!$A$5:$A$46,$A8,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$47,Meals!$A$5:$A$47,$A8,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -3222,11 +3277,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$46,Meals!$A$5:$A$46,$A8,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$47,Meals!$A$5:$A$47,$A8,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$46,Meals!$A$5:$A$46,$A8,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$47,Meals!$A$5:$A$47,$A8,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -3234,11 +3289,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$46,$A8,Meals!$M$5:$M$46,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$47,$A8,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$46,$A8,Meals!$M$5:$M$46,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$47,$A8,Meals!$M$5:$M$47,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -3251,11 +3306,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$46,Meals!$A$5:$A$46,$A9,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$47,Meals!$A$5:$A$47,$A9,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$46,Meals!$A$5:$A$46,$A9,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$47,Meals!$A$5:$A$47,$A9,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -3263,11 +3318,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$46,Meals!$A$5:$A$46,$A9,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$47,Meals!$A$5:$A$47,$A9,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$46,Meals!$A$5:$A$46,$A9,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$47,Meals!$A$5:$A$47,$A9,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -3275,11 +3330,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$46,Meals!$A$5:$A$46,$A9,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$47,Meals!$A$5:$A$47,$A9,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$46,Meals!$A$5:$A$46,$A9,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$47,Meals!$A$5:$A$47,$A9,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -3287,11 +3342,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$46,$A9,Meals!$M$5:$M$46,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$47,$A9,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$46,$A9,Meals!$M$5:$M$46,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$47,$A9,Meals!$M$5:$M$47,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -3304,11 +3359,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$46,Meals!$A$5:$A$46,$A10,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$47,Meals!$A$5:$A$47,$A10,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$46,Meals!$A$5:$A$46,$A10,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$47,Meals!$A$5:$A$47,$A10,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -3316,11 +3371,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$46,Meals!$A$5:$A$46,$A10,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$47,Meals!$A$5:$A$47,$A10,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$46,Meals!$A$5:$A$46,$A10,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$47,Meals!$A$5:$A$47,$A10,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -3328,11 +3383,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$46,Meals!$A$5:$A$46,$A10,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$47,Meals!$A$5:$A$47,$A10,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$46,Meals!$A$5:$A$46,$A10,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$47,Meals!$A$5:$A$47,$A10,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -3340,11 +3395,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$46,$A10,Meals!$M$5:$M$46,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$47,$A10,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$46,$A10,Meals!$M$5:$M$46,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$47,$A10,Meals!$M$5:$M$47,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -3357,11 +3412,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$46,Meals!$A$5:$A$46,$A11,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$47,Meals!$A$5:$A$47,$A11,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$46,Meals!$A$5:$A$46,$A11,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$47,Meals!$A$5:$A$47,$A11,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -3369,11 +3424,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$46,Meals!$A$5:$A$46,$A11,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$47,Meals!$A$5:$A$47,$A11,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$46,Meals!$A$5:$A$46,$A11,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$47,Meals!$A$5:$A$47,$A11,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -3381,11 +3436,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$46,Meals!$A$5:$A$46,$A11,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$47,Meals!$A$5:$A$47,$A11,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$46,Meals!$A$5:$A$46,$A11,Meals!$M$5:$M$46,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$47,Meals!$A$5:$A$47,$A11,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -3393,11 +3448,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$46,$A11,Meals!$M$5:$M$46,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$47,$A11,Meals!$M$5:$M$47,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$46,$A11,Meals!$M$5:$M$46,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$47,$A11,Meals!$M$5:$M$47,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">

</xml_diff>

<commit_message>
Revise the activity multiplier from measured step data: 1.45 -> 1.52
Apple Watch shows 8,237 steps/day averaged over 12 Aug-11 Sep, about 5.6 km.
The original 1.45 assumed a sedentary NEAT baseline that this clearly is
not. Rebuilt the maintenance breakdown to separate walking NEAT (~150/day)
from the training allowance, which now reads ~482 per session rather than
being inflated by miscounted walking.

Maintenance moves 2,550 -> 2,673 and the derived target 2,000 -> 2,125. The
six-day average intake of 2,193 is within 70 kcal of the new target, so
nothing about what to eat changes - but the deficit reads 480/day rather
than 357, and 0.44 kg/week rather than 0.32.

The extra-activity block is reset to zero walking, reserved for distance on
top of the usual 8,200 steps.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -4722,11 +4722,11 @@
         </is>
       </c>
       <c r="B9" s="34" t="n">
-        <v>1.45</v>
+        <v>1.52</v>
       </c>
       <c r="C9" s="33" t="inlineStr">
         <is>
-          <t>1.45 = desk job plus 6 lifting sessions/week. Lifting burns less than cardio-based charts assume; raise it only if the scale says so.</t>
+          <t>1.52, revised 2026-09-11 from Apple Watch: 8,237 steps/day averaged over a month is ~5.6 km, well above the sedentary baseline the old 1.45 assumed. Still an estimate - the trailing weight average is the arbiter.</t>
         </is>
       </c>
     </row>
@@ -4924,52 +4924,67 @@
       </c>
       <c r="C27" s="33" t="inlineStr">
         <is>
-          <t>Living, digestion, fidgeting, walking about - no training.</t>
+          <t>Living, digestion, and the ~3,500-5,000 steps a desk-bound day produces.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="29" t="inlineStr">
         <is>
-          <t>Training allowance</t>
-        </is>
-      </c>
-      <c r="B28" s="8">
-        <f>B15-B27</f>
-        <v/>
+          <t>Walking NEAT above sedentary</t>
+        </is>
+      </c>
+      <c r="B28" s="14" t="n">
+        <v>150</v>
       </c>
       <c r="C28" s="33" t="inlineStr">
         <is>
-          <t>The part of the multiplier that is the gym.</t>
+          <t>Apple Watch: 8,237 steps/day averaged over a month, ~5.6 km. The part above a sedentary baseline, at 0.5 kcal per kg per km.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="29" t="inlineStr">
         <is>
-          <t>Sessions per week</t>
-        </is>
-      </c>
-      <c r="B29" s="31" t="n">
-        <v>6</v>
+          <t>Training allowance</t>
+        </is>
+      </c>
+      <c r="B29" s="8">
+        <f>B15-B27-B28</f>
+        <v/>
       </c>
       <c r="C29" s="33" t="inlineStr">
         <is>
-          <t>6-day PPL split.</t>
+          <t>What is left for the gym once living and walking are paid for.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="29" t="inlineStr">
         <is>
+          <t>Sessions per week</t>
+        </is>
+      </c>
+      <c r="B30" s="31" t="n">
+        <v>6</v>
+      </c>
+      <c r="C30" s="33" t="inlineStr">
+        <is>
+          <t>6-day PPL split.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="29" t="inlineStr">
+        <is>
           <t>Implied kcal per session</t>
         </is>
       </c>
-      <c r="B30" s="8">
-        <f>B28*7/B29</f>
-        <v/>
-      </c>
-      <c r="C30" s="33" t="inlineStr">
+      <c r="B31" s="8">
+        <f>B29*7/B30</f>
+        <v/>
+      </c>
+      <c r="C31" s="33" t="inlineStr">
         <is>
           <t>Sanity check: resistance training runs ~5-7 kcal/min, so 45-90 min at this bodyweight is ~225-630 kcal. If sessions are short, this allowance is generous and the multiplier should come down - but let the scale decide, not this cell.</t>
         </is>
@@ -4994,11 +5009,11 @@
         </is>
       </c>
       <c r="B33" s="16" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C33" s="33" t="inlineStr">
         <is>
-          <t>Reported 5 km on 2026-09-07. ~50-60 min at a normal pace.</t>
+          <t>Now zero: the daily walk is inside the 1.52 multiplier, set from measured step count. Use this block only for walking ON TOP of the usual 8,200 steps.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log 90.05 kg weigh-in - fourth point, rate decelerating as forecast
91.50 -> 90.75 -> 90.30 -> 90.05, with interval changes of -0.75, -0.45 and
-0.25. Trailing average 90.65.

Across the six days the scale covers, intake was 13,642 kcal against
~16,038 of maintenance: a 2,396 kcal deficit, 0.31 kg of fat. The other
1.14 kg is water and glycogen, though the water share is falling (87% to
79%). Implied fat-loss rate 0.36 kg/week.

At 90.05 kg the targets re-derive to BMR 1,756, maintenance 2,669, target
2,120. BMI 34.1.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -3474,7 +3474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3603,8 +3603,33 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="27" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B8" s="24" t="n">
+        <v>90.05</v>
+      </c>
+      <c r="C8" s="25">
+        <f>B8-B7</f>
+        <v/>
+      </c>
+      <c r="D8" s="25">
+        <f>B8-$B$5</f>
+        <v/>
+      </c>
+      <c r="E8" s="26">
+        <f>AVERAGE(B5:B8)</f>
+        <v/>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Morning weigh-in</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="27" t="inlineStr">
         <is>
           <t>A drop in the first week is mostly water and glycogen, not fat. Judge the trend over 2-3 weeks, and change the activity multiplier on Targets only then.</t>
         </is>

</xml_diff>

<commit_message>
Log Day 8 breakfast: 2 set dosa with sambar
410-550 kcal (mid 480), 10-15 g protein, 11-24 g fat. Coconut chutney
skipped for the fourth time in eight days.

Friday is the roomiest day on the menu: biriyani carries protein and the
kadala dinner is light, so the mess as served plus 3 scoops lands 1,955 kcal
and 129 g protein - a 714 kcal deficit.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N47"/>
+  <dimension ref="A1:N48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2976,6 +2976,61 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" s="4" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Breakfast</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>2 set dosa + sambar + red chutney (coconut chutney skipped)</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="n">
+        <v>410</v>
+      </c>
+      <c r="E48" s="7" t="n">
+        <v>550</v>
+      </c>
+      <c r="F48" s="8">
+        <f>AVERAGE(D48:E48)</f>
+        <v/>
+      </c>
+      <c r="G48" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="H48" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="I48" s="10">
+        <f>AVERAGE(G48:H48)</f>
+        <v/>
+      </c>
+      <c r="J48" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="K48" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="L48" s="10">
+        <f>AVERAGE(J48:K48)</f>
+        <v/>
+      </c>
+      <c r="M48" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N48" s="6" t="inlineStr">
+        <is>
+          <t>Coconut chutney skipped again</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:N2"/>
@@ -2990,7 +3045,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3094,11 +3149,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$47,Meals!$A$5:$A$47,$A5,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$48,Meals!$A$5:$A$48,$A5,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$47,Meals!$A$5:$A$47,$A5,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$48,Meals!$A$5:$A$48,$A5,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -3106,11 +3161,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$47,Meals!$A$5:$A$47,$A5,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$48,Meals!$A$5:$A$48,$A5,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$47,Meals!$A$5:$A$47,$A5,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$48,Meals!$A$5:$A$48,$A5,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -3118,11 +3173,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$47,Meals!$A$5:$A$47,$A5,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$48,Meals!$A$5:$A$48,$A5,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$47,Meals!$A$5:$A$47,$A5,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$48,Meals!$A$5:$A$48,$A5,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -3130,11 +3185,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$47,$A5,Meals!$M$5:$M$47,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$48,$A5,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$47,$A5,Meals!$M$5:$M$47,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$48,$A5,Meals!$M$5:$M$48,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -3147,11 +3202,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$47,Meals!$A$5:$A$47,$A6,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$48,Meals!$A$5:$A$48,$A6,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$47,Meals!$A$5:$A$47,$A6,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$48,Meals!$A$5:$A$48,$A6,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -3159,11 +3214,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$47,Meals!$A$5:$A$47,$A6,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$48,Meals!$A$5:$A$48,$A6,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$47,Meals!$A$5:$A$47,$A6,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$48,Meals!$A$5:$A$48,$A6,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -3171,11 +3226,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$47,Meals!$A$5:$A$47,$A6,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$48,Meals!$A$5:$A$48,$A6,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$47,Meals!$A$5:$A$47,$A6,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$48,Meals!$A$5:$A$48,$A6,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -3183,11 +3238,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$47,$A6,Meals!$M$5:$M$47,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$48,$A6,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$47,$A6,Meals!$M$5:$M$47,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$48,$A6,Meals!$M$5:$M$48,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -3200,11 +3255,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$47,Meals!$A$5:$A$47,$A7,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$48,Meals!$A$5:$A$48,$A7,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$47,Meals!$A$5:$A$47,$A7,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$48,Meals!$A$5:$A$48,$A7,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -3212,11 +3267,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$47,Meals!$A$5:$A$47,$A7,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$48,Meals!$A$5:$A$48,$A7,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$47,Meals!$A$5:$A$47,$A7,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$48,Meals!$A$5:$A$48,$A7,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -3224,11 +3279,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$47,Meals!$A$5:$A$47,$A7,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$48,Meals!$A$5:$A$48,$A7,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$47,Meals!$A$5:$A$47,$A7,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$48,Meals!$A$5:$A$48,$A7,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -3236,11 +3291,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$47,$A7,Meals!$M$5:$M$47,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$48,$A7,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$47,$A7,Meals!$M$5:$M$47,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$48,$A7,Meals!$M$5:$M$48,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -3253,11 +3308,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$47,Meals!$A$5:$A$47,$A8,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$48,Meals!$A$5:$A$48,$A8,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$47,Meals!$A$5:$A$47,$A8,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$48,Meals!$A$5:$A$48,$A8,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -3265,11 +3320,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$47,Meals!$A$5:$A$47,$A8,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$48,Meals!$A$5:$A$48,$A8,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$47,Meals!$A$5:$A$47,$A8,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$48,Meals!$A$5:$A$48,$A8,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -3277,11 +3332,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$47,Meals!$A$5:$A$47,$A8,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$48,Meals!$A$5:$A$48,$A8,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$47,Meals!$A$5:$A$47,$A8,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$48,Meals!$A$5:$A$48,$A8,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -3289,11 +3344,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$47,$A8,Meals!$M$5:$M$47,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$48,$A8,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$47,$A8,Meals!$M$5:$M$47,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$48,$A8,Meals!$M$5:$M$48,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -3306,11 +3361,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$47,Meals!$A$5:$A$47,$A9,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$48,Meals!$A$5:$A$48,$A9,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$47,Meals!$A$5:$A$47,$A9,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$48,Meals!$A$5:$A$48,$A9,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -3318,11 +3373,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$47,Meals!$A$5:$A$47,$A9,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$48,Meals!$A$5:$A$48,$A9,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$47,Meals!$A$5:$A$47,$A9,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$48,Meals!$A$5:$A$48,$A9,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -3330,11 +3385,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$47,Meals!$A$5:$A$47,$A9,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$48,Meals!$A$5:$A$48,$A9,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$47,Meals!$A$5:$A$47,$A9,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$48,Meals!$A$5:$A$48,$A9,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -3342,11 +3397,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$47,$A9,Meals!$M$5:$M$47,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$48,$A9,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$47,$A9,Meals!$M$5:$M$47,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$48,$A9,Meals!$M$5:$M$48,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -3359,11 +3414,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$47,Meals!$A$5:$A$47,$A10,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$48,Meals!$A$5:$A$48,$A10,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$47,Meals!$A$5:$A$47,$A10,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$48,Meals!$A$5:$A$48,$A10,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -3371,11 +3426,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$47,Meals!$A$5:$A$47,$A10,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$48,Meals!$A$5:$A$48,$A10,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$47,Meals!$A$5:$A$47,$A10,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$48,Meals!$A$5:$A$48,$A10,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -3383,11 +3438,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$47,Meals!$A$5:$A$47,$A10,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$48,Meals!$A$5:$A$48,$A10,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$47,Meals!$A$5:$A$47,$A10,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$48,Meals!$A$5:$A$48,$A10,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -3395,11 +3450,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$47,$A10,Meals!$M$5:$M$47,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$48,$A10,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$47,$A10,Meals!$M$5:$M$47,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$48,$A10,Meals!$M$5:$M$48,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -3412,11 +3467,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$47,Meals!$A$5:$A$47,$A11,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$48,Meals!$A$5:$A$48,$A11,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$47,Meals!$A$5:$A$47,$A11,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$48,Meals!$A$5:$A$48,$A11,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -3424,11 +3479,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$47,Meals!$A$5:$A$47,$A11,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$48,Meals!$A$5:$A$48,$A11,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$47,Meals!$A$5:$A$47,$A11,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$48,Meals!$A$5:$A$48,$A11,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -3436,11 +3491,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$47,Meals!$A$5:$A$47,$A11,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$48,Meals!$A$5:$A$48,$A11,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$47,Meals!$A$5:$A$47,$A11,Meals!$M$5:$M$47,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$48,Meals!$A$5:$A$48,$A11,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -3448,15 +3503,68 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$47,$A11,Meals!$M$5:$M$47,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$48,$A11,Meals!$M$5:$M$48,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$47,$A11,Meals!$M$5:$M$47,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$48,$A11,Meals!$M$5:$M$48,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
         <f>D11-Targets!$B$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="20" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B12" s="21">
+        <f>SUMIFS(Meals!$D$5:$D$48,Meals!$A$5:$A$48,$A12,Meals!$M$5:$M$48,"logged")</f>
+        <v/>
+      </c>
+      <c r="C12" s="21">
+        <f>SUMIFS(Meals!$E$5:$E$48,Meals!$A$5:$A$48,$A12,Meals!$M$5:$M$48,"logged")</f>
+        <v/>
+      </c>
+      <c r="D12" s="21">
+        <f>AVERAGE(B12:C12)</f>
+        <v/>
+      </c>
+      <c r="E12" s="22">
+        <f>SUMIFS(Meals!$G$5:$G$48,Meals!$A$5:$A$48,$A12,Meals!$M$5:$M$48,"logged")</f>
+        <v/>
+      </c>
+      <c r="F12" s="22">
+        <f>SUMIFS(Meals!$H$5:$H$48,Meals!$A$5:$A$48,$A12,Meals!$M$5:$M$48,"logged")</f>
+        <v/>
+      </c>
+      <c r="G12" s="22">
+        <f>AVERAGE(E12:F12)</f>
+        <v/>
+      </c>
+      <c r="H12" s="22">
+        <f>SUMIFS(Meals!$J$5:$J$48,Meals!$A$5:$A$48,$A12,Meals!$M$5:$M$48,"logged")</f>
+        <v/>
+      </c>
+      <c r="I12" s="22">
+        <f>SUMIFS(Meals!$K$5:$K$48,Meals!$A$5:$A$48,$A12,Meals!$M$5:$M$48,"logged")</f>
+        <v/>
+      </c>
+      <c r="J12" s="22">
+        <f>AVERAGE(H12:I12)</f>
+        <v/>
+      </c>
+      <c r="K12" s="20">
+        <f>COUNTIFS(Meals!$A$5:$A$48,$A12,Meals!$M$5:$M$48,"logged")</f>
+        <v/>
+      </c>
+      <c r="L12" s="20">
+        <f>COUNTIFS(Meals!$A$5:$A$48,$A12,Meals!$M$5:$M$48,"pending")</f>
+        <v/>
+      </c>
+      <c r="M12" s="23">
+        <f>D12-Targets!$B$16</f>
         <v/>
       </c>
     </row>
@@ -4390,7 +4498,7 @@
         </is>
       </c>
       <c r="B5" s="18">
-        <f>COUNT(Daily!$A$5:$A$11)</f>
+        <f>COUNT(Daily!$A$5:$A$12)</f>
         <v/>
       </c>
     </row>
@@ -4401,7 +4509,7 @@
         </is>
       </c>
       <c r="B6" s="8">
-        <f>IFERROR(AVERAGE(Daily!$D$5:$D$11),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$D$5:$D$12),0)</f>
         <v/>
       </c>
     </row>
@@ -4412,7 +4520,7 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>IFERROR(AVERAGE(Daily!$G$5:$G$11),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$G$5:$G$12),0)</f>
         <v/>
       </c>
     </row>
@@ -4423,7 +4531,7 @@
         </is>
       </c>
       <c r="B8" s="10">
-        <f>IFERROR(AVERAGE(Daily!$J$5:$J$11),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$J$5:$J$12),0)</f>
         <v/>
       </c>
     </row>
@@ -4467,7 +4575,7 @@
         </is>
       </c>
       <c r="B12" s="18">
-        <f>COUNTIFS(Daily!$G$5:$G$11,"&gt;="&amp;Targets!$B$20)</f>
+        <f>COUNTIFS(Daily!$G$5:$G$12,"&gt;="&amp;Targets!$B$20)</f>
         <v/>
       </c>
     </row>
@@ -4478,7 +4586,7 @@
         </is>
       </c>
       <c r="B13" s="18">
-        <f>SUM(Daily!$L$5:$L$11)</f>
+        <f>SUM(Daily!$L$5:$L$12)</f>
         <v/>
       </c>
     </row>
@@ -4529,19 +4637,19 @@
         <v>46271</v>
       </c>
       <c r="C17" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$11,"&gt;="&amp;$A17,Daily!$A$5:$A$11,"&lt;="&amp;$B17)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$12,"&gt;="&amp;$A17,Daily!$A$5:$A$12,"&lt;="&amp;$B17)</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$11,Daily!$A$5:$A$11,"&gt;="&amp;$A17,Daily!$A$5:$A$11,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$12,Daily!$A$5:$A$12,"&gt;="&amp;$A17,Daily!$A$5:$A$12,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$11,Daily!$A$5:$A$11,"&gt;="&amp;$A17,Daily!$A$5:$A$11,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$12,Daily!$A$5:$A$12,"&gt;="&amp;$A17,Daily!$A$5:$A$12,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$11,Daily!$A$5:$A$11,"&gt;="&amp;$A17,Daily!$A$5:$A$11,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$12,Daily!$A$5:$A$12,"&gt;="&amp;$A17,Daily!$A$5:$A$12,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
     </row>
@@ -4553,19 +4661,19 @@
         <v>46278</v>
       </c>
       <c r="C18" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$11,"&gt;="&amp;$A18,Daily!$A$5:$A$11,"&lt;="&amp;$B18)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$12,"&gt;="&amp;$A18,Daily!$A$5:$A$12,"&lt;="&amp;$B18)</f>
         <v/>
       </c>
       <c r="D18" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$11,Daily!$A$5:$A$11,"&gt;="&amp;$A18,Daily!$A$5:$A$11,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$12,Daily!$A$5:$A$12,"&gt;="&amp;$A18,Daily!$A$5:$A$12,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="E18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$11,Daily!$A$5:$A$11,"&gt;="&amp;$A18,Daily!$A$5:$A$11,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$12,Daily!$A$5:$A$12,"&gt;="&amp;$A18,Daily!$A$5:$A$12,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="F18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$11,Daily!$A$5:$A$11,"&gt;="&amp;$A18,Daily!$A$5:$A$11,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$12,Daily!$A$5:$A$12,"&gt;="&amp;$A18,Daily!$A$5:$A$12,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
     </row>
@@ -4616,19 +4724,19 @@
         <v>46295</v>
       </c>
       <c r="C22" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$11,"&gt;="&amp;$A22,Daily!$A$5:$A$11,"&lt;="&amp;$B22)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$12,"&gt;="&amp;$A22,Daily!$A$5:$A$12,"&lt;="&amp;$B22)</f>
         <v/>
       </c>
       <c r="D22" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$11,Daily!$A$5:$A$11,"&gt;="&amp;$A22,Daily!$A$5:$A$11,"&lt;="&amp;$B22),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$12,Daily!$A$5:$A$12,"&gt;="&amp;$A22,Daily!$A$5:$A$12,"&lt;="&amp;$B22),0)</f>
         <v/>
       </c>
       <c r="E22" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$11,Daily!$A$5:$A$11,"&gt;="&amp;$A22,Daily!$A$5:$A$11,"&lt;="&amp;$B22),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$12,Daily!$A$5:$A$12,"&gt;="&amp;$A22,Daily!$A$5:$A$12,"&lt;="&amp;$B22),0)</f>
         <v/>
       </c>
       <c r="F22" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$11,Daily!$A$5:$A$11,"&gt;="&amp;$A22,Daily!$A$5:$A$11,"&lt;="&amp;$B22),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$12,Daily!$A$5:$A$12,"&gt;="&amp;$A22,Daily!$A$5:$A$12,"&lt;="&amp;$B22),0)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Log dry-fried egg on Day 8 breakfast
70-78 kcal, 6-6.5 g protein. Day 8 stands at 554 kcal and 18.75 g protein.
Reworked the day's plan around halving the biriyani rice: four scoops lands
1,954 kcal and 154 g protein, 715 under maintenance.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N48"/>
+  <dimension ref="A1:N49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3028,6 +3028,61 @@
       <c r="N48" s="6" t="inlineStr">
         <is>
           <t>Coconut chutney skipped again</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Breakfast</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>1 egg fried dry with no oil + pepper</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="E49" s="7" t="n">
+        <v>78</v>
+      </c>
+      <c r="F49" s="8">
+        <f>AVERAGE(D49:E49)</f>
+        <v/>
+      </c>
+      <c r="G49" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="H49" s="9" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="I49" s="10">
+        <f>AVERAGE(G49:H49)</f>
+        <v/>
+      </c>
+      <c r="J49" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="K49" s="9" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="L49" s="10">
+        <f>AVERAGE(J49:K49)</f>
+        <v/>
+      </c>
+      <c r="M49" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N49" s="6" t="inlineStr">
+        <is>
+          <t>Second time cooking eggs dry - saves ~20-25 kcal versus pan oil</t>
         </is>
       </c>
     </row>
@@ -3149,11 +3204,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$48,Meals!$A$5:$A$48,$A5,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$49,Meals!$A$5:$A$49,$A5,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$48,Meals!$A$5:$A$48,$A5,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$49,Meals!$A$5:$A$49,$A5,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -3161,11 +3216,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$48,Meals!$A$5:$A$48,$A5,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$49,Meals!$A$5:$A$49,$A5,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$48,Meals!$A$5:$A$48,$A5,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$49,Meals!$A$5:$A$49,$A5,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -3173,11 +3228,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$48,Meals!$A$5:$A$48,$A5,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$49,Meals!$A$5:$A$49,$A5,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$48,Meals!$A$5:$A$48,$A5,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$49,Meals!$A$5:$A$49,$A5,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -3185,11 +3240,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$48,$A5,Meals!$M$5:$M$48,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$49,$A5,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$48,$A5,Meals!$M$5:$M$48,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$49,$A5,Meals!$M$5:$M$49,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -3202,11 +3257,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$48,Meals!$A$5:$A$48,$A6,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$49,Meals!$A$5:$A$49,$A6,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$48,Meals!$A$5:$A$48,$A6,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$49,Meals!$A$5:$A$49,$A6,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -3214,11 +3269,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$48,Meals!$A$5:$A$48,$A6,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$49,Meals!$A$5:$A$49,$A6,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$48,Meals!$A$5:$A$48,$A6,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$49,Meals!$A$5:$A$49,$A6,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -3226,11 +3281,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$48,Meals!$A$5:$A$48,$A6,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$49,Meals!$A$5:$A$49,$A6,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$48,Meals!$A$5:$A$48,$A6,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$49,Meals!$A$5:$A$49,$A6,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -3238,11 +3293,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$48,$A6,Meals!$M$5:$M$48,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$49,$A6,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$48,$A6,Meals!$M$5:$M$48,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$49,$A6,Meals!$M$5:$M$49,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -3255,11 +3310,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$48,Meals!$A$5:$A$48,$A7,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$49,Meals!$A$5:$A$49,$A7,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$48,Meals!$A$5:$A$48,$A7,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$49,Meals!$A$5:$A$49,$A7,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -3267,11 +3322,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$48,Meals!$A$5:$A$48,$A7,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$49,Meals!$A$5:$A$49,$A7,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$48,Meals!$A$5:$A$48,$A7,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$49,Meals!$A$5:$A$49,$A7,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -3279,11 +3334,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$48,Meals!$A$5:$A$48,$A7,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$49,Meals!$A$5:$A$49,$A7,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$48,Meals!$A$5:$A$48,$A7,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$49,Meals!$A$5:$A$49,$A7,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -3291,11 +3346,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$48,$A7,Meals!$M$5:$M$48,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$49,$A7,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$48,$A7,Meals!$M$5:$M$48,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$49,$A7,Meals!$M$5:$M$49,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -3308,11 +3363,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$48,Meals!$A$5:$A$48,$A8,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$49,Meals!$A$5:$A$49,$A8,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$48,Meals!$A$5:$A$48,$A8,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$49,Meals!$A$5:$A$49,$A8,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -3320,11 +3375,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$48,Meals!$A$5:$A$48,$A8,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$49,Meals!$A$5:$A$49,$A8,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$48,Meals!$A$5:$A$48,$A8,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$49,Meals!$A$5:$A$49,$A8,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -3332,11 +3387,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$48,Meals!$A$5:$A$48,$A8,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$49,Meals!$A$5:$A$49,$A8,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$48,Meals!$A$5:$A$48,$A8,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$49,Meals!$A$5:$A$49,$A8,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -3344,11 +3399,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$48,$A8,Meals!$M$5:$M$48,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$49,$A8,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$48,$A8,Meals!$M$5:$M$48,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$49,$A8,Meals!$M$5:$M$49,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -3361,11 +3416,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$48,Meals!$A$5:$A$48,$A9,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$49,Meals!$A$5:$A$49,$A9,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$48,Meals!$A$5:$A$48,$A9,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$49,Meals!$A$5:$A$49,$A9,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -3373,11 +3428,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$48,Meals!$A$5:$A$48,$A9,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$49,Meals!$A$5:$A$49,$A9,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$48,Meals!$A$5:$A$48,$A9,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$49,Meals!$A$5:$A$49,$A9,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -3385,11 +3440,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$48,Meals!$A$5:$A$48,$A9,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$49,Meals!$A$5:$A$49,$A9,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$48,Meals!$A$5:$A$48,$A9,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$49,Meals!$A$5:$A$49,$A9,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -3397,11 +3452,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$48,$A9,Meals!$M$5:$M$48,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$49,$A9,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$48,$A9,Meals!$M$5:$M$48,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$49,$A9,Meals!$M$5:$M$49,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -3414,11 +3469,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$48,Meals!$A$5:$A$48,$A10,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$49,Meals!$A$5:$A$49,$A10,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$48,Meals!$A$5:$A$48,$A10,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$49,Meals!$A$5:$A$49,$A10,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -3426,11 +3481,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$48,Meals!$A$5:$A$48,$A10,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$49,Meals!$A$5:$A$49,$A10,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$48,Meals!$A$5:$A$48,$A10,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$49,Meals!$A$5:$A$49,$A10,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -3438,11 +3493,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$48,Meals!$A$5:$A$48,$A10,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$49,Meals!$A$5:$A$49,$A10,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$48,Meals!$A$5:$A$48,$A10,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$49,Meals!$A$5:$A$49,$A10,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -3450,11 +3505,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$48,$A10,Meals!$M$5:$M$48,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$49,$A10,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$48,$A10,Meals!$M$5:$M$48,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$49,$A10,Meals!$M$5:$M$49,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -3467,11 +3522,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$48,Meals!$A$5:$A$48,$A11,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$49,Meals!$A$5:$A$49,$A11,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$48,Meals!$A$5:$A$48,$A11,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$49,Meals!$A$5:$A$49,$A11,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -3479,11 +3534,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$48,Meals!$A$5:$A$48,$A11,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$49,Meals!$A$5:$A$49,$A11,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$48,Meals!$A$5:$A$48,$A11,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$49,Meals!$A$5:$A$49,$A11,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -3491,11 +3546,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$48,Meals!$A$5:$A$48,$A11,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$49,Meals!$A$5:$A$49,$A11,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$48,Meals!$A$5:$A$48,$A11,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$49,Meals!$A$5:$A$49,$A11,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -3503,11 +3558,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$48,$A11,Meals!$M$5:$M$48,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$49,$A11,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$48,$A11,Meals!$M$5:$M$48,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$49,$A11,Meals!$M$5:$M$49,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -3520,11 +3575,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$48,Meals!$A$5:$A$48,$A12,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$49,Meals!$A$5:$A$49,$A12,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$48,Meals!$A$5:$A$48,$A12,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$49,Meals!$A$5:$A$49,$A12,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -3532,11 +3587,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$48,Meals!$A$5:$A$48,$A12,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$49,Meals!$A$5:$A$49,$A12,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$48,Meals!$A$5:$A$48,$A12,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$49,Meals!$A$5:$A$49,$A12,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -3544,11 +3599,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$48,Meals!$A$5:$A$48,$A12,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$49,Meals!$A$5:$A$49,$A12,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$48,Meals!$A$5:$A$48,$A12,Meals!$M$5:$M$48,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$49,Meals!$A$5:$A$49,$A12,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -3556,11 +3611,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$48,$A12,Meals!$M$5:$M$48,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$49,$A12,Meals!$M$5:$M$49,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$48,$A12,Meals!$M$5:$M$48,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$49,$A12,Meals!$M$5:$M$49,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">

</xml_diff>

<commit_message>
Log Friday lunch: halved biriyani with 3 boiled eggs
700-954 kcal (mid 827), 45-57 g protein, 35-53 g fat. Rice halved as planned
and three eggs added, putting Day 8 at 1,381 kcal and 69.75 g protein by
lunch.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N49"/>
+  <dimension ref="A1:N50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3083,6 +3083,61 @@
       <c r="N49" s="6" t="inlineStr">
         <is>
           <t>Second time cooking eggs dry - saves ~20-25 kcal versus pan oil</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>Chicken biriyani with rice halved + 2 chicken pieces + 3 boiled eggs + curd salad</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="n">
+        <v>700</v>
+      </c>
+      <c r="E50" s="7" t="n">
+        <v>954</v>
+      </c>
+      <c r="F50" s="8">
+        <f>AVERAGE(D50:E50)</f>
+        <v/>
+      </c>
+      <c r="G50" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="H50" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="I50" s="10">
+        <f>AVERAGE(G50:H50)</f>
+        <v/>
+      </c>
+      <c r="J50" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="K50" s="9" t="n">
+        <v>53</v>
+      </c>
+      <c r="L50" s="10">
+        <f>AVERAGE(J50:K50)</f>
+        <v/>
+      </c>
+      <c r="M50" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N50" s="6" t="inlineStr">
+        <is>
+          <t>Rice halved; 3 eggs added</t>
         </is>
       </c>
     </row>
@@ -3204,11 +3259,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$49,Meals!$A$5:$A$49,$A5,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$50,Meals!$A$5:$A$50,$A5,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$49,Meals!$A$5:$A$49,$A5,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$50,Meals!$A$5:$A$50,$A5,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -3216,11 +3271,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$49,Meals!$A$5:$A$49,$A5,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$50,Meals!$A$5:$A$50,$A5,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$49,Meals!$A$5:$A$49,$A5,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$50,Meals!$A$5:$A$50,$A5,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -3228,11 +3283,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$49,Meals!$A$5:$A$49,$A5,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$50,Meals!$A$5:$A$50,$A5,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$49,Meals!$A$5:$A$49,$A5,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$50,Meals!$A$5:$A$50,$A5,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -3240,11 +3295,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$49,$A5,Meals!$M$5:$M$49,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$50,$A5,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$49,$A5,Meals!$M$5:$M$49,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$50,$A5,Meals!$M$5:$M$50,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -3257,11 +3312,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$49,Meals!$A$5:$A$49,$A6,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$50,Meals!$A$5:$A$50,$A6,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$49,Meals!$A$5:$A$49,$A6,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$50,Meals!$A$5:$A$50,$A6,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -3269,11 +3324,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$49,Meals!$A$5:$A$49,$A6,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$50,Meals!$A$5:$A$50,$A6,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$49,Meals!$A$5:$A$49,$A6,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$50,Meals!$A$5:$A$50,$A6,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -3281,11 +3336,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$49,Meals!$A$5:$A$49,$A6,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$50,Meals!$A$5:$A$50,$A6,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$49,Meals!$A$5:$A$49,$A6,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$50,Meals!$A$5:$A$50,$A6,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -3293,11 +3348,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$49,$A6,Meals!$M$5:$M$49,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$50,$A6,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$49,$A6,Meals!$M$5:$M$49,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$50,$A6,Meals!$M$5:$M$50,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -3310,11 +3365,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$49,Meals!$A$5:$A$49,$A7,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$50,Meals!$A$5:$A$50,$A7,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$49,Meals!$A$5:$A$49,$A7,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$50,Meals!$A$5:$A$50,$A7,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -3322,11 +3377,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$49,Meals!$A$5:$A$49,$A7,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$50,Meals!$A$5:$A$50,$A7,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$49,Meals!$A$5:$A$49,$A7,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$50,Meals!$A$5:$A$50,$A7,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -3334,11 +3389,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$49,Meals!$A$5:$A$49,$A7,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$50,Meals!$A$5:$A$50,$A7,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$49,Meals!$A$5:$A$49,$A7,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$50,Meals!$A$5:$A$50,$A7,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -3346,11 +3401,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$49,$A7,Meals!$M$5:$M$49,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$50,$A7,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$49,$A7,Meals!$M$5:$M$49,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$50,$A7,Meals!$M$5:$M$50,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -3363,11 +3418,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$49,Meals!$A$5:$A$49,$A8,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$50,Meals!$A$5:$A$50,$A8,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$49,Meals!$A$5:$A$49,$A8,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$50,Meals!$A$5:$A$50,$A8,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -3375,11 +3430,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$49,Meals!$A$5:$A$49,$A8,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$50,Meals!$A$5:$A$50,$A8,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$49,Meals!$A$5:$A$49,$A8,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$50,Meals!$A$5:$A$50,$A8,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -3387,11 +3442,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$49,Meals!$A$5:$A$49,$A8,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$50,Meals!$A$5:$A$50,$A8,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$49,Meals!$A$5:$A$49,$A8,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$50,Meals!$A$5:$A$50,$A8,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -3399,11 +3454,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$49,$A8,Meals!$M$5:$M$49,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$50,$A8,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$49,$A8,Meals!$M$5:$M$49,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$50,$A8,Meals!$M$5:$M$50,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -3416,11 +3471,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$49,Meals!$A$5:$A$49,$A9,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$50,Meals!$A$5:$A$50,$A9,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$49,Meals!$A$5:$A$49,$A9,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$50,Meals!$A$5:$A$50,$A9,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -3428,11 +3483,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$49,Meals!$A$5:$A$49,$A9,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$50,Meals!$A$5:$A$50,$A9,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$49,Meals!$A$5:$A$49,$A9,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$50,Meals!$A$5:$A$50,$A9,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -3440,11 +3495,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$49,Meals!$A$5:$A$49,$A9,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$50,Meals!$A$5:$A$50,$A9,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$49,Meals!$A$5:$A$49,$A9,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$50,Meals!$A$5:$A$50,$A9,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -3452,11 +3507,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$49,$A9,Meals!$M$5:$M$49,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$50,$A9,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$49,$A9,Meals!$M$5:$M$49,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$50,$A9,Meals!$M$5:$M$50,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -3469,11 +3524,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$49,Meals!$A$5:$A$49,$A10,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$50,Meals!$A$5:$A$50,$A10,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$49,Meals!$A$5:$A$49,$A10,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$50,Meals!$A$5:$A$50,$A10,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -3481,11 +3536,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$49,Meals!$A$5:$A$49,$A10,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$50,Meals!$A$5:$A$50,$A10,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$49,Meals!$A$5:$A$49,$A10,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$50,Meals!$A$5:$A$50,$A10,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -3493,11 +3548,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$49,Meals!$A$5:$A$49,$A10,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$50,Meals!$A$5:$A$50,$A10,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$49,Meals!$A$5:$A$49,$A10,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$50,Meals!$A$5:$A$50,$A10,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -3505,11 +3560,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$49,$A10,Meals!$M$5:$M$49,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$50,$A10,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$49,$A10,Meals!$M$5:$M$49,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$50,$A10,Meals!$M$5:$M$50,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -3522,11 +3577,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$49,Meals!$A$5:$A$49,$A11,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$50,Meals!$A$5:$A$50,$A11,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$49,Meals!$A$5:$A$49,$A11,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$50,Meals!$A$5:$A$50,$A11,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -3534,11 +3589,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$49,Meals!$A$5:$A$49,$A11,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$50,Meals!$A$5:$A$50,$A11,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$49,Meals!$A$5:$A$49,$A11,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$50,Meals!$A$5:$A$50,$A11,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -3546,11 +3601,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$49,Meals!$A$5:$A$49,$A11,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$50,Meals!$A$5:$A$50,$A11,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$49,Meals!$A$5:$A$49,$A11,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$50,Meals!$A$5:$A$50,$A11,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -3558,11 +3613,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$49,$A11,Meals!$M$5:$M$49,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$50,$A11,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$49,$A11,Meals!$M$5:$M$49,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$50,$A11,Meals!$M$5:$M$50,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -3575,11 +3630,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$49,Meals!$A$5:$A$49,$A12,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$50,Meals!$A$5:$A$50,$A12,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$49,Meals!$A$5:$A$49,$A12,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$50,Meals!$A$5:$A$50,$A12,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -3587,11 +3642,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$49,Meals!$A$5:$A$49,$A12,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$50,Meals!$A$5:$A$50,$A12,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$49,Meals!$A$5:$A$49,$A12,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$50,Meals!$A$5:$A$50,$A12,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -3599,11 +3654,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$49,Meals!$A$5:$A$49,$A12,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$50,Meals!$A$5:$A$50,$A12,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$49,Meals!$A$5:$A$49,$A12,Meals!$M$5:$M$49,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$50,Meals!$A$5:$A$50,$A12,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -3611,11 +3666,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$49,$A12,Meals!$M$5:$M$49,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$50,$A12,Meals!$M$5:$M$50,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$49,$A12,Meals!$M$5:$M$49,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$50,$A12,Meals!$M$5:$M$50,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">

</xml_diff>

<commit_message>
Add whole grilled chicken to the reference estimates
Skin eaten 1,200-1,600 kcal for ~125-140 g protein; skin removed 750-900
kcal for ~120-135 g. Half a skinless bird, 375-450 kcal for ~60-68 g, is
the realistic portion at 15.6 g of protein per 100 kcal.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -5364,7 +5364,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -6106,14 +6106,14 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Garlic sauce / toum (1 tbsp)</t>
+          <t>Whole grilled chicken - skin eaten</t>
         </is>
       </c>
       <c r="B31" s="7" t="n">
-        <v>90</v>
+        <v>1200</v>
       </c>
       <c r="C31" s="7" t="n">
-        <v>110</v>
+        <v>1600</v>
       </c>
       <c r="D31" s="8">
         <f>AVERAGE(B31:C31)</f>
@@ -6121,26 +6121,26 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>0 g</t>
+          <t>~125-140 g</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>Essentially emulsified oil - the hidden cost at a grill</t>
+          <t>A 900-1200 g raw bird. Skin carries most of the fat</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Khubz / pita (1 large)</t>
+          <t>Whole grilled chicken - skin removed</t>
         </is>
       </c>
       <c r="B32" s="7" t="n">
-        <v>250</v>
+        <v>750</v>
       </c>
       <c r="C32" s="7" t="n">
-        <v>300</v>
+        <v>900</v>
       </c>
       <c r="D32" s="8">
         <f>AVERAGE(B32:C32)</f>
@@ -6148,22 +6148,26 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>~8-9 g</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="inlineStr"/>
+          <t>~120-135 g</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>Same protein for roughly half the calories</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Barik/basmati rice (half container cooked)</t>
+          <t>Half grilled chicken - skin removed</t>
         </is>
       </c>
       <c r="B33" s="7" t="n">
-        <v>200</v>
+        <v>375</v>
       </c>
       <c r="C33" s="7" t="n">
-        <v>280</v>
+        <v>450</v>
       </c>
       <c r="D33" s="8">
         <f>AVERAGE(B33:C33)</f>
@@ -6171,22 +6175,26 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>~4-5 g</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="inlineStr"/>
+          <t>~60-68 g</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>The realistic single portion; 15.6 g protein per 100 kcal</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Fresh pineapple juice (350-450 ml)</t>
+          <t>Garlic sauce / toum (1 tbsp)</t>
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>175</v>
+        <v>90</v>
       </c>
       <c r="C34" s="7" t="n">
-        <v>240</v>
+        <v>110</v>
       </c>
       <c r="D34" s="8">
         <f>AVERAGE(B34:C34)</f>
@@ -6194,26 +6202,26 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>~1-2 g</t>
+          <t>0 g</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>No added sugar but ~35-45 g natural sugar; no fibre; almost no protein</t>
+          <t>Essentially emulsified oil - the hidden cost at a grill</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Fresh orange juice (350-450 ml)</t>
+          <t>Khubz / pita (1 large)</t>
         </is>
       </c>
       <c r="B35" s="7" t="n">
-        <v>155</v>
+        <v>250</v>
       </c>
       <c r="C35" s="7" t="n">
-        <v>205</v>
+        <v>300</v>
       </c>
       <c r="D35" s="8">
         <f>AVERAGE(B35:C35)</f>
@@ -6221,26 +6229,22 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>~2-3 g</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="inlineStr">
-        <is>
-          <t>No added sugar but ~32-40 g natural sugar; no fibre</t>
-        </is>
-      </c>
+          <t>~8-9 g</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in water)</t>
+          <t>Barik/basmati rice (half container cooked)</t>
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="C36" s="7" t="n">
-        <v>120</v>
+        <v>280</v>
       </c>
       <c r="D36" s="8">
         <f>AVERAGE(B36:C36)</f>
@@ -6248,7 +6252,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
+          <t>~4-5 g</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr"/>
@@ -6256,14 +6260,14 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Greek yogurt (200 g plain low-fat)</t>
+          <t>Fresh pineapple juice (350-450 ml)</t>
         </is>
       </c>
       <c r="B37" s="7" t="n">
-        <v>120</v>
+        <v>175</v>
       </c>
       <c r="C37" s="7" t="n">
-        <v>140</v>
+        <v>240</v>
       </c>
       <c r="D37" s="8">
         <f>AVERAGE(B37:C37)</f>
@@ -6271,26 +6275,26 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>~18-20 g</t>
+          <t>~1-2 g</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>Casein - digests slowly; good overnight</t>
+          <t>No added sugar but ~35-45 g natural sugar; no fibre; almost no protein</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>Boiled egg (1 large)</t>
+          <t>Fresh orange juice (350-450 ml)</t>
         </is>
       </c>
       <c r="B38" s="7" t="n">
-        <v>70</v>
+        <v>155</v>
       </c>
       <c r="C38" s="7" t="n">
-        <v>78</v>
+        <v>205</v>
       </c>
       <c r="D38" s="8">
         <f>AVERAGE(B38:C38)</f>
@@ -6298,26 +6302,26 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>~6-6.5 g</t>
+          <t>~2-3 g</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>~5 g fat each</t>
+          <t>No added sugar but ~32-40 g natural sugar; no fibre</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>Egg fried dry with no oil (1)</t>
+          <t>Whey scoop (in water)</t>
         </is>
       </c>
       <c r="B39" s="7" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="C39" s="7" t="n">
-        <v>78</v>
+        <v>120</v>
       </c>
       <c r="D39" s="8">
         <f>AVERAGE(B39:C39)</f>
@@ -6325,26 +6329,22 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>~6-6.5 g</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="inlineStr">
-        <is>
-          <t>Same as boiled - dry-frying saves the ~20-25 kcal per egg that pan oil adds</t>
-        </is>
-      </c>
+          <t>~20-25 g</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>Paneer (50 g full-fat)</t>
+          <t>Greek yogurt (200 g plain low-fat)</t>
         </is>
       </c>
       <c r="B40" s="7" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="C40" s="7" t="n">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="D40" s="8">
         <f>AVERAGE(B40:C40)</f>
@@ -6352,26 +6352,26 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>~8-9 g</t>
+          <t>~18-20 g</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>Fat-dense for the protein it gives</t>
+          <t>Casein - digests slowly; good overnight</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>Cucumber (1 medium)</t>
+          <t>Boiled egg (1 large)</t>
         </is>
       </c>
       <c r="B41" s="7" t="n">
-        <v>25</v>
+        <v>70</v>
       </c>
       <c r="C41" s="7" t="n">
-        <v>30</v>
+        <v>78</v>
       </c>
       <c r="D41" s="8">
         <f>AVERAGE(B41:C41)</f>
@@ -6379,26 +6379,26 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>~1.5 g</t>
+          <t>~6-6.5 g</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
-          <t>Volume with almost no calories</t>
+          <t>~5 g fat each</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Sweet melon / cantaloupe (1 wedge ~100-150 g)</t>
+          <t>Egg fried dry with no oil (1)</t>
         </is>
       </c>
       <c r="B42" s="7" t="n">
-        <v>35</v>
+        <v>70</v>
       </c>
       <c r="C42" s="7" t="n">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="D42" s="8">
         <f>AVERAGE(B42:C42)</f>
@@ -6406,26 +6406,26 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>~0.5-1 g</t>
+          <t>~6-6.5 g</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>Whole fruit - fibre and water intact; ~1/4 the calories of the same fruit juiced</t>
+          <t>Same as boiled - dry-frying saves the ~20-25 kcal per egg that pan oil adds</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>Grapes (~100 g / 15-20 grapes)</t>
+          <t>Paneer (50 g full-fat)</t>
         </is>
       </c>
       <c r="B43" s="7" t="n">
-        <v>60</v>
+        <v>130</v>
       </c>
       <c r="C43" s="7" t="n">
-        <v>75</v>
+        <v>150</v>
       </c>
       <c r="D43" s="8">
         <f>AVERAGE(B43:C43)</f>
@@ -6433,26 +6433,26 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>~0.6 g</t>
+          <t>~8-9 g</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t>Twice the calorie density of melon; easy to eat a large handful without noticing</t>
+          <t>Fat-dense for the protein it gives</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>Mango misiri (1 whole ~450-600 g)</t>
+          <t>Cucumber (1 medium)</t>
         </is>
       </c>
       <c r="B44" s="7" t="n">
-        <v>170</v>
+        <v>25</v>
       </c>
       <c r="C44" s="7" t="n">
-        <v>230</v>
+        <v>30</v>
       </c>
       <c r="D44" s="8">
         <f>AVERAGE(B44:C44)</f>
@@ -6460,26 +6460,26 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>~2-2.5 g</t>
+          <t>~1.5 g</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t>~60-65% is edible flesh; ~35-50 g sugar but fibre intact</t>
+          <t>Volume with almost no calories</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Diet/zero-sugar soft drink (330 ml)</t>
+          <t>Sweet melon / cantaloupe (1 wedge ~100-150 g)</t>
         </is>
       </c>
       <c r="B45" s="7" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="C45" s="7" t="n">
-        <v>2</v>
+        <v>55</v>
       </c>
       <c r="D45" s="8">
         <f>AVERAGE(B45:C45)</f>
@@ -6487,26 +6487,26 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>0 g</t>
+          <t>~0.5-1 g</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
         <is>
-          <t>Genuinely zero - unlike fruit juice sold as no added sugar</t>
+          <t>Whole fruit - fibre and water intact; ~1/4 the calories of the same fruit juiced</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in black coffee no sugar)</t>
+          <t>Grapes (~100 g / 15-20 grapes)</t>
         </is>
       </c>
       <c r="B46" s="7" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="C46" s="7" t="n">
-        <v>130</v>
+        <v>75</v>
       </c>
       <c r="D46" s="8">
         <f>AVERAGE(B46:C46)</f>
@@ -6514,22 +6514,26 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F46" s="6" t="inlineStr"/>
+          <t>~0.6 g</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>Twice the calorie density of melon; easy to eat a large handful without noticing</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>Cashew/almond biscuit (1)</t>
+          <t>Mango misiri (1 whole ~450-600 g)</t>
         </is>
       </c>
       <c r="B47" s="7" t="n">
-        <v>38</v>
+        <v>170</v>
       </c>
       <c r="C47" s="7" t="n">
-        <v>38</v>
+        <v>230</v>
       </c>
       <c r="D47" s="8">
         <f>AVERAGE(B47:C47)</f>
@@ -6537,22 +6541,26 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>~0.5 g</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="inlineStr"/>
+          <t>~2-2.5 g</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="inlineStr">
+        <is>
+          <t>~60-65% is edible flesh; ~35-50 g sugar but fibre intact</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (~50g standard)</t>
+          <t>Diet/zero-sugar soft drink (330 ml)</t>
         </is>
       </c>
       <c r="B48" s="7" t="n">
-        <v>245</v>
+        <v>0</v>
       </c>
       <c r="C48" s="7" t="n">
-        <v>250</v>
+        <v>2</v>
       </c>
       <c r="D48" s="8">
         <f>AVERAGE(B48:C48)</f>
@@ -6560,22 +6568,26 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>~4 g</t>
-        </is>
-      </c>
-      <c r="F48" s="6" t="inlineStr"/>
+          <t>0 g</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>Genuinely zero - unlike fruit juice sold as no added sugar</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (70g king-size)</t>
+          <t>Whey scoop (in black coffee no sugar)</t>
         </is>
       </c>
       <c r="B49" s="7" t="n">
-        <v>335</v>
+        <v>100</v>
       </c>
       <c r="C49" s="7" t="n">
-        <v>335</v>
+        <v>130</v>
       </c>
       <c r="D49" s="8">
         <f>AVERAGE(B49:C49)</f>
@@ -6583,7 +6595,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>~6 g</t>
+          <t>~20-25 g</t>
         </is>
       </c>
       <c r="F49" s="6" t="inlineStr"/>
@@ -6591,14 +6603,14 @@
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>Pre-workout scoop</t>
+          <t>Cashew/almond biscuit (1)</t>
         </is>
       </c>
       <c r="B50" s="7" t="n">
-        <v>5</v>
+        <v>38</v>
       </c>
       <c r="C50" s="7" t="n">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D50" s="8">
         <f>AVERAGE(B50:C50)</f>
@@ -6606,10 +6618,79 @@
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
+          <t>~0.5 g</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>Chocolate bar (~50g standard)</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="n">
+        <v>245</v>
+      </c>
+      <c r="C51" s="7" t="n">
+        <v>250</v>
+      </c>
+      <c r="D51" s="8">
+        <f>AVERAGE(B51:C51)</f>
+        <v/>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>~4 g</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>Chocolate bar (70g king-size)</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="n">
+        <v>335</v>
+      </c>
+      <c r="C52" s="7" t="n">
+        <v>335</v>
+      </c>
+      <c r="D52" s="8">
+        <f>AVERAGE(B52:C52)</f>
+        <v/>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>~6 g</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>Pre-workout scoop</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C53" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D53" s="8">
+        <f>AVERAGE(B53:C53)</f>
+        <v/>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
           <t>0 g</t>
         </is>
       </c>
-      <c r="F50" s="6" t="inlineStr">
+      <c r="F53" s="6" t="inlineStr">
         <is>
           <t>Negligible</t>
         </is>

</xml_diff>

<commit_message>
Log Day 9 breakfast and plan the Saturday menu
Saturday is one of the two tight days on the mess menu (2,100 kcal as
served). The dosa-set breakfast came in at 480 rather than the menu's
545 because the coconut chutney was skipped for the fifth time in nine
days.

The second cut Saturday needs is the roasted-coconut varutharachathu
gravy, not a chapati: lifting the chicken out of it saves ~100 kcal and
~11 g of fat for ~2 g of protein.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N50"/>
+  <dimension ref="A1:N51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3141,6 +3141,61 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" s="4" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>Breakfast</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>2 set dosa + sambar + red chutney (coconut chutney skipped)</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="n">
+        <v>410</v>
+      </c>
+      <c r="E51" s="7" t="n">
+        <v>550</v>
+      </c>
+      <c r="F51" s="8">
+        <f>AVERAGE(D51:E51)</f>
+        <v/>
+      </c>
+      <c r="G51" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="H51" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="I51" s="10">
+        <f>AVERAGE(G51:H51)</f>
+        <v/>
+      </c>
+      <c r="J51" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="K51" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="L51" s="10">
+        <f>AVERAGE(J51:K51)</f>
+        <v/>
+      </c>
+      <c r="M51" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N51" s="6" t="inlineStr">
+        <is>
+          <t>Fifth skip of the coconut chutney in nine days</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:N2"/>
@@ -3155,7 +3210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3259,11 +3314,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$50,Meals!$A$5:$A$50,$A5,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$51,Meals!$A$5:$A$51,$A5,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$50,Meals!$A$5:$A$50,$A5,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$51,Meals!$A$5:$A$51,$A5,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -3271,11 +3326,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$50,Meals!$A$5:$A$50,$A5,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$51,Meals!$A$5:$A$51,$A5,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$50,Meals!$A$5:$A$50,$A5,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$51,Meals!$A$5:$A$51,$A5,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -3283,11 +3338,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$50,Meals!$A$5:$A$50,$A5,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$51,Meals!$A$5:$A$51,$A5,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$50,Meals!$A$5:$A$50,$A5,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$51,Meals!$A$5:$A$51,$A5,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -3295,11 +3350,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$50,$A5,Meals!$M$5:$M$50,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$51,$A5,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$50,$A5,Meals!$M$5:$M$50,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$51,$A5,Meals!$M$5:$M$51,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -3312,11 +3367,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$50,Meals!$A$5:$A$50,$A6,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$51,Meals!$A$5:$A$51,$A6,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$50,Meals!$A$5:$A$50,$A6,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$51,Meals!$A$5:$A$51,$A6,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -3324,11 +3379,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$50,Meals!$A$5:$A$50,$A6,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$51,Meals!$A$5:$A$51,$A6,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$50,Meals!$A$5:$A$50,$A6,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$51,Meals!$A$5:$A$51,$A6,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -3336,11 +3391,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$50,Meals!$A$5:$A$50,$A6,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$51,Meals!$A$5:$A$51,$A6,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$50,Meals!$A$5:$A$50,$A6,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$51,Meals!$A$5:$A$51,$A6,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -3348,11 +3403,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$50,$A6,Meals!$M$5:$M$50,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$51,$A6,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$50,$A6,Meals!$M$5:$M$50,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$51,$A6,Meals!$M$5:$M$51,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -3365,11 +3420,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$50,Meals!$A$5:$A$50,$A7,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$51,Meals!$A$5:$A$51,$A7,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$50,Meals!$A$5:$A$50,$A7,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$51,Meals!$A$5:$A$51,$A7,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -3377,11 +3432,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$50,Meals!$A$5:$A$50,$A7,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$51,Meals!$A$5:$A$51,$A7,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$50,Meals!$A$5:$A$50,$A7,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$51,Meals!$A$5:$A$51,$A7,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -3389,11 +3444,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$50,Meals!$A$5:$A$50,$A7,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$51,Meals!$A$5:$A$51,$A7,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$50,Meals!$A$5:$A$50,$A7,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$51,Meals!$A$5:$A$51,$A7,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -3401,11 +3456,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$50,$A7,Meals!$M$5:$M$50,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$51,$A7,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$50,$A7,Meals!$M$5:$M$50,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$51,$A7,Meals!$M$5:$M$51,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -3418,11 +3473,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$50,Meals!$A$5:$A$50,$A8,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$51,Meals!$A$5:$A$51,$A8,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$50,Meals!$A$5:$A$50,$A8,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$51,Meals!$A$5:$A$51,$A8,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -3430,11 +3485,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$50,Meals!$A$5:$A$50,$A8,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$51,Meals!$A$5:$A$51,$A8,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$50,Meals!$A$5:$A$50,$A8,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$51,Meals!$A$5:$A$51,$A8,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -3442,11 +3497,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$50,Meals!$A$5:$A$50,$A8,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$51,Meals!$A$5:$A$51,$A8,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$50,Meals!$A$5:$A$50,$A8,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$51,Meals!$A$5:$A$51,$A8,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -3454,11 +3509,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$50,$A8,Meals!$M$5:$M$50,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$51,$A8,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$50,$A8,Meals!$M$5:$M$50,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$51,$A8,Meals!$M$5:$M$51,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -3471,11 +3526,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$50,Meals!$A$5:$A$50,$A9,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$51,Meals!$A$5:$A$51,$A9,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$50,Meals!$A$5:$A$50,$A9,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$51,Meals!$A$5:$A$51,$A9,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -3483,11 +3538,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$50,Meals!$A$5:$A$50,$A9,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$51,Meals!$A$5:$A$51,$A9,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$50,Meals!$A$5:$A$50,$A9,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$51,Meals!$A$5:$A$51,$A9,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -3495,11 +3550,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$50,Meals!$A$5:$A$50,$A9,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$51,Meals!$A$5:$A$51,$A9,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$50,Meals!$A$5:$A$50,$A9,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$51,Meals!$A$5:$A$51,$A9,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -3507,11 +3562,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$50,$A9,Meals!$M$5:$M$50,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$51,$A9,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$50,$A9,Meals!$M$5:$M$50,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$51,$A9,Meals!$M$5:$M$51,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -3524,11 +3579,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$50,Meals!$A$5:$A$50,$A10,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$51,Meals!$A$5:$A$51,$A10,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$50,Meals!$A$5:$A$50,$A10,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$51,Meals!$A$5:$A$51,$A10,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -3536,11 +3591,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$50,Meals!$A$5:$A$50,$A10,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$51,Meals!$A$5:$A$51,$A10,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$50,Meals!$A$5:$A$50,$A10,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$51,Meals!$A$5:$A$51,$A10,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -3548,11 +3603,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$50,Meals!$A$5:$A$50,$A10,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$51,Meals!$A$5:$A$51,$A10,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$50,Meals!$A$5:$A$50,$A10,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$51,Meals!$A$5:$A$51,$A10,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -3560,11 +3615,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$50,$A10,Meals!$M$5:$M$50,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$51,$A10,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$50,$A10,Meals!$M$5:$M$50,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$51,$A10,Meals!$M$5:$M$51,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -3577,11 +3632,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$50,Meals!$A$5:$A$50,$A11,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$51,Meals!$A$5:$A$51,$A11,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$50,Meals!$A$5:$A$50,$A11,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$51,Meals!$A$5:$A$51,$A11,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -3589,11 +3644,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$50,Meals!$A$5:$A$50,$A11,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$51,Meals!$A$5:$A$51,$A11,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$50,Meals!$A$5:$A$50,$A11,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$51,Meals!$A$5:$A$51,$A11,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -3601,11 +3656,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$50,Meals!$A$5:$A$50,$A11,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$51,Meals!$A$5:$A$51,$A11,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$50,Meals!$A$5:$A$50,$A11,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$51,Meals!$A$5:$A$51,$A11,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -3613,11 +3668,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$50,$A11,Meals!$M$5:$M$50,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$51,$A11,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$50,$A11,Meals!$M$5:$M$50,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$51,$A11,Meals!$M$5:$M$51,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -3630,11 +3685,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$50,Meals!$A$5:$A$50,$A12,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$51,Meals!$A$5:$A$51,$A12,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$50,Meals!$A$5:$A$50,$A12,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$51,Meals!$A$5:$A$51,$A12,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -3642,11 +3697,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$50,Meals!$A$5:$A$50,$A12,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$51,Meals!$A$5:$A$51,$A12,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$50,Meals!$A$5:$A$50,$A12,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$51,Meals!$A$5:$A$51,$A12,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -3654,11 +3709,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$50,Meals!$A$5:$A$50,$A12,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$51,Meals!$A$5:$A$51,$A12,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$50,Meals!$A$5:$A$50,$A12,Meals!$M$5:$M$50,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$51,Meals!$A$5:$A$51,$A12,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -3666,15 +3721,68 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$50,$A12,Meals!$M$5:$M$50,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$51,$A12,Meals!$M$5:$M$51,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$50,$A12,Meals!$M$5:$M$50,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$51,$A12,Meals!$M$5:$M$51,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
         <f>D12-Targets!$B$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="18" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B13" s="8">
+        <f>SUMIFS(Meals!$D$5:$D$51,Meals!$A$5:$A$51,$A13,Meals!$M$5:$M$51,"logged")</f>
+        <v/>
+      </c>
+      <c r="C13" s="8">
+        <f>SUMIFS(Meals!$E$5:$E$51,Meals!$A$5:$A$51,$A13,Meals!$M$5:$M$51,"logged")</f>
+        <v/>
+      </c>
+      <c r="D13" s="8">
+        <f>AVERAGE(B13:C13)</f>
+        <v/>
+      </c>
+      <c r="E13" s="10">
+        <f>SUMIFS(Meals!$G$5:$G$51,Meals!$A$5:$A$51,$A13,Meals!$M$5:$M$51,"logged")</f>
+        <v/>
+      </c>
+      <c r="F13" s="10">
+        <f>SUMIFS(Meals!$H$5:$H$51,Meals!$A$5:$A$51,$A13,Meals!$M$5:$M$51,"logged")</f>
+        <v/>
+      </c>
+      <c r="G13" s="10">
+        <f>AVERAGE(E13:F13)</f>
+        <v/>
+      </c>
+      <c r="H13" s="10">
+        <f>SUMIFS(Meals!$J$5:$J$51,Meals!$A$5:$A$51,$A13,Meals!$M$5:$M$51,"logged")</f>
+        <v/>
+      </c>
+      <c r="I13" s="10">
+        <f>SUMIFS(Meals!$K$5:$K$51,Meals!$A$5:$A$51,$A13,Meals!$M$5:$M$51,"logged")</f>
+        <v/>
+      </c>
+      <c r="J13" s="10">
+        <f>AVERAGE(H13:I13)</f>
+        <v/>
+      </c>
+      <c r="K13" s="18">
+        <f>COUNTIFS(Meals!$A$5:$A$51,$A13,Meals!$M$5:$M$51,"logged")</f>
+        <v/>
+      </c>
+      <c r="L13" s="18">
+        <f>COUNTIFS(Meals!$A$5:$A$51,$A13,Meals!$M$5:$M$51,"pending")</f>
+        <v/>
+      </c>
+      <c r="M13" s="19">
+        <f>D13-Targets!$B$16</f>
         <v/>
       </c>
     </row>
@@ -4608,7 +4716,7 @@
         </is>
       </c>
       <c r="B5" s="18">
-        <f>COUNT(Daily!$A$5:$A$12)</f>
+        <f>COUNT(Daily!$A$5:$A$13)</f>
         <v/>
       </c>
     </row>
@@ -4619,7 +4727,7 @@
         </is>
       </c>
       <c r="B6" s="8">
-        <f>IFERROR(AVERAGE(Daily!$D$5:$D$12),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$D$5:$D$13),0)</f>
         <v/>
       </c>
     </row>
@@ -4630,7 +4738,7 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>IFERROR(AVERAGE(Daily!$G$5:$G$12),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$G$5:$G$13),0)</f>
         <v/>
       </c>
     </row>
@@ -4641,7 +4749,7 @@
         </is>
       </c>
       <c r="B8" s="10">
-        <f>IFERROR(AVERAGE(Daily!$J$5:$J$12),0)</f>
+        <f>IFERROR(AVERAGE(Daily!$J$5:$J$13),0)</f>
         <v/>
       </c>
     </row>
@@ -4685,7 +4793,7 @@
         </is>
       </c>
       <c r="B12" s="18">
-        <f>COUNTIFS(Daily!$G$5:$G$12,"&gt;="&amp;Targets!$B$20)</f>
+        <f>COUNTIFS(Daily!$G$5:$G$13,"&gt;="&amp;Targets!$B$20)</f>
         <v/>
       </c>
     </row>
@@ -4696,7 +4804,7 @@
         </is>
       </c>
       <c r="B13" s="18">
-        <f>SUM(Daily!$L$5:$L$12)</f>
+        <f>SUM(Daily!$L$5:$L$13)</f>
         <v/>
       </c>
     </row>
@@ -4747,19 +4855,19 @@
         <v>46271</v>
       </c>
       <c r="C17" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$12,"&gt;="&amp;$A17,Daily!$A$5:$A$12,"&lt;="&amp;$B17)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$13,"&gt;="&amp;$A17,Daily!$A$5:$A$13,"&lt;="&amp;$B17)</f>
         <v/>
       </c>
       <c r="D17" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$12,Daily!$A$5:$A$12,"&gt;="&amp;$A17,Daily!$A$5:$A$12,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$13,Daily!$A$5:$A$13,"&gt;="&amp;$A17,Daily!$A$5:$A$13,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="E17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$12,Daily!$A$5:$A$12,"&gt;="&amp;$A17,Daily!$A$5:$A$12,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$13,Daily!$A$5:$A$13,"&gt;="&amp;$A17,Daily!$A$5:$A$13,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$12,Daily!$A$5:$A$12,"&gt;="&amp;$A17,Daily!$A$5:$A$12,"&lt;="&amp;$B17),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$13,Daily!$A$5:$A$13,"&gt;="&amp;$A17,Daily!$A$5:$A$13,"&lt;="&amp;$B17),0)</f>
         <v/>
       </c>
     </row>
@@ -4771,19 +4879,19 @@
         <v>46278</v>
       </c>
       <c r="C18" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$12,"&gt;="&amp;$A18,Daily!$A$5:$A$12,"&lt;="&amp;$B18)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$13,"&gt;="&amp;$A18,Daily!$A$5:$A$13,"&lt;="&amp;$B18)</f>
         <v/>
       </c>
       <c r="D18" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$12,Daily!$A$5:$A$12,"&gt;="&amp;$A18,Daily!$A$5:$A$12,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$13,Daily!$A$5:$A$13,"&gt;="&amp;$A18,Daily!$A$5:$A$13,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="E18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$12,Daily!$A$5:$A$12,"&gt;="&amp;$A18,Daily!$A$5:$A$12,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$13,Daily!$A$5:$A$13,"&gt;="&amp;$A18,Daily!$A$5:$A$13,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
       <c r="F18" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$12,Daily!$A$5:$A$12,"&gt;="&amp;$A18,Daily!$A$5:$A$12,"&lt;="&amp;$B18),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$13,Daily!$A$5:$A$13,"&gt;="&amp;$A18,Daily!$A$5:$A$13,"&lt;="&amp;$B18),0)</f>
         <v/>
       </c>
     </row>
@@ -4834,19 +4942,19 @@
         <v>46295</v>
       </c>
       <c r="C22" s="18">
-        <f>COUNTIFS(Daily!$A$5:$A$12,"&gt;="&amp;$A22,Daily!$A$5:$A$12,"&lt;="&amp;$B22)</f>
+        <f>COUNTIFS(Daily!$A$5:$A$13,"&gt;="&amp;$A22,Daily!$A$5:$A$13,"&lt;="&amp;$B22)</f>
         <v/>
       </c>
       <c r="D22" s="8">
-        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$12,Daily!$A$5:$A$12,"&gt;="&amp;$A22,Daily!$A$5:$A$12,"&lt;="&amp;$B22),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$D$5:$D$13,Daily!$A$5:$A$13,"&gt;="&amp;$A22,Daily!$A$5:$A$13,"&lt;="&amp;$B22),0)</f>
         <v/>
       </c>
       <c r="E22" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$12,Daily!$A$5:$A$12,"&gt;="&amp;$A22,Daily!$A$5:$A$12,"&lt;="&amp;$B22),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$G$5:$G$13,Daily!$A$5:$A$13,"&gt;="&amp;$A22,Daily!$A$5:$A$13,"&lt;="&amp;$B22),0)</f>
         <v/>
       </c>
       <c r="F22" s="10">
-        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$12,Daily!$A$5:$A$12,"&gt;="&amp;$A22,Daily!$A$5:$A$12,"&lt;="&amp;$B22),0)</f>
+        <f>IFERROR(AVERAGEIFS(Daily!$J$5:$J$13,Daily!$A$5:$A$13,"&gt;="&amp;$A22,Daily!$A$5:$A$13,"&lt;="&amp;$B22),0)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Log Day 9 lunch: halved meals plate with 2 eggs and fried fish
Both levers again - rice halved, 2 boiled eggs added. Revises the
Saturday plan: 825 kcal and 80.5 g of protein left, which lands on 3
scoops rather than 2 once the varutharachathu gravy is left behind.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N51"/>
+  <dimension ref="A1:N52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3193,6 +3193,61 @@
       <c r="N51" s="6" t="inlineStr">
         <is>
           <t>Fifth skip of the coconut chutney in nine days</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>Mess meals plate (rice halved) + 2 boiled eggs + 1 fried fish piece + sambar, curd, veg sides</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="n">
+        <v>665</v>
+      </c>
+      <c r="E52" s="7" t="n">
+        <v>965</v>
+      </c>
+      <c r="F52" s="8">
+        <f>AVERAGE(D52:E52)</f>
+        <v/>
+      </c>
+      <c r="G52" s="9" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="H52" s="9" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="I52" s="10">
+        <f>AVERAGE(G52:H52)</f>
+        <v/>
+      </c>
+      <c r="J52" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="K52" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="L52" s="10">
+        <f>AVERAGE(J52:K52)</f>
+        <v/>
+      </c>
+      <c r="M52" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N52" s="6" t="inlineStr">
+        <is>
+          <t>Rice halved and 2 eggs added - both levers again</t>
         </is>
       </c>
     </row>
@@ -3314,11 +3369,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$51,Meals!$A$5:$A$51,$A5,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$52,Meals!$A$5:$A$52,$A5,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$51,Meals!$A$5:$A$51,$A5,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$52,Meals!$A$5:$A$52,$A5,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -3326,11 +3381,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$51,Meals!$A$5:$A$51,$A5,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$52,Meals!$A$5:$A$52,$A5,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$51,Meals!$A$5:$A$51,$A5,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$52,Meals!$A$5:$A$52,$A5,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -3338,11 +3393,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$51,Meals!$A$5:$A$51,$A5,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$52,Meals!$A$5:$A$52,$A5,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$51,Meals!$A$5:$A$51,$A5,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$52,Meals!$A$5:$A$52,$A5,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -3350,11 +3405,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$51,$A5,Meals!$M$5:$M$51,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$52,$A5,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$51,$A5,Meals!$M$5:$M$51,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$52,$A5,Meals!$M$5:$M$52,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -3367,11 +3422,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$51,Meals!$A$5:$A$51,$A6,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$52,Meals!$A$5:$A$52,$A6,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$51,Meals!$A$5:$A$51,$A6,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$52,Meals!$A$5:$A$52,$A6,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -3379,11 +3434,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$51,Meals!$A$5:$A$51,$A6,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$52,Meals!$A$5:$A$52,$A6,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$51,Meals!$A$5:$A$51,$A6,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$52,Meals!$A$5:$A$52,$A6,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -3391,11 +3446,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$51,Meals!$A$5:$A$51,$A6,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$52,Meals!$A$5:$A$52,$A6,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$51,Meals!$A$5:$A$51,$A6,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$52,Meals!$A$5:$A$52,$A6,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -3403,11 +3458,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$51,$A6,Meals!$M$5:$M$51,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$52,$A6,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$51,$A6,Meals!$M$5:$M$51,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$52,$A6,Meals!$M$5:$M$52,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -3420,11 +3475,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$51,Meals!$A$5:$A$51,$A7,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$52,Meals!$A$5:$A$52,$A7,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$51,Meals!$A$5:$A$51,$A7,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$52,Meals!$A$5:$A$52,$A7,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -3432,11 +3487,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$51,Meals!$A$5:$A$51,$A7,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$52,Meals!$A$5:$A$52,$A7,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$51,Meals!$A$5:$A$51,$A7,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$52,Meals!$A$5:$A$52,$A7,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -3444,11 +3499,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$51,Meals!$A$5:$A$51,$A7,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$52,Meals!$A$5:$A$52,$A7,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$51,Meals!$A$5:$A$51,$A7,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$52,Meals!$A$5:$A$52,$A7,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -3456,11 +3511,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$51,$A7,Meals!$M$5:$M$51,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$52,$A7,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$51,$A7,Meals!$M$5:$M$51,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$52,$A7,Meals!$M$5:$M$52,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -3473,11 +3528,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$51,Meals!$A$5:$A$51,$A8,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$52,Meals!$A$5:$A$52,$A8,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$51,Meals!$A$5:$A$51,$A8,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$52,Meals!$A$5:$A$52,$A8,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -3485,11 +3540,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$51,Meals!$A$5:$A$51,$A8,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$52,Meals!$A$5:$A$52,$A8,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$51,Meals!$A$5:$A$51,$A8,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$52,Meals!$A$5:$A$52,$A8,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -3497,11 +3552,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$51,Meals!$A$5:$A$51,$A8,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$52,Meals!$A$5:$A$52,$A8,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$51,Meals!$A$5:$A$51,$A8,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$52,Meals!$A$5:$A$52,$A8,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -3509,11 +3564,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$51,$A8,Meals!$M$5:$M$51,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$52,$A8,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$51,$A8,Meals!$M$5:$M$51,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$52,$A8,Meals!$M$5:$M$52,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -3526,11 +3581,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$51,Meals!$A$5:$A$51,$A9,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$52,Meals!$A$5:$A$52,$A9,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$51,Meals!$A$5:$A$51,$A9,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$52,Meals!$A$5:$A$52,$A9,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -3538,11 +3593,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$51,Meals!$A$5:$A$51,$A9,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$52,Meals!$A$5:$A$52,$A9,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$51,Meals!$A$5:$A$51,$A9,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$52,Meals!$A$5:$A$52,$A9,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -3550,11 +3605,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$51,Meals!$A$5:$A$51,$A9,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$52,Meals!$A$5:$A$52,$A9,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$51,Meals!$A$5:$A$51,$A9,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$52,Meals!$A$5:$A$52,$A9,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -3562,11 +3617,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$51,$A9,Meals!$M$5:$M$51,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$52,$A9,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$51,$A9,Meals!$M$5:$M$51,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$52,$A9,Meals!$M$5:$M$52,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -3579,11 +3634,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$51,Meals!$A$5:$A$51,$A10,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$52,Meals!$A$5:$A$52,$A10,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$51,Meals!$A$5:$A$51,$A10,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$52,Meals!$A$5:$A$52,$A10,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -3591,11 +3646,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$51,Meals!$A$5:$A$51,$A10,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$52,Meals!$A$5:$A$52,$A10,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$51,Meals!$A$5:$A$51,$A10,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$52,Meals!$A$5:$A$52,$A10,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -3603,11 +3658,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$51,Meals!$A$5:$A$51,$A10,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$52,Meals!$A$5:$A$52,$A10,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$51,Meals!$A$5:$A$51,$A10,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$52,Meals!$A$5:$A$52,$A10,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -3615,11 +3670,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$51,$A10,Meals!$M$5:$M$51,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$52,$A10,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$51,$A10,Meals!$M$5:$M$51,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$52,$A10,Meals!$M$5:$M$52,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -3632,11 +3687,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$51,Meals!$A$5:$A$51,$A11,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$52,Meals!$A$5:$A$52,$A11,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$51,Meals!$A$5:$A$51,$A11,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$52,Meals!$A$5:$A$52,$A11,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -3644,11 +3699,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$51,Meals!$A$5:$A$51,$A11,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$52,Meals!$A$5:$A$52,$A11,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$51,Meals!$A$5:$A$51,$A11,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$52,Meals!$A$5:$A$52,$A11,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -3656,11 +3711,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$51,Meals!$A$5:$A$51,$A11,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$52,Meals!$A$5:$A$52,$A11,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$51,Meals!$A$5:$A$51,$A11,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$52,Meals!$A$5:$A$52,$A11,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -3668,11 +3723,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$51,$A11,Meals!$M$5:$M$51,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$52,$A11,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$51,$A11,Meals!$M$5:$M$51,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$52,$A11,Meals!$M$5:$M$52,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -3685,11 +3740,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$51,Meals!$A$5:$A$51,$A12,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$52,Meals!$A$5:$A$52,$A12,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$51,Meals!$A$5:$A$51,$A12,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$52,Meals!$A$5:$A$52,$A12,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -3697,11 +3752,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$51,Meals!$A$5:$A$51,$A12,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$52,Meals!$A$5:$A$52,$A12,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$51,Meals!$A$5:$A$51,$A12,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$52,Meals!$A$5:$A$52,$A12,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -3709,11 +3764,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$51,Meals!$A$5:$A$51,$A12,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$52,Meals!$A$5:$A$52,$A12,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$51,Meals!$A$5:$A$51,$A12,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$52,Meals!$A$5:$A$52,$A12,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -3721,11 +3776,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$51,$A12,Meals!$M$5:$M$51,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$52,$A12,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$51,$A12,Meals!$M$5:$M$51,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$52,$A12,Meals!$M$5:$M$52,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -3738,11 +3793,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$51,Meals!$A$5:$A$51,$A13,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$52,Meals!$A$5:$A$52,$A13,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$51,Meals!$A$5:$A$51,$A13,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$52,Meals!$A$5:$A$52,$A13,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -3750,11 +3805,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$51,Meals!$A$5:$A$51,$A13,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$52,Meals!$A$5:$A$52,$A13,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$51,Meals!$A$5:$A$51,$A13,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$52,Meals!$A$5:$A$52,$A13,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -3762,11 +3817,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$51,Meals!$A$5:$A$51,$A13,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$52,Meals!$A$5:$A$52,$A13,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$51,Meals!$A$5:$A$51,$A13,Meals!$M$5:$M$51,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$52,Meals!$A$5:$A$52,$A13,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -3774,11 +3829,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$51,$A13,Meals!$M$5:$M$51,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$52,$A13,Meals!$M$5:$M$52,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$51,$A13,Meals!$M$5:$M$51,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$52,$A13,Meals!$M$5:$M$52,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">

</xml_diff>

<commit_message>
Log 2 boiled eggs on Day 9 and drop the evening to 2 scoops
The afternoon eggs take the third scoop's place: 677 kcal and 68 g of
protein left rather than 825 and 80.5. Adds a note on the fat cost of
reaching the protein floor with eggs instead of whey.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N52"/>
+  <dimension ref="A1:N53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3248,6 +3248,61 @@
       <c r="N52" s="6" t="inlineStr">
         <is>
           <t>Rice halved and 2 eggs added - both levers again</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>2 boiled eggs</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="n">
+        <v>140</v>
+      </c>
+      <c r="E53" s="7" t="n">
+        <v>156</v>
+      </c>
+      <c r="F53" s="8">
+        <f>AVERAGE(D53:E53)</f>
+        <v/>
+      </c>
+      <c r="G53" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="H53" s="9" t="n">
+        <v>13</v>
+      </c>
+      <c r="I53" s="10">
+        <f>AVERAGE(G53:H53)</f>
+        <v/>
+      </c>
+      <c r="J53" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="K53" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="L53" s="10">
+        <f>AVERAGE(J53:K53)</f>
+        <v/>
+      </c>
+      <c r="M53" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N53" s="6" t="inlineStr">
+        <is>
+          <t>Eggs 3 and 4 of the day</t>
         </is>
       </c>
     </row>
@@ -3369,11 +3424,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$52,Meals!$A$5:$A$52,$A5,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$53,Meals!$A$5:$A$53,$A5,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$52,Meals!$A$5:$A$52,$A5,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$53,Meals!$A$5:$A$53,$A5,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -3381,11 +3436,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$52,Meals!$A$5:$A$52,$A5,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$53,Meals!$A$5:$A$53,$A5,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$52,Meals!$A$5:$A$52,$A5,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$53,Meals!$A$5:$A$53,$A5,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -3393,11 +3448,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$52,Meals!$A$5:$A$52,$A5,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$53,Meals!$A$5:$A$53,$A5,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$52,Meals!$A$5:$A$52,$A5,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$53,Meals!$A$5:$A$53,$A5,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -3405,11 +3460,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$52,$A5,Meals!$M$5:$M$52,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$53,$A5,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$52,$A5,Meals!$M$5:$M$52,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$53,$A5,Meals!$M$5:$M$53,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -3422,11 +3477,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$52,Meals!$A$5:$A$52,$A6,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$53,Meals!$A$5:$A$53,$A6,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$52,Meals!$A$5:$A$52,$A6,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$53,Meals!$A$5:$A$53,$A6,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -3434,11 +3489,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$52,Meals!$A$5:$A$52,$A6,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$53,Meals!$A$5:$A$53,$A6,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$52,Meals!$A$5:$A$52,$A6,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$53,Meals!$A$5:$A$53,$A6,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -3446,11 +3501,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$52,Meals!$A$5:$A$52,$A6,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$53,Meals!$A$5:$A$53,$A6,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$52,Meals!$A$5:$A$52,$A6,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$53,Meals!$A$5:$A$53,$A6,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -3458,11 +3513,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$52,$A6,Meals!$M$5:$M$52,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$53,$A6,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$52,$A6,Meals!$M$5:$M$52,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$53,$A6,Meals!$M$5:$M$53,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -3475,11 +3530,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$52,Meals!$A$5:$A$52,$A7,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$53,Meals!$A$5:$A$53,$A7,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$52,Meals!$A$5:$A$52,$A7,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$53,Meals!$A$5:$A$53,$A7,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -3487,11 +3542,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$52,Meals!$A$5:$A$52,$A7,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$53,Meals!$A$5:$A$53,$A7,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$52,Meals!$A$5:$A$52,$A7,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$53,Meals!$A$5:$A$53,$A7,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -3499,11 +3554,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$52,Meals!$A$5:$A$52,$A7,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$53,Meals!$A$5:$A$53,$A7,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$52,Meals!$A$5:$A$52,$A7,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$53,Meals!$A$5:$A$53,$A7,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -3511,11 +3566,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$52,$A7,Meals!$M$5:$M$52,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$53,$A7,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$52,$A7,Meals!$M$5:$M$52,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$53,$A7,Meals!$M$5:$M$53,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -3528,11 +3583,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$52,Meals!$A$5:$A$52,$A8,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$53,Meals!$A$5:$A$53,$A8,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$52,Meals!$A$5:$A$52,$A8,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$53,Meals!$A$5:$A$53,$A8,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -3540,11 +3595,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$52,Meals!$A$5:$A$52,$A8,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$53,Meals!$A$5:$A$53,$A8,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$52,Meals!$A$5:$A$52,$A8,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$53,Meals!$A$5:$A$53,$A8,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -3552,11 +3607,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$52,Meals!$A$5:$A$52,$A8,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$53,Meals!$A$5:$A$53,$A8,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$52,Meals!$A$5:$A$52,$A8,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$53,Meals!$A$5:$A$53,$A8,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -3564,11 +3619,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$52,$A8,Meals!$M$5:$M$52,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$53,$A8,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$52,$A8,Meals!$M$5:$M$52,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$53,$A8,Meals!$M$5:$M$53,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -3581,11 +3636,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$52,Meals!$A$5:$A$52,$A9,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$53,Meals!$A$5:$A$53,$A9,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$52,Meals!$A$5:$A$52,$A9,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$53,Meals!$A$5:$A$53,$A9,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -3593,11 +3648,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$52,Meals!$A$5:$A$52,$A9,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$53,Meals!$A$5:$A$53,$A9,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$52,Meals!$A$5:$A$52,$A9,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$53,Meals!$A$5:$A$53,$A9,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -3605,11 +3660,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$52,Meals!$A$5:$A$52,$A9,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$53,Meals!$A$5:$A$53,$A9,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$52,Meals!$A$5:$A$52,$A9,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$53,Meals!$A$5:$A$53,$A9,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -3617,11 +3672,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$52,$A9,Meals!$M$5:$M$52,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$53,$A9,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$52,$A9,Meals!$M$5:$M$52,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$53,$A9,Meals!$M$5:$M$53,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -3634,11 +3689,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$52,Meals!$A$5:$A$52,$A10,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$53,Meals!$A$5:$A$53,$A10,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$52,Meals!$A$5:$A$52,$A10,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$53,Meals!$A$5:$A$53,$A10,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -3646,11 +3701,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$52,Meals!$A$5:$A$52,$A10,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$53,Meals!$A$5:$A$53,$A10,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$52,Meals!$A$5:$A$52,$A10,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$53,Meals!$A$5:$A$53,$A10,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -3658,11 +3713,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$52,Meals!$A$5:$A$52,$A10,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$53,Meals!$A$5:$A$53,$A10,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$52,Meals!$A$5:$A$52,$A10,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$53,Meals!$A$5:$A$53,$A10,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -3670,11 +3725,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$52,$A10,Meals!$M$5:$M$52,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$53,$A10,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$52,$A10,Meals!$M$5:$M$52,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$53,$A10,Meals!$M$5:$M$53,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -3687,11 +3742,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$52,Meals!$A$5:$A$52,$A11,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$53,Meals!$A$5:$A$53,$A11,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$52,Meals!$A$5:$A$52,$A11,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$53,Meals!$A$5:$A$53,$A11,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -3699,11 +3754,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$52,Meals!$A$5:$A$52,$A11,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$53,Meals!$A$5:$A$53,$A11,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$52,Meals!$A$5:$A$52,$A11,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$53,Meals!$A$5:$A$53,$A11,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -3711,11 +3766,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$52,Meals!$A$5:$A$52,$A11,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$53,Meals!$A$5:$A$53,$A11,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$52,Meals!$A$5:$A$52,$A11,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$53,Meals!$A$5:$A$53,$A11,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -3723,11 +3778,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$52,$A11,Meals!$M$5:$M$52,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$53,$A11,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$52,$A11,Meals!$M$5:$M$52,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$53,$A11,Meals!$M$5:$M$53,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -3740,11 +3795,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$52,Meals!$A$5:$A$52,$A12,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$53,Meals!$A$5:$A$53,$A12,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$52,Meals!$A$5:$A$52,$A12,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$53,Meals!$A$5:$A$53,$A12,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -3752,11 +3807,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$52,Meals!$A$5:$A$52,$A12,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$53,Meals!$A$5:$A$53,$A12,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$52,Meals!$A$5:$A$52,$A12,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$53,Meals!$A$5:$A$53,$A12,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -3764,11 +3819,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$52,Meals!$A$5:$A$52,$A12,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$53,Meals!$A$5:$A$53,$A12,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$52,Meals!$A$5:$A$52,$A12,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$53,Meals!$A$5:$A$53,$A12,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -3776,11 +3831,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$52,$A12,Meals!$M$5:$M$52,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$53,$A12,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$52,$A12,Meals!$M$5:$M$52,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$53,$A12,Meals!$M$5:$M$53,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -3793,11 +3848,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$52,Meals!$A$5:$A$52,$A13,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$53,Meals!$A$5:$A$53,$A13,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$52,Meals!$A$5:$A$52,$A13,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$53,Meals!$A$5:$A$53,$A13,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -3805,11 +3860,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$52,Meals!$A$5:$A$52,$A13,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$53,Meals!$A$5:$A$53,$A13,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$52,Meals!$A$5:$A$52,$A13,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$53,Meals!$A$5:$A$53,$A13,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -3817,11 +3872,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$52,Meals!$A$5:$A$52,$A13,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$53,Meals!$A$5:$A$53,$A13,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$52,Meals!$A$5:$A$52,$A13,Meals!$M$5:$M$52,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$53,Meals!$A$5:$A$53,$A13,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -3829,11 +3884,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$52,$A13,Meals!$M$5:$M$52,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$53,$A13,Meals!$M$5:$M$53,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$52,$A13,Meals!$M$5:$M$52,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$53,$A13,Meals!$M$5:$M$53,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">

</xml_diff>

<commit_message>
Log Day 9 dinner: 2 chapati with chicken varutharachathu
Smaller chicken portion than the menu assumes, so the meal lands under
the 500-710 estimate even with the gravy poured over. Closes the day on
2 scoops and breaks out where the day's ~102 g of fat came from.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N53"/>
+  <dimension ref="A1:N54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3202,39 +3202,39 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>Lunch</t>
+          <t>Dinner</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>Mess meals plate (rice halved) + 2 boiled eggs + 1 fried fish piece + sambar, curd, veg sides</t>
+          <t>2 chapati + chicken varutharachathu (gravy poured over)</t>
         </is>
       </c>
       <c r="D52" s="7" t="n">
-        <v>665</v>
+        <v>460</v>
       </c>
       <c r="E52" s="7" t="n">
-        <v>965</v>
+        <v>650</v>
       </c>
       <c r="F52" s="8">
         <f>AVERAGE(D52:E52)</f>
         <v/>
       </c>
       <c r="G52" s="9" t="n">
-        <v>31.5</v>
+        <v>23</v>
       </c>
       <c r="H52" s="9" t="n">
-        <v>42.5</v>
+        <v>32</v>
       </c>
       <c r="I52" s="10">
         <f>AVERAGE(G52:H52)</f>
         <v/>
       </c>
       <c r="J52" s="9" t="n">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="K52" s="9" t="n">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="L52" s="10">
         <f>AVERAGE(J52:K52)</f>
@@ -3247,7 +3247,7 @@
       </c>
       <c r="N52" s="6" t="inlineStr">
         <is>
-          <t>Rice halved and 2 eggs added - both levers again</t>
+          <t>Mess Saturday dinner; whole container poured on rather than the chicken lifted out</t>
         </is>
       </c>
     </row>
@@ -3257,39 +3257,39 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>Snack</t>
+          <t>Lunch</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>2 boiled eggs</t>
+          <t>Mess meals plate (rice halved) + 2 boiled eggs + 1 fried fish piece + sambar, curd, veg sides</t>
         </is>
       </c>
       <c r="D53" s="7" t="n">
-        <v>140</v>
+        <v>665</v>
       </c>
       <c r="E53" s="7" t="n">
-        <v>156</v>
+        <v>965</v>
       </c>
       <c r="F53" s="8">
         <f>AVERAGE(D53:E53)</f>
         <v/>
       </c>
       <c r="G53" s="9" t="n">
-        <v>12</v>
+        <v>31.5</v>
       </c>
       <c r="H53" s="9" t="n">
-        <v>13</v>
+        <v>42.5</v>
       </c>
       <c r="I53" s="10">
         <f>AVERAGE(G53:H53)</f>
         <v/>
       </c>
       <c r="J53" s="9" t="n">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="K53" s="9" t="n">
-        <v>11</v>
+        <v>50</v>
       </c>
       <c r="L53" s="10">
         <f>AVERAGE(J53:K53)</f>
@@ -3301,6 +3301,61 @@
         </is>
       </c>
       <c r="N53" s="6" t="inlineStr">
+        <is>
+          <t>Rice halved and 2 eggs added - both levers again</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Snack</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>2 boiled eggs</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="n">
+        <v>140</v>
+      </c>
+      <c r="E54" s="7" t="n">
+        <v>156</v>
+      </c>
+      <c r="F54" s="8">
+        <f>AVERAGE(D54:E54)</f>
+        <v/>
+      </c>
+      <c r="G54" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="H54" s="9" t="n">
+        <v>13</v>
+      </c>
+      <c r="I54" s="10">
+        <f>AVERAGE(G54:H54)</f>
+        <v/>
+      </c>
+      <c r="J54" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="K54" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="L54" s="10">
+        <f>AVERAGE(J54:K54)</f>
+        <v/>
+      </c>
+      <c r="M54" s="5" t="inlineStr">
+        <is>
+          <t>logged</t>
+        </is>
+      </c>
+      <c r="N54" s="6" t="inlineStr">
         <is>
           <t>Eggs 3 and 4 of the day</t>
         </is>
@@ -3424,11 +3479,11 @@
         <v>46269</v>
       </c>
       <c r="B5" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$53,Meals!$A$5:$A$53,$A5,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$54,Meals!$A$5:$A$54,$A5,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$53,Meals!$A$5:$A$53,$A5,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$54,Meals!$A$5:$A$54,$A5,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="D5" s="8">
@@ -3436,11 +3491,11 @@
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$53,Meals!$A$5:$A$53,$A5,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$54,Meals!$A$5:$A$54,$A5,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$53,Meals!$A$5:$A$53,$A5,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$54,Meals!$A$5:$A$54,$A5,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="G5" s="10">
@@ -3448,11 +3503,11 @@
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$53,Meals!$A$5:$A$53,$A5,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$54,Meals!$A$5:$A$54,$A5,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$53,Meals!$A$5:$A$53,$A5,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$54,Meals!$A$5:$A$54,$A5,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="J5" s="10">
@@ -3460,11 +3515,11 @@
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$53,$A5,Meals!$M$5:$M$53,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$54,$A5,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$53,$A5,Meals!$M$5:$M$53,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$54,$A5,Meals!$M$5:$M$54,"pending")</f>
         <v/>
       </c>
       <c r="M5" s="19">
@@ -3477,11 +3532,11 @@
         <v>46270</v>
       </c>
       <c r="B6" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$53,Meals!$A$5:$A$53,$A6,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$54,Meals!$A$5:$A$54,$A6,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="C6" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$53,Meals!$A$5:$A$53,$A6,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$54,Meals!$A$5:$A$54,$A6,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="D6" s="21">
@@ -3489,11 +3544,11 @@
         <v/>
       </c>
       <c r="E6" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$53,Meals!$A$5:$A$53,$A6,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$54,Meals!$A$5:$A$54,$A6,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="F6" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$53,Meals!$A$5:$A$53,$A6,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$54,Meals!$A$5:$A$54,$A6,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="G6" s="22">
@@ -3501,11 +3556,11 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$53,Meals!$A$5:$A$53,$A6,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$54,Meals!$A$5:$A$54,$A6,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="I6" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$53,Meals!$A$5:$A$53,$A6,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$54,Meals!$A$5:$A$54,$A6,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="J6" s="22">
@@ -3513,11 +3568,11 @@
         <v/>
       </c>
       <c r="K6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$53,$A6,Meals!$M$5:$M$53,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$54,$A6,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="L6" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$53,$A6,Meals!$M$5:$M$53,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$54,$A6,Meals!$M$5:$M$54,"pending")</f>
         <v/>
       </c>
       <c r="M6" s="23">
@@ -3530,11 +3585,11 @@
         <v>46271</v>
       </c>
       <c r="B7" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$53,Meals!$A$5:$A$53,$A7,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$54,Meals!$A$5:$A$54,$A7,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="C7" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$53,Meals!$A$5:$A$53,$A7,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$54,Meals!$A$5:$A$54,$A7,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="D7" s="8">
@@ -3542,11 +3597,11 @@
         <v/>
       </c>
       <c r="E7" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$53,Meals!$A$5:$A$53,$A7,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$54,Meals!$A$5:$A$54,$A7,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$53,Meals!$A$5:$A$53,$A7,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$54,Meals!$A$5:$A$54,$A7,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -3554,11 +3609,11 @@
         <v/>
       </c>
       <c r="H7" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$53,Meals!$A$5:$A$53,$A7,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$54,Meals!$A$5:$A$54,$A7,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="I7" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$53,Meals!$A$5:$A$53,$A7,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$54,Meals!$A$5:$A$54,$A7,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="J7" s="10">
@@ -3566,11 +3621,11 @@
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$53,$A7,Meals!$M$5:$M$53,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$54,$A7,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$53,$A7,Meals!$M$5:$M$53,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$54,$A7,Meals!$M$5:$M$54,"pending")</f>
         <v/>
       </c>
       <c r="M7" s="19">
@@ -3583,11 +3638,11 @@
         <v>46272</v>
       </c>
       <c r="B8" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$53,Meals!$A$5:$A$53,$A8,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$54,Meals!$A$5:$A$54,$A8,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="C8" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$53,Meals!$A$5:$A$53,$A8,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$54,Meals!$A$5:$A$54,$A8,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="D8" s="21">
@@ -3595,11 +3650,11 @@
         <v/>
       </c>
       <c r="E8" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$53,Meals!$A$5:$A$53,$A8,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$54,Meals!$A$5:$A$54,$A8,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="F8" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$53,Meals!$A$5:$A$53,$A8,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$54,Meals!$A$5:$A$54,$A8,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="G8" s="22">
@@ -3607,11 +3662,11 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$53,Meals!$A$5:$A$53,$A8,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$54,Meals!$A$5:$A$54,$A8,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="I8" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$53,Meals!$A$5:$A$53,$A8,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$54,Meals!$A$5:$A$54,$A8,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="J8" s="22">
@@ -3619,11 +3674,11 @@
         <v/>
       </c>
       <c r="K8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$53,$A8,Meals!$M$5:$M$53,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$54,$A8,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="L8" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$53,$A8,Meals!$M$5:$M$53,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$54,$A8,Meals!$M$5:$M$54,"pending")</f>
         <v/>
       </c>
       <c r="M8" s="23">
@@ -3636,11 +3691,11 @@
         <v>46273</v>
       </c>
       <c r="B9" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$53,Meals!$A$5:$A$53,$A9,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$54,Meals!$A$5:$A$54,$A9,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="C9" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$53,Meals!$A$5:$A$53,$A9,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$54,Meals!$A$5:$A$54,$A9,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="D9" s="8">
@@ -3648,11 +3703,11 @@
         <v/>
       </c>
       <c r="E9" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$53,Meals!$A$5:$A$53,$A9,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$54,Meals!$A$5:$A$54,$A9,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$53,Meals!$A$5:$A$53,$A9,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$54,Meals!$A$5:$A$54,$A9,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="G9" s="10">
@@ -3660,11 +3715,11 @@
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$53,Meals!$A$5:$A$53,$A9,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$54,Meals!$A$5:$A$54,$A9,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$53,Meals!$A$5:$A$53,$A9,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$54,Meals!$A$5:$A$54,$A9,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="J9" s="10">
@@ -3672,11 +3727,11 @@
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$53,$A9,Meals!$M$5:$M$53,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$54,$A9,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$53,$A9,Meals!$M$5:$M$53,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$54,$A9,Meals!$M$5:$M$54,"pending")</f>
         <v/>
       </c>
       <c r="M9" s="19">
@@ -3689,11 +3744,11 @@
         <v>46274</v>
       </c>
       <c r="B10" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$53,Meals!$A$5:$A$53,$A10,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$54,Meals!$A$5:$A$54,$A10,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="C10" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$53,Meals!$A$5:$A$53,$A10,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$54,Meals!$A$5:$A$54,$A10,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="D10" s="21">
@@ -3701,11 +3756,11 @@
         <v/>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$53,Meals!$A$5:$A$53,$A10,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$54,Meals!$A$5:$A$54,$A10,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="F10" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$53,Meals!$A$5:$A$53,$A10,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$54,Meals!$A$5:$A$54,$A10,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="G10" s="22">
@@ -3713,11 +3768,11 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$53,Meals!$A$5:$A$53,$A10,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$54,Meals!$A$5:$A$54,$A10,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="I10" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$53,Meals!$A$5:$A$53,$A10,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$54,Meals!$A$5:$A$54,$A10,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="J10" s="22">
@@ -3725,11 +3780,11 @@
         <v/>
       </c>
       <c r="K10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$53,$A10,Meals!$M$5:$M$53,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$54,$A10,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="L10" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$53,$A10,Meals!$M$5:$M$53,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$54,$A10,Meals!$M$5:$M$54,"pending")</f>
         <v/>
       </c>
       <c r="M10" s="23">
@@ -3742,11 +3797,11 @@
         <v>46275</v>
       </c>
       <c r="B11" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$53,Meals!$A$5:$A$53,$A11,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$54,Meals!$A$5:$A$54,$A11,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="C11" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$53,Meals!$A$5:$A$53,$A11,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$54,Meals!$A$5:$A$54,$A11,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="D11" s="8">
@@ -3754,11 +3809,11 @@
         <v/>
       </c>
       <c r="E11" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$53,Meals!$A$5:$A$53,$A11,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$54,Meals!$A$5:$A$54,$A11,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$53,Meals!$A$5:$A$53,$A11,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$54,Meals!$A$5:$A$54,$A11,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="G11" s="10">
@@ -3766,11 +3821,11 @@
         <v/>
       </c>
       <c r="H11" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$53,Meals!$A$5:$A$53,$A11,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$54,Meals!$A$5:$A$54,$A11,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="I11" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$53,Meals!$A$5:$A$53,$A11,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$54,Meals!$A$5:$A$54,$A11,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="J11" s="10">
@@ -3778,11 +3833,11 @@
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$53,$A11,Meals!$M$5:$M$53,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$54,$A11,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$53,$A11,Meals!$M$5:$M$53,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$54,$A11,Meals!$M$5:$M$54,"pending")</f>
         <v/>
       </c>
       <c r="M11" s="19">
@@ -3795,11 +3850,11 @@
         <v>46276</v>
       </c>
       <c r="B12" s="21">
-        <f>SUMIFS(Meals!$D$5:$D$53,Meals!$A$5:$A$53,$A12,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$54,Meals!$A$5:$A$54,$A12,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="C12" s="21">
-        <f>SUMIFS(Meals!$E$5:$E$53,Meals!$A$5:$A$53,$A12,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$54,Meals!$A$5:$A$54,$A12,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="D12" s="21">
@@ -3807,11 +3862,11 @@
         <v/>
       </c>
       <c r="E12" s="22">
-        <f>SUMIFS(Meals!$G$5:$G$53,Meals!$A$5:$A$53,$A12,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$54,Meals!$A$5:$A$54,$A12,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="F12" s="22">
-        <f>SUMIFS(Meals!$H$5:$H$53,Meals!$A$5:$A$53,$A12,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$54,Meals!$A$5:$A$54,$A12,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="G12" s="22">
@@ -3819,11 +3874,11 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>SUMIFS(Meals!$J$5:$J$53,Meals!$A$5:$A$53,$A12,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$54,Meals!$A$5:$A$54,$A12,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="I12" s="22">
-        <f>SUMIFS(Meals!$K$5:$K$53,Meals!$A$5:$A$53,$A12,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$54,Meals!$A$5:$A$54,$A12,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="J12" s="22">
@@ -3831,11 +3886,11 @@
         <v/>
       </c>
       <c r="K12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$53,$A12,Meals!$M$5:$M$53,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$54,$A12,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="L12" s="20">
-        <f>COUNTIFS(Meals!$A$5:$A$53,$A12,Meals!$M$5:$M$53,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$54,$A12,Meals!$M$5:$M$54,"pending")</f>
         <v/>
       </c>
       <c r="M12" s="23">
@@ -3848,11 +3903,11 @@
         <v>46277</v>
       </c>
       <c r="B13" s="8">
-        <f>SUMIFS(Meals!$D$5:$D$53,Meals!$A$5:$A$53,$A13,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$D$5:$D$54,Meals!$A$5:$A$54,$A13,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="C13" s="8">
-        <f>SUMIFS(Meals!$E$5:$E$53,Meals!$A$5:$A$53,$A13,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$E$5:$E$54,Meals!$A$5:$A$54,$A13,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="D13" s="8">
@@ -3860,11 +3915,11 @@
         <v/>
       </c>
       <c r="E13" s="10">
-        <f>SUMIFS(Meals!$G$5:$G$53,Meals!$A$5:$A$53,$A13,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$G$5:$G$54,Meals!$A$5:$A$54,$A13,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>SUMIFS(Meals!$H$5:$H$53,Meals!$A$5:$A$53,$A13,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$H$5:$H$54,Meals!$A$5:$A$54,$A13,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="G13" s="10">
@@ -3872,11 +3927,11 @@
         <v/>
       </c>
       <c r="H13" s="10">
-        <f>SUMIFS(Meals!$J$5:$J$53,Meals!$A$5:$A$53,$A13,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$J$5:$J$54,Meals!$A$5:$A$54,$A13,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="I13" s="10">
-        <f>SUMIFS(Meals!$K$5:$K$53,Meals!$A$5:$A$53,$A13,Meals!$M$5:$M$53,"logged")</f>
+        <f>SUMIFS(Meals!$K$5:$K$54,Meals!$A$5:$A$54,$A13,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="J13" s="10">
@@ -3884,11 +3939,11 @@
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$53,$A13,Meals!$M$5:$M$53,"logged")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$54,$A13,Meals!$M$5:$M$54,"logged")</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>COUNTIFS(Meals!$A$5:$A$53,$A13,Meals!$M$5:$M$53,"pending")</f>
+        <f>COUNTIFS(Meals!$A$5:$A$54,$A13,Meals!$M$5:$M$54,"pending")</f>
         <v/>
       </c>
       <c r="M13" s="19">

</xml_diff>

<commit_message>
Add skin-on half chicken and quarter chicken to the reference table
The reference only carried the skin-removed half. Skin on is what gets
served by default and costs ~290 kcal and ~29 g of fat for ~2 g of
protein.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SP9bAzZw74ZesxXqcjX75N
</commit_message>
<xml_diff>
--- a/nutrition/calorie_tracker.xlsx
+++ b/nutrition/calorie_tracker.xlsx
@@ -5637,7 +5637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -6460,14 +6460,14 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Garlic sauce / toum (1 tbsp)</t>
+          <t>Half grilled chicken - skin on</t>
         </is>
       </c>
       <c r="B34" s="7" t="n">
-        <v>90</v>
+        <v>600</v>
       </c>
       <c r="C34" s="7" t="n">
-        <v>110</v>
+        <v>800</v>
       </c>
       <c r="D34" s="8">
         <f>AVERAGE(B34:C34)</f>
@@ -6475,26 +6475,26 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>0 g</t>
+          <t>~62-70 g</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>Essentially emulsified oil - the hidden cost at a grill</t>
+          <t>As served. The skin adds ~290 kcal and ~29 g fat for ~2 g protein</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Khubz / pita (1 large)</t>
+          <t>Quarter grilled chicken - skin removed</t>
         </is>
       </c>
       <c r="B35" s="7" t="n">
-        <v>250</v>
+        <v>190</v>
       </c>
       <c r="C35" s="7" t="n">
-        <v>300</v>
+        <v>225</v>
       </c>
       <c r="D35" s="8">
         <f>AVERAGE(B35:C35)</f>
@@ -6502,22 +6502,26 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>~8-9 g</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="inlineStr"/>
+          <t>~30-34 g</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>Half the above; the size that fits inside a normal day</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>Barik/basmati rice (half container cooked)</t>
+          <t>Garlic sauce / toum (1 tbsp)</t>
         </is>
       </c>
       <c r="B36" s="7" t="n">
-        <v>200</v>
+        <v>90</v>
       </c>
       <c r="C36" s="7" t="n">
-        <v>280</v>
+        <v>110</v>
       </c>
       <c r="D36" s="8">
         <f>AVERAGE(B36:C36)</f>
@@ -6525,22 +6529,26 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>~4-5 g</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="inlineStr"/>
+          <t>0 g</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>Essentially emulsified oil - the hidden cost at a grill</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Fresh pineapple juice (350-450 ml)</t>
+          <t>Khubz / pita (1 large)</t>
         </is>
       </c>
       <c r="B37" s="7" t="n">
-        <v>175</v>
+        <v>250</v>
       </c>
       <c r="C37" s="7" t="n">
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="D37" s="8">
         <f>AVERAGE(B37:C37)</f>
@@ -6548,26 +6556,22 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>~1-2 g</t>
-        </is>
-      </c>
-      <c r="F37" s="6" t="inlineStr">
-        <is>
-          <t>No added sugar but ~35-45 g natural sugar; no fibre; almost no protein</t>
-        </is>
-      </c>
+          <t>~8-9 g</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>Fresh orange juice (350-450 ml)</t>
+          <t>Barik/basmati rice (half container cooked)</t>
         </is>
       </c>
       <c r="B38" s="7" t="n">
-        <v>155</v>
+        <v>200</v>
       </c>
       <c r="C38" s="7" t="n">
-        <v>205</v>
+        <v>280</v>
       </c>
       <c r="D38" s="8">
         <f>AVERAGE(B38:C38)</f>
@@ -6575,26 +6579,22 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>~2-3 g</t>
-        </is>
-      </c>
-      <c r="F38" s="6" t="inlineStr">
-        <is>
-          <t>No added sugar but ~32-40 g natural sugar; no fibre</t>
-        </is>
-      </c>
+          <t>~4-5 g</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in water)</t>
+          <t>Fresh pineapple juice (350-450 ml)</t>
         </is>
       </c>
       <c r="B39" s="7" t="n">
-        <v>100</v>
+        <v>175</v>
       </c>
       <c r="C39" s="7" t="n">
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="D39" s="8">
         <f>AVERAGE(B39:C39)</f>
@@ -6602,22 +6602,26 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="inlineStr"/>
+          <t>~1-2 g</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>No added sugar but ~35-45 g natural sugar; no fibre; almost no protein</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>Greek yogurt (200 g plain low-fat)</t>
+          <t>Fresh orange juice (350-450 ml)</t>
         </is>
       </c>
       <c r="B40" s="7" t="n">
-        <v>120</v>
+        <v>155</v>
       </c>
       <c r="C40" s="7" t="n">
-        <v>140</v>
+        <v>205</v>
       </c>
       <c r="D40" s="8">
         <f>AVERAGE(B40:C40)</f>
@@ -6625,26 +6629,26 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>~18-20 g</t>
+          <t>~2-3 g</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>Casein - digests slowly; good overnight</t>
+          <t>No added sugar but ~32-40 g natural sugar; no fibre</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>Boiled egg (1 large)</t>
+          <t>Whey scoop (in water)</t>
         </is>
       </c>
       <c r="B41" s="7" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="C41" s="7" t="n">
-        <v>78</v>
+        <v>120</v>
       </c>
       <c r="D41" s="8">
         <f>AVERAGE(B41:C41)</f>
@@ -6652,26 +6656,22 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>~6-6.5 g</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="inlineStr">
-        <is>
-          <t>~5 g fat each</t>
-        </is>
-      </c>
+          <t>~20-25 g</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Egg fried dry with no oil (1)</t>
+          <t>Greek yogurt (200 g plain low-fat)</t>
         </is>
       </c>
       <c r="B42" s="7" t="n">
-        <v>70</v>
+        <v>120</v>
       </c>
       <c r="C42" s="7" t="n">
-        <v>78</v>
+        <v>140</v>
       </c>
       <c r="D42" s="8">
         <f>AVERAGE(B42:C42)</f>
@@ -6679,26 +6679,26 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>~6-6.5 g</t>
+          <t>~18-20 g</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>Same as boiled - dry-frying saves the ~20-25 kcal per egg that pan oil adds</t>
+          <t>Casein - digests slowly; good overnight</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>Paneer (50 g full-fat)</t>
+          <t>Boiled egg (1 large)</t>
         </is>
       </c>
       <c r="B43" s="7" t="n">
-        <v>130</v>
+        <v>70</v>
       </c>
       <c r="C43" s="7" t="n">
-        <v>150</v>
+        <v>78</v>
       </c>
       <c r="D43" s="8">
         <f>AVERAGE(B43:C43)</f>
@@ -6706,26 +6706,26 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>~8-9 g</t>
+          <t>~6-6.5 g</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t>Fat-dense for the protein it gives</t>
+          <t>~5 g fat each</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>Cucumber (1 medium)</t>
+          <t>Egg fried dry with no oil (1)</t>
         </is>
       </c>
       <c r="B44" s="7" t="n">
-        <v>25</v>
+        <v>70</v>
       </c>
       <c r="C44" s="7" t="n">
-        <v>30</v>
+        <v>78</v>
       </c>
       <c r="D44" s="8">
         <f>AVERAGE(B44:C44)</f>
@@ -6733,26 +6733,26 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>~1.5 g</t>
+          <t>~6-6.5 g</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t>Volume with almost no calories</t>
+          <t>Same as boiled - dry-frying saves the ~20-25 kcal per egg that pan oil adds</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Sweet melon / cantaloupe (1 wedge ~100-150 g)</t>
+          <t>Paneer (50 g full-fat)</t>
         </is>
       </c>
       <c r="B45" s="7" t="n">
-        <v>35</v>
+        <v>130</v>
       </c>
       <c r="C45" s="7" t="n">
-        <v>55</v>
+        <v>150</v>
       </c>
       <c r="D45" s="8">
         <f>AVERAGE(B45:C45)</f>
@@ -6760,26 +6760,26 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>~0.5-1 g</t>
+          <t>~8-9 g</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
         <is>
-          <t>Whole fruit - fibre and water intact; ~1/4 the calories of the same fruit juiced</t>
+          <t>Fat-dense for the protein it gives</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>Grapes (~100 g / 15-20 grapes)</t>
+          <t>Cucumber (1 medium)</t>
         </is>
       </c>
       <c r="B46" s="7" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="C46" s="7" t="n">
-        <v>75</v>
+        <v>30</v>
       </c>
       <c r="D46" s="8">
         <f>AVERAGE(B46:C46)</f>
@@ -6787,26 +6787,26 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>~0.6 g</t>
+          <t>~1.5 g</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>Twice the calorie density of melon; easy to eat a large handful without noticing</t>
+          <t>Volume with almost no calories</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>Mango misiri (1 whole ~450-600 g)</t>
+          <t>Sweet melon / cantaloupe (1 wedge ~100-150 g)</t>
         </is>
       </c>
       <c r="B47" s="7" t="n">
-        <v>170</v>
+        <v>35</v>
       </c>
       <c r="C47" s="7" t="n">
-        <v>230</v>
+        <v>55</v>
       </c>
       <c r="D47" s="8">
         <f>AVERAGE(B47:C47)</f>
@@ -6814,26 +6814,26 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>~2-2.5 g</t>
+          <t>~0.5-1 g</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr">
         <is>
-          <t>~60-65% is edible flesh; ~35-50 g sugar but fibre intact</t>
+          <t>Whole fruit - fibre and water intact; ~1/4 the calories of the same fruit juiced</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>Diet/zero-sugar soft drink (330 ml)</t>
+          <t>Grapes (~100 g / 15-20 grapes)</t>
         </is>
       </c>
       <c r="B48" s="7" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="C48" s="7" t="n">
-        <v>2</v>
+        <v>75</v>
       </c>
       <c r="D48" s="8">
         <f>AVERAGE(B48:C48)</f>
@@ -6841,26 +6841,26 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>0 g</t>
+          <t>~0.6 g</t>
         </is>
       </c>
       <c r="F48" s="6" t="inlineStr">
         <is>
-          <t>Genuinely zero - unlike fruit juice sold as no added sugar</t>
+          <t>Twice the calorie density of melon; easy to eat a large handful without noticing</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>Whey scoop (in black coffee no sugar)</t>
+          <t>Mango misiri (1 whole ~450-600 g)</t>
         </is>
       </c>
       <c r="B49" s="7" t="n">
-        <v>100</v>
+        <v>170</v>
       </c>
       <c r="C49" s="7" t="n">
-        <v>130</v>
+        <v>230</v>
       </c>
       <c r="D49" s="8">
         <f>AVERAGE(B49:C49)</f>
@@ -6868,22 +6868,26 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>~20-25 g</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="inlineStr"/>
+          <t>~2-2.5 g</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>~60-65% is edible flesh; ~35-50 g sugar but fibre intact</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>Cashew/almond biscuit (1)</t>
+          <t>Diet/zero-sugar soft drink (330 ml)</t>
         </is>
       </c>
       <c r="B50" s="7" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="C50" s="7" t="n">
-        <v>38</v>
+        <v>2</v>
       </c>
       <c r="D50" s="8">
         <f>AVERAGE(B50:C50)</f>
@@ -6891,22 +6895,26 @@
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>~0.5 g</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="inlineStr"/>
+          <t>0 g</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>Genuinely zero - unlike fruit juice sold as no added sugar</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (~50g standard)</t>
+          <t>Whey scoop (in black coffee no sugar)</t>
         </is>
       </c>
       <c r="B51" s="7" t="n">
-        <v>245</v>
+        <v>100</v>
       </c>
       <c r="C51" s="7" t="n">
-        <v>250</v>
+        <v>130</v>
       </c>
       <c r="D51" s="8">
         <f>AVERAGE(B51:C51)</f>
@@ -6914,7 +6922,7 @@
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>~4 g</t>
+          <t>~20-25 g</t>
         </is>
       </c>
       <c r="F51" s="6" t="inlineStr"/>
@@ -6922,14 +6930,14 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>Chocolate bar (70g king-size)</t>
+          <t>Cashew/almond biscuit (1)</t>
         </is>
       </c>
       <c r="B52" s="7" t="n">
-        <v>335</v>
+        <v>38</v>
       </c>
       <c r="C52" s="7" t="n">
-        <v>335</v>
+        <v>38</v>
       </c>
       <c r="D52" s="8">
         <f>AVERAGE(B52:C52)</f>
@@ -6937,7 +6945,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>~6 g</t>
+          <t>~0.5 g</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr"/>
@@ -6945,14 +6953,14 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>Pre-workout scoop</t>
+          <t>Chocolate bar (~50g standard)</t>
         </is>
       </c>
       <c r="B53" s="7" t="n">
-        <v>5</v>
+        <v>245</v>
       </c>
       <c r="C53" s="7" t="n">
-        <v>15</v>
+        <v>250</v>
       </c>
       <c r="D53" s="8">
         <f>AVERAGE(B53:C53)</f>
@@ -6960,10 +6968,56 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
+          <t>~4 g</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>Chocolate bar (70g king-size)</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="n">
+        <v>335</v>
+      </c>
+      <c r="C54" s="7" t="n">
+        <v>335</v>
+      </c>
+      <c r="D54" s="8">
+        <f>AVERAGE(B54:C54)</f>
+        <v/>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>~6 g</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>Pre-workout scoop</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C55" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="D55" s="8">
+        <f>AVERAGE(B55:C55)</f>
+        <v/>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
           <t>0 g</t>
         </is>
       </c>
-      <c r="F53" s="6" t="inlineStr">
+      <c r="F55" s="6" t="inlineStr">
         <is>
           <t>Negligible</t>
         </is>

</xml_diff>